<commit_message>
Publish site from 37850bd
</commit_message>
<xml_diff>
--- a/einnahmenueberschussrechnung/euer-vorlage-2026-firmendo.xlsx
+++ b/einnahmenueberschussrechnung/euer-vorlage-2026-firmendo.xlsx
@@ -518,7 +518,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="30">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -613,6 +613,30 @@
     </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -917,9 +941,11 @@
         <v>7</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B10" s="3" t="s">
-        <v>8</v>
+    <row r="10" customFormat="false" ht="42" hidden="false" customHeight="1" outlineLevel="0" collapsed="false">
+      <c r="B10" s="24" t="inlineStr">
+        <is>
+          <t>• Beispiele leeren: Kleinunternehmer A8:G10; Regelbesteuert A8:G11 und J8:J11. Nur Eingaben löschen, niemals ganze Zeilen, Formeln oder die Auswertung rechts.</t>
+        </is>
       </c>
     </row>
     <row r="11" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -952,9 +978,11 @@
         <v>14</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="3" t="s">
-        <v>15</v>
+    <row r="17" customFormat="false" ht="68" hidden="false" customHeight="1" outlineLevel="0" collapsed="false">
+      <c r="B17" s="24" t="inlineStr">
+        <is>
+          <t>• AfA: Nur den Jahresbetrag als „Abschreibung (AfA)“ erfassen, USt-Satz 0 %. Bei Regelbesteuerung die bezahlte, abziehbare Vorsteuer der Anschaffung separat als Ausgabe „Vorsteuer auf Anlagevermögen“ in F eintragen, ebenfalls mit 0 %. Beispiel: Kauf 3.000 € netto + 570 € USt, Jahres-AfA 300 € → zwei Einträge: 300 € AfA und 570 € Vorsteuer. In Folgejahren nur AfA, keine erneute Vorsteuer ohne neue Zahlung. GWG bis 800 € netto bleiben sofort abziehbar.</t>
+        </is>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -967,9 +995,11 @@
         <v>17</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B20" s="3" t="s">
-        <v>18</v>
+    <row r="20" customFormat="false" ht="44" hidden="false" customHeight="1" outlineLevel="0" collapsed="false">
+      <c r="B20" s="24" t="inlineStr">
+        <is>
+          <t>• Geldentnahmen und Einlagen verändern den Gewinn nicht und werden hier nicht mitgerechnet. Für die ergänzenden Angaben der Anlage EÜR gesondert aufzeichnen (Anlage EÜR 2025: Zeilen 106/107).</t>
+        </is>
       </c>
     </row>
     <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -992,8 +1022,13 @@
         <v>22</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B25" s="3"/>
+    <row r="25" customFormat="false" ht="44" hidden="false" customHeight="1" outlineLevel="0" collapsed="false">
+      <c r="B25" s="24" t="inlineStr">
+        <is>
+          <t>Quellen: https://www.elster.de/elsterweb/helpGlobal?themaGlobal=help_euer_ufa_77_2025
+https://www.gesetze-im-internet.de/estg/__4.html · geprüft am 07.10.2026</t>
+        </is>
+      </c>
     </row>
     <row r="26" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="2" t="s">
@@ -1050,8 +1085,10 @@
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="6" t="s">
-        <v>27</v>
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>Nur gelbe Beispiel-Eingaben A8:G10 leeren. Ganze Zeilen und die Auswertung I/J erhalten.</t>
+        </is>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5868,8 +5905,10 @@
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="6" t="s">
-        <v>27</v>
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>Nur gelbe Beispiel-Eingaben A8:G11 und J8:J11 leeren. Ganze Zeilen, H/I und Auswertung L/M erhalten.</t>
+        </is>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5877,7 +5916,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
         <v>29</v>
       </c>
@@ -5893,17 +5932,21 @@
       <c r="E7" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="F7" s="9" t="s">
-        <v>74</v>
-      </c>
-      <c r="G7" s="9" t="s">
+      <c r="F7" s="25" t="inlineStr">
+        <is>
+          <t>Netto / Sonderbetrag (€)</t>
+        </is>
+      </c>
+      <c r="G7" s="25" t="s">
         <v>75</v>
       </c>
-      <c r="H7" s="9" t="s">
+      <c r="H7" s="25" t="s">
         <v>76</v>
       </c>
-      <c r="I7" s="9" t="s">
-        <v>77</v>
+      <c r="I7" s="25" t="inlineStr">
+        <is>
+          <t>Betrag inkl. USt (€)</t>
+        </is>
       </c>
       <c r="J7" s="9" t="s">
         <v>35</v>
@@ -5938,7 +5981,7 @@
         <v>0.19</v>
       </c>
       <c r="H8" s="22" t="n">
-        <f aca="false">IF(F8="","",ROUND(F8*G8,2))</f>
+        <f>IF(F8="","",IF(OR(E8="Abschreibung (AfA)",E8="Vorsteuer auf Anlagevermögen"),0,ROUND(F8*G8,2)))</f>
         <v>380</v>
       </c>
       <c r="I8" s="22" t="n">
@@ -5953,38 +5996,40 @@
       </c>
       <c r="M8" s="15"/>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="32" hidden="false" customHeight="1" outlineLevel="0" collapsed="false">
       <c r="A9" s="11" t="n">
         <v>46042</v>
       </c>
       <c r="B9" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="C9" s="12" t="s">
+      <c r="C9" s="26" t="s">
         <v>79</v>
       </c>
-      <c r="D9" s="12" t="s">
+      <c r="D9" s="26" t="s">
         <v>46</v>
       </c>
-      <c r="E9" s="12" t="s">
+      <c r="E9" s="26" t="s">
         <v>63</v>
       </c>
-      <c r="F9" s="13" t="n">
+      <c r="F9" s="27" t="n">
         <v>1100</v>
       </c>
-      <c r="G9" s="21" t="n">
-        <v>0.19</v>
-      </c>
-      <c r="H9" s="22" t="n">
-        <f aca="false">IF(F9="","",ROUND(F9*G9,2))</f>
-        <v>209</v>
-      </c>
-      <c r="I9" s="22" t="n">
+      <c r="G9" s="28">
+        <v>0</v>
+      </c>
+      <c r="H9" s="29" t="n">
+        <f>IF(F9="","",IF(OR(E9="Abschreibung (AfA)",E9="Vorsteuer auf Anlagevermögen"),0,ROUND(F9*G9,2)))</f>
+        <v>0</v>
+      </c>
+      <c r="I9" s="29" t="n">
         <f aca="false">IF(F9="","",F9+H9)</f>
         <v>1309</v>
       </c>
-      <c r="J9" s="12" t="s">
-        <v>42</v>
+      <c r="J9" s="26" t="inlineStr">
+        <is>
+          <t>AfA; Vorsteuer separat in Zeile 11</t>
+        </is>
       </c>
       <c r="L9" s="16" t="s">
         <v>80</v>
@@ -5994,37 +6039,37 @@
         <v>2000</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="32" hidden="false" customHeight="1" outlineLevel="0" collapsed="false">
       <c r="A10" s="11" t="n">
         <v>46063</v>
       </c>
       <c r="B10" s="12" t="s">
         <v>81</v>
       </c>
-      <c r="C10" s="12" t="s">
+      <c r="C10" s="26" t="s">
         <v>82</v>
       </c>
-      <c r="D10" s="12" t="s">
+      <c r="D10" s="26" t="s">
         <v>46</v>
       </c>
-      <c r="E10" s="12" t="s">
+      <c r="E10" s="26" t="s">
         <v>83</v>
       </c>
-      <c r="F10" s="13" t="n">
+      <c r="F10" s="27" t="n">
         <v>171</v>
       </c>
-      <c r="G10" s="21" t="n">
+      <c r="G10" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="H10" s="22" t="n">
-        <f aca="false">IF(F10="","",ROUND(F10*G10,2))</f>
+      <c r="H10" s="29" t="n">
+        <f>IF(F10="","",IF(OR(E10="Abschreibung (AfA)",E10="Vorsteuer auf Anlagevermögen"),0,ROUND(F10*G10,2)))</f>
         <v>0</v>
       </c>
-      <c r="I10" s="22" t="n">
+      <c r="I10" s="29" t="n">
         <f aca="false">IF(F10="","",F10+H10)</f>
         <v>171</v>
       </c>
-      <c r="J10" s="12" t="s">
+      <c r="J10" s="26" t="s">
         <v>42</v>
       </c>
       <c r="L10" s="16" t="s">
@@ -6035,23 +6080,49 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="11"/>
-      <c r="B11" s="12"/>
-      <c r="C11" s="12"/>
-      <c r="D11" s="12"/>
-      <c r="E11" s="12"/>
-      <c r="F11" s="13"/>
-      <c r="G11" s="21"/>
-      <c r="H11" s="22" t="str">
-        <f aca="false">IF(F11="","",ROUND(F11*G11,2))</f>
-        <v/>
-      </c>
-      <c r="I11" s="22" t="str">
+    <row r="11" customFormat="false" ht="32" hidden="false" customHeight="1" outlineLevel="0" collapsed="false">
+      <c r="A11" s="11">
+        <v>46042</v>
+      </c>
+      <c r="B11" s="12" t="inlineStr">
+        <is>
+          <t>E-001</t>
+        </is>
+      </c>
+      <c r="C11" s="26" t="inlineStr">
+        <is>
+          <t>Vorsteuer aus Laptop-Kauf</t>
+        </is>
+      </c>
+      <c r="D11" s="26" t="inlineStr">
+        <is>
+          <t>Ausgabe</t>
+        </is>
+      </c>
+      <c r="E11" s="26" t="inlineStr">
+        <is>
+          <t>Vorsteuer auf Anlagevermögen</t>
+        </is>
+      </c>
+      <c r="F11" s="27">
+        <v>209</v>
+      </c>
+      <c r="G11" s="28">
+        <v>0</v>
+      </c>
+      <c r="H11" s="29" t="n">
+        <f>IF(F11="","",IF(OR(E11="Abschreibung (AfA)",E11="Vorsteuer auf Anlagevermögen"),0,ROUND(F11*G11,2)))</f>
+        <v>0</v>
+      </c>
+      <c r="I11" s="29" t="n">
         <f aca="false">IF(F11="","",F11+H11)</f>
-        <v/>
-      </c>
-      <c r="J11" s="12"/>
+        <v>209</v>
+      </c>
+      <c r="J11" s="26" t="inlineStr">
+        <is>
+          <t>Beispiel – Eingaben löschen</t>
+        </is>
+      </c>
       <c r="L11" s="16" t="s">
         <v>85</v>
       </c>
@@ -6069,7 +6140,7 @@
       <c r="F12" s="13"/>
       <c r="G12" s="21"/>
       <c r="H12" s="22" t="str">
-        <f aca="false">IF(F12="","",ROUND(F12*G12,2))</f>
+        <f>IF(F12="","",IF(OR(E12="Abschreibung (AfA)",E12="Vorsteuer auf Anlagevermögen"),0,ROUND(F12*G12,2)))</f>
         <v/>
       </c>
       <c r="I12" s="22" t="str">
@@ -6094,7 +6165,7 @@
       <c r="F13" s="13"/>
       <c r="G13" s="21"/>
       <c r="H13" s="22" t="str">
-        <f aca="false">IF(F13="","",ROUND(F13*G13,2))</f>
+        <f>IF(F13="","",IF(OR(E13="Abschreibung (AfA)",E13="Vorsteuer auf Anlagevermögen"),0,ROUND(F13*G13,2)))</f>
         <v/>
       </c>
       <c r="I13" s="22" t="str">
@@ -6119,7 +6190,7 @@
       <c r="F14" s="13"/>
       <c r="G14" s="21"/>
       <c r="H14" s="22" t="str">
-        <f aca="false">IF(F14="","",ROUND(F14*G14,2))</f>
+        <f>IF(F14="","",IF(OR(E14="Abschreibung (AfA)",E14="Vorsteuer auf Anlagevermögen"),0,ROUND(F14*G14,2)))</f>
         <v/>
       </c>
       <c r="I14" s="22" t="str">
@@ -6139,7 +6210,7 @@
       <c r="F15" s="13"/>
       <c r="G15" s="21"/>
       <c r="H15" s="22" t="str">
-        <f aca="false">IF(F15="","",ROUND(F15*G15,2))</f>
+        <f>IF(F15="","",IF(OR(E15="Abschreibung (AfA)",E15="Vorsteuer auf Anlagevermögen"),0,ROUND(F15*G15,2)))</f>
         <v/>
       </c>
       <c r="I15" s="22" t="str">
@@ -6161,7 +6232,7 @@
       <c r="F16" s="13"/>
       <c r="G16" s="21"/>
       <c r="H16" s="22" t="str">
-        <f aca="false">IF(F16="","",ROUND(F16*G16,2))</f>
+        <f>IF(F16="","",IF(OR(E16="Abschreibung (AfA)",E16="Vorsteuer auf Anlagevermögen"),0,ROUND(F16*G16,2)))</f>
         <v/>
       </c>
       <c r="I16" s="22" t="str">
@@ -6186,7 +6257,7 @@
       <c r="F17" s="13"/>
       <c r="G17" s="21"/>
       <c r="H17" s="22" t="str">
-        <f aca="false">IF(F17="","",ROUND(F17*G17,2))</f>
+        <f>IF(F17="","",IF(OR(E17="Abschreibung (AfA)",E17="Vorsteuer auf Anlagevermögen"),0,ROUND(F17*G17,2)))</f>
         <v/>
       </c>
       <c r="I17" s="22" t="str">
@@ -6211,7 +6282,7 @@
       <c r="F18" s="13"/>
       <c r="G18" s="21"/>
       <c r="H18" s="22" t="str">
-        <f aca="false">IF(F18="","",ROUND(F18*G18,2))</f>
+        <f>IF(F18="","",IF(OR(E18="Abschreibung (AfA)",E18="Vorsteuer auf Anlagevermögen"),0,ROUND(F18*G18,2)))</f>
         <v/>
       </c>
       <c r="I18" s="22" t="str">
@@ -6236,7 +6307,7 @@
       <c r="F19" s="13"/>
       <c r="G19" s="21"/>
       <c r="H19" s="22" t="str">
-        <f aca="false">IF(F19="","",ROUND(F19*G19,2))</f>
+        <f>IF(F19="","",IF(OR(E19="Abschreibung (AfA)",E19="Vorsteuer auf Anlagevermögen"),0,ROUND(F19*G19,2)))</f>
         <v/>
       </c>
       <c r="I19" s="22" t="str">
@@ -6261,7 +6332,7 @@
       <c r="F20" s="13"/>
       <c r="G20" s="21"/>
       <c r="H20" s="22" t="str">
-        <f aca="false">IF(F20="","",ROUND(F20*G20,2))</f>
+        <f>IF(F20="","",IF(OR(E20="Abschreibung (AfA)",E20="Vorsteuer auf Anlagevermögen"),0,ROUND(F20*G20,2)))</f>
         <v/>
       </c>
       <c r="I20" s="22" t="str">
@@ -6286,7 +6357,7 @@
       <c r="F21" s="13"/>
       <c r="G21" s="21"/>
       <c r="H21" s="22" t="str">
-        <f aca="false">IF(F21="","",ROUND(F21*G21,2))</f>
+        <f>IF(F21="","",IF(OR(E21="Abschreibung (AfA)",E21="Vorsteuer auf Anlagevermögen"),0,ROUND(F21*G21,2)))</f>
         <v/>
       </c>
       <c r="I21" s="22" t="str">
@@ -6311,7 +6382,7 @@
       <c r="F22" s="13"/>
       <c r="G22" s="21"/>
       <c r="H22" s="22" t="str">
-        <f aca="false">IF(F22="","",ROUND(F22*G22,2))</f>
+        <f>IF(F22="","",IF(OR(E22="Abschreibung (AfA)",E22="Vorsteuer auf Anlagevermögen"),0,ROUND(F22*G22,2)))</f>
         <v/>
       </c>
       <c r="I22" s="22" t="str">
@@ -6336,7 +6407,7 @@
       <c r="F23" s="13"/>
       <c r="G23" s="21"/>
       <c r="H23" s="22" t="str">
-        <f aca="false">IF(F23="","",ROUND(F23*G23,2))</f>
+        <f>IF(F23="","",IF(OR(E23="Abschreibung (AfA)",E23="Vorsteuer auf Anlagevermögen"),0,ROUND(F23*G23,2)))</f>
         <v/>
       </c>
       <c r="I23" s="22" t="str">
@@ -6361,7 +6432,7 @@
       <c r="F24" s="13"/>
       <c r="G24" s="21"/>
       <c r="H24" s="22" t="str">
-        <f aca="false">IF(F24="","",ROUND(F24*G24,2))</f>
+        <f>IF(F24="","",IF(OR(E24="Abschreibung (AfA)",E24="Vorsteuer auf Anlagevermögen"),0,ROUND(F24*G24,2)))</f>
         <v/>
       </c>
       <c r="I24" s="22" t="str">
@@ -6386,7 +6457,7 @@
       <c r="F25" s="13"/>
       <c r="G25" s="21"/>
       <c r="H25" s="22" t="str">
-        <f aca="false">IF(F25="","",ROUND(F25*G25,2))</f>
+        <f>IF(F25="","",IF(OR(E25="Abschreibung (AfA)",E25="Vorsteuer auf Anlagevermögen"),0,ROUND(F25*G25,2)))</f>
         <v/>
       </c>
       <c r="I25" s="22" t="str">
@@ -6411,7 +6482,7 @@
       <c r="F26" s="13"/>
       <c r="G26" s="21"/>
       <c r="H26" s="22" t="str">
-        <f aca="false">IF(F26="","",ROUND(F26*G26,2))</f>
+        <f>IF(F26="","",IF(OR(E26="Abschreibung (AfA)",E26="Vorsteuer auf Anlagevermögen"),0,ROUND(F26*G26,2)))</f>
         <v/>
       </c>
       <c r="I26" s="22" t="str">
@@ -6436,7 +6507,7 @@
       <c r="F27" s="13"/>
       <c r="G27" s="21"/>
       <c r="H27" s="22" t="str">
-        <f aca="false">IF(F27="","",ROUND(F27*G27,2))</f>
+        <f>IF(F27="","",IF(OR(E27="Abschreibung (AfA)",E27="Vorsteuer auf Anlagevermögen"),0,ROUND(F27*G27,2)))</f>
         <v/>
       </c>
       <c r="I27" s="22" t="str">
@@ -6461,7 +6532,7 @@
       <c r="F28" s="13"/>
       <c r="G28" s="21"/>
       <c r="H28" s="22" t="str">
-        <f aca="false">IF(F28="","",ROUND(F28*G28,2))</f>
+        <f>IF(F28="","",IF(OR(E28="Abschreibung (AfA)",E28="Vorsteuer auf Anlagevermögen"),0,ROUND(F28*G28,2)))</f>
         <v/>
       </c>
       <c r="I28" s="22" t="str">
@@ -6486,7 +6557,7 @@
       <c r="F29" s="13"/>
       <c r="G29" s="21"/>
       <c r="H29" s="22" t="str">
-        <f aca="false">IF(F29="","",ROUND(F29*G29,2))</f>
+        <f>IF(F29="","",IF(OR(E29="Abschreibung (AfA)",E29="Vorsteuer auf Anlagevermögen"),0,ROUND(F29*G29,2)))</f>
         <v/>
       </c>
       <c r="I29" s="22" t="str">
@@ -6511,7 +6582,7 @@
       <c r="F30" s="13"/>
       <c r="G30" s="21"/>
       <c r="H30" s="22" t="str">
-        <f aca="false">IF(F30="","",ROUND(F30*G30,2))</f>
+        <f>IF(F30="","",IF(OR(E30="Abschreibung (AfA)",E30="Vorsteuer auf Anlagevermögen"),0,ROUND(F30*G30,2)))</f>
         <v/>
       </c>
       <c r="I30" s="22" t="str">
@@ -6536,7 +6607,7 @@
       <c r="F31" s="13"/>
       <c r="G31" s="21"/>
       <c r="H31" s="22" t="str">
-        <f aca="false">IF(F31="","",ROUND(F31*G31,2))</f>
+        <f>IF(F31="","",IF(OR(E31="Abschreibung (AfA)",E31="Vorsteuer auf Anlagevermögen"),0,ROUND(F31*G31,2)))</f>
         <v/>
       </c>
       <c r="I31" s="22" t="str">
@@ -6548,7 +6619,7 @@
         <v>101</v>
       </c>
       <c r="M31" s="15" t="n">
-        <f aca="false">SUMIFS($H$8:$H$507,$D$8:$D$507,"Ausgabe")</f>
+        <f>SUMIFS($H$8:$H$507,$D$8:$D$507,"Ausgabe")+SUMIFS($F$8:$F$507,$D$8:$D$507,"Ausgabe",$E$8:$E$507,"Vorsteuer auf Anlagevermögen")</f>
         <v>209</v>
       </c>
     </row>
@@ -6561,7 +6632,7 @@
       <c r="F32" s="13"/>
       <c r="G32" s="21"/>
       <c r="H32" s="22" t="str">
-        <f aca="false">IF(F32="","",ROUND(F32*G32,2))</f>
+        <f>IF(F32="","",IF(OR(E32="Abschreibung (AfA)",E32="Vorsteuer auf Anlagevermögen"),0,ROUND(F32*G32,2)))</f>
         <v/>
       </c>
       <c r="I32" s="22" t="str">
@@ -6586,7 +6657,7 @@
       <c r="F33" s="13"/>
       <c r="G33" s="21"/>
       <c r="H33" s="22" t="str">
-        <f aca="false">IF(F33="","",ROUND(F33*G33,2))</f>
+        <f>IF(F33="","",IF(OR(E33="Abschreibung (AfA)",E33="Vorsteuer auf Anlagevermögen"),0,ROUND(F33*G33,2)))</f>
         <v/>
       </c>
       <c r="I33" s="22" t="str">
@@ -6611,7 +6682,7 @@
       <c r="F34" s="13"/>
       <c r="G34" s="21"/>
       <c r="H34" s="22" t="str">
-        <f aca="false">IF(F34="","",ROUND(F34*G34,2))</f>
+        <f>IF(F34="","",IF(OR(E34="Abschreibung (AfA)",E34="Vorsteuer auf Anlagevermögen"),0,ROUND(F34*G34,2)))</f>
         <v/>
       </c>
       <c r="I34" s="22" t="str">
@@ -6636,7 +6707,7 @@
       <c r="F35" s="13"/>
       <c r="G35" s="21"/>
       <c r="H35" s="22" t="str">
-        <f aca="false">IF(F35="","",ROUND(F35*G35,2))</f>
+        <f>IF(F35="","",IF(OR(E35="Abschreibung (AfA)",E35="Vorsteuer auf Anlagevermögen"),0,ROUND(F35*G35,2)))</f>
         <v/>
       </c>
       <c r="I35" s="22" t="str">
@@ -6656,7 +6727,7 @@
       <c r="F36" s="13"/>
       <c r="G36" s="21"/>
       <c r="H36" s="22" t="str">
-        <f aca="false">IF(F36="","",ROUND(F36*G36,2))</f>
+        <f>IF(F36="","",IF(OR(E36="Abschreibung (AfA)",E36="Vorsteuer auf Anlagevermögen"),0,ROUND(F36*G36,2)))</f>
         <v/>
       </c>
       <c r="I36" s="22" t="str">
@@ -6681,7 +6752,7 @@
       <c r="F37" s="13"/>
       <c r="G37" s="21"/>
       <c r="H37" s="22" t="str">
-        <f aca="false">IF(F37="","",ROUND(F37*G37,2))</f>
+        <f>IF(F37="","",IF(OR(E37="Abschreibung (AfA)",E37="Vorsteuer auf Anlagevermögen"),0,ROUND(F37*G37,2)))</f>
         <v/>
       </c>
       <c r="I37" s="22" t="str">
@@ -6701,7 +6772,7 @@
       <c r="F38" s="13"/>
       <c r="G38" s="21"/>
       <c r="H38" s="22" t="str">
-        <f aca="false">IF(F38="","",ROUND(F38*G38,2))</f>
+        <f>IF(F38="","",IF(OR(E38="Abschreibung (AfA)",E38="Vorsteuer auf Anlagevermögen"),0,ROUND(F38*G38,2)))</f>
         <v/>
       </c>
       <c r="I38" s="22" t="str">
@@ -6726,7 +6797,7 @@
       <c r="F39" s="13"/>
       <c r="G39" s="21"/>
       <c r="H39" s="22" t="str">
-        <f aca="false">IF(F39="","",ROUND(F39*G39,2))</f>
+        <f>IF(F39="","",IF(OR(E39="Abschreibung (AfA)",E39="Vorsteuer auf Anlagevermögen"),0,ROUND(F39*G39,2)))</f>
         <v/>
       </c>
       <c r="I39" s="22" t="str">
@@ -6744,7 +6815,7 @@
       <c r="F40" s="13"/>
       <c r="G40" s="21"/>
       <c r="H40" s="22" t="str">
-        <f aca="false">IF(F40="","",ROUND(F40*G40,2))</f>
+        <f>IF(F40="","",IF(OR(E40="Abschreibung (AfA)",E40="Vorsteuer auf Anlagevermögen"),0,ROUND(F40*G40,2)))</f>
         <v/>
       </c>
       <c r="I40" s="22" t="str">
@@ -6762,7 +6833,7 @@
       <c r="F41" s="13"/>
       <c r="G41" s="21"/>
       <c r="H41" s="22" t="str">
-        <f aca="false">IF(F41="","",ROUND(F41*G41,2))</f>
+        <f>IF(F41="","",IF(OR(E41="Abschreibung (AfA)",E41="Vorsteuer auf Anlagevermögen"),0,ROUND(F41*G41,2)))</f>
         <v/>
       </c>
       <c r="I41" s="22" t="str">
@@ -6780,7 +6851,7 @@
       <c r="F42" s="13"/>
       <c r="G42" s="21"/>
       <c r="H42" s="22" t="str">
-        <f aca="false">IF(F42="","",ROUND(F42*G42,2))</f>
+        <f>IF(F42="","",IF(OR(E42="Abschreibung (AfA)",E42="Vorsteuer auf Anlagevermögen"),0,ROUND(F42*G42,2)))</f>
         <v/>
       </c>
       <c r="I42" s="22" t="str">
@@ -6798,7 +6869,7 @@
       <c r="F43" s="13"/>
       <c r="G43" s="21"/>
       <c r="H43" s="22" t="str">
-        <f aca="false">IF(F43="","",ROUND(F43*G43,2))</f>
+        <f>IF(F43="","",IF(OR(E43="Abschreibung (AfA)",E43="Vorsteuer auf Anlagevermögen"),0,ROUND(F43*G43,2)))</f>
         <v/>
       </c>
       <c r="I43" s="22" t="str">
@@ -6816,7 +6887,7 @@
       <c r="F44" s="13"/>
       <c r="G44" s="21"/>
       <c r="H44" s="22" t="str">
-        <f aca="false">IF(F44="","",ROUND(F44*G44,2))</f>
+        <f>IF(F44="","",IF(OR(E44="Abschreibung (AfA)",E44="Vorsteuer auf Anlagevermögen"),0,ROUND(F44*G44,2)))</f>
         <v/>
       </c>
       <c r="I44" s="22" t="str">
@@ -6834,7 +6905,7 @@
       <c r="F45" s="13"/>
       <c r="G45" s="21"/>
       <c r="H45" s="22" t="str">
-        <f aca="false">IF(F45="","",ROUND(F45*G45,2))</f>
+        <f>IF(F45="","",IF(OR(E45="Abschreibung (AfA)",E45="Vorsteuer auf Anlagevermögen"),0,ROUND(F45*G45,2)))</f>
         <v/>
       </c>
       <c r="I45" s="22" t="str">
@@ -6852,7 +6923,7 @@
       <c r="F46" s="13"/>
       <c r="G46" s="21"/>
       <c r="H46" s="22" t="str">
-        <f aca="false">IF(F46="","",ROUND(F46*G46,2))</f>
+        <f>IF(F46="","",IF(OR(E46="Abschreibung (AfA)",E46="Vorsteuer auf Anlagevermögen"),0,ROUND(F46*G46,2)))</f>
         <v/>
       </c>
       <c r="I46" s="22" t="str">
@@ -6870,7 +6941,7 @@
       <c r="F47" s="13"/>
       <c r="G47" s="21"/>
       <c r="H47" s="22" t="str">
-        <f aca="false">IF(F47="","",ROUND(F47*G47,2))</f>
+        <f>IF(F47="","",IF(OR(E47="Abschreibung (AfA)",E47="Vorsteuer auf Anlagevermögen"),0,ROUND(F47*G47,2)))</f>
         <v/>
       </c>
       <c r="I47" s="22" t="str">
@@ -6888,7 +6959,7 @@
       <c r="F48" s="13"/>
       <c r="G48" s="21"/>
       <c r="H48" s="22" t="str">
-        <f aca="false">IF(F48="","",ROUND(F48*G48,2))</f>
+        <f>IF(F48="","",IF(OR(E48="Abschreibung (AfA)",E48="Vorsteuer auf Anlagevermögen"),0,ROUND(F48*G48,2)))</f>
         <v/>
       </c>
       <c r="I48" s="22" t="str">
@@ -6906,7 +6977,7 @@
       <c r="F49" s="13"/>
       <c r="G49" s="21"/>
       <c r="H49" s="22" t="str">
-        <f aca="false">IF(F49="","",ROUND(F49*G49,2))</f>
+        <f>IF(F49="","",IF(OR(E49="Abschreibung (AfA)",E49="Vorsteuer auf Anlagevermögen"),0,ROUND(F49*G49,2)))</f>
         <v/>
       </c>
       <c r="I49" s="22" t="str">
@@ -6924,7 +6995,7 @@
       <c r="F50" s="13"/>
       <c r="G50" s="21"/>
       <c r="H50" s="22" t="str">
-        <f aca="false">IF(F50="","",ROUND(F50*G50,2))</f>
+        <f>IF(F50="","",IF(OR(E50="Abschreibung (AfA)",E50="Vorsteuer auf Anlagevermögen"),0,ROUND(F50*G50,2)))</f>
         <v/>
       </c>
       <c r="I50" s="22" t="str">
@@ -6942,7 +7013,7 @@
       <c r="F51" s="13"/>
       <c r="G51" s="21"/>
       <c r="H51" s="22" t="str">
-        <f aca="false">IF(F51="","",ROUND(F51*G51,2))</f>
+        <f>IF(F51="","",IF(OR(E51="Abschreibung (AfA)",E51="Vorsteuer auf Anlagevermögen"),0,ROUND(F51*G51,2)))</f>
         <v/>
       </c>
       <c r="I51" s="22" t="str">
@@ -6960,7 +7031,7 @@
       <c r="F52" s="13"/>
       <c r="G52" s="21"/>
       <c r="H52" s="22" t="str">
-        <f aca="false">IF(F52="","",ROUND(F52*G52,2))</f>
+        <f>IF(F52="","",IF(OR(E52="Abschreibung (AfA)",E52="Vorsteuer auf Anlagevermögen"),0,ROUND(F52*G52,2)))</f>
         <v/>
       </c>
       <c r="I52" s="22" t="str">
@@ -6978,7 +7049,7 @@
       <c r="F53" s="13"/>
       <c r="G53" s="21"/>
       <c r="H53" s="22" t="str">
-        <f aca="false">IF(F53="","",ROUND(F53*G53,2))</f>
+        <f>IF(F53="","",IF(OR(E53="Abschreibung (AfA)",E53="Vorsteuer auf Anlagevermögen"),0,ROUND(F53*G53,2)))</f>
         <v/>
       </c>
       <c r="I53" s="22" t="str">
@@ -6996,7 +7067,7 @@
       <c r="F54" s="13"/>
       <c r="G54" s="21"/>
       <c r="H54" s="22" t="str">
-        <f aca="false">IF(F54="","",ROUND(F54*G54,2))</f>
+        <f>IF(F54="","",IF(OR(E54="Abschreibung (AfA)",E54="Vorsteuer auf Anlagevermögen"),0,ROUND(F54*G54,2)))</f>
         <v/>
       </c>
       <c r="I54" s="22" t="str">
@@ -7014,7 +7085,7 @@
       <c r="F55" s="13"/>
       <c r="G55" s="21"/>
       <c r="H55" s="22" t="str">
-        <f aca="false">IF(F55="","",ROUND(F55*G55,2))</f>
+        <f>IF(F55="","",IF(OR(E55="Abschreibung (AfA)",E55="Vorsteuer auf Anlagevermögen"),0,ROUND(F55*G55,2)))</f>
         <v/>
       </c>
       <c r="I55" s="22" t="str">
@@ -7032,7 +7103,7 @@
       <c r="F56" s="13"/>
       <c r="G56" s="21"/>
       <c r="H56" s="22" t="str">
-        <f aca="false">IF(F56="","",ROUND(F56*G56,2))</f>
+        <f>IF(F56="","",IF(OR(E56="Abschreibung (AfA)",E56="Vorsteuer auf Anlagevermögen"),0,ROUND(F56*G56,2)))</f>
         <v/>
       </c>
       <c r="I56" s="22" t="str">
@@ -7050,7 +7121,7 @@
       <c r="F57" s="13"/>
       <c r="G57" s="21"/>
       <c r="H57" s="22" t="str">
-        <f aca="false">IF(F57="","",ROUND(F57*G57,2))</f>
+        <f>IF(F57="","",IF(OR(E57="Abschreibung (AfA)",E57="Vorsteuer auf Anlagevermögen"),0,ROUND(F57*G57,2)))</f>
         <v/>
       </c>
       <c r="I57" s="22" t="str">
@@ -7068,7 +7139,7 @@
       <c r="F58" s="13"/>
       <c r="G58" s="21"/>
       <c r="H58" s="22" t="str">
-        <f aca="false">IF(F58="","",ROUND(F58*G58,2))</f>
+        <f>IF(F58="","",IF(OR(E58="Abschreibung (AfA)",E58="Vorsteuer auf Anlagevermögen"),0,ROUND(F58*G58,2)))</f>
         <v/>
       </c>
       <c r="I58" s="22" t="str">
@@ -7086,7 +7157,7 @@
       <c r="F59" s="13"/>
       <c r="G59" s="21"/>
       <c r="H59" s="22" t="str">
-        <f aca="false">IF(F59="","",ROUND(F59*G59,2))</f>
+        <f>IF(F59="","",IF(OR(E59="Abschreibung (AfA)",E59="Vorsteuer auf Anlagevermögen"),0,ROUND(F59*G59,2)))</f>
         <v/>
       </c>
       <c r="I59" s="22" t="str">
@@ -7104,7 +7175,7 @@
       <c r="F60" s="13"/>
       <c r="G60" s="21"/>
       <c r="H60" s="22" t="str">
-        <f aca="false">IF(F60="","",ROUND(F60*G60,2))</f>
+        <f>IF(F60="","",IF(OR(E60="Abschreibung (AfA)",E60="Vorsteuer auf Anlagevermögen"),0,ROUND(F60*G60,2)))</f>
         <v/>
       </c>
       <c r="I60" s="22" t="str">
@@ -7122,7 +7193,7 @@
       <c r="F61" s="13"/>
       <c r="G61" s="21"/>
       <c r="H61" s="22" t="str">
-        <f aca="false">IF(F61="","",ROUND(F61*G61,2))</f>
+        <f>IF(F61="","",IF(OR(E61="Abschreibung (AfA)",E61="Vorsteuer auf Anlagevermögen"),0,ROUND(F61*G61,2)))</f>
         <v/>
       </c>
       <c r="I61" s="22" t="str">
@@ -7140,7 +7211,7 @@
       <c r="F62" s="13"/>
       <c r="G62" s="21"/>
       <c r="H62" s="22" t="str">
-        <f aca="false">IF(F62="","",ROUND(F62*G62,2))</f>
+        <f>IF(F62="","",IF(OR(E62="Abschreibung (AfA)",E62="Vorsteuer auf Anlagevermögen"),0,ROUND(F62*G62,2)))</f>
         <v/>
       </c>
       <c r="I62" s="22" t="str">
@@ -7158,7 +7229,7 @@
       <c r="F63" s="13"/>
       <c r="G63" s="21"/>
       <c r="H63" s="22" t="str">
-        <f aca="false">IF(F63="","",ROUND(F63*G63,2))</f>
+        <f>IF(F63="","",IF(OR(E63="Abschreibung (AfA)",E63="Vorsteuer auf Anlagevermögen"),0,ROUND(F63*G63,2)))</f>
         <v/>
       </c>
       <c r="I63" s="22" t="str">
@@ -7176,7 +7247,7 @@
       <c r="F64" s="13"/>
       <c r="G64" s="21"/>
       <c r="H64" s="22" t="str">
-        <f aca="false">IF(F64="","",ROUND(F64*G64,2))</f>
+        <f>IF(F64="","",IF(OR(E64="Abschreibung (AfA)",E64="Vorsteuer auf Anlagevermögen"),0,ROUND(F64*G64,2)))</f>
         <v/>
       </c>
       <c r="I64" s="22" t="str">
@@ -7194,7 +7265,7 @@
       <c r="F65" s="13"/>
       <c r="G65" s="21"/>
       <c r="H65" s="22" t="str">
-        <f aca="false">IF(F65="","",ROUND(F65*G65,2))</f>
+        <f>IF(F65="","",IF(OR(E65="Abschreibung (AfA)",E65="Vorsteuer auf Anlagevermögen"),0,ROUND(F65*G65,2)))</f>
         <v/>
       </c>
       <c r="I65" s="22" t="str">
@@ -7212,7 +7283,7 @@
       <c r="F66" s="13"/>
       <c r="G66" s="21"/>
       <c r="H66" s="22" t="str">
-        <f aca="false">IF(F66="","",ROUND(F66*G66,2))</f>
+        <f>IF(F66="","",IF(OR(E66="Abschreibung (AfA)",E66="Vorsteuer auf Anlagevermögen"),0,ROUND(F66*G66,2)))</f>
         <v/>
       </c>
       <c r="I66" s="22" t="str">
@@ -7230,7 +7301,7 @@
       <c r="F67" s="13"/>
       <c r="G67" s="21"/>
       <c r="H67" s="22" t="str">
-        <f aca="false">IF(F67="","",ROUND(F67*G67,2))</f>
+        <f>IF(F67="","",IF(OR(E67="Abschreibung (AfA)",E67="Vorsteuer auf Anlagevermögen"),0,ROUND(F67*G67,2)))</f>
         <v/>
       </c>
       <c r="I67" s="22" t="str">
@@ -7248,7 +7319,7 @@
       <c r="F68" s="13"/>
       <c r="G68" s="21"/>
       <c r="H68" s="22" t="str">
-        <f aca="false">IF(F68="","",ROUND(F68*G68,2))</f>
+        <f>IF(F68="","",IF(OR(E68="Abschreibung (AfA)",E68="Vorsteuer auf Anlagevermögen"),0,ROUND(F68*G68,2)))</f>
         <v/>
       </c>
       <c r="I68" s="22" t="str">
@@ -7266,7 +7337,7 @@
       <c r="F69" s="13"/>
       <c r="G69" s="21"/>
       <c r="H69" s="22" t="str">
-        <f aca="false">IF(F69="","",ROUND(F69*G69,2))</f>
+        <f>IF(F69="","",IF(OR(E69="Abschreibung (AfA)",E69="Vorsteuer auf Anlagevermögen"),0,ROUND(F69*G69,2)))</f>
         <v/>
       </c>
       <c r="I69" s="22" t="str">
@@ -7284,7 +7355,7 @@
       <c r="F70" s="13"/>
       <c r="G70" s="21"/>
       <c r="H70" s="22" t="str">
-        <f aca="false">IF(F70="","",ROUND(F70*G70,2))</f>
+        <f>IF(F70="","",IF(OR(E70="Abschreibung (AfA)",E70="Vorsteuer auf Anlagevermögen"),0,ROUND(F70*G70,2)))</f>
         <v/>
       </c>
       <c r="I70" s="22" t="str">
@@ -7302,7 +7373,7 @@
       <c r="F71" s="13"/>
       <c r="G71" s="21"/>
       <c r="H71" s="22" t="str">
-        <f aca="false">IF(F71="","",ROUND(F71*G71,2))</f>
+        <f>IF(F71="","",IF(OR(E71="Abschreibung (AfA)",E71="Vorsteuer auf Anlagevermögen"),0,ROUND(F71*G71,2)))</f>
         <v/>
       </c>
       <c r="I71" s="22" t="str">
@@ -7320,7 +7391,7 @@
       <c r="F72" s="13"/>
       <c r="G72" s="21"/>
       <c r="H72" s="22" t="str">
-        <f aca="false">IF(F72="","",ROUND(F72*G72,2))</f>
+        <f>IF(F72="","",IF(OR(E72="Abschreibung (AfA)",E72="Vorsteuer auf Anlagevermögen"),0,ROUND(F72*G72,2)))</f>
         <v/>
       </c>
       <c r="I72" s="22" t="str">
@@ -7338,7 +7409,7 @@
       <c r="F73" s="13"/>
       <c r="G73" s="21"/>
       <c r="H73" s="22" t="str">
-        <f aca="false">IF(F73="","",ROUND(F73*G73,2))</f>
+        <f>IF(F73="","",IF(OR(E73="Abschreibung (AfA)",E73="Vorsteuer auf Anlagevermögen"),0,ROUND(F73*G73,2)))</f>
         <v/>
       </c>
       <c r="I73" s="22" t="str">
@@ -7356,7 +7427,7 @@
       <c r="F74" s="13"/>
       <c r="G74" s="21"/>
       <c r="H74" s="22" t="str">
-        <f aca="false">IF(F74="","",ROUND(F74*G74,2))</f>
+        <f>IF(F74="","",IF(OR(E74="Abschreibung (AfA)",E74="Vorsteuer auf Anlagevermögen"),0,ROUND(F74*G74,2)))</f>
         <v/>
       </c>
       <c r="I74" s="22" t="str">
@@ -7374,7 +7445,7 @@
       <c r="F75" s="13"/>
       <c r="G75" s="21"/>
       <c r="H75" s="22" t="str">
-        <f aca="false">IF(F75="","",ROUND(F75*G75,2))</f>
+        <f>IF(F75="","",IF(OR(E75="Abschreibung (AfA)",E75="Vorsteuer auf Anlagevermögen"),0,ROUND(F75*G75,2)))</f>
         <v/>
       </c>
       <c r="I75" s="22" t="str">
@@ -7392,7 +7463,7 @@
       <c r="F76" s="13"/>
       <c r="G76" s="21"/>
       <c r="H76" s="22" t="str">
-        <f aca="false">IF(F76="","",ROUND(F76*G76,2))</f>
+        <f>IF(F76="","",IF(OR(E76="Abschreibung (AfA)",E76="Vorsteuer auf Anlagevermögen"),0,ROUND(F76*G76,2)))</f>
         <v/>
       </c>
       <c r="I76" s="22" t="str">
@@ -7410,7 +7481,7 @@
       <c r="F77" s="13"/>
       <c r="G77" s="21"/>
       <c r="H77" s="22" t="str">
-        <f aca="false">IF(F77="","",ROUND(F77*G77,2))</f>
+        <f>IF(F77="","",IF(OR(E77="Abschreibung (AfA)",E77="Vorsteuer auf Anlagevermögen"),0,ROUND(F77*G77,2)))</f>
         <v/>
       </c>
       <c r="I77" s="22" t="str">
@@ -7428,7 +7499,7 @@
       <c r="F78" s="13"/>
       <c r="G78" s="21"/>
       <c r="H78" s="22" t="str">
-        <f aca="false">IF(F78="","",ROUND(F78*G78,2))</f>
+        <f>IF(F78="","",IF(OR(E78="Abschreibung (AfA)",E78="Vorsteuer auf Anlagevermögen"),0,ROUND(F78*G78,2)))</f>
         <v/>
       </c>
       <c r="I78" s="22" t="str">
@@ -7446,7 +7517,7 @@
       <c r="F79" s="13"/>
       <c r="G79" s="21"/>
       <c r="H79" s="22" t="str">
-        <f aca="false">IF(F79="","",ROUND(F79*G79,2))</f>
+        <f>IF(F79="","",IF(OR(E79="Abschreibung (AfA)",E79="Vorsteuer auf Anlagevermögen"),0,ROUND(F79*G79,2)))</f>
         <v/>
       </c>
       <c r="I79" s="22" t="str">
@@ -7464,7 +7535,7 @@
       <c r="F80" s="13"/>
       <c r="G80" s="21"/>
       <c r="H80" s="22" t="str">
-        <f aca="false">IF(F80="","",ROUND(F80*G80,2))</f>
+        <f>IF(F80="","",IF(OR(E80="Abschreibung (AfA)",E80="Vorsteuer auf Anlagevermögen"),0,ROUND(F80*G80,2)))</f>
         <v/>
       </c>
       <c r="I80" s="22" t="str">
@@ -7482,7 +7553,7 @@
       <c r="F81" s="13"/>
       <c r="G81" s="21"/>
       <c r="H81" s="22" t="str">
-        <f aca="false">IF(F81="","",ROUND(F81*G81,2))</f>
+        <f>IF(F81="","",IF(OR(E81="Abschreibung (AfA)",E81="Vorsteuer auf Anlagevermögen"),0,ROUND(F81*G81,2)))</f>
         <v/>
       </c>
       <c r="I81" s="22" t="str">
@@ -7500,7 +7571,7 @@
       <c r="F82" s="13"/>
       <c r="G82" s="21"/>
       <c r="H82" s="22" t="str">
-        <f aca="false">IF(F82="","",ROUND(F82*G82,2))</f>
+        <f>IF(F82="","",IF(OR(E82="Abschreibung (AfA)",E82="Vorsteuer auf Anlagevermögen"),0,ROUND(F82*G82,2)))</f>
         <v/>
       </c>
       <c r="I82" s="22" t="str">
@@ -7518,7 +7589,7 @@
       <c r="F83" s="13"/>
       <c r="G83" s="21"/>
       <c r="H83" s="22" t="str">
-        <f aca="false">IF(F83="","",ROUND(F83*G83,2))</f>
+        <f>IF(F83="","",IF(OR(E83="Abschreibung (AfA)",E83="Vorsteuer auf Anlagevermögen"),0,ROUND(F83*G83,2)))</f>
         <v/>
       </c>
       <c r="I83" s="22" t="str">
@@ -7536,7 +7607,7 @@
       <c r="F84" s="13"/>
       <c r="G84" s="21"/>
       <c r="H84" s="22" t="str">
-        <f aca="false">IF(F84="","",ROUND(F84*G84,2))</f>
+        <f>IF(F84="","",IF(OR(E84="Abschreibung (AfA)",E84="Vorsteuer auf Anlagevermögen"),0,ROUND(F84*G84,2)))</f>
         <v/>
       </c>
       <c r="I84" s="22" t="str">
@@ -7554,7 +7625,7 @@
       <c r="F85" s="13"/>
       <c r="G85" s="21"/>
       <c r="H85" s="22" t="str">
-        <f aca="false">IF(F85="","",ROUND(F85*G85,2))</f>
+        <f>IF(F85="","",IF(OR(E85="Abschreibung (AfA)",E85="Vorsteuer auf Anlagevermögen"),0,ROUND(F85*G85,2)))</f>
         <v/>
       </c>
       <c r="I85" s="22" t="str">
@@ -7572,7 +7643,7 @@
       <c r="F86" s="13"/>
       <c r="G86" s="21"/>
       <c r="H86" s="22" t="str">
-        <f aca="false">IF(F86="","",ROUND(F86*G86,2))</f>
+        <f>IF(F86="","",IF(OR(E86="Abschreibung (AfA)",E86="Vorsteuer auf Anlagevermögen"),0,ROUND(F86*G86,2)))</f>
         <v/>
       </c>
       <c r="I86" s="22" t="str">
@@ -7590,7 +7661,7 @@
       <c r="F87" s="13"/>
       <c r="G87" s="21"/>
       <c r="H87" s="22" t="str">
-        <f aca="false">IF(F87="","",ROUND(F87*G87,2))</f>
+        <f>IF(F87="","",IF(OR(E87="Abschreibung (AfA)",E87="Vorsteuer auf Anlagevermögen"),0,ROUND(F87*G87,2)))</f>
         <v/>
       </c>
       <c r="I87" s="22" t="str">
@@ -7608,7 +7679,7 @@
       <c r="F88" s="13"/>
       <c r="G88" s="21"/>
       <c r="H88" s="22" t="str">
-        <f aca="false">IF(F88="","",ROUND(F88*G88,2))</f>
+        <f>IF(F88="","",IF(OR(E88="Abschreibung (AfA)",E88="Vorsteuer auf Anlagevermögen"),0,ROUND(F88*G88,2)))</f>
         <v/>
       </c>
       <c r="I88" s="22" t="str">
@@ -7626,7 +7697,7 @@
       <c r="F89" s="13"/>
       <c r="G89" s="21"/>
       <c r="H89" s="22" t="str">
-        <f aca="false">IF(F89="","",ROUND(F89*G89,2))</f>
+        <f>IF(F89="","",IF(OR(E89="Abschreibung (AfA)",E89="Vorsteuer auf Anlagevermögen"),0,ROUND(F89*G89,2)))</f>
         <v/>
       </c>
       <c r="I89" s="22" t="str">
@@ -7644,7 +7715,7 @@
       <c r="F90" s="13"/>
       <c r="G90" s="21"/>
       <c r="H90" s="22" t="str">
-        <f aca="false">IF(F90="","",ROUND(F90*G90,2))</f>
+        <f>IF(F90="","",IF(OR(E90="Abschreibung (AfA)",E90="Vorsteuer auf Anlagevermögen"),0,ROUND(F90*G90,2)))</f>
         <v/>
       </c>
       <c r="I90" s="22" t="str">
@@ -7662,7 +7733,7 @@
       <c r="F91" s="13"/>
       <c r="G91" s="21"/>
       <c r="H91" s="22" t="str">
-        <f aca="false">IF(F91="","",ROUND(F91*G91,2))</f>
+        <f>IF(F91="","",IF(OR(E91="Abschreibung (AfA)",E91="Vorsteuer auf Anlagevermögen"),0,ROUND(F91*G91,2)))</f>
         <v/>
       </c>
       <c r="I91" s="22" t="str">
@@ -7680,7 +7751,7 @@
       <c r="F92" s="13"/>
       <c r="G92" s="21"/>
       <c r="H92" s="22" t="str">
-        <f aca="false">IF(F92="","",ROUND(F92*G92,2))</f>
+        <f>IF(F92="","",IF(OR(E92="Abschreibung (AfA)",E92="Vorsteuer auf Anlagevermögen"),0,ROUND(F92*G92,2)))</f>
         <v/>
       </c>
       <c r="I92" s="22" t="str">
@@ -7698,7 +7769,7 @@
       <c r="F93" s="13"/>
       <c r="G93" s="21"/>
       <c r="H93" s="22" t="str">
-        <f aca="false">IF(F93="","",ROUND(F93*G93,2))</f>
+        <f>IF(F93="","",IF(OR(E93="Abschreibung (AfA)",E93="Vorsteuer auf Anlagevermögen"),0,ROUND(F93*G93,2)))</f>
         <v/>
       </c>
       <c r="I93" s="22" t="str">
@@ -7716,7 +7787,7 @@
       <c r="F94" s="13"/>
       <c r="G94" s="21"/>
       <c r="H94" s="22" t="str">
-        <f aca="false">IF(F94="","",ROUND(F94*G94,2))</f>
+        <f>IF(F94="","",IF(OR(E94="Abschreibung (AfA)",E94="Vorsteuer auf Anlagevermögen"),0,ROUND(F94*G94,2)))</f>
         <v/>
       </c>
       <c r="I94" s="22" t="str">
@@ -7734,7 +7805,7 @@
       <c r="F95" s="13"/>
       <c r="G95" s="21"/>
       <c r="H95" s="22" t="str">
-        <f aca="false">IF(F95="","",ROUND(F95*G95,2))</f>
+        <f>IF(F95="","",IF(OR(E95="Abschreibung (AfA)",E95="Vorsteuer auf Anlagevermögen"),0,ROUND(F95*G95,2)))</f>
         <v/>
       </c>
       <c r="I95" s="22" t="str">
@@ -7752,7 +7823,7 @@
       <c r="F96" s="13"/>
       <c r="G96" s="21"/>
       <c r="H96" s="22" t="str">
-        <f aca="false">IF(F96="","",ROUND(F96*G96,2))</f>
+        <f>IF(F96="","",IF(OR(E96="Abschreibung (AfA)",E96="Vorsteuer auf Anlagevermögen"),0,ROUND(F96*G96,2)))</f>
         <v/>
       </c>
       <c r="I96" s="22" t="str">
@@ -7770,7 +7841,7 @@
       <c r="F97" s="13"/>
       <c r="G97" s="21"/>
       <c r="H97" s="22" t="str">
-        <f aca="false">IF(F97="","",ROUND(F97*G97,2))</f>
+        <f>IF(F97="","",IF(OR(E97="Abschreibung (AfA)",E97="Vorsteuer auf Anlagevermögen"),0,ROUND(F97*G97,2)))</f>
         <v/>
       </c>
       <c r="I97" s="22" t="str">
@@ -7788,7 +7859,7 @@
       <c r="F98" s="13"/>
       <c r="G98" s="21"/>
       <c r="H98" s="22" t="str">
-        <f aca="false">IF(F98="","",ROUND(F98*G98,2))</f>
+        <f>IF(F98="","",IF(OR(E98="Abschreibung (AfA)",E98="Vorsteuer auf Anlagevermögen"),0,ROUND(F98*G98,2)))</f>
         <v/>
       </c>
       <c r="I98" s="22" t="str">
@@ -7806,7 +7877,7 @@
       <c r="F99" s="13"/>
       <c r="G99" s="21"/>
       <c r="H99" s="22" t="str">
-        <f aca="false">IF(F99="","",ROUND(F99*G99,2))</f>
+        <f>IF(F99="","",IF(OR(E99="Abschreibung (AfA)",E99="Vorsteuer auf Anlagevermögen"),0,ROUND(F99*G99,2)))</f>
         <v/>
       </c>
       <c r="I99" s="22" t="str">
@@ -7824,7 +7895,7 @@
       <c r="F100" s="13"/>
       <c r="G100" s="21"/>
       <c r="H100" s="22" t="str">
-        <f aca="false">IF(F100="","",ROUND(F100*G100,2))</f>
+        <f>IF(F100="","",IF(OR(E100="Abschreibung (AfA)",E100="Vorsteuer auf Anlagevermögen"),0,ROUND(F100*G100,2)))</f>
         <v/>
       </c>
       <c r="I100" s="22" t="str">
@@ -7842,7 +7913,7 @@
       <c r="F101" s="13"/>
       <c r="G101" s="21"/>
       <c r="H101" s="22" t="str">
-        <f aca="false">IF(F101="","",ROUND(F101*G101,2))</f>
+        <f>IF(F101="","",IF(OR(E101="Abschreibung (AfA)",E101="Vorsteuer auf Anlagevermögen"),0,ROUND(F101*G101,2)))</f>
         <v/>
       </c>
       <c r="I101" s="22" t="str">
@@ -7860,7 +7931,7 @@
       <c r="F102" s="13"/>
       <c r="G102" s="21"/>
       <c r="H102" s="22" t="str">
-        <f aca="false">IF(F102="","",ROUND(F102*G102,2))</f>
+        <f>IF(F102="","",IF(OR(E102="Abschreibung (AfA)",E102="Vorsteuer auf Anlagevermögen"),0,ROUND(F102*G102,2)))</f>
         <v/>
       </c>
       <c r="I102" s="22" t="str">
@@ -7878,7 +7949,7 @@
       <c r="F103" s="13"/>
       <c r="G103" s="21"/>
       <c r="H103" s="22" t="str">
-        <f aca="false">IF(F103="","",ROUND(F103*G103,2))</f>
+        <f>IF(F103="","",IF(OR(E103="Abschreibung (AfA)",E103="Vorsteuer auf Anlagevermögen"),0,ROUND(F103*G103,2)))</f>
         <v/>
       </c>
       <c r="I103" s="22" t="str">
@@ -7896,7 +7967,7 @@
       <c r="F104" s="13"/>
       <c r="G104" s="21"/>
       <c r="H104" s="22" t="str">
-        <f aca="false">IF(F104="","",ROUND(F104*G104,2))</f>
+        <f>IF(F104="","",IF(OR(E104="Abschreibung (AfA)",E104="Vorsteuer auf Anlagevermögen"),0,ROUND(F104*G104,2)))</f>
         <v/>
       </c>
       <c r="I104" s="22" t="str">
@@ -7914,7 +7985,7 @@
       <c r="F105" s="13"/>
       <c r="G105" s="21"/>
       <c r="H105" s="22" t="str">
-        <f aca="false">IF(F105="","",ROUND(F105*G105,2))</f>
+        <f>IF(F105="","",IF(OR(E105="Abschreibung (AfA)",E105="Vorsteuer auf Anlagevermögen"),0,ROUND(F105*G105,2)))</f>
         <v/>
       </c>
       <c r="I105" s="22" t="str">
@@ -7932,7 +8003,7 @@
       <c r="F106" s="13"/>
       <c r="G106" s="21"/>
       <c r="H106" s="22" t="str">
-        <f aca="false">IF(F106="","",ROUND(F106*G106,2))</f>
+        <f>IF(F106="","",IF(OR(E106="Abschreibung (AfA)",E106="Vorsteuer auf Anlagevermögen"),0,ROUND(F106*G106,2)))</f>
         <v/>
       </c>
       <c r="I106" s="22" t="str">
@@ -7950,7 +8021,7 @@
       <c r="F107" s="13"/>
       <c r="G107" s="21"/>
       <c r="H107" s="22" t="str">
-        <f aca="false">IF(F107="","",ROUND(F107*G107,2))</f>
+        <f>IF(F107="","",IF(OR(E107="Abschreibung (AfA)",E107="Vorsteuer auf Anlagevermögen"),0,ROUND(F107*G107,2)))</f>
         <v/>
       </c>
       <c r="I107" s="22" t="str">
@@ -7968,7 +8039,7 @@
       <c r="F108" s="13"/>
       <c r="G108" s="21"/>
       <c r="H108" s="22" t="str">
-        <f aca="false">IF(F108="","",ROUND(F108*G108,2))</f>
+        <f>IF(F108="","",IF(OR(E108="Abschreibung (AfA)",E108="Vorsteuer auf Anlagevermögen"),0,ROUND(F108*G108,2)))</f>
         <v/>
       </c>
       <c r="I108" s="22" t="str">
@@ -7986,7 +8057,7 @@
       <c r="F109" s="13"/>
       <c r="G109" s="21"/>
       <c r="H109" s="22" t="str">
-        <f aca="false">IF(F109="","",ROUND(F109*G109,2))</f>
+        <f>IF(F109="","",IF(OR(E109="Abschreibung (AfA)",E109="Vorsteuer auf Anlagevermögen"),0,ROUND(F109*G109,2)))</f>
         <v/>
       </c>
       <c r="I109" s="22" t="str">
@@ -8004,7 +8075,7 @@
       <c r="F110" s="13"/>
       <c r="G110" s="21"/>
       <c r="H110" s="22" t="str">
-        <f aca="false">IF(F110="","",ROUND(F110*G110,2))</f>
+        <f>IF(F110="","",IF(OR(E110="Abschreibung (AfA)",E110="Vorsteuer auf Anlagevermögen"),0,ROUND(F110*G110,2)))</f>
         <v/>
       </c>
       <c r="I110" s="22" t="str">
@@ -8022,7 +8093,7 @@
       <c r="F111" s="13"/>
       <c r="G111" s="21"/>
       <c r="H111" s="22" t="str">
-        <f aca="false">IF(F111="","",ROUND(F111*G111,2))</f>
+        <f>IF(F111="","",IF(OR(E111="Abschreibung (AfA)",E111="Vorsteuer auf Anlagevermögen"),0,ROUND(F111*G111,2)))</f>
         <v/>
       </c>
       <c r="I111" s="22" t="str">
@@ -8040,7 +8111,7 @@
       <c r="F112" s="13"/>
       <c r="G112" s="21"/>
       <c r="H112" s="22" t="str">
-        <f aca="false">IF(F112="","",ROUND(F112*G112,2))</f>
+        <f>IF(F112="","",IF(OR(E112="Abschreibung (AfA)",E112="Vorsteuer auf Anlagevermögen"),0,ROUND(F112*G112,2)))</f>
         <v/>
       </c>
       <c r="I112" s="22" t="str">
@@ -8058,7 +8129,7 @@
       <c r="F113" s="13"/>
       <c r="G113" s="21"/>
       <c r="H113" s="22" t="str">
-        <f aca="false">IF(F113="","",ROUND(F113*G113,2))</f>
+        <f>IF(F113="","",IF(OR(E113="Abschreibung (AfA)",E113="Vorsteuer auf Anlagevermögen"),0,ROUND(F113*G113,2)))</f>
         <v/>
       </c>
       <c r="I113" s="22" t="str">
@@ -8076,7 +8147,7 @@
       <c r="F114" s="13"/>
       <c r="G114" s="21"/>
       <c r="H114" s="22" t="str">
-        <f aca="false">IF(F114="","",ROUND(F114*G114,2))</f>
+        <f>IF(F114="","",IF(OR(E114="Abschreibung (AfA)",E114="Vorsteuer auf Anlagevermögen"),0,ROUND(F114*G114,2)))</f>
         <v/>
       </c>
       <c r="I114" s="22" t="str">
@@ -8094,7 +8165,7 @@
       <c r="F115" s="13"/>
       <c r="G115" s="21"/>
       <c r="H115" s="22" t="str">
-        <f aca="false">IF(F115="","",ROUND(F115*G115,2))</f>
+        <f>IF(F115="","",IF(OR(E115="Abschreibung (AfA)",E115="Vorsteuer auf Anlagevermögen"),0,ROUND(F115*G115,2)))</f>
         <v/>
       </c>
       <c r="I115" s="22" t="str">
@@ -8112,7 +8183,7 @@
       <c r="F116" s="13"/>
       <c r="G116" s="21"/>
       <c r="H116" s="22" t="str">
-        <f aca="false">IF(F116="","",ROUND(F116*G116,2))</f>
+        <f>IF(F116="","",IF(OR(E116="Abschreibung (AfA)",E116="Vorsteuer auf Anlagevermögen"),0,ROUND(F116*G116,2)))</f>
         <v/>
       </c>
       <c r="I116" s="22" t="str">
@@ -8130,7 +8201,7 @@
       <c r="F117" s="13"/>
       <c r="G117" s="21"/>
       <c r="H117" s="22" t="str">
-        <f aca="false">IF(F117="","",ROUND(F117*G117,2))</f>
+        <f>IF(F117="","",IF(OR(E117="Abschreibung (AfA)",E117="Vorsteuer auf Anlagevermögen"),0,ROUND(F117*G117,2)))</f>
         <v/>
       </c>
       <c r="I117" s="22" t="str">
@@ -8148,7 +8219,7 @@
       <c r="F118" s="13"/>
       <c r="G118" s="21"/>
       <c r="H118" s="22" t="str">
-        <f aca="false">IF(F118="","",ROUND(F118*G118,2))</f>
+        <f>IF(F118="","",IF(OR(E118="Abschreibung (AfA)",E118="Vorsteuer auf Anlagevermögen"),0,ROUND(F118*G118,2)))</f>
         <v/>
       </c>
       <c r="I118" s="22" t="str">
@@ -8166,7 +8237,7 @@
       <c r="F119" s="13"/>
       <c r="G119" s="21"/>
       <c r="H119" s="22" t="str">
-        <f aca="false">IF(F119="","",ROUND(F119*G119,2))</f>
+        <f>IF(F119="","",IF(OR(E119="Abschreibung (AfA)",E119="Vorsteuer auf Anlagevermögen"),0,ROUND(F119*G119,2)))</f>
         <v/>
       </c>
       <c r="I119" s="22" t="str">
@@ -8184,7 +8255,7 @@
       <c r="F120" s="13"/>
       <c r="G120" s="21"/>
       <c r="H120" s="22" t="str">
-        <f aca="false">IF(F120="","",ROUND(F120*G120,2))</f>
+        <f>IF(F120="","",IF(OR(E120="Abschreibung (AfA)",E120="Vorsteuer auf Anlagevermögen"),0,ROUND(F120*G120,2)))</f>
         <v/>
       </c>
       <c r="I120" s="22" t="str">
@@ -8202,7 +8273,7 @@
       <c r="F121" s="13"/>
       <c r="G121" s="21"/>
       <c r="H121" s="22" t="str">
-        <f aca="false">IF(F121="","",ROUND(F121*G121,2))</f>
+        <f>IF(F121="","",IF(OR(E121="Abschreibung (AfA)",E121="Vorsteuer auf Anlagevermögen"),0,ROUND(F121*G121,2)))</f>
         <v/>
       </c>
       <c r="I121" s="22" t="str">
@@ -8220,7 +8291,7 @@
       <c r="F122" s="13"/>
       <c r="G122" s="21"/>
       <c r="H122" s="22" t="str">
-        <f aca="false">IF(F122="","",ROUND(F122*G122,2))</f>
+        <f>IF(F122="","",IF(OR(E122="Abschreibung (AfA)",E122="Vorsteuer auf Anlagevermögen"),0,ROUND(F122*G122,2)))</f>
         <v/>
       </c>
       <c r="I122" s="22" t="str">
@@ -8238,7 +8309,7 @@
       <c r="F123" s="13"/>
       <c r="G123" s="21"/>
       <c r="H123" s="22" t="str">
-        <f aca="false">IF(F123="","",ROUND(F123*G123,2))</f>
+        <f>IF(F123="","",IF(OR(E123="Abschreibung (AfA)",E123="Vorsteuer auf Anlagevermögen"),0,ROUND(F123*G123,2)))</f>
         <v/>
       </c>
       <c r="I123" s="22" t="str">
@@ -8256,7 +8327,7 @@
       <c r="F124" s="13"/>
       <c r="G124" s="21"/>
       <c r="H124" s="22" t="str">
-        <f aca="false">IF(F124="","",ROUND(F124*G124,2))</f>
+        <f>IF(F124="","",IF(OR(E124="Abschreibung (AfA)",E124="Vorsteuer auf Anlagevermögen"),0,ROUND(F124*G124,2)))</f>
         <v/>
       </c>
       <c r="I124" s="22" t="str">
@@ -8274,7 +8345,7 @@
       <c r="F125" s="13"/>
       <c r="G125" s="21"/>
       <c r="H125" s="22" t="str">
-        <f aca="false">IF(F125="","",ROUND(F125*G125,2))</f>
+        <f>IF(F125="","",IF(OR(E125="Abschreibung (AfA)",E125="Vorsteuer auf Anlagevermögen"),0,ROUND(F125*G125,2)))</f>
         <v/>
       </c>
       <c r="I125" s="22" t="str">
@@ -8292,7 +8363,7 @@
       <c r="F126" s="13"/>
       <c r="G126" s="21"/>
       <c r="H126" s="22" t="str">
-        <f aca="false">IF(F126="","",ROUND(F126*G126,2))</f>
+        <f>IF(F126="","",IF(OR(E126="Abschreibung (AfA)",E126="Vorsteuer auf Anlagevermögen"),0,ROUND(F126*G126,2)))</f>
         <v/>
       </c>
       <c r="I126" s="22" t="str">
@@ -8310,7 +8381,7 @@
       <c r="F127" s="13"/>
       <c r="G127" s="21"/>
       <c r="H127" s="22" t="str">
-        <f aca="false">IF(F127="","",ROUND(F127*G127,2))</f>
+        <f>IF(F127="","",IF(OR(E127="Abschreibung (AfA)",E127="Vorsteuer auf Anlagevermögen"),0,ROUND(F127*G127,2)))</f>
         <v/>
       </c>
       <c r="I127" s="22" t="str">
@@ -8328,7 +8399,7 @@
       <c r="F128" s="13"/>
       <c r="G128" s="21"/>
       <c r="H128" s="22" t="str">
-        <f aca="false">IF(F128="","",ROUND(F128*G128,2))</f>
+        <f>IF(F128="","",IF(OR(E128="Abschreibung (AfA)",E128="Vorsteuer auf Anlagevermögen"),0,ROUND(F128*G128,2)))</f>
         <v/>
       </c>
       <c r="I128" s="22" t="str">
@@ -8346,7 +8417,7 @@
       <c r="F129" s="13"/>
       <c r="G129" s="21"/>
       <c r="H129" s="22" t="str">
-        <f aca="false">IF(F129="","",ROUND(F129*G129,2))</f>
+        <f>IF(F129="","",IF(OR(E129="Abschreibung (AfA)",E129="Vorsteuer auf Anlagevermögen"),0,ROUND(F129*G129,2)))</f>
         <v/>
       </c>
       <c r="I129" s="22" t="str">
@@ -8364,7 +8435,7 @@
       <c r="F130" s="13"/>
       <c r="G130" s="21"/>
       <c r="H130" s="22" t="str">
-        <f aca="false">IF(F130="","",ROUND(F130*G130,2))</f>
+        <f>IF(F130="","",IF(OR(E130="Abschreibung (AfA)",E130="Vorsteuer auf Anlagevermögen"),0,ROUND(F130*G130,2)))</f>
         <v/>
       </c>
       <c r="I130" s="22" t="str">
@@ -8382,7 +8453,7 @@
       <c r="F131" s="13"/>
       <c r="G131" s="21"/>
       <c r="H131" s="22" t="str">
-        <f aca="false">IF(F131="","",ROUND(F131*G131,2))</f>
+        <f>IF(F131="","",IF(OR(E131="Abschreibung (AfA)",E131="Vorsteuer auf Anlagevermögen"),0,ROUND(F131*G131,2)))</f>
         <v/>
       </c>
       <c r="I131" s="22" t="str">
@@ -8400,7 +8471,7 @@
       <c r="F132" s="13"/>
       <c r="G132" s="21"/>
       <c r="H132" s="22" t="str">
-        <f aca="false">IF(F132="","",ROUND(F132*G132,2))</f>
+        <f>IF(F132="","",IF(OR(E132="Abschreibung (AfA)",E132="Vorsteuer auf Anlagevermögen"),0,ROUND(F132*G132,2)))</f>
         <v/>
       </c>
       <c r="I132" s="22" t="str">
@@ -8418,7 +8489,7 @@
       <c r="F133" s="13"/>
       <c r="G133" s="21"/>
       <c r="H133" s="22" t="str">
-        <f aca="false">IF(F133="","",ROUND(F133*G133,2))</f>
+        <f>IF(F133="","",IF(OR(E133="Abschreibung (AfA)",E133="Vorsteuer auf Anlagevermögen"),0,ROUND(F133*G133,2)))</f>
         <v/>
       </c>
       <c r="I133" s="22" t="str">
@@ -8436,7 +8507,7 @@
       <c r="F134" s="13"/>
       <c r="G134" s="21"/>
       <c r="H134" s="22" t="str">
-        <f aca="false">IF(F134="","",ROUND(F134*G134,2))</f>
+        <f>IF(F134="","",IF(OR(E134="Abschreibung (AfA)",E134="Vorsteuer auf Anlagevermögen"),0,ROUND(F134*G134,2)))</f>
         <v/>
       </c>
       <c r="I134" s="22" t="str">
@@ -8454,7 +8525,7 @@
       <c r="F135" s="13"/>
       <c r="G135" s="21"/>
       <c r="H135" s="22" t="str">
-        <f aca="false">IF(F135="","",ROUND(F135*G135,2))</f>
+        <f>IF(F135="","",IF(OR(E135="Abschreibung (AfA)",E135="Vorsteuer auf Anlagevermögen"),0,ROUND(F135*G135,2)))</f>
         <v/>
       </c>
       <c r="I135" s="22" t="str">
@@ -8472,7 +8543,7 @@
       <c r="F136" s="13"/>
       <c r="G136" s="21"/>
       <c r="H136" s="22" t="str">
-        <f aca="false">IF(F136="","",ROUND(F136*G136,2))</f>
+        <f>IF(F136="","",IF(OR(E136="Abschreibung (AfA)",E136="Vorsteuer auf Anlagevermögen"),0,ROUND(F136*G136,2)))</f>
         <v/>
       </c>
       <c r="I136" s="22" t="str">
@@ -8490,7 +8561,7 @@
       <c r="F137" s="13"/>
       <c r="G137" s="21"/>
       <c r="H137" s="22" t="str">
-        <f aca="false">IF(F137="","",ROUND(F137*G137,2))</f>
+        <f>IF(F137="","",IF(OR(E137="Abschreibung (AfA)",E137="Vorsteuer auf Anlagevermögen"),0,ROUND(F137*G137,2)))</f>
         <v/>
       </c>
       <c r="I137" s="22" t="str">
@@ -8508,7 +8579,7 @@
       <c r="F138" s="13"/>
       <c r="G138" s="21"/>
       <c r="H138" s="22" t="str">
-        <f aca="false">IF(F138="","",ROUND(F138*G138,2))</f>
+        <f>IF(F138="","",IF(OR(E138="Abschreibung (AfA)",E138="Vorsteuer auf Anlagevermögen"),0,ROUND(F138*G138,2)))</f>
         <v/>
       </c>
       <c r="I138" s="22" t="str">
@@ -8526,7 +8597,7 @@
       <c r="F139" s="13"/>
       <c r="G139" s="21"/>
       <c r="H139" s="22" t="str">
-        <f aca="false">IF(F139="","",ROUND(F139*G139,2))</f>
+        <f>IF(F139="","",IF(OR(E139="Abschreibung (AfA)",E139="Vorsteuer auf Anlagevermögen"),0,ROUND(F139*G139,2)))</f>
         <v/>
       </c>
       <c r="I139" s="22" t="str">
@@ -8544,7 +8615,7 @@
       <c r="F140" s="13"/>
       <c r="G140" s="21"/>
       <c r="H140" s="22" t="str">
-        <f aca="false">IF(F140="","",ROUND(F140*G140,2))</f>
+        <f>IF(F140="","",IF(OR(E140="Abschreibung (AfA)",E140="Vorsteuer auf Anlagevermögen"),0,ROUND(F140*G140,2)))</f>
         <v/>
       </c>
       <c r="I140" s="22" t="str">
@@ -8562,7 +8633,7 @@
       <c r="F141" s="13"/>
       <c r="G141" s="21"/>
       <c r="H141" s="22" t="str">
-        <f aca="false">IF(F141="","",ROUND(F141*G141,2))</f>
+        <f>IF(F141="","",IF(OR(E141="Abschreibung (AfA)",E141="Vorsteuer auf Anlagevermögen"),0,ROUND(F141*G141,2)))</f>
         <v/>
       </c>
       <c r="I141" s="22" t="str">
@@ -8580,7 +8651,7 @@
       <c r="F142" s="13"/>
       <c r="G142" s="21"/>
       <c r="H142" s="22" t="str">
-        <f aca="false">IF(F142="","",ROUND(F142*G142,2))</f>
+        <f>IF(F142="","",IF(OR(E142="Abschreibung (AfA)",E142="Vorsteuer auf Anlagevermögen"),0,ROUND(F142*G142,2)))</f>
         <v/>
       </c>
       <c r="I142" s="22" t="str">
@@ -8598,7 +8669,7 @@
       <c r="F143" s="13"/>
       <c r="G143" s="21"/>
       <c r="H143" s="22" t="str">
-        <f aca="false">IF(F143="","",ROUND(F143*G143,2))</f>
+        <f>IF(F143="","",IF(OR(E143="Abschreibung (AfA)",E143="Vorsteuer auf Anlagevermögen"),0,ROUND(F143*G143,2)))</f>
         <v/>
       </c>
       <c r="I143" s="22" t="str">
@@ -8616,7 +8687,7 @@
       <c r="F144" s="13"/>
       <c r="G144" s="21"/>
       <c r="H144" s="22" t="str">
-        <f aca="false">IF(F144="","",ROUND(F144*G144,2))</f>
+        <f>IF(F144="","",IF(OR(E144="Abschreibung (AfA)",E144="Vorsteuer auf Anlagevermögen"),0,ROUND(F144*G144,2)))</f>
         <v/>
       </c>
       <c r="I144" s="22" t="str">
@@ -8634,7 +8705,7 @@
       <c r="F145" s="13"/>
       <c r="G145" s="21"/>
       <c r="H145" s="22" t="str">
-        <f aca="false">IF(F145="","",ROUND(F145*G145,2))</f>
+        <f>IF(F145="","",IF(OR(E145="Abschreibung (AfA)",E145="Vorsteuer auf Anlagevermögen"),0,ROUND(F145*G145,2)))</f>
         <v/>
       </c>
       <c r="I145" s="22" t="str">
@@ -8652,7 +8723,7 @@
       <c r="F146" s="13"/>
       <c r="G146" s="21"/>
       <c r="H146" s="22" t="str">
-        <f aca="false">IF(F146="","",ROUND(F146*G146,2))</f>
+        <f>IF(F146="","",IF(OR(E146="Abschreibung (AfA)",E146="Vorsteuer auf Anlagevermögen"),0,ROUND(F146*G146,2)))</f>
         <v/>
       </c>
       <c r="I146" s="22" t="str">
@@ -8670,7 +8741,7 @@
       <c r="F147" s="13"/>
       <c r="G147" s="21"/>
       <c r="H147" s="22" t="str">
-        <f aca="false">IF(F147="","",ROUND(F147*G147,2))</f>
+        <f>IF(F147="","",IF(OR(E147="Abschreibung (AfA)",E147="Vorsteuer auf Anlagevermögen"),0,ROUND(F147*G147,2)))</f>
         <v/>
       </c>
       <c r="I147" s="22" t="str">
@@ -8688,7 +8759,7 @@
       <c r="F148" s="13"/>
       <c r="G148" s="21"/>
       <c r="H148" s="22" t="str">
-        <f aca="false">IF(F148="","",ROUND(F148*G148,2))</f>
+        <f>IF(F148="","",IF(OR(E148="Abschreibung (AfA)",E148="Vorsteuer auf Anlagevermögen"),0,ROUND(F148*G148,2)))</f>
         <v/>
       </c>
       <c r="I148" s="22" t="str">
@@ -8706,7 +8777,7 @@
       <c r="F149" s="13"/>
       <c r="G149" s="21"/>
       <c r="H149" s="22" t="str">
-        <f aca="false">IF(F149="","",ROUND(F149*G149,2))</f>
+        <f>IF(F149="","",IF(OR(E149="Abschreibung (AfA)",E149="Vorsteuer auf Anlagevermögen"),0,ROUND(F149*G149,2)))</f>
         <v/>
       </c>
       <c r="I149" s="22" t="str">
@@ -8724,7 +8795,7 @@
       <c r="F150" s="13"/>
       <c r="G150" s="21"/>
       <c r="H150" s="22" t="str">
-        <f aca="false">IF(F150="","",ROUND(F150*G150,2))</f>
+        <f>IF(F150="","",IF(OR(E150="Abschreibung (AfA)",E150="Vorsteuer auf Anlagevermögen"),0,ROUND(F150*G150,2)))</f>
         <v/>
       </c>
       <c r="I150" s="22" t="str">
@@ -8742,7 +8813,7 @@
       <c r="F151" s="13"/>
       <c r="G151" s="21"/>
       <c r="H151" s="22" t="str">
-        <f aca="false">IF(F151="","",ROUND(F151*G151,2))</f>
+        <f>IF(F151="","",IF(OR(E151="Abschreibung (AfA)",E151="Vorsteuer auf Anlagevermögen"),0,ROUND(F151*G151,2)))</f>
         <v/>
       </c>
       <c r="I151" s="22" t="str">
@@ -8760,7 +8831,7 @@
       <c r="F152" s="13"/>
       <c r="G152" s="21"/>
       <c r="H152" s="22" t="str">
-        <f aca="false">IF(F152="","",ROUND(F152*G152,2))</f>
+        <f>IF(F152="","",IF(OR(E152="Abschreibung (AfA)",E152="Vorsteuer auf Anlagevermögen"),0,ROUND(F152*G152,2)))</f>
         <v/>
       </c>
       <c r="I152" s="22" t="str">
@@ -8778,7 +8849,7 @@
       <c r="F153" s="13"/>
       <c r="G153" s="21"/>
       <c r="H153" s="22" t="str">
-        <f aca="false">IF(F153="","",ROUND(F153*G153,2))</f>
+        <f>IF(F153="","",IF(OR(E153="Abschreibung (AfA)",E153="Vorsteuer auf Anlagevermögen"),0,ROUND(F153*G153,2)))</f>
         <v/>
       </c>
       <c r="I153" s="22" t="str">
@@ -8796,7 +8867,7 @@
       <c r="F154" s="13"/>
       <c r="G154" s="21"/>
       <c r="H154" s="22" t="str">
-        <f aca="false">IF(F154="","",ROUND(F154*G154,2))</f>
+        <f>IF(F154="","",IF(OR(E154="Abschreibung (AfA)",E154="Vorsteuer auf Anlagevermögen"),0,ROUND(F154*G154,2)))</f>
         <v/>
       </c>
       <c r="I154" s="22" t="str">
@@ -8814,7 +8885,7 @@
       <c r="F155" s="13"/>
       <c r="G155" s="21"/>
       <c r="H155" s="22" t="str">
-        <f aca="false">IF(F155="","",ROUND(F155*G155,2))</f>
+        <f>IF(F155="","",IF(OR(E155="Abschreibung (AfA)",E155="Vorsteuer auf Anlagevermögen"),0,ROUND(F155*G155,2)))</f>
         <v/>
       </c>
       <c r="I155" s="22" t="str">
@@ -8832,7 +8903,7 @@
       <c r="F156" s="13"/>
       <c r="G156" s="21"/>
       <c r="H156" s="22" t="str">
-        <f aca="false">IF(F156="","",ROUND(F156*G156,2))</f>
+        <f>IF(F156="","",IF(OR(E156="Abschreibung (AfA)",E156="Vorsteuer auf Anlagevermögen"),0,ROUND(F156*G156,2)))</f>
         <v/>
       </c>
       <c r="I156" s="22" t="str">
@@ -8850,7 +8921,7 @@
       <c r="F157" s="13"/>
       <c r="G157" s="21"/>
       <c r="H157" s="22" t="str">
-        <f aca="false">IF(F157="","",ROUND(F157*G157,2))</f>
+        <f>IF(F157="","",IF(OR(E157="Abschreibung (AfA)",E157="Vorsteuer auf Anlagevermögen"),0,ROUND(F157*G157,2)))</f>
         <v/>
       </c>
       <c r="I157" s="22" t="str">
@@ -8868,7 +8939,7 @@
       <c r="F158" s="13"/>
       <c r="G158" s="21"/>
       <c r="H158" s="22" t="str">
-        <f aca="false">IF(F158="","",ROUND(F158*G158,2))</f>
+        <f>IF(F158="","",IF(OR(E158="Abschreibung (AfA)",E158="Vorsteuer auf Anlagevermögen"),0,ROUND(F158*G158,2)))</f>
         <v/>
       </c>
       <c r="I158" s="22" t="str">
@@ -8886,7 +8957,7 @@
       <c r="F159" s="13"/>
       <c r="G159" s="21"/>
       <c r="H159" s="22" t="str">
-        <f aca="false">IF(F159="","",ROUND(F159*G159,2))</f>
+        <f>IF(F159="","",IF(OR(E159="Abschreibung (AfA)",E159="Vorsteuer auf Anlagevermögen"),0,ROUND(F159*G159,2)))</f>
         <v/>
       </c>
       <c r="I159" s="22" t="str">
@@ -8904,7 +8975,7 @@
       <c r="F160" s="13"/>
       <c r="G160" s="21"/>
       <c r="H160" s="22" t="str">
-        <f aca="false">IF(F160="","",ROUND(F160*G160,2))</f>
+        <f>IF(F160="","",IF(OR(E160="Abschreibung (AfA)",E160="Vorsteuer auf Anlagevermögen"),0,ROUND(F160*G160,2)))</f>
         <v/>
       </c>
       <c r="I160" s="22" t="str">
@@ -8922,7 +8993,7 @@
       <c r="F161" s="13"/>
       <c r="G161" s="21"/>
       <c r="H161" s="22" t="str">
-        <f aca="false">IF(F161="","",ROUND(F161*G161,2))</f>
+        <f>IF(F161="","",IF(OR(E161="Abschreibung (AfA)",E161="Vorsteuer auf Anlagevermögen"),0,ROUND(F161*G161,2)))</f>
         <v/>
       </c>
       <c r="I161" s="22" t="str">
@@ -8940,7 +9011,7 @@
       <c r="F162" s="13"/>
       <c r="G162" s="21"/>
       <c r="H162" s="22" t="str">
-        <f aca="false">IF(F162="","",ROUND(F162*G162,2))</f>
+        <f>IF(F162="","",IF(OR(E162="Abschreibung (AfA)",E162="Vorsteuer auf Anlagevermögen"),0,ROUND(F162*G162,2)))</f>
         <v/>
       </c>
       <c r="I162" s="22" t="str">
@@ -8958,7 +9029,7 @@
       <c r="F163" s="13"/>
       <c r="G163" s="21"/>
       <c r="H163" s="22" t="str">
-        <f aca="false">IF(F163="","",ROUND(F163*G163,2))</f>
+        <f>IF(F163="","",IF(OR(E163="Abschreibung (AfA)",E163="Vorsteuer auf Anlagevermögen"),0,ROUND(F163*G163,2)))</f>
         <v/>
       </c>
       <c r="I163" s="22" t="str">
@@ -8976,7 +9047,7 @@
       <c r="F164" s="13"/>
       <c r="G164" s="21"/>
       <c r="H164" s="22" t="str">
-        <f aca="false">IF(F164="","",ROUND(F164*G164,2))</f>
+        <f>IF(F164="","",IF(OR(E164="Abschreibung (AfA)",E164="Vorsteuer auf Anlagevermögen"),0,ROUND(F164*G164,2)))</f>
         <v/>
       </c>
       <c r="I164" s="22" t="str">
@@ -8994,7 +9065,7 @@
       <c r="F165" s="13"/>
       <c r="G165" s="21"/>
       <c r="H165" s="22" t="str">
-        <f aca="false">IF(F165="","",ROUND(F165*G165,2))</f>
+        <f>IF(F165="","",IF(OR(E165="Abschreibung (AfA)",E165="Vorsteuer auf Anlagevermögen"),0,ROUND(F165*G165,2)))</f>
         <v/>
       </c>
       <c r="I165" s="22" t="str">
@@ -9012,7 +9083,7 @@
       <c r="F166" s="13"/>
       <c r="G166" s="21"/>
       <c r="H166" s="22" t="str">
-        <f aca="false">IF(F166="","",ROUND(F166*G166,2))</f>
+        <f>IF(F166="","",IF(OR(E166="Abschreibung (AfA)",E166="Vorsteuer auf Anlagevermögen"),0,ROUND(F166*G166,2)))</f>
         <v/>
       </c>
       <c r="I166" s="22" t="str">
@@ -9030,7 +9101,7 @@
       <c r="F167" s="13"/>
       <c r="G167" s="21"/>
       <c r="H167" s="22" t="str">
-        <f aca="false">IF(F167="","",ROUND(F167*G167,2))</f>
+        <f>IF(F167="","",IF(OR(E167="Abschreibung (AfA)",E167="Vorsteuer auf Anlagevermögen"),0,ROUND(F167*G167,2)))</f>
         <v/>
       </c>
       <c r="I167" s="22" t="str">
@@ -9048,7 +9119,7 @@
       <c r="F168" s="13"/>
       <c r="G168" s="21"/>
       <c r="H168" s="22" t="str">
-        <f aca="false">IF(F168="","",ROUND(F168*G168,2))</f>
+        <f>IF(F168="","",IF(OR(E168="Abschreibung (AfA)",E168="Vorsteuer auf Anlagevermögen"),0,ROUND(F168*G168,2)))</f>
         <v/>
       </c>
       <c r="I168" s="22" t="str">
@@ -9066,7 +9137,7 @@
       <c r="F169" s="13"/>
       <c r="G169" s="21"/>
       <c r="H169" s="22" t="str">
-        <f aca="false">IF(F169="","",ROUND(F169*G169,2))</f>
+        <f>IF(F169="","",IF(OR(E169="Abschreibung (AfA)",E169="Vorsteuer auf Anlagevermögen"),0,ROUND(F169*G169,2)))</f>
         <v/>
       </c>
       <c r="I169" s="22" t="str">
@@ -9084,7 +9155,7 @@
       <c r="F170" s="13"/>
       <c r="G170" s="21"/>
       <c r="H170" s="22" t="str">
-        <f aca="false">IF(F170="","",ROUND(F170*G170,2))</f>
+        <f>IF(F170="","",IF(OR(E170="Abschreibung (AfA)",E170="Vorsteuer auf Anlagevermögen"),0,ROUND(F170*G170,2)))</f>
         <v/>
       </c>
       <c r="I170" s="22" t="str">
@@ -9102,7 +9173,7 @@
       <c r="F171" s="13"/>
       <c r="G171" s="21"/>
       <c r="H171" s="22" t="str">
-        <f aca="false">IF(F171="","",ROUND(F171*G171,2))</f>
+        <f>IF(F171="","",IF(OR(E171="Abschreibung (AfA)",E171="Vorsteuer auf Anlagevermögen"),0,ROUND(F171*G171,2)))</f>
         <v/>
       </c>
       <c r="I171" s="22" t="str">
@@ -9120,7 +9191,7 @@
       <c r="F172" s="13"/>
       <c r="G172" s="21"/>
       <c r="H172" s="22" t="str">
-        <f aca="false">IF(F172="","",ROUND(F172*G172,2))</f>
+        <f>IF(F172="","",IF(OR(E172="Abschreibung (AfA)",E172="Vorsteuer auf Anlagevermögen"),0,ROUND(F172*G172,2)))</f>
         <v/>
       </c>
       <c r="I172" s="22" t="str">
@@ -9138,7 +9209,7 @@
       <c r="F173" s="13"/>
       <c r="G173" s="21"/>
       <c r="H173" s="22" t="str">
-        <f aca="false">IF(F173="","",ROUND(F173*G173,2))</f>
+        <f>IF(F173="","",IF(OR(E173="Abschreibung (AfA)",E173="Vorsteuer auf Anlagevermögen"),0,ROUND(F173*G173,2)))</f>
         <v/>
       </c>
       <c r="I173" s="22" t="str">
@@ -9156,7 +9227,7 @@
       <c r="F174" s="13"/>
       <c r="G174" s="21"/>
       <c r="H174" s="22" t="str">
-        <f aca="false">IF(F174="","",ROUND(F174*G174,2))</f>
+        <f>IF(F174="","",IF(OR(E174="Abschreibung (AfA)",E174="Vorsteuer auf Anlagevermögen"),0,ROUND(F174*G174,2)))</f>
         <v/>
       </c>
       <c r="I174" s="22" t="str">
@@ -9174,7 +9245,7 @@
       <c r="F175" s="13"/>
       <c r="G175" s="21"/>
       <c r="H175" s="22" t="str">
-        <f aca="false">IF(F175="","",ROUND(F175*G175,2))</f>
+        <f>IF(F175="","",IF(OR(E175="Abschreibung (AfA)",E175="Vorsteuer auf Anlagevermögen"),0,ROUND(F175*G175,2)))</f>
         <v/>
       </c>
       <c r="I175" s="22" t="str">
@@ -9192,7 +9263,7 @@
       <c r="F176" s="13"/>
       <c r="G176" s="21"/>
       <c r="H176" s="22" t="str">
-        <f aca="false">IF(F176="","",ROUND(F176*G176,2))</f>
+        <f>IF(F176="","",IF(OR(E176="Abschreibung (AfA)",E176="Vorsteuer auf Anlagevermögen"),0,ROUND(F176*G176,2)))</f>
         <v/>
       </c>
       <c r="I176" s="22" t="str">
@@ -9210,7 +9281,7 @@
       <c r="F177" s="13"/>
       <c r="G177" s="21"/>
       <c r="H177" s="22" t="str">
-        <f aca="false">IF(F177="","",ROUND(F177*G177,2))</f>
+        <f>IF(F177="","",IF(OR(E177="Abschreibung (AfA)",E177="Vorsteuer auf Anlagevermögen"),0,ROUND(F177*G177,2)))</f>
         <v/>
       </c>
       <c r="I177" s="22" t="str">
@@ -9228,7 +9299,7 @@
       <c r="F178" s="13"/>
       <c r="G178" s="21"/>
       <c r="H178" s="22" t="str">
-        <f aca="false">IF(F178="","",ROUND(F178*G178,2))</f>
+        <f>IF(F178="","",IF(OR(E178="Abschreibung (AfA)",E178="Vorsteuer auf Anlagevermögen"),0,ROUND(F178*G178,2)))</f>
         <v/>
       </c>
       <c r="I178" s="22" t="str">
@@ -9246,7 +9317,7 @@
       <c r="F179" s="13"/>
       <c r="G179" s="21"/>
       <c r="H179" s="22" t="str">
-        <f aca="false">IF(F179="","",ROUND(F179*G179,2))</f>
+        <f>IF(F179="","",IF(OR(E179="Abschreibung (AfA)",E179="Vorsteuer auf Anlagevermögen"),0,ROUND(F179*G179,2)))</f>
         <v/>
       </c>
       <c r="I179" s="22" t="str">
@@ -9264,7 +9335,7 @@
       <c r="F180" s="13"/>
       <c r="G180" s="21"/>
       <c r="H180" s="22" t="str">
-        <f aca="false">IF(F180="","",ROUND(F180*G180,2))</f>
+        <f>IF(F180="","",IF(OR(E180="Abschreibung (AfA)",E180="Vorsteuer auf Anlagevermögen"),0,ROUND(F180*G180,2)))</f>
         <v/>
       </c>
       <c r="I180" s="22" t="str">
@@ -9282,7 +9353,7 @@
       <c r="F181" s="13"/>
       <c r="G181" s="21"/>
       <c r="H181" s="22" t="str">
-        <f aca="false">IF(F181="","",ROUND(F181*G181,2))</f>
+        <f>IF(F181="","",IF(OR(E181="Abschreibung (AfA)",E181="Vorsteuer auf Anlagevermögen"),0,ROUND(F181*G181,2)))</f>
         <v/>
       </c>
       <c r="I181" s="22" t="str">
@@ -9300,7 +9371,7 @@
       <c r="F182" s="13"/>
       <c r="G182" s="21"/>
       <c r="H182" s="22" t="str">
-        <f aca="false">IF(F182="","",ROUND(F182*G182,2))</f>
+        <f>IF(F182="","",IF(OR(E182="Abschreibung (AfA)",E182="Vorsteuer auf Anlagevermögen"),0,ROUND(F182*G182,2)))</f>
         <v/>
       </c>
       <c r="I182" s="22" t="str">
@@ -9318,7 +9389,7 @@
       <c r="F183" s="13"/>
       <c r="G183" s="21"/>
       <c r="H183" s="22" t="str">
-        <f aca="false">IF(F183="","",ROUND(F183*G183,2))</f>
+        <f>IF(F183="","",IF(OR(E183="Abschreibung (AfA)",E183="Vorsteuer auf Anlagevermögen"),0,ROUND(F183*G183,2)))</f>
         <v/>
       </c>
       <c r="I183" s="22" t="str">
@@ -9336,7 +9407,7 @@
       <c r="F184" s="13"/>
       <c r="G184" s="21"/>
       <c r="H184" s="22" t="str">
-        <f aca="false">IF(F184="","",ROUND(F184*G184,2))</f>
+        <f>IF(F184="","",IF(OR(E184="Abschreibung (AfA)",E184="Vorsteuer auf Anlagevermögen"),0,ROUND(F184*G184,2)))</f>
         <v/>
       </c>
       <c r="I184" s="22" t="str">
@@ -9354,7 +9425,7 @@
       <c r="F185" s="13"/>
       <c r="G185" s="21"/>
       <c r="H185" s="22" t="str">
-        <f aca="false">IF(F185="","",ROUND(F185*G185,2))</f>
+        <f>IF(F185="","",IF(OR(E185="Abschreibung (AfA)",E185="Vorsteuer auf Anlagevermögen"),0,ROUND(F185*G185,2)))</f>
         <v/>
       </c>
       <c r="I185" s="22" t="str">
@@ -9372,7 +9443,7 @@
       <c r="F186" s="13"/>
       <c r="G186" s="21"/>
       <c r="H186" s="22" t="str">
-        <f aca="false">IF(F186="","",ROUND(F186*G186,2))</f>
+        <f>IF(F186="","",IF(OR(E186="Abschreibung (AfA)",E186="Vorsteuer auf Anlagevermögen"),0,ROUND(F186*G186,2)))</f>
         <v/>
       </c>
       <c r="I186" s="22" t="str">
@@ -9390,7 +9461,7 @@
       <c r="F187" s="13"/>
       <c r="G187" s="21"/>
       <c r="H187" s="22" t="str">
-        <f aca="false">IF(F187="","",ROUND(F187*G187,2))</f>
+        <f>IF(F187="","",IF(OR(E187="Abschreibung (AfA)",E187="Vorsteuer auf Anlagevermögen"),0,ROUND(F187*G187,2)))</f>
         <v/>
       </c>
       <c r="I187" s="22" t="str">
@@ -9408,7 +9479,7 @@
       <c r="F188" s="13"/>
       <c r="G188" s="21"/>
       <c r="H188" s="22" t="str">
-        <f aca="false">IF(F188="","",ROUND(F188*G188,2))</f>
+        <f>IF(F188="","",IF(OR(E188="Abschreibung (AfA)",E188="Vorsteuer auf Anlagevermögen"),0,ROUND(F188*G188,2)))</f>
         <v/>
       </c>
       <c r="I188" s="22" t="str">
@@ -9426,7 +9497,7 @@
       <c r="F189" s="13"/>
       <c r="G189" s="21"/>
       <c r="H189" s="22" t="str">
-        <f aca="false">IF(F189="","",ROUND(F189*G189,2))</f>
+        <f>IF(F189="","",IF(OR(E189="Abschreibung (AfA)",E189="Vorsteuer auf Anlagevermögen"),0,ROUND(F189*G189,2)))</f>
         <v/>
       </c>
       <c r="I189" s="22" t="str">
@@ -9444,7 +9515,7 @@
       <c r="F190" s="13"/>
       <c r="G190" s="21"/>
       <c r="H190" s="22" t="str">
-        <f aca="false">IF(F190="","",ROUND(F190*G190,2))</f>
+        <f>IF(F190="","",IF(OR(E190="Abschreibung (AfA)",E190="Vorsteuer auf Anlagevermögen"),0,ROUND(F190*G190,2)))</f>
         <v/>
       </c>
       <c r="I190" s="22" t="str">
@@ -9462,7 +9533,7 @@
       <c r="F191" s="13"/>
       <c r="G191" s="21"/>
       <c r="H191" s="22" t="str">
-        <f aca="false">IF(F191="","",ROUND(F191*G191,2))</f>
+        <f>IF(F191="","",IF(OR(E191="Abschreibung (AfA)",E191="Vorsteuer auf Anlagevermögen"),0,ROUND(F191*G191,2)))</f>
         <v/>
       </c>
       <c r="I191" s="22" t="str">
@@ -9480,7 +9551,7 @@
       <c r="F192" s="13"/>
       <c r="G192" s="21"/>
       <c r="H192" s="22" t="str">
-        <f aca="false">IF(F192="","",ROUND(F192*G192,2))</f>
+        <f>IF(F192="","",IF(OR(E192="Abschreibung (AfA)",E192="Vorsteuer auf Anlagevermögen"),0,ROUND(F192*G192,2)))</f>
         <v/>
       </c>
       <c r="I192" s="22" t="str">
@@ -9498,7 +9569,7 @@
       <c r="F193" s="13"/>
       <c r="G193" s="21"/>
       <c r="H193" s="22" t="str">
-        <f aca="false">IF(F193="","",ROUND(F193*G193,2))</f>
+        <f>IF(F193="","",IF(OR(E193="Abschreibung (AfA)",E193="Vorsteuer auf Anlagevermögen"),0,ROUND(F193*G193,2)))</f>
         <v/>
       </c>
       <c r="I193" s="22" t="str">
@@ -9516,7 +9587,7 @@
       <c r="F194" s="13"/>
       <c r="G194" s="21"/>
       <c r="H194" s="22" t="str">
-        <f aca="false">IF(F194="","",ROUND(F194*G194,2))</f>
+        <f>IF(F194="","",IF(OR(E194="Abschreibung (AfA)",E194="Vorsteuer auf Anlagevermögen"),0,ROUND(F194*G194,2)))</f>
         <v/>
       </c>
       <c r="I194" s="22" t="str">
@@ -9534,7 +9605,7 @@
       <c r="F195" s="13"/>
       <c r="G195" s="21"/>
       <c r="H195" s="22" t="str">
-        <f aca="false">IF(F195="","",ROUND(F195*G195,2))</f>
+        <f>IF(F195="","",IF(OR(E195="Abschreibung (AfA)",E195="Vorsteuer auf Anlagevermögen"),0,ROUND(F195*G195,2)))</f>
         <v/>
       </c>
       <c r="I195" s="22" t="str">
@@ -9552,7 +9623,7 @@
       <c r="F196" s="13"/>
       <c r="G196" s="21"/>
       <c r="H196" s="22" t="str">
-        <f aca="false">IF(F196="","",ROUND(F196*G196,2))</f>
+        <f>IF(F196="","",IF(OR(E196="Abschreibung (AfA)",E196="Vorsteuer auf Anlagevermögen"),0,ROUND(F196*G196,2)))</f>
         <v/>
       </c>
       <c r="I196" s="22" t="str">
@@ -9570,7 +9641,7 @@
       <c r="F197" s="13"/>
       <c r="G197" s="21"/>
       <c r="H197" s="22" t="str">
-        <f aca="false">IF(F197="","",ROUND(F197*G197,2))</f>
+        <f>IF(F197="","",IF(OR(E197="Abschreibung (AfA)",E197="Vorsteuer auf Anlagevermögen"),0,ROUND(F197*G197,2)))</f>
         <v/>
       </c>
       <c r="I197" s="22" t="str">
@@ -9588,7 +9659,7 @@
       <c r="F198" s="13"/>
       <c r="G198" s="21"/>
       <c r="H198" s="22" t="str">
-        <f aca="false">IF(F198="","",ROUND(F198*G198,2))</f>
+        <f>IF(F198="","",IF(OR(E198="Abschreibung (AfA)",E198="Vorsteuer auf Anlagevermögen"),0,ROUND(F198*G198,2)))</f>
         <v/>
       </c>
       <c r="I198" s="22" t="str">
@@ -9606,7 +9677,7 @@
       <c r="F199" s="13"/>
       <c r="G199" s="21"/>
       <c r="H199" s="22" t="str">
-        <f aca="false">IF(F199="","",ROUND(F199*G199,2))</f>
+        <f>IF(F199="","",IF(OR(E199="Abschreibung (AfA)",E199="Vorsteuer auf Anlagevermögen"),0,ROUND(F199*G199,2)))</f>
         <v/>
       </c>
       <c r="I199" s="22" t="str">
@@ -9624,7 +9695,7 @@
       <c r="F200" s="13"/>
       <c r="G200" s="21"/>
       <c r="H200" s="22" t="str">
-        <f aca="false">IF(F200="","",ROUND(F200*G200,2))</f>
+        <f>IF(F200="","",IF(OR(E200="Abschreibung (AfA)",E200="Vorsteuer auf Anlagevermögen"),0,ROUND(F200*G200,2)))</f>
         <v/>
       </c>
       <c r="I200" s="22" t="str">
@@ -9642,7 +9713,7 @@
       <c r="F201" s="13"/>
       <c r="G201" s="21"/>
       <c r="H201" s="22" t="str">
-        <f aca="false">IF(F201="","",ROUND(F201*G201,2))</f>
+        <f>IF(F201="","",IF(OR(E201="Abschreibung (AfA)",E201="Vorsteuer auf Anlagevermögen"),0,ROUND(F201*G201,2)))</f>
         <v/>
       </c>
       <c r="I201" s="22" t="str">
@@ -9660,7 +9731,7 @@
       <c r="F202" s="13"/>
       <c r="G202" s="21"/>
       <c r="H202" s="22" t="str">
-        <f aca="false">IF(F202="","",ROUND(F202*G202,2))</f>
+        <f>IF(F202="","",IF(OR(E202="Abschreibung (AfA)",E202="Vorsteuer auf Anlagevermögen"),0,ROUND(F202*G202,2)))</f>
         <v/>
       </c>
       <c r="I202" s="22" t="str">
@@ -9678,7 +9749,7 @@
       <c r="F203" s="13"/>
       <c r="G203" s="21"/>
       <c r="H203" s="22" t="str">
-        <f aca="false">IF(F203="","",ROUND(F203*G203,2))</f>
+        <f>IF(F203="","",IF(OR(E203="Abschreibung (AfA)",E203="Vorsteuer auf Anlagevermögen"),0,ROUND(F203*G203,2)))</f>
         <v/>
       </c>
       <c r="I203" s="22" t="str">
@@ -9696,7 +9767,7 @@
       <c r="F204" s="13"/>
       <c r="G204" s="21"/>
       <c r="H204" s="22" t="str">
-        <f aca="false">IF(F204="","",ROUND(F204*G204,2))</f>
+        <f>IF(F204="","",IF(OR(E204="Abschreibung (AfA)",E204="Vorsteuer auf Anlagevermögen"),0,ROUND(F204*G204,2)))</f>
         <v/>
       </c>
       <c r="I204" s="22" t="str">
@@ -9714,7 +9785,7 @@
       <c r="F205" s="13"/>
       <c r="G205" s="21"/>
       <c r="H205" s="22" t="str">
-        <f aca="false">IF(F205="","",ROUND(F205*G205,2))</f>
+        <f>IF(F205="","",IF(OR(E205="Abschreibung (AfA)",E205="Vorsteuer auf Anlagevermögen"),0,ROUND(F205*G205,2)))</f>
         <v/>
       </c>
       <c r="I205" s="22" t="str">
@@ -9732,7 +9803,7 @@
       <c r="F206" s="13"/>
       <c r="G206" s="21"/>
       <c r="H206" s="22" t="str">
-        <f aca="false">IF(F206="","",ROUND(F206*G206,2))</f>
+        <f>IF(F206="","",IF(OR(E206="Abschreibung (AfA)",E206="Vorsteuer auf Anlagevermögen"),0,ROUND(F206*G206,2)))</f>
         <v/>
       </c>
       <c r="I206" s="22" t="str">
@@ -9750,7 +9821,7 @@
       <c r="F207" s="13"/>
       <c r="G207" s="21"/>
       <c r="H207" s="22" t="str">
-        <f aca="false">IF(F207="","",ROUND(F207*G207,2))</f>
+        <f>IF(F207="","",IF(OR(E207="Abschreibung (AfA)",E207="Vorsteuer auf Anlagevermögen"),0,ROUND(F207*G207,2)))</f>
         <v/>
       </c>
       <c r="I207" s="22" t="str">
@@ -9768,7 +9839,7 @@
       <c r="F208" s="13"/>
       <c r="G208" s="21"/>
       <c r="H208" s="22" t="str">
-        <f aca="false">IF(F208="","",ROUND(F208*G208,2))</f>
+        <f>IF(F208="","",IF(OR(E208="Abschreibung (AfA)",E208="Vorsteuer auf Anlagevermögen"),0,ROUND(F208*G208,2)))</f>
         <v/>
       </c>
       <c r="I208" s="22" t="str">
@@ -9786,7 +9857,7 @@
       <c r="F209" s="13"/>
       <c r="G209" s="21"/>
       <c r="H209" s="22" t="str">
-        <f aca="false">IF(F209="","",ROUND(F209*G209,2))</f>
+        <f>IF(F209="","",IF(OR(E209="Abschreibung (AfA)",E209="Vorsteuer auf Anlagevermögen"),0,ROUND(F209*G209,2)))</f>
         <v/>
       </c>
       <c r="I209" s="22" t="str">
@@ -9804,7 +9875,7 @@
       <c r="F210" s="13"/>
       <c r="G210" s="21"/>
       <c r="H210" s="22" t="str">
-        <f aca="false">IF(F210="","",ROUND(F210*G210,2))</f>
+        <f>IF(F210="","",IF(OR(E210="Abschreibung (AfA)",E210="Vorsteuer auf Anlagevermögen"),0,ROUND(F210*G210,2)))</f>
         <v/>
       </c>
       <c r="I210" s="22" t="str">
@@ -9822,7 +9893,7 @@
       <c r="F211" s="13"/>
       <c r="G211" s="21"/>
       <c r="H211" s="22" t="str">
-        <f aca="false">IF(F211="","",ROUND(F211*G211,2))</f>
+        <f>IF(F211="","",IF(OR(E211="Abschreibung (AfA)",E211="Vorsteuer auf Anlagevermögen"),0,ROUND(F211*G211,2)))</f>
         <v/>
       </c>
       <c r="I211" s="22" t="str">
@@ -9840,7 +9911,7 @@
       <c r="F212" s="13"/>
       <c r="G212" s="21"/>
       <c r="H212" s="22" t="str">
-        <f aca="false">IF(F212="","",ROUND(F212*G212,2))</f>
+        <f>IF(F212="","",IF(OR(E212="Abschreibung (AfA)",E212="Vorsteuer auf Anlagevermögen"),0,ROUND(F212*G212,2)))</f>
         <v/>
       </c>
       <c r="I212" s="22" t="str">
@@ -9858,7 +9929,7 @@
       <c r="F213" s="13"/>
       <c r="G213" s="21"/>
       <c r="H213" s="22" t="str">
-        <f aca="false">IF(F213="","",ROUND(F213*G213,2))</f>
+        <f>IF(F213="","",IF(OR(E213="Abschreibung (AfA)",E213="Vorsteuer auf Anlagevermögen"),0,ROUND(F213*G213,2)))</f>
         <v/>
       </c>
       <c r="I213" s="22" t="str">
@@ -9876,7 +9947,7 @@
       <c r="F214" s="13"/>
       <c r="G214" s="21"/>
       <c r="H214" s="22" t="str">
-        <f aca="false">IF(F214="","",ROUND(F214*G214,2))</f>
+        <f>IF(F214="","",IF(OR(E214="Abschreibung (AfA)",E214="Vorsteuer auf Anlagevermögen"),0,ROUND(F214*G214,2)))</f>
         <v/>
       </c>
       <c r="I214" s="22" t="str">
@@ -9894,7 +9965,7 @@
       <c r="F215" s="13"/>
       <c r="G215" s="21"/>
       <c r="H215" s="22" t="str">
-        <f aca="false">IF(F215="","",ROUND(F215*G215,2))</f>
+        <f>IF(F215="","",IF(OR(E215="Abschreibung (AfA)",E215="Vorsteuer auf Anlagevermögen"),0,ROUND(F215*G215,2)))</f>
         <v/>
       </c>
       <c r="I215" s="22" t="str">
@@ -9912,7 +9983,7 @@
       <c r="F216" s="13"/>
       <c r="G216" s="21"/>
       <c r="H216" s="22" t="str">
-        <f aca="false">IF(F216="","",ROUND(F216*G216,2))</f>
+        <f>IF(F216="","",IF(OR(E216="Abschreibung (AfA)",E216="Vorsteuer auf Anlagevermögen"),0,ROUND(F216*G216,2)))</f>
         <v/>
       </c>
       <c r="I216" s="22" t="str">
@@ -9930,7 +10001,7 @@
       <c r="F217" s="13"/>
       <c r="G217" s="21"/>
       <c r="H217" s="22" t="str">
-        <f aca="false">IF(F217="","",ROUND(F217*G217,2))</f>
+        <f>IF(F217="","",IF(OR(E217="Abschreibung (AfA)",E217="Vorsteuer auf Anlagevermögen"),0,ROUND(F217*G217,2)))</f>
         <v/>
       </c>
       <c r="I217" s="22" t="str">
@@ -9948,7 +10019,7 @@
       <c r="F218" s="13"/>
       <c r="G218" s="21"/>
       <c r="H218" s="22" t="str">
-        <f aca="false">IF(F218="","",ROUND(F218*G218,2))</f>
+        <f>IF(F218="","",IF(OR(E218="Abschreibung (AfA)",E218="Vorsteuer auf Anlagevermögen"),0,ROUND(F218*G218,2)))</f>
         <v/>
       </c>
       <c r="I218" s="22" t="str">
@@ -9966,7 +10037,7 @@
       <c r="F219" s="13"/>
       <c r="G219" s="21"/>
       <c r="H219" s="22" t="str">
-        <f aca="false">IF(F219="","",ROUND(F219*G219,2))</f>
+        <f>IF(F219="","",IF(OR(E219="Abschreibung (AfA)",E219="Vorsteuer auf Anlagevermögen"),0,ROUND(F219*G219,2)))</f>
         <v/>
       </c>
       <c r="I219" s="22" t="str">
@@ -9984,7 +10055,7 @@
       <c r="F220" s="13"/>
       <c r="G220" s="21"/>
       <c r="H220" s="22" t="str">
-        <f aca="false">IF(F220="","",ROUND(F220*G220,2))</f>
+        <f>IF(F220="","",IF(OR(E220="Abschreibung (AfA)",E220="Vorsteuer auf Anlagevermögen"),0,ROUND(F220*G220,2)))</f>
         <v/>
       </c>
       <c r="I220" s="22" t="str">
@@ -10002,7 +10073,7 @@
       <c r="F221" s="13"/>
       <c r="G221" s="21"/>
       <c r="H221" s="22" t="str">
-        <f aca="false">IF(F221="","",ROUND(F221*G221,2))</f>
+        <f>IF(F221="","",IF(OR(E221="Abschreibung (AfA)",E221="Vorsteuer auf Anlagevermögen"),0,ROUND(F221*G221,2)))</f>
         <v/>
       </c>
       <c r="I221" s="22" t="str">
@@ -10020,7 +10091,7 @@
       <c r="F222" s="13"/>
       <c r="G222" s="21"/>
       <c r="H222" s="22" t="str">
-        <f aca="false">IF(F222="","",ROUND(F222*G222,2))</f>
+        <f>IF(F222="","",IF(OR(E222="Abschreibung (AfA)",E222="Vorsteuer auf Anlagevermögen"),0,ROUND(F222*G222,2)))</f>
         <v/>
       </c>
       <c r="I222" s="22" t="str">
@@ -10038,7 +10109,7 @@
       <c r="F223" s="13"/>
       <c r="G223" s="21"/>
       <c r="H223" s="22" t="str">
-        <f aca="false">IF(F223="","",ROUND(F223*G223,2))</f>
+        <f>IF(F223="","",IF(OR(E223="Abschreibung (AfA)",E223="Vorsteuer auf Anlagevermögen"),0,ROUND(F223*G223,2)))</f>
         <v/>
       </c>
       <c r="I223" s="22" t="str">
@@ -10056,7 +10127,7 @@
       <c r="F224" s="13"/>
       <c r="G224" s="21"/>
       <c r="H224" s="22" t="str">
-        <f aca="false">IF(F224="","",ROUND(F224*G224,2))</f>
+        <f>IF(F224="","",IF(OR(E224="Abschreibung (AfA)",E224="Vorsteuer auf Anlagevermögen"),0,ROUND(F224*G224,2)))</f>
         <v/>
       </c>
       <c r="I224" s="22" t="str">
@@ -10074,7 +10145,7 @@
       <c r="F225" s="13"/>
       <c r="G225" s="21"/>
       <c r="H225" s="22" t="str">
-        <f aca="false">IF(F225="","",ROUND(F225*G225,2))</f>
+        <f>IF(F225="","",IF(OR(E225="Abschreibung (AfA)",E225="Vorsteuer auf Anlagevermögen"),0,ROUND(F225*G225,2)))</f>
         <v/>
       </c>
       <c r="I225" s="22" t="str">
@@ -10092,7 +10163,7 @@
       <c r="F226" s="13"/>
       <c r="G226" s="21"/>
       <c r="H226" s="22" t="str">
-        <f aca="false">IF(F226="","",ROUND(F226*G226,2))</f>
+        <f>IF(F226="","",IF(OR(E226="Abschreibung (AfA)",E226="Vorsteuer auf Anlagevermögen"),0,ROUND(F226*G226,2)))</f>
         <v/>
       </c>
       <c r="I226" s="22" t="str">
@@ -10110,7 +10181,7 @@
       <c r="F227" s="13"/>
       <c r="G227" s="21"/>
       <c r="H227" s="22" t="str">
-        <f aca="false">IF(F227="","",ROUND(F227*G227,2))</f>
+        <f>IF(F227="","",IF(OR(E227="Abschreibung (AfA)",E227="Vorsteuer auf Anlagevermögen"),0,ROUND(F227*G227,2)))</f>
         <v/>
       </c>
       <c r="I227" s="22" t="str">
@@ -10128,7 +10199,7 @@
       <c r="F228" s="13"/>
       <c r="G228" s="21"/>
       <c r="H228" s="22" t="str">
-        <f aca="false">IF(F228="","",ROUND(F228*G228,2))</f>
+        <f>IF(F228="","",IF(OR(E228="Abschreibung (AfA)",E228="Vorsteuer auf Anlagevermögen"),0,ROUND(F228*G228,2)))</f>
         <v/>
       </c>
       <c r="I228" s="22" t="str">
@@ -10146,7 +10217,7 @@
       <c r="F229" s="13"/>
       <c r="G229" s="21"/>
       <c r="H229" s="22" t="str">
-        <f aca="false">IF(F229="","",ROUND(F229*G229,2))</f>
+        <f>IF(F229="","",IF(OR(E229="Abschreibung (AfA)",E229="Vorsteuer auf Anlagevermögen"),0,ROUND(F229*G229,2)))</f>
         <v/>
       </c>
       <c r="I229" s="22" t="str">
@@ -10164,7 +10235,7 @@
       <c r="F230" s="13"/>
       <c r="G230" s="21"/>
       <c r="H230" s="22" t="str">
-        <f aca="false">IF(F230="","",ROUND(F230*G230,2))</f>
+        <f>IF(F230="","",IF(OR(E230="Abschreibung (AfA)",E230="Vorsteuer auf Anlagevermögen"),0,ROUND(F230*G230,2)))</f>
         <v/>
       </c>
       <c r="I230" s="22" t="str">
@@ -10182,7 +10253,7 @@
       <c r="F231" s="13"/>
       <c r="G231" s="21"/>
       <c r="H231" s="22" t="str">
-        <f aca="false">IF(F231="","",ROUND(F231*G231,2))</f>
+        <f>IF(F231="","",IF(OR(E231="Abschreibung (AfA)",E231="Vorsteuer auf Anlagevermögen"),0,ROUND(F231*G231,2)))</f>
         <v/>
       </c>
       <c r="I231" s="22" t="str">
@@ -10200,7 +10271,7 @@
       <c r="F232" s="13"/>
       <c r="G232" s="21"/>
       <c r="H232" s="22" t="str">
-        <f aca="false">IF(F232="","",ROUND(F232*G232,2))</f>
+        <f>IF(F232="","",IF(OR(E232="Abschreibung (AfA)",E232="Vorsteuer auf Anlagevermögen"),0,ROUND(F232*G232,2)))</f>
         <v/>
       </c>
       <c r="I232" s="22" t="str">
@@ -10218,7 +10289,7 @@
       <c r="F233" s="13"/>
       <c r="G233" s="21"/>
       <c r="H233" s="22" t="str">
-        <f aca="false">IF(F233="","",ROUND(F233*G233,2))</f>
+        <f>IF(F233="","",IF(OR(E233="Abschreibung (AfA)",E233="Vorsteuer auf Anlagevermögen"),0,ROUND(F233*G233,2)))</f>
         <v/>
       </c>
       <c r="I233" s="22" t="str">
@@ -10236,7 +10307,7 @@
       <c r="F234" s="13"/>
       <c r="G234" s="21"/>
       <c r="H234" s="22" t="str">
-        <f aca="false">IF(F234="","",ROUND(F234*G234,2))</f>
+        <f>IF(F234="","",IF(OR(E234="Abschreibung (AfA)",E234="Vorsteuer auf Anlagevermögen"),0,ROUND(F234*G234,2)))</f>
         <v/>
       </c>
       <c r="I234" s="22" t="str">
@@ -10254,7 +10325,7 @@
       <c r="F235" s="13"/>
       <c r="G235" s="21"/>
       <c r="H235" s="22" t="str">
-        <f aca="false">IF(F235="","",ROUND(F235*G235,2))</f>
+        <f>IF(F235="","",IF(OR(E235="Abschreibung (AfA)",E235="Vorsteuer auf Anlagevermögen"),0,ROUND(F235*G235,2)))</f>
         <v/>
       </c>
       <c r="I235" s="22" t="str">
@@ -10272,7 +10343,7 @@
       <c r="F236" s="13"/>
       <c r="G236" s="21"/>
       <c r="H236" s="22" t="str">
-        <f aca="false">IF(F236="","",ROUND(F236*G236,2))</f>
+        <f>IF(F236="","",IF(OR(E236="Abschreibung (AfA)",E236="Vorsteuer auf Anlagevermögen"),0,ROUND(F236*G236,2)))</f>
         <v/>
       </c>
       <c r="I236" s="22" t="str">
@@ -10290,7 +10361,7 @@
       <c r="F237" s="13"/>
       <c r="G237" s="21"/>
       <c r="H237" s="22" t="str">
-        <f aca="false">IF(F237="","",ROUND(F237*G237,2))</f>
+        <f>IF(F237="","",IF(OR(E237="Abschreibung (AfA)",E237="Vorsteuer auf Anlagevermögen"),0,ROUND(F237*G237,2)))</f>
         <v/>
       </c>
       <c r="I237" s="22" t="str">
@@ -10308,7 +10379,7 @@
       <c r="F238" s="13"/>
       <c r="G238" s="21"/>
       <c r="H238" s="22" t="str">
-        <f aca="false">IF(F238="","",ROUND(F238*G238,2))</f>
+        <f>IF(F238="","",IF(OR(E238="Abschreibung (AfA)",E238="Vorsteuer auf Anlagevermögen"),0,ROUND(F238*G238,2)))</f>
         <v/>
       </c>
       <c r="I238" s="22" t="str">
@@ -10326,7 +10397,7 @@
       <c r="F239" s="13"/>
       <c r="G239" s="21"/>
       <c r="H239" s="22" t="str">
-        <f aca="false">IF(F239="","",ROUND(F239*G239,2))</f>
+        <f>IF(F239="","",IF(OR(E239="Abschreibung (AfA)",E239="Vorsteuer auf Anlagevermögen"),0,ROUND(F239*G239,2)))</f>
         <v/>
       </c>
       <c r="I239" s="22" t="str">
@@ -10344,7 +10415,7 @@
       <c r="F240" s="13"/>
       <c r="G240" s="21"/>
       <c r="H240" s="22" t="str">
-        <f aca="false">IF(F240="","",ROUND(F240*G240,2))</f>
+        <f>IF(F240="","",IF(OR(E240="Abschreibung (AfA)",E240="Vorsteuer auf Anlagevermögen"),0,ROUND(F240*G240,2)))</f>
         <v/>
       </c>
       <c r="I240" s="22" t="str">
@@ -10362,7 +10433,7 @@
       <c r="F241" s="13"/>
       <c r="G241" s="21"/>
       <c r="H241" s="22" t="str">
-        <f aca="false">IF(F241="","",ROUND(F241*G241,2))</f>
+        <f>IF(F241="","",IF(OR(E241="Abschreibung (AfA)",E241="Vorsteuer auf Anlagevermögen"),0,ROUND(F241*G241,2)))</f>
         <v/>
       </c>
       <c r="I241" s="22" t="str">
@@ -10380,7 +10451,7 @@
       <c r="F242" s="13"/>
       <c r="G242" s="21"/>
       <c r="H242" s="22" t="str">
-        <f aca="false">IF(F242="","",ROUND(F242*G242,2))</f>
+        <f>IF(F242="","",IF(OR(E242="Abschreibung (AfA)",E242="Vorsteuer auf Anlagevermögen"),0,ROUND(F242*G242,2)))</f>
         <v/>
       </c>
       <c r="I242" s="22" t="str">
@@ -10398,7 +10469,7 @@
       <c r="F243" s="13"/>
       <c r="G243" s="21"/>
       <c r="H243" s="22" t="str">
-        <f aca="false">IF(F243="","",ROUND(F243*G243,2))</f>
+        <f>IF(F243="","",IF(OR(E243="Abschreibung (AfA)",E243="Vorsteuer auf Anlagevermögen"),0,ROUND(F243*G243,2)))</f>
         <v/>
       </c>
       <c r="I243" s="22" t="str">
@@ -10416,7 +10487,7 @@
       <c r="F244" s="13"/>
       <c r="G244" s="21"/>
       <c r="H244" s="22" t="str">
-        <f aca="false">IF(F244="","",ROUND(F244*G244,2))</f>
+        <f>IF(F244="","",IF(OR(E244="Abschreibung (AfA)",E244="Vorsteuer auf Anlagevermögen"),0,ROUND(F244*G244,2)))</f>
         <v/>
       </c>
       <c r="I244" s="22" t="str">
@@ -10434,7 +10505,7 @@
       <c r="F245" s="13"/>
       <c r="G245" s="21"/>
       <c r="H245" s="22" t="str">
-        <f aca="false">IF(F245="","",ROUND(F245*G245,2))</f>
+        <f>IF(F245="","",IF(OR(E245="Abschreibung (AfA)",E245="Vorsteuer auf Anlagevermögen"),0,ROUND(F245*G245,2)))</f>
         <v/>
       </c>
       <c r="I245" s="22" t="str">
@@ -10452,7 +10523,7 @@
       <c r="F246" s="13"/>
       <c r="G246" s="21"/>
       <c r="H246" s="22" t="str">
-        <f aca="false">IF(F246="","",ROUND(F246*G246,2))</f>
+        <f>IF(F246="","",IF(OR(E246="Abschreibung (AfA)",E246="Vorsteuer auf Anlagevermögen"),0,ROUND(F246*G246,2)))</f>
         <v/>
       </c>
       <c r="I246" s="22" t="str">
@@ -10470,7 +10541,7 @@
       <c r="F247" s="13"/>
       <c r="G247" s="21"/>
       <c r="H247" s="22" t="str">
-        <f aca="false">IF(F247="","",ROUND(F247*G247,2))</f>
+        <f>IF(F247="","",IF(OR(E247="Abschreibung (AfA)",E247="Vorsteuer auf Anlagevermögen"),0,ROUND(F247*G247,2)))</f>
         <v/>
       </c>
       <c r="I247" s="22" t="str">
@@ -10488,7 +10559,7 @@
       <c r="F248" s="13"/>
       <c r="G248" s="21"/>
       <c r="H248" s="22" t="str">
-        <f aca="false">IF(F248="","",ROUND(F248*G248,2))</f>
+        <f>IF(F248="","",IF(OR(E248="Abschreibung (AfA)",E248="Vorsteuer auf Anlagevermögen"),0,ROUND(F248*G248,2)))</f>
         <v/>
       </c>
       <c r="I248" s="22" t="str">
@@ -10506,7 +10577,7 @@
       <c r="F249" s="13"/>
       <c r="G249" s="21"/>
       <c r="H249" s="22" t="str">
-        <f aca="false">IF(F249="","",ROUND(F249*G249,2))</f>
+        <f>IF(F249="","",IF(OR(E249="Abschreibung (AfA)",E249="Vorsteuer auf Anlagevermögen"),0,ROUND(F249*G249,2)))</f>
         <v/>
       </c>
       <c r="I249" s="22" t="str">
@@ -10524,7 +10595,7 @@
       <c r="F250" s="13"/>
       <c r="G250" s="21"/>
       <c r="H250" s="22" t="str">
-        <f aca="false">IF(F250="","",ROUND(F250*G250,2))</f>
+        <f>IF(F250="","",IF(OR(E250="Abschreibung (AfA)",E250="Vorsteuer auf Anlagevermögen"),0,ROUND(F250*G250,2)))</f>
         <v/>
       </c>
       <c r="I250" s="22" t="str">
@@ -10542,7 +10613,7 @@
       <c r="F251" s="13"/>
       <c r="G251" s="21"/>
       <c r="H251" s="22" t="str">
-        <f aca="false">IF(F251="","",ROUND(F251*G251,2))</f>
+        <f>IF(F251="","",IF(OR(E251="Abschreibung (AfA)",E251="Vorsteuer auf Anlagevermögen"),0,ROUND(F251*G251,2)))</f>
         <v/>
       </c>
       <c r="I251" s="22" t="str">
@@ -10560,7 +10631,7 @@
       <c r="F252" s="13"/>
       <c r="G252" s="21"/>
       <c r="H252" s="22" t="str">
-        <f aca="false">IF(F252="","",ROUND(F252*G252,2))</f>
+        <f>IF(F252="","",IF(OR(E252="Abschreibung (AfA)",E252="Vorsteuer auf Anlagevermögen"),0,ROUND(F252*G252,2)))</f>
         <v/>
       </c>
       <c r="I252" s="22" t="str">
@@ -10578,7 +10649,7 @@
       <c r="F253" s="13"/>
       <c r="G253" s="21"/>
       <c r="H253" s="22" t="str">
-        <f aca="false">IF(F253="","",ROUND(F253*G253,2))</f>
+        <f>IF(F253="","",IF(OR(E253="Abschreibung (AfA)",E253="Vorsteuer auf Anlagevermögen"),0,ROUND(F253*G253,2)))</f>
         <v/>
       </c>
       <c r="I253" s="22" t="str">
@@ -10596,7 +10667,7 @@
       <c r="F254" s="13"/>
       <c r="G254" s="21"/>
       <c r="H254" s="22" t="str">
-        <f aca="false">IF(F254="","",ROUND(F254*G254,2))</f>
+        <f>IF(F254="","",IF(OR(E254="Abschreibung (AfA)",E254="Vorsteuer auf Anlagevermögen"),0,ROUND(F254*G254,2)))</f>
         <v/>
       </c>
       <c r="I254" s="22" t="str">
@@ -10614,7 +10685,7 @@
       <c r="F255" s="13"/>
       <c r="G255" s="21"/>
       <c r="H255" s="22" t="str">
-        <f aca="false">IF(F255="","",ROUND(F255*G255,2))</f>
+        <f>IF(F255="","",IF(OR(E255="Abschreibung (AfA)",E255="Vorsteuer auf Anlagevermögen"),0,ROUND(F255*G255,2)))</f>
         <v/>
       </c>
       <c r="I255" s="22" t="str">
@@ -10632,7 +10703,7 @@
       <c r="F256" s="13"/>
       <c r="G256" s="21"/>
       <c r="H256" s="22" t="str">
-        <f aca="false">IF(F256="","",ROUND(F256*G256,2))</f>
+        <f>IF(F256="","",IF(OR(E256="Abschreibung (AfA)",E256="Vorsteuer auf Anlagevermögen"),0,ROUND(F256*G256,2)))</f>
         <v/>
       </c>
       <c r="I256" s="22" t="str">
@@ -10650,7 +10721,7 @@
       <c r="F257" s="13"/>
       <c r="G257" s="21"/>
       <c r="H257" s="22" t="str">
-        <f aca="false">IF(F257="","",ROUND(F257*G257,2))</f>
+        <f>IF(F257="","",IF(OR(E257="Abschreibung (AfA)",E257="Vorsteuer auf Anlagevermögen"),0,ROUND(F257*G257,2)))</f>
         <v/>
       </c>
       <c r="I257" s="22" t="str">
@@ -10668,7 +10739,7 @@
       <c r="F258" s="13"/>
       <c r="G258" s="21"/>
       <c r="H258" s="22" t="str">
-        <f aca="false">IF(F258="","",ROUND(F258*G258,2))</f>
+        <f>IF(F258="","",IF(OR(E258="Abschreibung (AfA)",E258="Vorsteuer auf Anlagevermögen"),0,ROUND(F258*G258,2)))</f>
         <v/>
       </c>
       <c r="I258" s="22" t="str">
@@ -10686,7 +10757,7 @@
       <c r="F259" s="13"/>
       <c r="G259" s="21"/>
       <c r="H259" s="22" t="str">
-        <f aca="false">IF(F259="","",ROUND(F259*G259,2))</f>
+        <f>IF(F259="","",IF(OR(E259="Abschreibung (AfA)",E259="Vorsteuer auf Anlagevermögen"),0,ROUND(F259*G259,2)))</f>
         <v/>
       </c>
       <c r="I259" s="22" t="str">
@@ -10704,7 +10775,7 @@
       <c r="F260" s="13"/>
       <c r="G260" s="21"/>
       <c r="H260" s="22" t="str">
-        <f aca="false">IF(F260="","",ROUND(F260*G260,2))</f>
+        <f>IF(F260="","",IF(OR(E260="Abschreibung (AfA)",E260="Vorsteuer auf Anlagevermögen"),0,ROUND(F260*G260,2)))</f>
         <v/>
       </c>
       <c r="I260" s="22" t="str">
@@ -10722,7 +10793,7 @@
       <c r="F261" s="13"/>
       <c r="G261" s="21"/>
       <c r="H261" s="22" t="str">
-        <f aca="false">IF(F261="","",ROUND(F261*G261,2))</f>
+        <f>IF(F261="","",IF(OR(E261="Abschreibung (AfA)",E261="Vorsteuer auf Anlagevermögen"),0,ROUND(F261*G261,2)))</f>
         <v/>
       </c>
       <c r="I261" s="22" t="str">
@@ -10740,7 +10811,7 @@
       <c r="F262" s="13"/>
       <c r="G262" s="21"/>
       <c r="H262" s="22" t="str">
-        <f aca="false">IF(F262="","",ROUND(F262*G262,2))</f>
+        <f>IF(F262="","",IF(OR(E262="Abschreibung (AfA)",E262="Vorsteuer auf Anlagevermögen"),0,ROUND(F262*G262,2)))</f>
         <v/>
       </c>
       <c r="I262" s="22" t="str">
@@ -10758,7 +10829,7 @@
       <c r="F263" s="13"/>
       <c r="G263" s="21"/>
       <c r="H263" s="22" t="str">
-        <f aca="false">IF(F263="","",ROUND(F263*G263,2))</f>
+        <f>IF(F263="","",IF(OR(E263="Abschreibung (AfA)",E263="Vorsteuer auf Anlagevermögen"),0,ROUND(F263*G263,2)))</f>
         <v/>
       </c>
       <c r="I263" s="22" t="str">
@@ -10776,7 +10847,7 @@
       <c r="F264" s="13"/>
       <c r="G264" s="21"/>
       <c r="H264" s="22" t="str">
-        <f aca="false">IF(F264="","",ROUND(F264*G264,2))</f>
+        <f>IF(F264="","",IF(OR(E264="Abschreibung (AfA)",E264="Vorsteuer auf Anlagevermögen"),0,ROUND(F264*G264,2)))</f>
         <v/>
       </c>
       <c r="I264" s="22" t="str">
@@ -10794,7 +10865,7 @@
       <c r="F265" s="13"/>
       <c r="G265" s="21"/>
       <c r="H265" s="22" t="str">
-        <f aca="false">IF(F265="","",ROUND(F265*G265,2))</f>
+        <f>IF(F265="","",IF(OR(E265="Abschreibung (AfA)",E265="Vorsteuer auf Anlagevermögen"),0,ROUND(F265*G265,2)))</f>
         <v/>
       </c>
       <c r="I265" s="22" t="str">
@@ -10812,7 +10883,7 @@
       <c r="F266" s="13"/>
       <c r="G266" s="21"/>
       <c r="H266" s="22" t="str">
-        <f aca="false">IF(F266="","",ROUND(F266*G266,2))</f>
+        <f>IF(F266="","",IF(OR(E266="Abschreibung (AfA)",E266="Vorsteuer auf Anlagevermögen"),0,ROUND(F266*G266,2)))</f>
         <v/>
       </c>
       <c r="I266" s="22" t="str">
@@ -10830,7 +10901,7 @@
       <c r="F267" s="13"/>
       <c r="G267" s="21"/>
       <c r="H267" s="22" t="str">
-        <f aca="false">IF(F267="","",ROUND(F267*G267,2))</f>
+        <f>IF(F267="","",IF(OR(E267="Abschreibung (AfA)",E267="Vorsteuer auf Anlagevermögen"),0,ROUND(F267*G267,2)))</f>
         <v/>
       </c>
       <c r="I267" s="22" t="str">
@@ -10848,7 +10919,7 @@
       <c r="F268" s="13"/>
       <c r="G268" s="21"/>
       <c r="H268" s="22" t="str">
-        <f aca="false">IF(F268="","",ROUND(F268*G268,2))</f>
+        <f>IF(F268="","",IF(OR(E268="Abschreibung (AfA)",E268="Vorsteuer auf Anlagevermögen"),0,ROUND(F268*G268,2)))</f>
         <v/>
       </c>
       <c r="I268" s="22" t="str">
@@ -10866,7 +10937,7 @@
       <c r="F269" s="13"/>
       <c r="G269" s="21"/>
       <c r="H269" s="22" t="str">
-        <f aca="false">IF(F269="","",ROUND(F269*G269,2))</f>
+        <f>IF(F269="","",IF(OR(E269="Abschreibung (AfA)",E269="Vorsteuer auf Anlagevermögen"),0,ROUND(F269*G269,2)))</f>
         <v/>
       </c>
       <c r="I269" s="22" t="str">
@@ -10884,7 +10955,7 @@
       <c r="F270" s="13"/>
       <c r="G270" s="21"/>
       <c r="H270" s="22" t="str">
-        <f aca="false">IF(F270="","",ROUND(F270*G270,2))</f>
+        <f>IF(F270="","",IF(OR(E270="Abschreibung (AfA)",E270="Vorsteuer auf Anlagevermögen"),0,ROUND(F270*G270,2)))</f>
         <v/>
       </c>
       <c r="I270" s="22" t="str">
@@ -10902,7 +10973,7 @@
       <c r="F271" s="13"/>
       <c r="G271" s="21"/>
       <c r="H271" s="22" t="str">
-        <f aca="false">IF(F271="","",ROUND(F271*G271,2))</f>
+        <f>IF(F271="","",IF(OR(E271="Abschreibung (AfA)",E271="Vorsteuer auf Anlagevermögen"),0,ROUND(F271*G271,2)))</f>
         <v/>
       </c>
       <c r="I271" s="22" t="str">
@@ -10920,7 +10991,7 @@
       <c r="F272" s="13"/>
       <c r="G272" s="21"/>
       <c r="H272" s="22" t="str">
-        <f aca="false">IF(F272="","",ROUND(F272*G272,2))</f>
+        <f>IF(F272="","",IF(OR(E272="Abschreibung (AfA)",E272="Vorsteuer auf Anlagevermögen"),0,ROUND(F272*G272,2)))</f>
         <v/>
       </c>
       <c r="I272" s="22" t="str">
@@ -10938,7 +11009,7 @@
       <c r="F273" s="13"/>
       <c r="G273" s="21"/>
       <c r="H273" s="22" t="str">
-        <f aca="false">IF(F273="","",ROUND(F273*G273,2))</f>
+        <f>IF(F273="","",IF(OR(E273="Abschreibung (AfA)",E273="Vorsteuer auf Anlagevermögen"),0,ROUND(F273*G273,2)))</f>
         <v/>
       </c>
       <c r="I273" s="22" t="str">
@@ -10956,7 +11027,7 @@
       <c r="F274" s="13"/>
       <c r="G274" s="21"/>
       <c r="H274" s="22" t="str">
-        <f aca="false">IF(F274="","",ROUND(F274*G274,2))</f>
+        <f>IF(F274="","",IF(OR(E274="Abschreibung (AfA)",E274="Vorsteuer auf Anlagevermögen"),0,ROUND(F274*G274,2)))</f>
         <v/>
       </c>
       <c r="I274" s="22" t="str">
@@ -10974,7 +11045,7 @@
       <c r="F275" s="13"/>
       <c r="G275" s="21"/>
       <c r="H275" s="22" t="str">
-        <f aca="false">IF(F275="","",ROUND(F275*G275,2))</f>
+        <f>IF(F275="","",IF(OR(E275="Abschreibung (AfA)",E275="Vorsteuer auf Anlagevermögen"),0,ROUND(F275*G275,2)))</f>
         <v/>
       </c>
       <c r="I275" s="22" t="str">
@@ -10992,7 +11063,7 @@
       <c r="F276" s="13"/>
       <c r="G276" s="21"/>
       <c r="H276" s="22" t="str">
-        <f aca="false">IF(F276="","",ROUND(F276*G276,2))</f>
+        <f>IF(F276="","",IF(OR(E276="Abschreibung (AfA)",E276="Vorsteuer auf Anlagevermögen"),0,ROUND(F276*G276,2)))</f>
         <v/>
       </c>
       <c r="I276" s="22" t="str">
@@ -11010,7 +11081,7 @@
       <c r="F277" s="13"/>
       <c r="G277" s="21"/>
       <c r="H277" s="22" t="str">
-        <f aca="false">IF(F277="","",ROUND(F277*G277,2))</f>
+        <f>IF(F277="","",IF(OR(E277="Abschreibung (AfA)",E277="Vorsteuer auf Anlagevermögen"),0,ROUND(F277*G277,2)))</f>
         <v/>
       </c>
       <c r="I277" s="22" t="str">
@@ -11028,7 +11099,7 @@
       <c r="F278" s="13"/>
       <c r="G278" s="21"/>
       <c r="H278" s="22" t="str">
-        <f aca="false">IF(F278="","",ROUND(F278*G278,2))</f>
+        <f>IF(F278="","",IF(OR(E278="Abschreibung (AfA)",E278="Vorsteuer auf Anlagevermögen"),0,ROUND(F278*G278,2)))</f>
         <v/>
       </c>
       <c r="I278" s="22" t="str">
@@ -11046,7 +11117,7 @@
       <c r="F279" s="13"/>
       <c r="G279" s="21"/>
       <c r="H279" s="22" t="str">
-        <f aca="false">IF(F279="","",ROUND(F279*G279,2))</f>
+        <f>IF(F279="","",IF(OR(E279="Abschreibung (AfA)",E279="Vorsteuer auf Anlagevermögen"),0,ROUND(F279*G279,2)))</f>
         <v/>
       </c>
       <c r="I279" s="22" t="str">
@@ -11064,7 +11135,7 @@
       <c r="F280" s="13"/>
       <c r="G280" s="21"/>
       <c r="H280" s="22" t="str">
-        <f aca="false">IF(F280="","",ROUND(F280*G280,2))</f>
+        <f>IF(F280="","",IF(OR(E280="Abschreibung (AfA)",E280="Vorsteuer auf Anlagevermögen"),0,ROUND(F280*G280,2)))</f>
         <v/>
       </c>
       <c r="I280" s="22" t="str">
@@ -11082,7 +11153,7 @@
       <c r="F281" s="13"/>
       <c r="G281" s="21"/>
       <c r="H281" s="22" t="str">
-        <f aca="false">IF(F281="","",ROUND(F281*G281,2))</f>
+        <f>IF(F281="","",IF(OR(E281="Abschreibung (AfA)",E281="Vorsteuer auf Anlagevermögen"),0,ROUND(F281*G281,2)))</f>
         <v/>
       </c>
       <c r="I281" s="22" t="str">
@@ -11100,7 +11171,7 @@
       <c r="F282" s="13"/>
       <c r="G282" s="21"/>
       <c r="H282" s="22" t="str">
-        <f aca="false">IF(F282="","",ROUND(F282*G282,2))</f>
+        <f>IF(F282="","",IF(OR(E282="Abschreibung (AfA)",E282="Vorsteuer auf Anlagevermögen"),0,ROUND(F282*G282,2)))</f>
         <v/>
       </c>
       <c r="I282" s="22" t="str">
@@ -11118,7 +11189,7 @@
       <c r="F283" s="13"/>
       <c r="G283" s="21"/>
       <c r="H283" s="22" t="str">
-        <f aca="false">IF(F283="","",ROUND(F283*G283,2))</f>
+        <f>IF(F283="","",IF(OR(E283="Abschreibung (AfA)",E283="Vorsteuer auf Anlagevermögen"),0,ROUND(F283*G283,2)))</f>
         <v/>
       </c>
       <c r="I283" s="22" t="str">
@@ -11136,7 +11207,7 @@
       <c r="F284" s="13"/>
       <c r="G284" s="21"/>
       <c r="H284" s="22" t="str">
-        <f aca="false">IF(F284="","",ROUND(F284*G284,2))</f>
+        <f>IF(F284="","",IF(OR(E284="Abschreibung (AfA)",E284="Vorsteuer auf Anlagevermögen"),0,ROUND(F284*G284,2)))</f>
         <v/>
       </c>
       <c r="I284" s="22" t="str">
@@ -11154,7 +11225,7 @@
       <c r="F285" s="13"/>
       <c r="G285" s="21"/>
       <c r="H285" s="22" t="str">
-        <f aca="false">IF(F285="","",ROUND(F285*G285,2))</f>
+        <f>IF(F285="","",IF(OR(E285="Abschreibung (AfA)",E285="Vorsteuer auf Anlagevermögen"),0,ROUND(F285*G285,2)))</f>
         <v/>
       </c>
       <c r="I285" s="22" t="str">
@@ -11172,7 +11243,7 @@
       <c r="F286" s="13"/>
       <c r="G286" s="21"/>
       <c r="H286" s="22" t="str">
-        <f aca="false">IF(F286="","",ROUND(F286*G286,2))</f>
+        <f>IF(F286="","",IF(OR(E286="Abschreibung (AfA)",E286="Vorsteuer auf Anlagevermögen"),0,ROUND(F286*G286,2)))</f>
         <v/>
       </c>
       <c r="I286" s="22" t="str">
@@ -11190,7 +11261,7 @@
       <c r="F287" s="13"/>
       <c r="G287" s="21"/>
       <c r="H287" s="22" t="str">
-        <f aca="false">IF(F287="","",ROUND(F287*G287,2))</f>
+        <f>IF(F287="","",IF(OR(E287="Abschreibung (AfA)",E287="Vorsteuer auf Anlagevermögen"),0,ROUND(F287*G287,2)))</f>
         <v/>
       </c>
       <c r="I287" s="22" t="str">
@@ -11208,7 +11279,7 @@
       <c r="F288" s="13"/>
       <c r="G288" s="21"/>
       <c r="H288" s="22" t="str">
-        <f aca="false">IF(F288="","",ROUND(F288*G288,2))</f>
+        <f>IF(F288="","",IF(OR(E288="Abschreibung (AfA)",E288="Vorsteuer auf Anlagevermögen"),0,ROUND(F288*G288,2)))</f>
         <v/>
       </c>
       <c r="I288" s="22" t="str">
@@ -11226,7 +11297,7 @@
       <c r="F289" s="13"/>
       <c r="G289" s="21"/>
       <c r="H289" s="22" t="str">
-        <f aca="false">IF(F289="","",ROUND(F289*G289,2))</f>
+        <f>IF(F289="","",IF(OR(E289="Abschreibung (AfA)",E289="Vorsteuer auf Anlagevermögen"),0,ROUND(F289*G289,2)))</f>
         <v/>
       </c>
       <c r="I289" s="22" t="str">
@@ -11244,7 +11315,7 @@
       <c r="F290" s="13"/>
       <c r="G290" s="21"/>
       <c r="H290" s="22" t="str">
-        <f aca="false">IF(F290="","",ROUND(F290*G290,2))</f>
+        <f>IF(F290="","",IF(OR(E290="Abschreibung (AfA)",E290="Vorsteuer auf Anlagevermögen"),0,ROUND(F290*G290,2)))</f>
         <v/>
       </c>
       <c r="I290" s="22" t="str">
@@ -11262,7 +11333,7 @@
       <c r="F291" s="13"/>
       <c r="G291" s="21"/>
       <c r="H291" s="22" t="str">
-        <f aca="false">IF(F291="","",ROUND(F291*G291,2))</f>
+        <f>IF(F291="","",IF(OR(E291="Abschreibung (AfA)",E291="Vorsteuer auf Anlagevermögen"),0,ROUND(F291*G291,2)))</f>
         <v/>
       </c>
       <c r="I291" s="22" t="str">
@@ -11280,7 +11351,7 @@
       <c r="F292" s="13"/>
       <c r="G292" s="21"/>
       <c r="H292" s="22" t="str">
-        <f aca="false">IF(F292="","",ROUND(F292*G292,2))</f>
+        <f>IF(F292="","",IF(OR(E292="Abschreibung (AfA)",E292="Vorsteuer auf Anlagevermögen"),0,ROUND(F292*G292,2)))</f>
         <v/>
       </c>
       <c r="I292" s="22" t="str">
@@ -11298,7 +11369,7 @@
       <c r="F293" s="13"/>
       <c r="G293" s="21"/>
       <c r="H293" s="22" t="str">
-        <f aca="false">IF(F293="","",ROUND(F293*G293,2))</f>
+        <f>IF(F293="","",IF(OR(E293="Abschreibung (AfA)",E293="Vorsteuer auf Anlagevermögen"),0,ROUND(F293*G293,2)))</f>
         <v/>
       </c>
       <c r="I293" s="22" t="str">
@@ -11316,7 +11387,7 @@
       <c r="F294" s="13"/>
       <c r="G294" s="21"/>
       <c r="H294" s="22" t="str">
-        <f aca="false">IF(F294="","",ROUND(F294*G294,2))</f>
+        <f>IF(F294="","",IF(OR(E294="Abschreibung (AfA)",E294="Vorsteuer auf Anlagevermögen"),0,ROUND(F294*G294,2)))</f>
         <v/>
       </c>
       <c r="I294" s="22" t="str">
@@ -11334,7 +11405,7 @@
       <c r="F295" s="13"/>
       <c r="G295" s="21"/>
       <c r="H295" s="22" t="str">
-        <f aca="false">IF(F295="","",ROUND(F295*G295,2))</f>
+        <f>IF(F295="","",IF(OR(E295="Abschreibung (AfA)",E295="Vorsteuer auf Anlagevermögen"),0,ROUND(F295*G295,2)))</f>
         <v/>
       </c>
       <c r="I295" s="22" t="str">
@@ -11352,7 +11423,7 @@
       <c r="F296" s="13"/>
       <c r="G296" s="21"/>
       <c r="H296" s="22" t="str">
-        <f aca="false">IF(F296="","",ROUND(F296*G296,2))</f>
+        <f>IF(F296="","",IF(OR(E296="Abschreibung (AfA)",E296="Vorsteuer auf Anlagevermögen"),0,ROUND(F296*G296,2)))</f>
         <v/>
       </c>
       <c r="I296" s="22" t="str">
@@ -11370,7 +11441,7 @@
       <c r="F297" s="13"/>
       <c r="G297" s="21"/>
       <c r="H297" s="22" t="str">
-        <f aca="false">IF(F297="","",ROUND(F297*G297,2))</f>
+        <f>IF(F297="","",IF(OR(E297="Abschreibung (AfA)",E297="Vorsteuer auf Anlagevermögen"),0,ROUND(F297*G297,2)))</f>
         <v/>
       </c>
       <c r="I297" s="22" t="str">
@@ -11388,7 +11459,7 @@
       <c r="F298" s="13"/>
       <c r="G298" s="21"/>
       <c r="H298" s="22" t="str">
-        <f aca="false">IF(F298="","",ROUND(F298*G298,2))</f>
+        <f>IF(F298="","",IF(OR(E298="Abschreibung (AfA)",E298="Vorsteuer auf Anlagevermögen"),0,ROUND(F298*G298,2)))</f>
         <v/>
       </c>
       <c r="I298" s="22" t="str">
@@ -11406,7 +11477,7 @@
       <c r="F299" s="13"/>
       <c r="G299" s="21"/>
       <c r="H299" s="22" t="str">
-        <f aca="false">IF(F299="","",ROUND(F299*G299,2))</f>
+        <f>IF(F299="","",IF(OR(E299="Abschreibung (AfA)",E299="Vorsteuer auf Anlagevermögen"),0,ROUND(F299*G299,2)))</f>
         <v/>
       </c>
       <c r="I299" s="22" t="str">
@@ -11424,7 +11495,7 @@
       <c r="F300" s="13"/>
       <c r="G300" s="21"/>
       <c r="H300" s="22" t="str">
-        <f aca="false">IF(F300="","",ROUND(F300*G300,2))</f>
+        <f>IF(F300="","",IF(OR(E300="Abschreibung (AfA)",E300="Vorsteuer auf Anlagevermögen"),0,ROUND(F300*G300,2)))</f>
         <v/>
       </c>
       <c r="I300" s="22" t="str">
@@ -11442,7 +11513,7 @@
       <c r="F301" s="13"/>
       <c r="G301" s="21"/>
       <c r="H301" s="22" t="str">
-        <f aca="false">IF(F301="","",ROUND(F301*G301,2))</f>
+        <f>IF(F301="","",IF(OR(E301="Abschreibung (AfA)",E301="Vorsteuer auf Anlagevermögen"),0,ROUND(F301*G301,2)))</f>
         <v/>
       </c>
       <c r="I301" s="22" t="str">
@@ -11460,7 +11531,7 @@
       <c r="F302" s="13"/>
       <c r="G302" s="21"/>
       <c r="H302" s="22" t="str">
-        <f aca="false">IF(F302="","",ROUND(F302*G302,2))</f>
+        <f>IF(F302="","",IF(OR(E302="Abschreibung (AfA)",E302="Vorsteuer auf Anlagevermögen"),0,ROUND(F302*G302,2)))</f>
         <v/>
       </c>
       <c r="I302" s="22" t="str">
@@ -11478,7 +11549,7 @@
       <c r="F303" s="13"/>
       <c r="G303" s="21"/>
       <c r="H303" s="22" t="str">
-        <f aca="false">IF(F303="","",ROUND(F303*G303,2))</f>
+        <f>IF(F303="","",IF(OR(E303="Abschreibung (AfA)",E303="Vorsteuer auf Anlagevermögen"),0,ROUND(F303*G303,2)))</f>
         <v/>
       </c>
       <c r="I303" s="22" t="str">
@@ -11496,7 +11567,7 @@
       <c r="F304" s="13"/>
       <c r="G304" s="21"/>
       <c r="H304" s="22" t="str">
-        <f aca="false">IF(F304="","",ROUND(F304*G304,2))</f>
+        <f>IF(F304="","",IF(OR(E304="Abschreibung (AfA)",E304="Vorsteuer auf Anlagevermögen"),0,ROUND(F304*G304,2)))</f>
         <v/>
       </c>
       <c r="I304" s="22" t="str">
@@ -11514,7 +11585,7 @@
       <c r="F305" s="13"/>
       <c r="G305" s="21"/>
       <c r="H305" s="22" t="str">
-        <f aca="false">IF(F305="","",ROUND(F305*G305,2))</f>
+        <f>IF(F305="","",IF(OR(E305="Abschreibung (AfA)",E305="Vorsteuer auf Anlagevermögen"),0,ROUND(F305*G305,2)))</f>
         <v/>
       </c>
       <c r="I305" s="22" t="str">
@@ -11532,7 +11603,7 @@
       <c r="F306" s="13"/>
       <c r="G306" s="21"/>
       <c r="H306" s="22" t="str">
-        <f aca="false">IF(F306="","",ROUND(F306*G306,2))</f>
+        <f>IF(F306="","",IF(OR(E306="Abschreibung (AfA)",E306="Vorsteuer auf Anlagevermögen"),0,ROUND(F306*G306,2)))</f>
         <v/>
       </c>
       <c r="I306" s="22" t="str">
@@ -11550,7 +11621,7 @@
       <c r="F307" s="13"/>
       <c r="G307" s="21"/>
       <c r="H307" s="22" t="str">
-        <f aca="false">IF(F307="","",ROUND(F307*G307,2))</f>
+        <f>IF(F307="","",IF(OR(E307="Abschreibung (AfA)",E307="Vorsteuer auf Anlagevermögen"),0,ROUND(F307*G307,2)))</f>
         <v/>
       </c>
       <c r="I307" s="22" t="str">
@@ -11568,7 +11639,7 @@
       <c r="F308" s="13"/>
       <c r="G308" s="21"/>
       <c r="H308" s="22" t="str">
-        <f aca="false">IF(F308="","",ROUND(F308*G308,2))</f>
+        <f>IF(F308="","",IF(OR(E308="Abschreibung (AfA)",E308="Vorsteuer auf Anlagevermögen"),0,ROUND(F308*G308,2)))</f>
         <v/>
       </c>
       <c r="I308" s="22" t="str">
@@ -11586,7 +11657,7 @@
       <c r="F309" s="13"/>
       <c r="G309" s="21"/>
       <c r="H309" s="22" t="str">
-        <f aca="false">IF(F309="","",ROUND(F309*G309,2))</f>
+        <f>IF(F309="","",IF(OR(E309="Abschreibung (AfA)",E309="Vorsteuer auf Anlagevermögen"),0,ROUND(F309*G309,2)))</f>
         <v/>
       </c>
       <c r="I309" s="22" t="str">
@@ -11604,7 +11675,7 @@
       <c r="F310" s="13"/>
       <c r="G310" s="21"/>
       <c r="H310" s="22" t="str">
-        <f aca="false">IF(F310="","",ROUND(F310*G310,2))</f>
+        <f>IF(F310="","",IF(OR(E310="Abschreibung (AfA)",E310="Vorsteuer auf Anlagevermögen"),0,ROUND(F310*G310,2)))</f>
         <v/>
       </c>
       <c r="I310" s="22" t="str">
@@ -11622,7 +11693,7 @@
       <c r="F311" s="13"/>
       <c r="G311" s="21"/>
       <c r="H311" s="22" t="str">
-        <f aca="false">IF(F311="","",ROUND(F311*G311,2))</f>
+        <f>IF(F311="","",IF(OR(E311="Abschreibung (AfA)",E311="Vorsteuer auf Anlagevermögen"),0,ROUND(F311*G311,2)))</f>
         <v/>
       </c>
       <c r="I311" s="22" t="str">
@@ -11640,7 +11711,7 @@
       <c r="F312" s="13"/>
       <c r="G312" s="21"/>
       <c r="H312" s="22" t="str">
-        <f aca="false">IF(F312="","",ROUND(F312*G312,2))</f>
+        <f>IF(F312="","",IF(OR(E312="Abschreibung (AfA)",E312="Vorsteuer auf Anlagevermögen"),0,ROUND(F312*G312,2)))</f>
         <v/>
       </c>
       <c r="I312" s="22" t="str">
@@ -11658,7 +11729,7 @@
       <c r="F313" s="13"/>
       <c r="G313" s="21"/>
       <c r="H313" s="22" t="str">
-        <f aca="false">IF(F313="","",ROUND(F313*G313,2))</f>
+        <f>IF(F313="","",IF(OR(E313="Abschreibung (AfA)",E313="Vorsteuer auf Anlagevermögen"),0,ROUND(F313*G313,2)))</f>
         <v/>
       </c>
       <c r="I313" s="22" t="str">
@@ -11676,7 +11747,7 @@
       <c r="F314" s="13"/>
       <c r="G314" s="21"/>
       <c r="H314" s="22" t="str">
-        <f aca="false">IF(F314="","",ROUND(F314*G314,2))</f>
+        <f>IF(F314="","",IF(OR(E314="Abschreibung (AfA)",E314="Vorsteuer auf Anlagevermögen"),0,ROUND(F314*G314,2)))</f>
         <v/>
       </c>
       <c r="I314" s="22" t="str">
@@ -11694,7 +11765,7 @@
       <c r="F315" s="13"/>
       <c r="G315" s="21"/>
       <c r="H315" s="22" t="str">
-        <f aca="false">IF(F315="","",ROUND(F315*G315,2))</f>
+        <f>IF(F315="","",IF(OR(E315="Abschreibung (AfA)",E315="Vorsteuer auf Anlagevermögen"),0,ROUND(F315*G315,2)))</f>
         <v/>
       </c>
       <c r="I315" s="22" t="str">
@@ -11712,7 +11783,7 @@
       <c r="F316" s="13"/>
       <c r="G316" s="21"/>
       <c r="H316" s="22" t="str">
-        <f aca="false">IF(F316="","",ROUND(F316*G316,2))</f>
+        <f>IF(F316="","",IF(OR(E316="Abschreibung (AfA)",E316="Vorsteuer auf Anlagevermögen"),0,ROUND(F316*G316,2)))</f>
         <v/>
       </c>
       <c r="I316" s="22" t="str">
@@ -11730,7 +11801,7 @@
       <c r="F317" s="13"/>
       <c r="G317" s="21"/>
       <c r="H317" s="22" t="str">
-        <f aca="false">IF(F317="","",ROUND(F317*G317,2))</f>
+        <f>IF(F317="","",IF(OR(E317="Abschreibung (AfA)",E317="Vorsteuer auf Anlagevermögen"),0,ROUND(F317*G317,2)))</f>
         <v/>
       </c>
       <c r="I317" s="22" t="str">
@@ -11748,7 +11819,7 @@
       <c r="F318" s="13"/>
       <c r="G318" s="21"/>
       <c r="H318" s="22" t="str">
-        <f aca="false">IF(F318="","",ROUND(F318*G318,2))</f>
+        <f>IF(F318="","",IF(OR(E318="Abschreibung (AfA)",E318="Vorsteuer auf Anlagevermögen"),0,ROUND(F318*G318,2)))</f>
         <v/>
       </c>
       <c r="I318" s="22" t="str">
@@ -11766,7 +11837,7 @@
       <c r="F319" s="13"/>
       <c r="G319" s="21"/>
       <c r="H319" s="22" t="str">
-        <f aca="false">IF(F319="","",ROUND(F319*G319,2))</f>
+        <f>IF(F319="","",IF(OR(E319="Abschreibung (AfA)",E319="Vorsteuer auf Anlagevermögen"),0,ROUND(F319*G319,2)))</f>
         <v/>
       </c>
       <c r="I319" s="22" t="str">
@@ -11784,7 +11855,7 @@
       <c r="F320" s="13"/>
       <c r="G320" s="21"/>
       <c r="H320" s="22" t="str">
-        <f aca="false">IF(F320="","",ROUND(F320*G320,2))</f>
+        <f>IF(F320="","",IF(OR(E320="Abschreibung (AfA)",E320="Vorsteuer auf Anlagevermögen"),0,ROUND(F320*G320,2)))</f>
         <v/>
       </c>
       <c r="I320" s="22" t="str">
@@ -11802,7 +11873,7 @@
       <c r="F321" s="13"/>
       <c r="G321" s="21"/>
       <c r="H321" s="22" t="str">
-        <f aca="false">IF(F321="","",ROUND(F321*G321,2))</f>
+        <f>IF(F321="","",IF(OR(E321="Abschreibung (AfA)",E321="Vorsteuer auf Anlagevermögen"),0,ROUND(F321*G321,2)))</f>
         <v/>
       </c>
       <c r="I321" s="22" t="str">
@@ -11820,7 +11891,7 @@
       <c r="F322" s="13"/>
       <c r="G322" s="21"/>
       <c r="H322" s="22" t="str">
-        <f aca="false">IF(F322="","",ROUND(F322*G322,2))</f>
+        <f>IF(F322="","",IF(OR(E322="Abschreibung (AfA)",E322="Vorsteuer auf Anlagevermögen"),0,ROUND(F322*G322,2)))</f>
         <v/>
       </c>
       <c r="I322" s="22" t="str">
@@ -11838,7 +11909,7 @@
       <c r="F323" s="13"/>
       <c r="G323" s="21"/>
       <c r="H323" s="22" t="str">
-        <f aca="false">IF(F323="","",ROUND(F323*G323,2))</f>
+        <f>IF(F323="","",IF(OR(E323="Abschreibung (AfA)",E323="Vorsteuer auf Anlagevermögen"),0,ROUND(F323*G323,2)))</f>
         <v/>
       </c>
       <c r="I323" s="22" t="str">
@@ -11856,7 +11927,7 @@
       <c r="F324" s="13"/>
       <c r="G324" s="21"/>
       <c r="H324" s="22" t="str">
-        <f aca="false">IF(F324="","",ROUND(F324*G324,2))</f>
+        <f>IF(F324="","",IF(OR(E324="Abschreibung (AfA)",E324="Vorsteuer auf Anlagevermögen"),0,ROUND(F324*G324,2)))</f>
         <v/>
       </c>
       <c r="I324" s="22" t="str">
@@ -11874,7 +11945,7 @@
       <c r="F325" s="13"/>
       <c r="G325" s="21"/>
       <c r="H325" s="22" t="str">
-        <f aca="false">IF(F325="","",ROUND(F325*G325,2))</f>
+        <f>IF(F325="","",IF(OR(E325="Abschreibung (AfA)",E325="Vorsteuer auf Anlagevermögen"),0,ROUND(F325*G325,2)))</f>
         <v/>
       </c>
       <c r="I325" s="22" t="str">
@@ -11892,7 +11963,7 @@
       <c r="F326" s="13"/>
       <c r="G326" s="21"/>
       <c r="H326" s="22" t="str">
-        <f aca="false">IF(F326="","",ROUND(F326*G326,2))</f>
+        <f>IF(F326="","",IF(OR(E326="Abschreibung (AfA)",E326="Vorsteuer auf Anlagevermögen"),0,ROUND(F326*G326,2)))</f>
         <v/>
       </c>
       <c r="I326" s="22" t="str">
@@ -11910,7 +11981,7 @@
       <c r="F327" s="13"/>
       <c r="G327" s="21"/>
       <c r="H327" s="22" t="str">
-        <f aca="false">IF(F327="","",ROUND(F327*G327,2))</f>
+        <f>IF(F327="","",IF(OR(E327="Abschreibung (AfA)",E327="Vorsteuer auf Anlagevermögen"),0,ROUND(F327*G327,2)))</f>
         <v/>
       </c>
       <c r="I327" s="22" t="str">
@@ -11928,7 +11999,7 @@
       <c r="F328" s="13"/>
       <c r="G328" s="21"/>
       <c r="H328" s="22" t="str">
-        <f aca="false">IF(F328="","",ROUND(F328*G328,2))</f>
+        <f>IF(F328="","",IF(OR(E328="Abschreibung (AfA)",E328="Vorsteuer auf Anlagevermögen"),0,ROUND(F328*G328,2)))</f>
         <v/>
       </c>
       <c r="I328" s="22" t="str">
@@ -11946,7 +12017,7 @@
       <c r="F329" s="13"/>
       <c r="G329" s="21"/>
       <c r="H329" s="22" t="str">
-        <f aca="false">IF(F329="","",ROUND(F329*G329,2))</f>
+        <f>IF(F329="","",IF(OR(E329="Abschreibung (AfA)",E329="Vorsteuer auf Anlagevermögen"),0,ROUND(F329*G329,2)))</f>
         <v/>
       </c>
       <c r="I329" s="22" t="str">
@@ -11964,7 +12035,7 @@
       <c r="F330" s="13"/>
       <c r="G330" s="21"/>
       <c r="H330" s="22" t="str">
-        <f aca="false">IF(F330="","",ROUND(F330*G330,2))</f>
+        <f>IF(F330="","",IF(OR(E330="Abschreibung (AfA)",E330="Vorsteuer auf Anlagevermögen"),0,ROUND(F330*G330,2)))</f>
         <v/>
       </c>
       <c r="I330" s="22" t="str">
@@ -11982,7 +12053,7 @@
       <c r="F331" s="13"/>
       <c r="G331" s="21"/>
       <c r="H331" s="22" t="str">
-        <f aca="false">IF(F331="","",ROUND(F331*G331,2))</f>
+        <f>IF(F331="","",IF(OR(E331="Abschreibung (AfA)",E331="Vorsteuer auf Anlagevermögen"),0,ROUND(F331*G331,2)))</f>
         <v/>
       </c>
       <c r="I331" s="22" t="str">
@@ -12000,7 +12071,7 @@
       <c r="F332" s="13"/>
       <c r="G332" s="21"/>
       <c r="H332" s="22" t="str">
-        <f aca="false">IF(F332="","",ROUND(F332*G332,2))</f>
+        <f>IF(F332="","",IF(OR(E332="Abschreibung (AfA)",E332="Vorsteuer auf Anlagevermögen"),0,ROUND(F332*G332,2)))</f>
         <v/>
       </c>
       <c r="I332" s="22" t="str">
@@ -12018,7 +12089,7 @@
       <c r="F333" s="13"/>
       <c r="G333" s="21"/>
       <c r="H333" s="22" t="str">
-        <f aca="false">IF(F333="","",ROUND(F333*G333,2))</f>
+        <f>IF(F333="","",IF(OR(E333="Abschreibung (AfA)",E333="Vorsteuer auf Anlagevermögen"),0,ROUND(F333*G333,2)))</f>
         <v/>
       </c>
       <c r="I333" s="22" t="str">
@@ -12036,7 +12107,7 @@
       <c r="F334" s="13"/>
       <c r="G334" s="21"/>
       <c r="H334" s="22" t="str">
-        <f aca="false">IF(F334="","",ROUND(F334*G334,2))</f>
+        <f>IF(F334="","",IF(OR(E334="Abschreibung (AfA)",E334="Vorsteuer auf Anlagevermögen"),0,ROUND(F334*G334,2)))</f>
         <v/>
       </c>
       <c r="I334" s="22" t="str">
@@ -12054,7 +12125,7 @@
       <c r="F335" s="13"/>
       <c r="G335" s="21"/>
       <c r="H335" s="22" t="str">
-        <f aca="false">IF(F335="","",ROUND(F335*G335,2))</f>
+        <f>IF(F335="","",IF(OR(E335="Abschreibung (AfA)",E335="Vorsteuer auf Anlagevermögen"),0,ROUND(F335*G335,2)))</f>
         <v/>
       </c>
       <c r="I335" s="22" t="str">
@@ -12072,7 +12143,7 @@
       <c r="F336" s="13"/>
       <c r="G336" s="21"/>
       <c r="H336" s="22" t="str">
-        <f aca="false">IF(F336="","",ROUND(F336*G336,2))</f>
+        <f>IF(F336="","",IF(OR(E336="Abschreibung (AfA)",E336="Vorsteuer auf Anlagevermögen"),0,ROUND(F336*G336,2)))</f>
         <v/>
       </c>
       <c r="I336" s="22" t="str">
@@ -12090,7 +12161,7 @@
       <c r="F337" s="13"/>
       <c r="G337" s="21"/>
       <c r="H337" s="22" t="str">
-        <f aca="false">IF(F337="","",ROUND(F337*G337,2))</f>
+        <f>IF(F337="","",IF(OR(E337="Abschreibung (AfA)",E337="Vorsteuer auf Anlagevermögen"),0,ROUND(F337*G337,2)))</f>
         <v/>
       </c>
       <c r="I337" s="22" t="str">
@@ -12108,7 +12179,7 @@
       <c r="F338" s="13"/>
       <c r="G338" s="21"/>
       <c r="H338" s="22" t="str">
-        <f aca="false">IF(F338="","",ROUND(F338*G338,2))</f>
+        <f>IF(F338="","",IF(OR(E338="Abschreibung (AfA)",E338="Vorsteuer auf Anlagevermögen"),0,ROUND(F338*G338,2)))</f>
         <v/>
       </c>
       <c r="I338" s="22" t="str">
@@ -12126,7 +12197,7 @@
       <c r="F339" s="13"/>
       <c r="G339" s="21"/>
       <c r="H339" s="22" t="str">
-        <f aca="false">IF(F339="","",ROUND(F339*G339,2))</f>
+        <f>IF(F339="","",IF(OR(E339="Abschreibung (AfA)",E339="Vorsteuer auf Anlagevermögen"),0,ROUND(F339*G339,2)))</f>
         <v/>
       </c>
       <c r="I339" s="22" t="str">
@@ -12144,7 +12215,7 @@
       <c r="F340" s="13"/>
       <c r="G340" s="21"/>
       <c r="H340" s="22" t="str">
-        <f aca="false">IF(F340="","",ROUND(F340*G340,2))</f>
+        <f>IF(F340="","",IF(OR(E340="Abschreibung (AfA)",E340="Vorsteuer auf Anlagevermögen"),0,ROUND(F340*G340,2)))</f>
         <v/>
       </c>
       <c r="I340" s="22" t="str">
@@ -12162,7 +12233,7 @@
       <c r="F341" s="13"/>
       <c r="G341" s="21"/>
       <c r="H341" s="22" t="str">
-        <f aca="false">IF(F341="","",ROUND(F341*G341,2))</f>
+        <f>IF(F341="","",IF(OR(E341="Abschreibung (AfA)",E341="Vorsteuer auf Anlagevermögen"),0,ROUND(F341*G341,2)))</f>
         <v/>
       </c>
       <c r="I341" s="22" t="str">
@@ -12180,7 +12251,7 @@
       <c r="F342" s="13"/>
       <c r="G342" s="21"/>
       <c r="H342" s="22" t="str">
-        <f aca="false">IF(F342="","",ROUND(F342*G342,2))</f>
+        <f>IF(F342="","",IF(OR(E342="Abschreibung (AfA)",E342="Vorsteuer auf Anlagevermögen"),0,ROUND(F342*G342,2)))</f>
         <v/>
       </c>
       <c r="I342" s="22" t="str">
@@ -12198,7 +12269,7 @@
       <c r="F343" s="13"/>
       <c r="G343" s="21"/>
       <c r="H343" s="22" t="str">
-        <f aca="false">IF(F343="","",ROUND(F343*G343,2))</f>
+        <f>IF(F343="","",IF(OR(E343="Abschreibung (AfA)",E343="Vorsteuer auf Anlagevermögen"),0,ROUND(F343*G343,2)))</f>
         <v/>
       </c>
       <c r="I343" s="22" t="str">
@@ -12216,7 +12287,7 @@
       <c r="F344" s="13"/>
       <c r="G344" s="21"/>
       <c r="H344" s="22" t="str">
-        <f aca="false">IF(F344="","",ROUND(F344*G344,2))</f>
+        <f>IF(F344="","",IF(OR(E344="Abschreibung (AfA)",E344="Vorsteuer auf Anlagevermögen"),0,ROUND(F344*G344,2)))</f>
         <v/>
       </c>
       <c r="I344" s="22" t="str">
@@ -12234,7 +12305,7 @@
       <c r="F345" s="13"/>
       <c r="G345" s="21"/>
       <c r="H345" s="22" t="str">
-        <f aca="false">IF(F345="","",ROUND(F345*G345,2))</f>
+        <f>IF(F345="","",IF(OR(E345="Abschreibung (AfA)",E345="Vorsteuer auf Anlagevermögen"),0,ROUND(F345*G345,2)))</f>
         <v/>
       </c>
       <c r="I345" s="22" t="str">
@@ -12252,7 +12323,7 @@
       <c r="F346" s="13"/>
       <c r="G346" s="21"/>
       <c r="H346" s="22" t="str">
-        <f aca="false">IF(F346="","",ROUND(F346*G346,2))</f>
+        <f>IF(F346="","",IF(OR(E346="Abschreibung (AfA)",E346="Vorsteuer auf Anlagevermögen"),0,ROUND(F346*G346,2)))</f>
         <v/>
       </c>
       <c r="I346" s="22" t="str">
@@ -12270,7 +12341,7 @@
       <c r="F347" s="13"/>
       <c r="G347" s="21"/>
       <c r="H347" s="22" t="str">
-        <f aca="false">IF(F347="","",ROUND(F347*G347,2))</f>
+        <f>IF(F347="","",IF(OR(E347="Abschreibung (AfA)",E347="Vorsteuer auf Anlagevermögen"),0,ROUND(F347*G347,2)))</f>
         <v/>
       </c>
       <c r="I347" s="22" t="str">
@@ -12288,7 +12359,7 @@
       <c r="F348" s="13"/>
       <c r="G348" s="21"/>
       <c r="H348" s="22" t="str">
-        <f aca="false">IF(F348="","",ROUND(F348*G348,2))</f>
+        <f>IF(F348="","",IF(OR(E348="Abschreibung (AfA)",E348="Vorsteuer auf Anlagevermögen"),0,ROUND(F348*G348,2)))</f>
         <v/>
       </c>
       <c r="I348" s="22" t="str">
@@ -12306,7 +12377,7 @@
       <c r="F349" s="13"/>
       <c r="G349" s="21"/>
       <c r="H349" s="22" t="str">
-        <f aca="false">IF(F349="","",ROUND(F349*G349,2))</f>
+        <f>IF(F349="","",IF(OR(E349="Abschreibung (AfA)",E349="Vorsteuer auf Anlagevermögen"),0,ROUND(F349*G349,2)))</f>
         <v/>
       </c>
       <c r="I349" s="22" t="str">
@@ -12324,7 +12395,7 @@
       <c r="F350" s="13"/>
       <c r="G350" s="21"/>
       <c r="H350" s="22" t="str">
-        <f aca="false">IF(F350="","",ROUND(F350*G350,2))</f>
+        <f>IF(F350="","",IF(OR(E350="Abschreibung (AfA)",E350="Vorsteuer auf Anlagevermögen"),0,ROUND(F350*G350,2)))</f>
         <v/>
       </c>
       <c r="I350" s="22" t="str">
@@ -12342,7 +12413,7 @@
       <c r="F351" s="13"/>
       <c r="G351" s="21"/>
       <c r="H351" s="22" t="str">
-        <f aca="false">IF(F351="","",ROUND(F351*G351,2))</f>
+        <f>IF(F351="","",IF(OR(E351="Abschreibung (AfA)",E351="Vorsteuer auf Anlagevermögen"),0,ROUND(F351*G351,2)))</f>
         <v/>
       </c>
       <c r="I351" s="22" t="str">
@@ -12360,7 +12431,7 @@
       <c r="F352" s="13"/>
       <c r="G352" s="21"/>
       <c r="H352" s="22" t="str">
-        <f aca="false">IF(F352="","",ROUND(F352*G352,2))</f>
+        <f>IF(F352="","",IF(OR(E352="Abschreibung (AfA)",E352="Vorsteuer auf Anlagevermögen"),0,ROUND(F352*G352,2)))</f>
         <v/>
       </c>
       <c r="I352" s="22" t="str">
@@ -12378,7 +12449,7 @@
       <c r="F353" s="13"/>
       <c r="G353" s="21"/>
       <c r="H353" s="22" t="str">
-        <f aca="false">IF(F353="","",ROUND(F353*G353,2))</f>
+        <f>IF(F353="","",IF(OR(E353="Abschreibung (AfA)",E353="Vorsteuer auf Anlagevermögen"),0,ROUND(F353*G353,2)))</f>
         <v/>
       </c>
       <c r="I353" s="22" t="str">
@@ -12396,7 +12467,7 @@
       <c r="F354" s="13"/>
       <c r="G354" s="21"/>
       <c r="H354" s="22" t="str">
-        <f aca="false">IF(F354="","",ROUND(F354*G354,2))</f>
+        <f>IF(F354="","",IF(OR(E354="Abschreibung (AfA)",E354="Vorsteuer auf Anlagevermögen"),0,ROUND(F354*G354,2)))</f>
         <v/>
       </c>
       <c r="I354" s="22" t="str">
@@ -12414,7 +12485,7 @@
       <c r="F355" s="13"/>
       <c r="G355" s="21"/>
       <c r="H355" s="22" t="str">
-        <f aca="false">IF(F355="","",ROUND(F355*G355,2))</f>
+        <f>IF(F355="","",IF(OR(E355="Abschreibung (AfA)",E355="Vorsteuer auf Anlagevermögen"),0,ROUND(F355*G355,2)))</f>
         <v/>
       </c>
       <c r="I355" s="22" t="str">
@@ -12432,7 +12503,7 @@
       <c r="F356" s="13"/>
       <c r="G356" s="21"/>
       <c r="H356" s="22" t="str">
-        <f aca="false">IF(F356="","",ROUND(F356*G356,2))</f>
+        <f>IF(F356="","",IF(OR(E356="Abschreibung (AfA)",E356="Vorsteuer auf Anlagevermögen"),0,ROUND(F356*G356,2)))</f>
         <v/>
       </c>
       <c r="I356" s="22" t="str">
@@ -12450,7 +12521,7 @@
       <c r="F357" s="13"/>
       <c r="G357" s="21"/>
       <c r="H357" s="22" t="str">
-        <f aca="false">IF(F357="","",ROUND(F357*G357,2))</f>
+        <f>IF(F357="","",IF(OR(E357="Abschreibung (AfA)",E357="Vorsteuer auf Anlagevermögen"),0,ROUND(F357*G357,2)))</f>
         <v/>
       </c>
       <c r="I357" s="22" t="str">
@@ -12468,7 +12539,7 @@
       <c r="F358" s="13"/>
       <c r="G358" s="21"/>
       <c r="H358" s="22" t="str">
-        <f aca="false">IF(F358="","",ROUND(F358*G358,2))</f>
+        <f>IF(F358="","",IF(OR(E358="Abschreibung (AfA)",E358="Vorsteuer auf Anlagevermögen"),0,ROUND(F358*G358,2)))</f>
         <v/>
       </c>
       <c r="I358" s="22" t="str">
@@ -12486,7 +12557,7 @@
       <c r="F359" s="13"/>
       <c r="G359" s="21"/>
       <c r="H359" s="22" t="str">
-        <f aca="false">IF(F359="","",ROUND(F359*G359,2))</f>
+        <f>IF(F359="","",IF(OR(E359="Abschreibung (AfA)",E359="Vorsteuer auf Anlagevermögen"),0,ROUND(F359*G359,2)))</f>
         <v/>
       </c>
       <c r="I359" s="22" t="str">
@@ -12504,7 +12575,7 @@
       <c r="F360" s="13"/>
       <c r="G360" s="21"/>
       <c r="H360" s="22" t="str">
-        <f aca="false">IF(F360="","",ROUND(F360*G360,2))</f>
+        <f>IF(F360="","",IF(OR(E360="Abschreibung (AfA)",E360="Vorsteuer auf Anlagevermögen"),0,ROUND(F360*G360,2)))</f>
         <v/>
       </c>
       <c r="I360" s="22" t="str">
@@ -12522,7 +12593,7 @@
       <c r="F361" s="13"/>
       <c r="G361" s="21"/>
       <c r="H361" s="22" t="str">
-        <f aca="false">IF(F361="","",ROUND(F361*G361,2))</f>
+        <f>IF(F361="","",IF(OR(E361="Abschreibung (AfA)",E361="Vorsteuer auf Anlagevermögen"),0,ROUND(F361*G361,2)))</f>
         <v/>
       </c>
       <c r="I361" s="22" t="str">
@@ -12540,7 +12611,7 @@
       <c r="F362" s="13"/>
       <c r="G362" s="21"/>
       <c r="H362" s="22" t="str">
-        <f aca="false">IF(F362="","",ROUND(F362*G362,2))</f>
+        <f>IF(F362="","",IF(OR(E362="Abschreibung (AfA)",E362="Vorsteuer auf Anlagevermögen"),0,ROUND(F362*G362,2)))</f>
         <v/>
       </c>
       <c r="I362" s="22" t="str">
@@ -12558,7 +12629,7 @@
       <c r="F363" s="13"/>
       <c r="G363" s="21"/>
       <c r="H363" s="22" t="str">
-        <f aca="false">IF(F363="","",ROUND(F363*G363,2))</f>
+        <f>IF(F363="","",IF(OR(E363="Abschreibung (AfA)",E363="Vorsteuer auf Anlagevermögen"),0,ROUND(F363*G363,2)))</f>
         <v/>
       </c>
       <c r="I363" s="22" t="str">
@@ -12576,7 +12647,7 @@
       <c r="F364" s="13"/>
       <c r="G364" s="21"/>
       <c r="H364" s="22" t="str">
-        <f aca="false">IF(F364="","",ROUND(F364*G364,2))</f>
+        <f>IF(F364="","",IF(OR(E364="Abschreibung (AfA)",E364="Vorsteuer auf Anlagevermögen"),0,ROUND(F364*G364,2)))</f>
         <v/>
       </c>
       <c r="I364" s="22" t="str">
@@ -12594,7 +12665,7 @@
       <c r="F365" s="13"/>
       <c r="G365" s="21"/>
       <c r="H365" s="22" t="str">
-        <f aca="false">IF(F365="","",ROUND(F365*G365,2))</f>
+        <f>IF(F365="","",IF(OR(E365="Abschreibung (AfA)",E365="Vorsteuer auf Anlagevermögen"),0,ROUND(F365*G365,2)))</f>
         <v/>
       </c>
       <c r="I365" s="22" t="str">
@@ -12612,7 +12683,7 @@
       <c r="F366" s="13"/>
       <c r="G366" s="21"/>
       <c r="H366" s="22" t="str">
-        <f aca="false">IF(F366="","",ROUND(F366*G366,2))</f>
+        <f>IF(F366="","",IF(OR(E366="Abschreibung (AfA)",E366="Vorsteuer auf Anlagevermögen"),0,ROUND(F366*G366,2)))</f>
         <v/>
       </c>
       <c r="I366" s="22" t="str">
@@ -12630,7 +12701,7 @@
       <c r="F367" s="13"/>
       <c r="G367" s="21"/>
       <c r="H367" s="22" t="str">
-        <f aca="false">IF(F367="","",ROUND(F367*G367,2))</f>
+        <f>IF(F367="","",IF(OR(E367="Abschreibung (AfA)",E367="Vorsteuer auf Anlagevermögen"),0,ROUND(F367*G367,2)))</f>
         <v/>
       </c>
       <c r="I367" s="22" t="str">
@@ -12648,7 +12719,7 @@
       <c r="F368" s="13"/>
       <c r="G368" s="21"/>
       <c r="H368" s="22" t="str">
-        <f aca="false">IF(F368="","",ROUND(F368*G368,2))</f>
+        <f>IF(F368="","",IF(OR(E368="Abschreibung (AfA)",E368="Vorsteuer auf Anlagevermögen"),0,ROUND(F368*G368,2)))</f>
         <v/>
       </c>
       <c r="I368" s="22" t="str">
@@ -12666,7 +12737,7 @@
       <c r="F369" s="13"/>
       <c r="G369" s="21"/>
       <c r="H369" s="22" t="str">
-        <f aca="false">IF(F369="","",ROUND(F369*G369,2))</f>
+        <f>IF(F369="","",IF(OR(E369="Abschreibung (AfA)",E369="Vorsteuer auf Anlagevermögen"),0,ROUND(F369*G369,2)))</f>
         <v/>
       </c>
       <c r="I369" s="22" t="str">
@@ -12684,7 +12755,7 @@
       <c r="F370" s="13"/>
       <c r="G370" s="21"/>
       <c r="H370" s="22" t="str">
-        <f aca="false">IF(F370="","",ROUND(F370*G370,2))</f>
+        <f>IF(F370="","",IF(OR(E370="Abschreibung (AfA)",E370="Vorsteuer auf Anlagevermögen"),0,ROUND(F370*G370,2)))</f>
         <v/>
       </c>
       <c r="I370" s="22" t="str">
@@ -12702,7 +12773,7 @@
       <c r="F371" s="13"/>
       <c r="G371" s="21"/>
       <c r="H371" s="22" t="str">
-        <f aca="false">IF(F371="","",ROUND(F371*G371,2))</f>
+        <f>IF(F371="","",IF(OR(E371="Abschreibung (AfA)",E371="Vorsteuer auf Anlagevermögen"),0,ROUND(F371*G371,2)))</f>
         <v/>
       </c>
       <c r="I371" s="22" t="str">
@@ -12720,7 +12791,7 @@
       <c r="F372" s="13"/>
       <c r="G372" s="21"/>
       <c r="H372" s="22" t="str">
-        <f aca="false">IF(F372="","",ROUND(F372*G372,2))</f>
+        <f>IF(F372="","",IF(OR(E372="Abschreibung (AfA)",E372="Vorsteuer auf Anlagevermögen"),0,ROUND(F372*G372,2)))</f>
         <v/>
       </c>
       <c r="I372" s="22" t="str">
@@ -12738,7 +12809,7 @@
       <c r="F373" s="13"/>
       <c r="G373" s="21"/>
       <c r="H373" s="22" t="str">
-        <f aca="false">IF(F373="","",ROUND(F373*G373,2))</f>
+        <f>IF(F373="","",IF(OR(E373="Abschreibung (AfA)",E373="Vorsteuer auf Anlagevermögen"),0,ROUND(F373*G373,2)))</f>
         <v/>
       </c>
       <c r="I373" s="22" t="str">
@@ -12756,7 +12827,7 @@
       <c r="F374" s="13"/>
       <c r="G374" s="21"/>
       <c r="H374" s="22" t="str">
-        <f aca="false">IF(F374="","",ROUND(F374*G374,2))</f>
+        <f>IF(F374="","",IF(OR(E374="Abschreibung (AfA)",E374="Vorsteuer auf Anlagevermögen"),0,ROUND(F374*G374,2)))</f>
         <v/>
       </c>
       <c r="I374" s="22" t="str">
@@ -12774,7 +12845,7 @@
       <c r="F375" s="13"/>
       <c r="G375" s="21"/>
       <c r="H375" s="22" t="str">
-        <f aca="false">IF(F375="","",ROUND(F375*G375,2))</f>
+        <f>IF(F375="","",IF(OR(E375="Abschreibung (AfA)",E375="Vorsteuer auf Anlagevermögen"),0,ROUND(F375*G375,2)))</f>
         <v/>
       </c>
       <c r="I375" s="22" t="str">
@@ -12792,7 +12863,7 @@
       <c r="F376" s="13"/>
       <c r="G376" s="21"/>
       <c r="H376" s="22" t="str">
-        <f aca="false">IF(F376="","",ROUND(F376*G376,2))</f>
+        <f>IF(F376="","",IF(OR(E376="Abschreibung (AfA)",E376="Vorsteuer auf Anlagevermögen"),0,ROUND(F376*G376,2)))</f>
         <v/>
       </c>
       <c r="I376" s="22" t="str">
@@ -12810,7 +12881,7 @@
       <c r="F377" s="13"/>
       <c r="G377" s="21"/>
       <c r="H377" s="22" t="str">
-        <f aca="false">IF(F377="","",ROUND(F377*G377,2))</f>
+        <f>IF(F377="","",IF(OR(E377="Abschreibung (AfA)",E377="Vorsteuer auf Anlagevermögen"),0,ROUND(F377*G377,2)))</f>
         <v/>
       </c>
       <c r="I377" s="22" t="str">
@@ -12828,7 +12899,7 @@
       <c r="F378" s="13"/>
       <c r="G378" s="21"/>
       <c r="H378" s="22" t="str">
-        <f aca="false">IF(F378="","",ROUND(F378*G378,2))</f>
+        <f>IF(F378="","",IF(OR(E378="Abschreibung (AfA)",E378="Vorsteuer auf Anlagevermögen"),0,ROUND(F378*G378,2)))</f>
         <v/>
       </c>
       <c r="I378" s="22" t="str">
@@ -12846,7 +12917,7 @@
       <c r="F379" s="13"/>
       <c r="G379" s="21"/>
       <c r="H379" s="22" t="str">
-        <f aca="false">IF(F379="","",ROUND(F379*G379,2))</f>
+        <f>IF(F379="","",IF(OR(E379="Abschreibung (AfA)",E379="Vorsteuer auf Anlagevermögen"),0,ROUND(F379*G379,2)))</f>
         <v/>
       </c>
       <c r="I379" s="22" t="str">
@@ -12864,7 +12935,7 @@
       <c r="F380" s="13"/>
       <c r="G380" s="21"/>
       <c r="H380" s="22" t="str">
-        <f aca="false">IF(F380="","",ROUND(F380*G380,2))</f>
+        <f>IF(F380="","",IF(OR(E380="Abschreibung (AfA)",E380="Vorsteuer auf Anlagevermögen"),0,ROUND(F380*G380,2)))</f>
         <v/>
       </c>
       <c r="I380" s="22" t="str">
@@ -12882,7 +12953,7 @@
       <c r="F381" s="13"/>
       <c r="G381" s="21"/>
       <c r="H381" s="22" t="str">
-        <f aca="false">IF(F381="","",ROUND(F381*G381,2))</f>
+        <f>IF(F381="","",IF(OR(E381="Abschreibung (AfA)",E381="Vorsteuer auf Anlagevermögen"),0,ROUND(F381*G381,2)))</f>
         <v/>
       </c>
       <c r="I381" s="22" t="str">
@@ -12900,7 +12971,7 @@
       <c r="F382" s="13"/>
       <c r="G382" s="21"/>
       <c r="H382" s="22" t="str">
-        <f aca="false">IF(F382="","",ROUND(F382*G382,2))</f>
+        <f>IF(F382="","",IF(OR(E382="Abschreibung (AfA)",E382="Vorsteuer auf Anlagevermögen"),0,ROUND(F382*G382,2)))</f>
         <v/>
       </c>
       <c r="I382" s="22" t="str">
@@ -12918,7 +12989,7 @@
       <c r="F383" s="13"/>
       <c r="G383" s="21"/>
       <c r="H383" s="22" t="str">
-        <f aca="false">IF(F383="","",ROUND(F383*G383,2))</f>
+        <f>IF(F383="","",IF(OR(E383="Abschreibung (AfA)",E383="Vorsteuer auf Anlagevermögen"),0,ROUND(F383*G383,2)))</f>
         <v/>
       </c>
       <c r="I383" s="22" t="str">
@@ -12936,7 +13007,7 @@
       <c r="F384" s="13"/>
       <c r="G384" s="21"/>
       <c r="H384" s="22" t="str">
-        <f aca="false">IF(F384="","",ROUND(F384*G384,2))</f>
+        <f>IF(F384="","",IF(OR(E384="Abschreibung (AfA)",E384="Vorsteuer auf Anlagevermögen"),0,ROUND(F384*G384,2)))</f>
         <v/>
       </c>
       <c r="I384" s="22" t="str">
@@ -12954,7 +13025,7 @@
       <c r="F385" s="13"/>
       <c r="G385" s="21"/>
       <c r="H385" s="22" t="str">
-        <f aca="false">IF(F385="","",ROUND(F385*G385,2))</f>
+        <f>IF(F385="","",IF(OR(E385="Abschreibung (AfA)",E385="Vorsteuer auf Anlagevermögen"),0,ROUND(F385*G385,2)))</f>
         <v/>
       </c>
       <c r="I385" s="22" t="str">
@@ -12972,7 +13043,7 @@
       <c r="F386" s="13"/>
       <c r="G386" s="21"/>
       <c r="H386" s="22" t="str">
-        <f aca="false">IF(F386="","",ROUND(F386*G386,2))</f>
+        <f>IF(F386="","",IF(OR(E386="Abschreibung (AfA)",E386="Vorsteuer auf Anlagevermögen"),0,ROUND(F386*G386,2)))</f>
         <v/>
       </c>
       <c r="I386" s="22" t="str">
@@ -12990,7 +13061,7 @@
       <c r="F387" s="13"/>
       <c r="G387" s="21"/>
       <c r="H387" s="22" t="str">
-        <f aca="false">IF(F387="","",ROUND(F387*G387,2))</f>
+        <f>IF(F387="","",IF(OR(E387="Abschreibung (AfA)",E387="Vorsteuer auf Anlagevermögen"),0,ROUND(F387*G387,2)))</f>
         <v/>
       </c>
       <c r="I387" s="22" t="str">
@@ -13008,7 +13079,7 @@
       <c r="F388" s="13"/>
       <c r="G388" s="21"/>
       <c r="H388" s="22" t="str">
-        <f aca="false">IF(F388="","",ROUND(F388*G388,2))</f>
+        <f>IF(F388="","",IF(OR(E388="Abschreibung (AfA)",E388="Vorsteuer auf Anlagevermögen"),0,ROUND(F388*G388,2)))</f>
         <v/>
       </c>
       <c r="I388" s="22" t="str">
@@ -13026,7 +13097,7 @@
       <c r="F389" s="13"/>
       <c r="G389" s="21"/>
       <c r="H389" s="22" t="str">
-        <f aca="false">IF(F389="","",ROUND(F389*G389,2))</f>
+        <f>IF(F389="","",IF(OR(E389="Abschreibung (AfA)",E389="Vorsteuer auf Anlagevermögen"),0,ROUND(F389*G389,2)))</f>
         <v/>
       </c>
       <c r="I389" s="22" t="str">
@@ -13044,7 +13115,7 @@
       <c r="F390" s="13"/>
       <c r="G390" s="21"/>
       <c r="H390" s="22" t="str">
-        <f aca="false">IF(F390="","",ROUND(F390*G390,2))</f>
+        <f>IF(F390="","",IF(OR(E390="Abschreibung (AfA)",E390="Vorsteuer auf Anlagevermögen"),0,ROUND(F390*G390,2)))</f>
         <v/>
       </c>
       <c r="I390" s="22" t="str">
@@ -13062,7 +13133,7 @@
       <c r="F391" s="13"/>
       <c r="G391" s="21"/>
       <c r="H391" s="22" t="str">
-        <f aca="false">IF(F391="","",ROUND(F391*G391,2))</f>
+        <f>IF(F391="","",IF(OR(E391="Abschreibung (AfA)",E391="Vorsteuer auf Anlagevermögen"),0,ROUND(F391*G391,2)))</f>
         <v/>
       </c>
       <c r="I391" s="22" t="str">
@@ -13080,7 +13151,7 @@
       <c r="F392" s="13"/>
       <c r="G392" s="21"/>
       <c r="H392" s="22" t="str">
-        <f aca="false">IF(F392="","",ROUND(F392*G392,2))</f>
+        <f>IF(F392="","",IF(OR(E392="Abschreibung (AfA)",E392="Vorsteuer auf Anlagevermögen"),0,ROUND(F392*G392,2)))</f>
         <v/>
       </c>
       <c r="I392" s="22" t="str">
@@ -13098,7 +13169,7 @@
       <c r="F393" s="13"/>
       <c r="G393" s="21"/>
       <c r="H393" s="22" t="str">
-        <f aca="false">IF(F393="","",ROUND(F393*G393,2))</f>
+        <f>IF(F393="","",IF(OR(E393="Abschreibung (AfA)",E393="Vorsteuer auf Anlagevermögen"),0,ROUND(F393*G393,2)))</f>
         <v/>
       </c>
       <c r="I393" s="22" t="str">
@@ -13116,7 +13187,7 @@
       <c r="F394" s="13"/>
       <c r="G394" s="21"/>
       <c r="H394" s="22" t="str">
-        <f aca="false">IF(F394="","",ROUND(F394*G394,2))</f>
+        <f>IF(F394="","",IF(OR(E394="Abschreibung (AfA)",E394="Vorsteuer auf Anlagevermögen"),0,ROUND(F394*G394,2)))</f>
         <v/>
       </c>
       <c r="I394" s="22" t="str">
@@ -13134,7 +13205,7 @@
       <c r="F395" s="13"/>
       <c r="G395" s="21"/>
       <c r="H395" s="22" t="str">
-        <f aca="false">IF(F395="","",ROUND(F395*G395,2))</f>
+        <f>IF(F395="","",IF(OR(E395="Abschreibung (AfA)",E395="Vorsteuer auf Anlagevermögen"),0,ROUND(F395*G395,2)))</f>
         <v/>
       </c>
       <c r="I395" s="22" t="str">
@@ -13152,7 +13223,7 @@
       <c r="F396" s="13"/>
       <c r="G396" s="21"/>
       <c r="H396" s="22" t="str">
-        <f aca="false">IF(F396="","",ROUND(F396*G396,2))</f>
+        <f>IF(F396="","",IF(OR(E396="Abschreibung (AfA)",E396="Vorsteuer auf Anlagevermögen"),0,ROUND(F396*G396,2)))</f>
         <v/>
       </c>
       <c r="I396" s="22" t="str">
@@ -13170,7 +13241,7 @@
       <c r="F397" s="13"/>
       <c r="G397" s="21"/>
       <c r="H397" s="22" t="str">
-        <f aca="false">IF(F397="","",ROUND(F397*G397,2))</f>
+        <f>IF(F397="","",IF(OR(E397="Abschreibung (AfA)",E397="Vorsteuer auf Anlagevermögen"),0,ROUND(F397*G397,2)))</f>
         <v/>
       </c>
       <c r="I397" s="22" t="str">
@@ -13188,7 +13259,7 @@
       <c r="F398" s="13"/>
       <c r="G398" s="21"/>
       <c r="H398" s="22" t="str">
-        <f aca="false">IF(F398="","",ROUND(F398*G398,2))</f>
+        <f>IF(F398="","",IF(OR(E398="Abschreibung (AfA)",E398="Vorsteuer auf Anlagevermögen"),0,ROUND(F398*G398,2)))</f>
         <v/>
       </c>
       <c r="I398" s="22" t="str">
@@ -13206,7 +13277,7 @@
       <c r="F399" s="13"/>
       <c r="G399" s="21"/>
       <c r="H399" s="22" t="str">
-        <f aca="false">IF(F399="","",ROUND(F399*G399,2))</f>
+        <f>IF(F399="","",IF(OR(E399="Abschreibung (AfA)",E399="Vorsteuer auf Anlagevermögen"),0,ROUND(F399*G399,2)))</f>
         <v/>
       </c>
       <c r="I399" s="22" t="str">
@@ -13224,7 +13295,7 @@
       <c r="F400" s="13"/>
       <c r="G400" s="21"/>
       <c r="H400" s="22" t="str">
-        <f aca="false">IF(F400="","",ROUND(F400*G400,2))</f>
+        <f>IF(F400="","",IF(OR(E400="Abschreibung (AfA)",E400="Vorsteuer auf Anlagevermögen"),0,ROUND(F400*G400,2)))</f>
         <v/>
       </c>
       <c r="I400" s="22" t="str">
@@ -13242,7 +13313,7 @@
       <c r="F401" s="13"/>
       <c r="G401" s="21"/>
       <c r="H401" s="22" t="str">
-        <f aca="false">IF(F401="","",ROUND(F401*G401,2))</f>
+        <f>IF(F401="","",IF(OR(E401="Abschreibung (AfA)",E401="Vorsteuer auf Anlagevermögen"),0,ROUND(F401*G401,2)))</f>
         <v/>
       </c>
       <c r="I401" s="22" t="str">
@@ -13260,7 +13331,7 @@
       <c r="F402" s="13"/>
       <c r="G402" s="21"/>
       <c r="H402" s="22" t="str">
-        <f aca="false">IF(F402="","",ROUND(F402*G402,2))</f>
+        <f>IF(F402="","",IF(OR(E402="Abschreibung (AfA)",E402="Vorsteuer auf Anlagevermögen"),0,ROUND(F402*G402,2)))</f>
         <v/>
       </c>
       <c r="I402" s="22" t="str">
@@ -13278,7 +13349,7 @@
       <c r="F403" s="13"/>
       <c r="G403" s="21"/>
       <c r="H403" s="22" t="str">
-        <f aca="false">IF(F403="","",ROUND(F403*G403,2))</f>
+        <f>IF(F403="","",IF(OR(E403="Abschreibung (AfA)",E403="Vorsteuer auf Anlagevermögen"),0,ROUND(F403*G403,2)))</f>
         <v/>
       </c>
       <c r="I403" s="22" t="str">
@@ -13296,7 +13367,7 @@
       <c r="F404" s="13"/>
       <c r="G404" s="21"/>
       <c r="H404" s="22" t="str">
-        <f aca="false">IF(F404="","",ROUND(F404*G404,2))</f>
+        <f>IF(F404="","",IF(OR(E404="Abschreibung (AfA)",E404="Vorsteuer auf Anlagevermögen"),0,ROUND(F404*G404,2)))</f>
         <v/>
       </c>
       <c r="I404" s="22" t="str">
@@ -13314,7 +13385,7 @@
       <c r="F405" s="13"/>
       <c r="G405" s="21"/>
       <c r="H405" s="22" t="str">
-        <f aca="false">IF(F405="","",ROUND(F405*G405,2))</f>
+        <f>IF(F405="","",IF(OR(E405="Abschreibung (AfA)",E405="Vorsteuer auf Anlagevermögen"),0,ROUND(F405*G405,2)))</f>
         <v/>
       </c>
       <c r="I405" s="22" t="str">
@@ -13332,7 +13403,7 @@
       <c r="F406" s="13"/>
       <c r="G406" s="21"/>
       <c r="H406" s="22" t="str">
-        <f aca="false">IF(F406="","",ROUND(F406*G406,2))</f>
+        <f>IF(F406="","",IF(OR(E406="Abschreibung (AfA)",E406="Vorsteuer auf Anlagevermögen"),0,ROUND(F406*G406,2)))</f>
         <v/>
       </c>
       <c r="I406" s="22" t="str">
@@ -13350,7 +13421,7 @@
       <c r="F407" s="13"/>
       <c r="G407" s="21"/>
       <c r="H407" s="22" t="str">
-        <f aca="false">IF(F407="","",ROUND(F407*G407,2))</f>
+        <f>IF(F407="","",IF(OR(E407="Abschreibung (AfA)",E407="Vorsteuer auf Anlagevermögen"),0,ROUND(F407*G407,2)))</f>
         <v/>
       </c>
       <c r="I407" s="22" t="str">
@@ -13368,7 +13439,7 @@
       <c r="F408" s="13"/>
       <c r="G408" s="21"/>
       <c r="H408" s="22" t="str">
-        <f aca="false">IF(F408="","",ROUND(F408*G408,2))</f>
+        <f>IF(F408="","",IF(OR(E408="Abschreibung (AfA)",E408="Vorsteuer auf Anlagevermögen"),0,ROUND(F408*G408,2)))</f>
         <v/>
       </c>
       <c r="I408" s="22" t="str">
@@ -13386,7 +13457,7 @@
       <c r="F409" s="13"/>
       <c r="G409" s="21"/>
       <c r="H409" s="22" t="str">
-        <f aca="false">IF(F409="","",ROUND(F409*G409,2))</f>
+        <f>IF(F409="","",IF(OR(E409="Abschreibung (AfA)",E409="Vorsteuer auf Anlagevermögen"),0,ROUND(F409*G409,2)))</f>
         <v/>
       </c>
       <c r="I409" s="22" t="str">
@@ -13404,7 +13475,7 @@
       <c r="F410" s="13"/>
       <c r="G410" s="21"/>
       <c r="H410" s="22" t="str">
-        <f aca="false">IF(F410="","",ROUND(F410*G410,2))</f>
+        <f>IF(F410="","",IF(OR(E410="Abschreibung (AfA)",E410="Vorsteuer auf Anlagevermögen"),0,ROUND(F410*G410,2)))</f>
         <v/>
       </c>
       <c r="I410" s="22" t="str">
@@ -13422,7 +13493,7 @@
       <c r="F411" s="13"/>
       <c r="G411" s="21"/>
       <c r="H411" s="22" t="str">
-        <f aca="false">IF(F411="","",ROUND(F411*G411,2))</f>
+        <f>IF(F411="","",IF(OR(E411="Abschreibung (AfA)",E411="Vorsteuer auf Anlagevermögen"),0,ROUND(F411*G411,2)))</f>
         <v/>
       </c>
       <c r="I411" s="22" t="str">
@@ -13440,7 +13511,7 @@
       <c r="F412" s="13"/>
       <c r="G412" s="21"/>
       <c r="H412" s="22" t="str">
-        <f aca="false">IF(F412="","",ROUND(F412*G412,2))</f>
+        <f>IF(F412="","",IF(OR(E412="Abschreibung (AfA)",E412="Vorsteuer auf Anlagevermögen"),0,ROUND(F412*G412,2)))</f>
         <v/>
       </c>
       <c r="I412" s="22" t="str">
@@ -13458,7 +13529,7 @@
       <c r="F413" s="13"/>
       <c r="G413" s="21"/>
       <c r="H413" s="22" t="str">
-        <f aca="false">IF(F413="","",ROUND(F413*G413,2))</f>
+        <f>IF(F413="","",IF(OR(E413="Abschreibung (AfA)",E413="Vorsteuer auf Anlagevermögen"),0,ROUND(F413*G413,2)))</f>
         <v/>
       </c>
       <c r="I413" s="22" t="str">
@@ -13476,7 +13547,7 @@
       <c r="F414" s="13"/>
       <c r="G414" s="21"/>
       <c r="H414" s="22" t="str">
-        <f aca="false">IF(F414="","",ROUND(F414*G414,2))</f>
+        <f>IF(F414="","",IF(OR(E414="Abschreibung (AfA)",E414="Vorsteuer auf Anlagevermögen"),0,ROUND(F414*G414,2)))</f>
         <v/>
       </c>
       <c r="I414" s="22" t="str">
@@ -13494,7 +13565,7 @@
       <c r="F415" s="13"/>
       <c r="G415" s="21"/>
       <c r="H415" s="22" t="str">
-        <f aca="false">IF(F415="","",ROUND(F415*G415,2))</f>
+        <f>IF(F415="","",IF(OR(E415="Abschreibung (AfA)",E415="Vorsteuer auf Anlagevermögen"),0,ROUND(F415*G415,2)))</f>
         <v/>
       </c>
       <c r="I415" s="22" t="str">
@@ -13512,7 +13583,7 @@
       <c r="F416" s="13"/>
       <c r="G416" s="21"/>
       <c r="H416" s="22" t="str">
-        <f aca="false">IF(F416="","",ROUND(F416*G416,2))</f>
+        <f>IF(F416="","",IF(OR(E416="Abschreibung (AfA)",E416="Vorsteuer auf Anlagevermögen"),0,ROUND(F416*G416,2)))</f>
         <v/>
       </c>
       <c r="I416" s="22" t="str">
@@ -13530,7 +13601,7 @@
       <c r="F417" s="13"/>
       <c r="G417" s="21"/>
       <c r="H417" s="22" t="str">
-        <f aca="false">IF(F417="","",ROUND(F417*G417,2))</f>
+        <f>IF(F417="","",IF(OR(E417="Abschreibung (AfA)",E417="Vorsteuer auf Anlagevermögen"),0,ROUND(F417*G417,2)))</f>
         <v/>
       </c>
       <c r="I417" s="22" t="str">
@@ -13548,7 +13619,7 @@
       <c r="F418" s="13"/>
       <c r="G418" s="21"/>
       <c r="H418" s="22" t="str">
-        <f aca="false">IF(F418="","",ROUND(F418*G418,2))</f>
+        <f>IF(F418="","",IF(OR(E418="Abschreibung (AfA)",E418="Vorsteuer auf Anlagevermögen"),0,ROUND(F418*G418,2)))</f>
         <v/>
       </c>
       <c r="I418" s="22" t="str">
@@ -13566,7 +13637,7 @@
       <c r="F419" s="13"/>
       <c r="G419" s="21"/>
       <c r="H419" s="22" t="str">
-        <f aca="false">IF(F419="","",ROUND(F419*G419,2))</f>
+        <f>IF(F419="","",IF(OR(E419="Abschreibung (AfA)",E419="Vorsteuer auf Anlagevermögen"),0,ROUND(F419*G419,2)))</f>
         <v/>
       </c>
       <c r="I419" s="22" t="str">
@@ -13584,7 +13655,7 @@
       <c r="F420" s="13"/>
       <c r="G420" s="21"/>
       <c r="H420" s="22" t="str">
-        <f aca="false">IF(F420="","",ROUND(F420*G420,2))</f>
+        <f>IF(F420="","",IF(OR(E420="Abschreibung (AfA)",E420="Vorsteuer auf Anlagevermögen"),0,ROUND(F420*G420,2)))</f>
         <v/>
       </c>
       <c r="I420" s="22" t="str">
@@ -13602,7 +13673,7 @@
       <c r="F421" s="13"/>
       <c r="G421" s="21"/>
       <c r="H421" s="22" t="str">
-        <f aca="false">IF(F421="","",ROUND(F421*G421,2))</f>
+        <f>IF(F421="","",IF(OR(E421="Abschreibung (AfA)",E421="Vorsteuer auf Anlagevermögen"),0,ROUND(F421*G421,2)))</f>
         <v/>
       </c>
       <c r="I421" s="22" t="str">
@@ -13620,7 +13691,7 @@
       <c r="F422" s="13"/>
       <c r="G422" s="21"/>
       <c r="H422" s="22" t="str">
-        <f aca="false">IF(F422="","",ROUND(F422*G422,2))</f>
+        <f>IF(F422="","",IF(OR(E422="Abschreibung (AfA)",E422="Vorsteuer auf Anlagevermögen"),0,ROUND(F422*G422,2)))</f>
         <v/>
       </c>
       <c r="I422" s="22" t="str">
@@ -13638,7 +13709,7 @@
       <c r="F423" s="13"/>
       <c r="G423" s="21"/>
       <c r="H423" s="22" t="str">
-        <f aca="false">IF(F423="","",ROUND(F423*G423,2))</f>
+        <f>IF(F423="","",IF(OR(E423="Abschreibung (AfA)",E423="Vorsteuer auf Anlagevermögen"),0,ROUND(F423*G423,2)))</f>
         <v/>
       </c>
       <c r="I423" s="22" t="str">
@@ -13656,7 +13727,7 @@
       <c r="F424" s="13"/>
       <c r="G424" s="21"/>
       <c r="H424" s="22" t="str">
-        <f aca="false">IF(F424="","",ROUND(F424*G424,2))</f>
+        <f>IF(F424="","",IF(OR(E424="Abschreibung (AfA)",E424="Vorsteuer auf Anlagevermögen"),0,ROUND(F424*G424,2)))</f>
         <v/>
       </c>
       <c r="I424" s="22" t="str">
@@ -13674,7 +13745,7 @@
       <c r="F425" s="13"/>
       <c r="G425" s="21"/>
       <c r="H425" s="22" t="str">
-        <f aca="false">IF(F425="","",ROUND(F425*G425,2))</f>
+        <f>IF(F425="","",IF(OR(E425="Abschreibung (AfA)",E425="Vorsteuer auf Anlagevermögen"),0,ROUND(F425*G425,2)))</f>
         <v/>
       </c>
       <c r="I425" s="22" t="str">
@@ -13692,7 +13763,7 @@
       <c r="F426" s="13"/>
       <c r="G426" s="21"/>
       <c r="H426" s="22" t="str">
-        <f aca="false">IF(F426="","",ROUND(F426*G426,2))</f>
+        <f>IF(F426="","",IF(OR(E426="Abschreibung (AfA)",E426="Vorsteuer auf Anlagevermögen"),0,ROUND(F426*G426,2)))</f>
         <v/>
       </c>
       <c r="I426" s="22" t="str">
@@ -13710,7 +13781,7 @@
       <c r="F427" s="13"/>
       <c r="G427" s="21"/>
       <c r="H427" s="22" t="str">
-        <f aca="false">IF(F427="","",ROUND(F427*G427,2))</f>
+        <f>IF(F427="","",IF(OR(E427="Abschreibung (AfA)",E427="Vorsteuer auf Anlagevermögen"),0,ROUND(F427*G427,2)))</f>
         <v/>
       </c>
       <c r="I427" s="22" t="str">
@@ -13728,7 +13799,7 @@
       <c r="F428" s="13"/>
       <c r="G428" s="21"/>
       <c r="H428" s="22" t="str">
-        <f aca="false">IF(F428="","",ROUND(F428*G428,2))</f>
+        <f>IF(F428="","",IF(OR(E428="Abschreibung (AfA)",E428="Vorsteuer auf Anlagevermögen"),0,ROUND(F428*G428,2)))</f>
         <v/>
       </c>
       <c r="I428" s="22" t="str">
@@ -13746,7 +13817,7 @@
       <c r="F429" s="13"/>
       <c r="G429" s="21"/>
       <c r="H429" s="22" t="str">
-        <f aca="false">IF(F429="","",ROUND(F429*G429,2))</f>
+        <f>IF(F429="","",IF(OR(E429="Abschreibung (AfA)",E429="Vorsteuer auf Anlagevermögen"),0,ROUND(F429*G429,2)))</f>
         <v/>
       </c>
       <c r="I429" s="22" t="str">
@@ -13764,7 +13835,7 @@
       <c r="F430" s="13"/>
       <c r="G430" s="21"/>
       <c r="H430" s="22" t="str">
-        <f aca="false">IF(F430="","",ROUND(F430*G430,2))</f>
+        <f>IF(F430="","",IF(OR(E430="Abschreibung (AfA)",E430="Vorsteuer auf Anlagevermögen"),0,ROUND(F430*G430,2)))</f>
         <v/>
       </c>
       <c r="I430" s="22" t="str">
@@ -13782,7 +13853,7 @@
       <c r="F431" s="13"/>
       <c r="G431" s="21"/>
       <c r="H431" s="22" t="str">
-        <f aca="false">IF(F431="","",ROUND(F431*G431,2))</f>
+        <f>IF(F431="","",IF(OR(E431="Abschreibung (AfA)",E431="Vorsteuer auf Anlagevermögen"),0,ROUND(F431*G431,2)))</f>
         <v/>
       </c>
       <c r="I431" s="22" t="str">
@@ -13800,7 +13871,7 @@
       <c r="F432" s="13"/>
       <c r="G432" s="21"/>
       <c r="H432" s="22" t="str">
-        <f aca="false">IF(F432="","",ROUND(F432*G432,2))</f>
+        <f>IF(F432="","",IF(OR(E432="Abschreibung (AfA)",E432="Vorsteuer auf Anlagevermögen"),0,ROUND(F432*G432,2)))</f>
         <v/>
       </c>
       <c r="I432" s="22" t="str">
@@ -13818,7 +13889,7 @@
       <c r="F433" s="13"/>
       <c r="G433" s="21"/>
       <c r="H433" s="22" t="str">
-        <f aca="false">IF(F433="","",ROUND(F433*G433,2))</f>
+        <f>IF(F433="","",IF(OR(E433="Abschreibung (AfA)",E433="Vorsteuer auf Anlagevermögen"),0,ROUND(F433*G433,2)))</f>
         <v/>
       </c>
       <c r="I433" s="22" t="str">
@@ -13836,7 +13907,7 @@
       <c r="F434" s="13"/>
       <c r="G434" s="21"/>
       <c r="H434" s="22" t="str">
-        <f aca="false">IF(F434="","",ROUND(F434*G434,2))</f>
+        <f>IF(F434="","",IF(OR(E434="Abschreibung (AfA)",E434="Vorsteuer auf Anlagevermögen"),0,ROUND(F434*G434,2)))</f>
         <v/>
       </c>
       <c r="I434" s="22" t="str">
@@ -13854,7 +13925,7 @@
       <c r="F435" s="13"/>
       <c r="G435" s="21"/>
       <c r="H435" s="22" t="str">
-        <f aca="false">IF(F435="","",ROUND(F435*G435,2))</f>
+        <f>IF(F435="","",IF(OR(E435="Abschreibung (AfA)",E435="Vorsteuer auf Anlagevermögen"),0,ROUND(F435*G435,2)))</f>
         <v/>
       </c>
       <c r="I435" s="22" t="str">
@@ -13872,7 +13943,7 @@
       <c r="F436" s="13"/>
       <c r="G436" s="21"/>
       <c r="H436" s="22" t="str">
-        <f aca="false">IF(F436="","",ROUND(F436*G436,2))</f>
+        <f>IF(F436="","",IF(OR(E436="Abschreibung (AfA)",E436="Vorsteuer auf Anlagevermögen"),0,ROUND(F436*G436,2)))</f>
         <v/>
       </c>
       <c r="I436" s="22" t="str">
@@ -13890,7 +13961,7 @@
       <c r="F437" s="13"/>
       <c r="G437" s="21"/>
       <c r="H437" s="22" t="str">
-        <f aca="false">IF(F437="","",ROUND(F437*G437,2))</f>
+        <f>IF(F437="","",IF(OR(E437="Abschreibung (AfA)",E437="Vorsteuer auf Anlagevermögen"),0,ROUND(F437*G437,2)))</f>
         <v/>
       </c>
       <c r="I437" s="22" t="str">
@@ -13908,7 +13979,7 @@
       <c r="F438" s="13"/>
       <c r="G438" s="21"/>
       <c r="H438" s="22" t="str">
-        <f aca="false">IF(F438="","",ROUND(F438*G438,2))</f>
+        <f>IF(F438="","",IF(OR(E438="Abschreibung (AfA)",E438="Vorsteuer auf Anlagevermögen"),0,ROUND(F438*G438,2)))</f>
         <v/>
       </c>
       <c r="I438" s="22" t="str">
@@ -13926,7 +13997,7 @@
       <c r="F439" s="13"/>
       <c r="G439" s="21"/>
       <c r="H439" s="22" t="str">
-        <f aca="false">IF(F439="","",ROUND(F439*G439,2))</f>
+        <f>IF(F439="","",IF(OR(E439="Abschreibung (AfA)",E439="Vorsteuer auf Anlagevermögen"),0,ROUND(F439*G439,2)))</f>
         <v/>
       </c>
       <c r="I439" s="22" t="str">
@@ -13944,7 +14015,7 @@
       <c r="F440" s="13"/>
       <c r="G440" s="21"/>
       <c r="H440" s="22" t="str">
-        <f aca="false">IF(F440="","",ROUND(F440*G440,2))</f>
+        <f>IF(F440="","",IF(OR(E440="Abschreibung (AfA)",E440="Vorsteuer auf Anlagevermögen"),0,ROUND(F440*G440,2)))</f>
         <v/>
       </c>
       <c r="I440" s="22" t="str">
@@ -13962,7 +14033,7 @@
       <c r="F441" s="13"/>
       <c r="G441" s="21"/>
       <c r="H441" s="22" t="str">
-        <f aca="false">IF(F441="","",ROUND(F441*G441,2))</f>
+        <f>IF(F441="","",IF(OR(E441="Abschreibung (AfA)",E441="Vorsteuer auf Anlagevermögen"),0,ROUND(F441*G441,2)))</f>
         <v/>
       </c>
       <c r="I441" s="22" t="str">
@@ -13980,7 +14051,7 @@
       <c r="F442" s="13"/>
       <c r="G442" s="21"/>
       <c r="H442" s="22" t="str">
-        <f aca="false">IF(F442="","",ROUND(F442*G442,2))</f>
+        <f>IF(F442="","",IF(OR(E442="Abschreibung (AfA)",E442="Vorsteuer auf Anlagevermögen"),0,ROUND(F442*G442,2)))</f>
         <v/>
       </c>
       <c r="I442" s="22" t="str">
@@ -13998,7 +14069,7 @@
       <c r="F443" s="13"/>
       <c r="G443" s="21"/>
       <c r="H443" s="22" t="str">
-        <f aca="false">IF(F443="","",ROUND(F443*G443,2))</f>
+        <f>IF(F443="","",IF(OR(E443="Abschreibung (AfA)",E443="Vorsteuer auf Anlagevermögen"),0,ROUND(F443*G443,2)))</f>
         <v/>
       </c>
       <c r="I443" s="22" t="str">
@@ -14016,7 +14087,7 @@
       <c r="F444" s="13"/>
       <c r="G444" s="21"/>
       <c r="H444" s="22" t="str">
-        <f aca="false">IF(F444="","",ROUND(F444*G444,2))</f>
+        <f>IF(F444="","",IF(OR(E444="Abschreibung (AfA)",E444="Vorsteuer auf Anlagevermögen"),0,ROUND(F444*G444,2)))</f>
         <v/>
       </c>
       <c r="I444" s="22" t="str">
@@ -14034,7 +14105,7 @@
       <c r="F445" s="13"/>
       <c r="G445" s="21"/>
       <c r="H445" s="22" t="str">
-        <f aca="false">IF(F445="","",ROUND(F445*G445,2))</f>
+        <f>IF(F445="","",IF(OR(E445="Abschreibung (AfA)",E445="Vorsteuer auf Anlagevermögen"),0,ROUND(F445*G445,2)))</f>
         <v/>
       </c>
       <c r="I445" s="22" t="str">
@@ -14052,7 +14123,7 @@
       <c r="F446" s="13"/>
       <c r="G446" s="21"/>
       <c r="H446" s="22" t="str">
-        <f aca="false">IF(F446="","",ROUND(F446*G446,2))</f>
+        <f>IF(F446="","",IF(OR(E446="Abschreibung (AfA)",E446="Vorsteuer auf Anlagevermögen"),0,ROUND(F446*G446,2)))</f>
         <v/>
       </c>
       <c r="I446" s="22" t="str">
@@ -14070,7 +14141,7 @@
       <c r="F447" s="13"/>
       <c r="G447" s="21"/>
       <c r="H447" s="22" t="str">
-        <f aca="false">IF(F447="","",ROUND(F447*G447,2))</f>
+        <f>IF(F447="","",IF(OR(E447="Abschreibung (AfA)",E447="Vorsteuer auf Anlagevermögen"),0,ROUND(F447*G447,2)))</f>
         <v/>
       </c>
       <c r="I447" s="22" t="str">
@@ -14088,7 +14159,7 @@
       <c r="F448" s="13"/>
       <c r="G448" s="21"/>
       <c r="H448" s="22" t="str">
-        <f aca="false">IF(F448="","",ROUND(F448*G448,2))</f>
+        <f>IF(F448="","",IF(OR(E448="Abschreibung (AfA)",E448="Vorsteuer auf Anlagevermögen"),0,ROUND(F448*G448,2)))</f>
         <v/>
       </c>
       <c r="I448" s="22" t="str">
@@ -14106,7 +14177,7 @@
       <c r="F449" s="13"/>
       <c r="G449" s="21"/>
       <c r="H449" s="22" t="str">
-        <f aca="false">IF(F449="","",ROUND(F449*G449,2))</f>
+        <f>IF(F449="","",IF(OR(E449="Abschreibung (AfA)",E449="Vorsteuer auf Anlagevermögen"),0,ROUND(F449*G449,2)))</f>
         <v/>
       </c>
       <c r="I449" s="22" t="str">
@@ -14124,7 +14195,7 @@
       <c r="F450" s="13"/>
       <c r="G450" s="21"/>
       <c r="H450" s="22" t="str">
-        <f aca="false">IF(F450="","",ROUND(F450*G450,2))</f>
+        <f>IF(F450="","",IF(OR(E450="Abschreibung (AfA)",E450="Vorsteuer auf Anlagevermögen"),0,ROUND(F450*G450,2)))</f>
         <v/>
       </c>
       <c r="I450" s="22" t="str">
@@ -14142,7 +14213,7 @@
       <c r="F451" s="13"/>
       <c r="G451" s="21"/>
       <c r="H451" s="22" t="str">
-        <f aca="false">IF(F451="","",ROUND(F451*G451,2))</f>
+        <f>IF(F451="","",IF(OR(E451="Abschreibung (AfA)",E451="Vorsteuer auf Anlagevermögen"),0,ROUND(F451*G451,2)))</f>
         <v/>
       </c>
       <c r="I451" s="22" t="str">
@@ -14160,7 +14231,7 @@
       <c r="F452" s="13"/>
       <c r="G452" s="21"/>
       <c r="H452" s="22" t="str">
-        <f aca="false">IF(F452="","",ROUND(F452*G452,2))</f>
+        <f>IF(F452="","",IF(OR(E452="Abschreibung (AfA)",E452="Vorsteuer auf Anlagevermögen"),0,ROUND(F452*G452,2)))</f>
         <v/>
       </c>
       <c r="I452" s="22" t="str">
@@ -14178,7 +14249,7 @@
       <c r="F453" s="13"/>
       <c r="G453" s="21"/>
       <c r="H453" s="22" t="str">
-        <f aca="false">IF(F453="","",ROUND(F453*G453,2))</f>
+        <f>IF(F453="","",IF(OR(E453="Abschreibung (AfA)",E453="Vorsteuer auf Anlagevermögen"),0,ROUND(F453*G453,2)))</f>
         <v/>
       </c>
       <c r="I453" s="22" t="str">
@@ -14196,7 +14267,7 @@
       <c r="F454" s="13"/>
       <c r="G454" s="21"/>
       <c r="H454" s="22" t="str">
-        <f aca="false">IF(F454="","",ROUND(F454*G454,2))</f>
+        <f>IF(F454="","",IF(OR(E454="Abschreibung (AfA)",E454="Vorsteuer auf Anlagevermögen"),0,ROUND(F454*G454,2)))</f>
         <v/>
       </c>
       <c r="I454" s="22" t="str">
@@ -14214,7 +14285,7 @@
       <c r="F455" s="13"/>
       <c r="G455" s="21"/>
       <c r="H455" s="22" t="str">
-        <f aca="false">IF(F455="","",ROUND(F455*G455,2))</f>
+        <f>IF(F455="","",IF(OR(E455="Abschreibung (AfA)",E455="Vorsteuer auf Anlagevermögen"),0,ROUND(F455*G455,2)))</f>
         <v/>
       </c>
       <c r="I455" s="22" t="str">
@@ -14232,7 +14303,7 @@
       <c r="F456" s="13"/>
       <c r="G456" s="21"/>
       <c r="H456" s="22" t="str">
-        <f aca="false">IF(F456="","",ROUND(F456*G456,2))</f>
+        <f>IF(F456="","",IF(OR(E456="Abschreibung (AfA)",E456="Vorsteuer auf Anlagevermögen"),0,ROUND(F456*G456,2)))</f>
         <v/>
       </c>
       <c r="I456" s="22" t="str">
@@ -14250,7 +14321,7 @@
       <c r="F457" s="13"/>
       <c r="G457" s="21"/>
       <c r="H457" s="22" t="str">
-        <f aca="false">IF(F457="","",ROUND(F457*G457,2))</f>
+        <f>IF(F457="","",IF(OR(E457="Abschreibung (AfA)",E457="Vorsteuer auf Anlagevermögen"),0,ROUND(F457*G457,2)))</f>
         <v/>
       </c>
       <c r="I457" s="22" t="str">
@@ -14268,7 +14339,7 @@
       <c r="F458" s="13"/>
       <c r="G458" s="21"/>
       <c r="H458" s="22" t="str">
-        <f aca="false">IF(F458="","",ROUND(F458*G458,2))</f>
+        <f>IF(F458="","",IF(OR(E458="Abschreibung (AfA)",E458="Vorsteuer auf Anlagevermögen"),0,ROUND(F458*G458,2)))</f>
         <v/>
       </c>
       <c r="I458" s="22" t="str">
@@ -14286,7 +14357,7 @@
       <c r="F459" s="13"/>
       <c r="G459" s="21"/>
       <c r="H459" s="22" t="str">
-        <f aca="false">IF(F459="","",ROUND(F459*G459,2))</f>
+        <f>IF(F459="","",IF(OR(E459="Abschreibung (AfA)",E459="Vorsteuer auf Anlagevermögen"),0,ROUND(F459*G459,2)))</f>
         <v/>
       </c>
       <c r="I459" s="22" t="str">
@@ -14304,7 +14375,7 @@
       <c r="F460" s="13"/>
       <c r="G460" s="21"/>
       <c r="H460" s="22" t="str">
-        <f aca="false">IF(F460="","",ROUND(F460*G460,2))</f>
+        <f>IF(F460="","",IF(OR(E460="Abschreibung (AfA)",E460="Vorsteuer auf Anlagevermögen"),0,ROUND(F460*G460,2)))</f>
         <v/>
       </c>
       <c r="I460" s="22" t="str">
@@ -14322,7 +14393,7 @@
       <c r="F461" s="13"/>
       <c r="G461" s="21"/>
       <c r="H461" s="22" t="str">
-        <f aca="false">IF(F461="","",ROUND(F461*G461,2))</f>
+        <f>IF(F461="","",IF(OR(E461="Abschreibung (AfA)",E461="Vorsteuer auf Anlagevermögen"),0,ROUND(F461*G461,2)))</f>
         <v/>
       </c>
       <c r="I461" s="22" t="str">
@@ -14340,7 +14411,7 @@
       <c r="F462" s="13"/>
       <c r="G462" s="21"/>
       <c r="H462" s="22" t="str">
-        <f aca="false">IF(F462="","",ROUND(F462*G462,2))</f>
+        <f>IF(F462="","",IF(OR(E462="Abschreibung (AfA)",E462="Vorsteuer auf Anlagevermögen"),0,ROUND(F462*G462,2)))</f>
         <v/>
       </c>
       <c r="I462" s="22" t="str">
@@ -14358,7 +14429,7 @@
       <c r="F463" s="13"/>
       <c r="G463" s="21"/>
       <c r="H463" s="22" t="str">
-        <f aca="false">IF(F463="","",ROUND(F463*G463,2))</f>
+        <f>IF(F463="","",IF(OR(E463="Abschreibung (AfA)",E463="Vorsteuer auf Anlagevermögen"),0,ROUND(F463*G463,2)))</f>
         <v/>
       </c>
       <c r="I463" s="22" t="str">
@@ -14376,7 +14447,7 @@
       <c r="F464" s="13"/>
       <c r="G464" s="21"/>
       <c r="H464" s="22" t="str">
-        <f aca="false">IF(F464="","",ROUND(F464*G464,2))</f>
+        <f>IF(F464="","",IF(OR(E464="Abschreibung (AfA)",E464="Vorsteuer auf Anlagevermögen"),0,ROUND(F464*G464,2)))</f>
         <v/>
       </c>
       <c r="I464" s="22" t="str">
@@ -14394,7 +14465,7 @@
       <c r="F465" s="13"/>
       <c r="G465" s="21"/>
       <c r="H465" s="22" t="str">
-        <f aca="false">IF(F465="","",ROUND(F465*G465,2))</f>
+        <f>IF(F465="","",IF(OR(E465="Abschreibung (AfA)",E465="Vorsteuer auf Anlagevermögen"),0,ROUND(F465*G465,2)))</f>
         <v/>
       </c>
       <c r="I465" s="22" t="str">
@@ -14412,7 +14483,7 @@
       <c r="F466" s="13"/>
       <c r="G466" s="21"/>
       <c r="H466" s="22" t="str">
-        <f aca="false">IF(F466="","",ROUND(F466*G466,2))</f>
+        <f>IF(F466="","",IF(OR(E466="Abschreibung (AfA)",E466="Vorsteuer auf Anlagevermögen"),0,ROUND(F466*G466,2)))</f>
         <v/>
       </c>
       <c r="I466" s="22" t="str">
@@ -14430,7 +14501,7 @@
       <c r="F467" s="13"/>
       <c r="G467" s="21"/>
       <c r="H467" s="22" t="str">
-        <f aca="false">IF(F467="","",ROUND(F467*G467,2))</f>
+        <f>IF(F467="","",IF(OR(E467="Abschreibung (AfA)",E467="Vorsteuer auf Anlagevermögen"),0,ROUND(F467*G467,2)))</f>
         <v/>
       </c>
       <c r="I467" s="22" t="str">
@@ -14448,7 +14519,7 @@
       <c r="F468" s="13"/>
       <c r="G468" s="21"/>
       <c r="H468" s="22" t="str">
-        <f aca="false">IF(F468="","",ROUND(F468*G468,2))</f>
+        <f>IF(F468="","",IF(OR(E468="Abschreibung (AfA)",E468="Vorsteuer auf Anlagevermögen"),0,ROUND(F468*G468,2)))</f>
         <v/>
       </c>
       <c r="I468" s="22" t="str">
@@ -14466,7 +14537,7 @@
       <c r="F469" s="13"/>
       <c r="G469" s="21"/>
       <c r="H469" s="22" t="str">
-        <f aca="false">IF(F469="","",ROUND(F469*G469,2))</f>
+        <f>IF(F469="","",IF(OR(E469="Abschreibung (AfA)",E469="Vorsteuer auf Anlagevermögen"),0,ROUND(F469*G469,2)))</f>
         <v/>
       </c>
       <c r="I469" s="22" t="str">
@@ -14484,7 +14555,7 @@
       <c r="F470" s="13"/>
       <c r="G470" s="21"/>
       <c r="H470" s="22" t="str">
-        <f aca="false">IF(F470="","",ROUND(F470*G470,2))</f>
+        <f>IF(F470="","",IF(OR(E470="Abschreibung (AfA)",E470="Vorsteuer auf Anlagevermögen"),0,ROUND(F470*G470,2)))</f>
         <v/>
       </c>
       <c r="I470" s="22" t="str">
@@ -14502,7 +14573,7 @@
       <c r="F471" s="13"/>
       <c r="G471" s="21"/>
       <c r="H471" s="22" t="str">
-        <f aca="false">IF(F471="","",ROUND(F471*G471,2))</f>
+        <f>IF(F471="","",IF(OR(E471="Abschreibung (AfA)",E471="Vorsteuer auf Anlagevermögen"),0,ROUND(F471*G471,2)))</f>
         <v/>
       </c>
       <c r="I471" s="22" t="str">
@@ -14520,7 +14591,7 @@
       <c r="F472" s="13"/>
       <c r="G472" s="21"/>
       <c r="H472" s="22" t="str">
-        <f aca="false">IF(F472="","",ROUND(F472*G472,2))</f>
+        <f>IF(F472="","",IF(OR(E472="Abschreibung (AfA)",E472="Vorsteuer auf Anlagevermögen"),0,ROUND(F472*G472,2)))</f>
         <v/>
       </c>
       <c r="I472" s="22" t="str">
@@ -14538,7 +14609,7 @@
       <c r="F473" s="13"/>
       <c r="G473" s="21"/>
       <c r="H473" s="22" t="str">
-        <f aca="false">IF(F473="","",ROUND(F473*G473,2))</f>
+        <f>IF(F473="","",IF(OR(E473="Abschreibung (AfA)",E473="Vorsteuer auf Anlagevermögen"),0,ROUND(F473*G473,2)))</f>
         <v/>
       </c>
       <c r="I473" s="22" t="str">
@@ -14556,7 +14627,7 @@
       <c r="F474" s="13"/>
       <c r="G474" s="21"/>
       <c r="H474" s="22" t="str">
-        <f aca="false">IF(F474="","",ROUND(F474*G474,2))</f>
+        <f>IF(F474="","",IF(OR(E474="Abschreibung (AfA)",E474="Vorsteuer auf Anlagevermögen"),0,ROUND(F474*G474,2)))</f>
         <v/>
       </c>
       <c r="I474" s="22" t="str">
@@ -14574,7 +14645,7 @@
       <c r="F475" s="13"/>
       <c r="G475" s="21"/>
       <c r="H475" s="22" t="str">
-        <f aca="false">IF(F475="","",ROUND(F475*G475,2))</f>
+        <f>IF(F475="","",IF(OR(E475="Abschreibung (AfA)",E475="Vorsteuer auf Anlagevermögen"),0,ROUND(F475*G475,2)))</f>
         <v/>
       </c>
       <c r="I475" s="22" t="str">
@@ -14592,7 +14663,7 @@
       <c r="F476" s="13"/>
       <c r="G476" s="21"/>
       <c r="H476" s="22" t="str">
-        <f aca="false">IF(F476="","",ROUND(F476*G476,2))</f>
+        <f>IF(F476="","",IF(OR(E476="Abschreibung (AfA)",E476="Vorsteuer auf Anlagevermögen"),0,ROUND(F476*G476,2)))</f>
         <v/>
       </c>
       <c r="I476" s="22" t="str">
@@ -14610,7 +14681,7 @@
       <c r="F477" s="13"/>
       <c r="G477" s="21"/>
       <c r="H477" s="22" t="str">
-        <f aca="false">IF(F477="","",ROUND(F477*G477,2))</f>
+        <f>IF(F477="","",IF(OR(E477="Abschreibung (AfA)",E477="Vorsteuer auf Anlagevermögen"),0,ROUND(F477*G477,2)))</f>
         <v/>
       </c>
       <c r="I477" s="22" t="str">
@@ -14628,7 +14699,7 @@
       <c r="F478" s="13"/>
       <c r="G478" s="21"/>
       <c r="H478" s="22" t="str">
-        <f aca="false">IF(F478="","",ROUND(F478*G478,2))</f>
+        <f>IF(F478="","",IF(OR(E478="Abschreibung (AfA)",E478="Vorsteuer auf Anlagevermögen"),0,ROUND(F478*G478,2)))</f>
         <v/>
       </c>
       <c r="I478" s="22" t="str">
@@ -14646,7 +14717,7 @@
       <c r="F479" s="13"/>
       <c r="G479" s="21"/>
       <c r="H479" s="22" t="str">
-        <f aca="false">IF(F479="","",ROUND(F479*G479,2))</f>
+        <f>IF(F479="","",IF(OR(E479="Abschreibung (AfA)",E479="Vorsteuer auf Anlagevermögen"),0,ROUND(F479*G479,2)))</f>
         <v/>
       </c>
       <c r="I479" s="22" t="str">
@@ -14664,7 +14735,7 @@
       <c r="F480" s="13"/>
       <c r="G480" s="21"/>
       <c r="H480" s="22" t="str">
-        <f aca="false">IF(F480="","",ROUND(F480*G480,2))</f>
+        <f>IF(F480="","",IF(OR(E480="Abschreibung (AfA)",E480="Vorsteuer auf Anlagevermögen"),0,ROUND(F480*G480,2)))</f>
         <v/>
       </c>
       <c r="I480" s="22" t="str">
@@ -14682,7 +14753,7 @@
       <c r="F481" s="13"/>
       <c r="G481" s="21"/>
       <c r="H481" s="22" t="str">
-        <f aca="false">IF(F481="","",ROUND(F481*G481,2))</f>
+        <f>IF(F481="","",IF(OR(E481="Abschreibung (AfA)",E481="Vorsteuer auf Anlagevermögen"),0,ROUND(F481*G481,2)))</f>
         <v/>
       </c>
       <c r="I481" s="22" t="str">
@@ -14700,7 +14771,7 @@
       <c r="F482" s="13"/>
       <c r="G482" s="21"/>
       <c r="H482" s="22" t="str">
-        <f aca="false">IF(F482="","",ROUND(F482*G482,2))</f>
+        <f>IF(F482="","",IF(OR(E482="Abschreibung (AfA)",E482="Vorsteuer auf Anlagevermögen"),0,ROUND(F482*G482,2)))</f>
         <v/>
       </c>
       <c r="I482" s="22" t="str">
@@ -14718,7 +14789,7 @@
       <c r="F483" s="13"/>
       <c r="G483" s="21"/>
       <c r="H483" s="22" t="str">
-        <f aca="false">IF(F483="","",ROUND(F483*G483,2))</f>
+        <f>IF(F483="","",IF(OR(E483="Abschreibung (AfA)",E483="Vorsteuer auf Anlagevermögen"),0,ROUND(F483*G483,2)))</f>
         <v/>
       </c>
       <c r="I483" s="22" t="str">
@@ -14736,7 +14807,7 @@
       <c r="F484" s="13"/>
       <c r="G484" s="21"/>
       <c r="H484" s="22" t="str">
-        <f aca="false">IF(F484="","",ROUND(F484*G484,2))</f>
+        <f>IF(F484="","",IF(OR(E484="Abschreibung (AfA)",E484="Vorsteuer auf Anlagevermögen"),0,ROUND(F484*G484,2)))</f>
         <v/>
       </c>
       <c r="I484" s="22" t="str">
@@ -14754,7 +14825,7 @@
       <c r="F485" s="13"/>
       <c r="G485" s="21"/>
       <c r="H485" s="22" t="str">
-        <f aca="false">IF(F485="","",ROUND(F485*G485,2))</f>
+        <f>IF(F485="","",IF(OR(E485="Abschreibung (AfA)",E485="Vorsteuer auf Anlagevermögen"),0,ROUND(F485*G485,2)))</f>
         <v/>
       </c>
       <c r="I485" s="22" t="str">
@@ -14772,7 +14843,7 @@
       <c r="F486" s="13"/>
       <c r="G486" s="21"/>
       <c r="H486" s="22" t="str">
-        <f aca="false">IF(F486="","",ROUND(F486*G486,2))</f>
+        <f>IF(F486="","",IF(OR(E486="Abschreibung (AfA)",E486="Vorsteuer auf Anlagevermögen"),0,ROUND(F486*G486,2)))</f>
         <v/>
       </c>
       <c r="I486" s="22" t="str">
@@ -14790,7 +14861,7 @@
       <c r="F487" s="13"/>
       <c r="G487" s="21"/>
       <c r="H487" s="22" t="str">
-        <f aca="false">IF(F487="","",ROUND(F487*G487,2))</f>
+        <f>IF(F487="","",IF(OR(E487="Abschreibung (AfA)",E487="Vorsteuer auf Anlagevermögen"),0,ROUND(F487*G487,2)))</f>
         <v/>
       </c>
       <c r="I487" s="22" t="str">
@@ -14808,7 +14879,7 @@
       <c r="F488" s="13"/>
       <c r="G488" s="21"/>
       <c r="H488" s="22" t="str">
-        <f aca="false">IF(F488="","",ROUND(F488*G488,2))</f>
+        <f>IF(F488="","",IF(OR(E488="Abschreibung (AfA)",E488="Vorsteuer auf Anlagevermögen"),0,ROUND(F488*G488,2)))</f>
         <v/>
       </c>
       <c r="I488" s="22" t="str">
@@ -14826,7 +14897,7 @@
       <c r="F489" s="13"/>
       <c r="G489" s="21"/>
       <c r="H489" s="22" t="str">
-        <f aca="false">IF(F489="","",ROUND(F489*G489,2))</f>
+        <f>IF(F489="","",IF(OR(E489="Abschreibung (AfA)",E489="Vorsteuer auf Anlagevermögen"),0,ROUND(F489*G489,2)))</f>
         <v/>
       </c>
       <c r="I489" s="22" t="str">
@@ -14844,7 +14915,7 @@
       <c r="F490" s="13"/>
       <c r="G490" s="21"/>
       <c r="H490" s="22" t="str">
-        <f aca="false">IF(F490="","",ROUND(F490*G490,2))</f>
+        <f>IF(F490="","",IF(OR(E490="Abschreibung (AfA)",E490="Vorsteuer auf Anlagevermögen"),0,ROUND(F490*G490,2)))</f>
         <v/>
       </c>
       <c r="I490" s="22" t="str">
@@ -14862,7 +14933,7 @@
       <c r="F491" s="13"/>
       <c r="G491" s="21"/>
       <c r="H491" s="22" t="str">
-        <f aca="false">IF(F491="","",ROUND(F491*G491,2))</f>
+        <f>IF(F491="","",IF(OR(E491="Abschreibung (AfA)",E491="Vorsteuer auf Anlagevermögen"),0,ROUND(F491*G491,2)))</f>
         <v/>
       </c>
       <c r="I491" s="22" t="str">
@@ -14880,7 +14951,7 @@
       <c r="F492" s="13"/>
       <c r="G492" s="21"/>
       <c r="H492" s="22" t="str">
-        <f aca="false">IF(F492="","",ROUND(F492*G492,2))</f>
+        <f>IF(F492="","",IF(OR(E492="Abschreibung (AfA)",E492="Vorsteuer auf Anlagevermögen"),0,ROUND(F492*G492,2)))</f>
         <v/>
       </c>
       <c r="I492" s="22" t="str">
@@ -14898,7 +14969,7 @@
       <c r="F493" s="13"/>
       <c r="G493" s="21"/>
       <c r="H493" s="22" t="str">
-        <f aca="false">IF(F493="","",ROUND(F493*G493,2))</f>
+        <f>IF(F493="","",IF(OR(E493="Abschreibung (AfA)",E493="Vorsteuer auf Anlagevermögen"),0,ROUND(F493*G493,2)))</f>
         <v/>
       </c>
       <c r="I493" s="22" t="str">
@@ -14916,7 +14987,7 @@
       <c r="F494" s="13"/>
       <c r="G494" s="21"/>
       <c r="H494" s="22" t="str">
-        <f aca="false">IF(F494="","",ROUND(F494*G494,2))</f>
+        <f>IF(F494="","",IF(OR(E494="Abschreibung (AfA)",E494="Vorsteuer auf Anlagevermögen"),0,ROUND(F494*G494,2)))</f>
         <v/>
       </c>
       <c r="I494" s="22" t="str">
@@ -14934,7 +15005,7 @@
       <c r="F495" s="13"/>
       <c r="G495" s="21"/>
       <c r="H495" s="22" t="str">
-        <f aca="false">IF(F495="","",ROUND(F495*G495,2))</f>
+        <f>IF(F495="","",IF(OR(E495="Abschreibung (AfA)",E495="Vorsteuer auf Anlagevermögen"),0,ROUND(F495*G495,2)))</f>
         <v/>
       </c>
       <c r="I495" s="22" t="str">
@@ -14952,7 +15023,7 @@
       <c r="F496" s="13"/>
       <c r="G496" s="21"/>
       <c r="H496" s="22" t="str">
-        <f aca="false">IF(F496="","",ROUND(F496*G496,2))</f>
+        <f>IF(F496="","",IF(OR(E496="Abschreibung (AfA)",E496="Vorsteuer auf Anlagevermögen"),0,ROUND(F496*G496,2)))</f>
         <v/>
       </c>
       <c r="I496" s="22" t="str">
@@ -14970,7 +15041,7 @@
       <c r="F497" s="13"/>
       <c r="G497" s="21"/>
       <c r="H497" s="22" t="str">
-        <f aca="false">IF(F497="","",ROUND(F497*G497,2))</f>
+        <f>IF(F497="","",IF(OR(E497="Abschreibung (AfA)",E497="Vorsteuer auf Anlagevermögen"),0,ROUND(F497*G497,2)))</f>
         <v/>
       </c>
       <c r="I497" s="22" t="str">
@@ -14988,7 +15059,7 @@
       <c r="F498" s="13"/>
       <c r="G498" s="21"/>
       <c r="H498" s="22" t="str">
-        <f aca="false">IF(F498="","",ROUND(F498*G498,2))</f>
+        <f>IF(F498="","",IF(OR(E498="Abschreibung (AfA)",E498="Vorsteuer auf Anlagevermögen"),0,ROUND(F498*G498,2)))</f>
         <v/>
       </c>
       <c r="I498" s="22" t="str">
@@ -15006,7 +15077,7 @@
       <c r="F499" s="13"/>
       <c r="G499" s="21"/>
       <c r="H499" s="22" t="str">
-        <f aca="false">IF(F499="","",ROUND(F499*G499,2))</f>
+        <f>IF(F499="","",IF(OR(E499="Abschreibung (AfA)",E499="Vorsteuer auf Anlagevermögen"),0,ROUND(F499*G499,2)))</f>
         <v/>
       </c>
       <c r="I499" s="22" t="str">
@@ -15024,7 +15095,7 @@
       <c r="F500" s="13"/>
       <c r="G500" s="21"/>
       <c r="H500" s="22" t="str">
-        <f aca="false">IF(F500="","",ROUND(F500*G500,2))</f>
+        <f>IF(F500="","",IF(OR(E500="Abschreibung (AfA)",E500="Vorsteuer auf Anlagevermögen"),0,ROUND(F500*G500,2)))</f>
         <v/>
       </c>
       <c r="I500" s="22" t="str">
@@ -15042,7 +15113,7 @@
       <c r="F501" s="13"/>
       <c r="G501" s="21"/>
       <c r="H501" s="22" t="str">
-        <f aca="false">IF(F501="","",ROUND(F501*G501,2))</f>
+        <f>IF(F501="","",IF(OR(E501="Abschreibung (AfA)",E501="Vorsteuer auf Anlagevermögen"),0,ROUND(F501*G501,2)))</f>
         <v/>
       </c>
       <c r="I501" s="22" t="str">
@@ -15060,7 +15131,7 @@
       <c r="F502" s="13"/>
       <c r="G502" s="21"/>
       <c r="H502" s="22" t="str">
-        <f aca="false">IF(F502="","",ROUND(F502*G502,2))</f>
+        <f>IF(F502="","",IF(OR(E502="Abschreibung (AfA)",E502="Vorsteuer auf Anlagevermögen"),0,ROUND(F502*G502,2)))</f>
         <v/>
       </c>
       <c r="I502" s="22" t="str">
@@ -15078,7 +15149,7 @@
       <c r="F503" s="13"/>
       <c r="G503" s="21"/>
       <c r="H503" s="22" t="str">
-        <f aca="false">IF(F503="","",ROUND(F503*G503,2))</f>
+        <f>IF(F503="","",IF(OR(E503="Abschreibung (AfA)",E503="Vorsteuer auf Anlagevermögen"),0,ROUND(F503*G503,2)))</f>
         <v/>
       </c>
       <c r="I503" s="22" t="str">
@@ -15096,7 +15167,7 @@
       <c r="F504" s="13"/>
       <c r="G504" s="21"/>
       <c r="H504" s="22" t="str">
-        <f aca="false">IF(F504="","",ROUND(F504*G504,2))</f>
+        <f>IF(F504="","",IF(OR(E504="Abschreibung (AfA)",E504="Vorsteuer auf Anlagevermögen"),0,ROUND(F504*G504,2)))</f>
         <v/>
       </c>
       <c r="I504" s="22" t="str">
@@ -15114,7 +15185,7 @@
       <c r="F505" s="13"/>
       <c r="G505" s="21"/>
       <c r="H505" s="22" t="str">
-        <f aca="false">IF(F505="","",ROUND(F505*G505,2))</f>
+        <f>IF(F505="","",IF(OR(E505="Abschreibung (AfA)",E505="Vorsteuer auf Anlagevermögen"),0,ROUND(F505*G505,2)))</f>
         <v/>
       </c>
       <c r="I505" s="22" t="str">
@@ -15132,7 +15203,7 @@
       <c r="F506" s="13"/>
       <c r="G506" s="21"/>
       <c r="H506" s="22" t="str">
-        <f aca="false">IF(F506="","",ROUND(F506*G506,2))</f>
+        <f>IF(F506="","",IF(OR(E506="Abschreibung (AfA)",E506="Vorsteuer auf Anlagevermögen"),0,ROUND(F506*G506,2)))</f>
         <v/>
       </c>
       <c r="I506" s="22" t="str">
@@ -15150,7 +15221,7 @@
       <c r="F507" s="13"/>
       <c r="G507" s="21"/>
       <c r="H507" s="22" t="str">
-        <f aca="false">IF(F507="","",ROUND(F507*G507,2))</f>
+        <f>IF(F507="","",IF(OR(E507="Abschreibung (AfA)",E507="Vorsteuer auf Anlagevermögen"),0,ROUND(F507*G507,2)))</f>
         <v/>
       </c>
       <c r="I507" s="22" t="str">
@@ -15166,7 +15237,7 @@
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" error="Bitte einen Wert aus der Liste wählen." errorStyle="stop" errorTitle="Ungültiger Eintrag" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E8:E507" type="list">
-      <formula1>Listen!$C$2:$C$20</formula1>
+      <formula1>'Listen'!$C$2:$C$21</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" error="Bitte einen Wert aus der Liste wählen." errorStyle="stop" errorTitle="Ungültiger Eintrag" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="G8:G507" type="list">
@@ -15189,7 +15260,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D20"/>
+  <dimension ref="A1:D21"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15401,6 +15472,13 @@
         <v>83</v>
       </c>
       <c r="D20" s="23"/>
+    </row>
+    <row r="21">
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Vorsteuer auf Anlagevermögen</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
Publish site from 02f5cfd
</commit_message>
<xml_diff>
--- a/einnahmenueberschussrechnung/euer-vorlage-2026-firmendo.xlsx
+++ b/einnahmenueberschussrechnung/euer-vorlage-2026-firmendo.xlsx
@@ -518,7 +518,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="24">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -613,30 +613,6 @@
     </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -941,11 +917,9 @@
         <v>7</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="42" hidden="false" customHeight="1" outlineLevel="0" collapsed="false">
-      <c r="B10" s="24" t="inlineStr">
-        <is>
-          <t>• Beispiele leeren: Kleinunternehmer A8:G10; Regelbesteuert A8:G11 und J8:J11. Nur Eingaben löschen, niemals ganze Zeilen, Formeln oder die Auswertung rechts.</t>
-        </is>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B10" s="3" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -978,11 +952,9 @@
         <v>14</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="68" hidden="false" customHeight="1" outlineLevel="0" collapsed="false">
-      <c r="B17" s="24" t="inlineStr">
-        <is>
-          <t>• AfA: Nur den Jahresbetrag als „Abschreibung (AfA)“ erfassen, USt-Satz 0 %. Bei Regelbesteuerung die bezahlte, abziehbare Vorsteuer der Anschaffung separat als Ausgabe „Vorsteuer auf Anlagevermögen“ in F eintragen, ebenfalls mit 0 %. Beispiel: Kauf 3.000 € netto + 570 € USt, Jahres-AfA 300 € → zwei Einträge: 300 € AfA und 570 € Vorsteuer. In Folgejahren nur AfA, keine erneute Vorsteuer ohne neue Zahlung. GWG bis 800 € netto bleiben sofort abziehbar.</t>
-        </is>
+    <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B17" s="3" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -995,11 +967,9 @@
         <v>17</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="44" hidden="false" customHeight="1" outlineLevel="0" collapsed="false">
-      <c r="B20" s="24" t="inlineStr">
-        <is>
-          <t>• Geldentnahmen und Einlagen verändern den Gewinn nicht und werden hier nicht mitgerechnet. Für die ergänzenden Angaben der Anlage EÜR gesondert aufzeichnen (Anlage EÜR 2025: Zeilen 106/107).</t>
-        </is>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B20" s="3" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1022,13 +992,8 @@
         <v>22</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="44" hidden="false" customHeight="1" outlineLevel="0" collapsed="false">
-      <c r="B25" s="24" t="inlineStr">
-        <is>
-          <t>Quellen: https://www.elster.de/elsterweb/helpGlobal?themaGlobal=help_euer_ufa_77_2025
-https://www.gesetze-im-internet.de/estg/__4.html · geprüft am 07.10.2026</t>
-        </is>
-      </c>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B25" s="3"/>
     </row>
     <row r="26" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="2" t="s">
@@ -1085,10 +1050,8 @@
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="6" t="inlineStr">
-        <is>
-          <t>Nur gelbe Beispiel-Eingaben A8:G10 leeren. Ganze Zeilen und die Auswertung I/J erhalten.</t>
-        </is>
+      <c r="A4" s="6" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5905,10 +5868,8 @@
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="6" t="inlineStr">
-        <is>
-          <t>Nur gelbe Beispiel-Eingaben A8:G11 und J8:J11 leeren. Ganze Zeilen, H/I und Auswertung L/M erhalten.</t>
-        </is>
+      <c r="A4" s="6" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5916,7 +5877,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
         <v>29</v>
       </c>
@@ -5932,21 +5893,17 @@
       <c r="E7" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="F7" s="25" t="inlineStr">
-        <is>
-          <t>Netto / Sonderbetrag (€)</t>
-        </is>
-      </c>
-      <c r="G7" s="25" t="s">
+      <c r="F7" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="G7" s="9" t="s">
         <v>75</v>
       </c>
-      <c r="H7" s="25" t="s">
+      <c r="H7" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="I7" s="25" t="inlineStr">
-        <is>
-          <t>Betrag inkl. USt (€)</t>
-        </is>
+      <c r="I7" s="9" t="s">
+        <v>77</v>
       </c>
       <c r="J7" s="9" t="s">
         <v>35</v>
@@ -5981,7 +5938,7 @@
         <v>0.19</v>
       </c>
       <c r="H8" s="22" t="n">
-        <f>IF(F8="","",IF(OR(E8="Abschreibung (AfA)",E8="Vorsteuer auf Anlagevermögen"),0,ROUND(F8*G8,2)))</f>
+        <f aca="false">IF(F8="","",ROUND(F8*G8,2))</f>
         <v>380</v>
       </c>
       <c r="I8" s="22" t="n">
@@ -5996,40 +5953,38 @@
       </c>
       <c r="M8" s="15"/>
     </row>
-    <row r="9" customFormat="false" ht="32" hidden="false" customHeight="1" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="11" t="n">
         <v>46042</v>
       </c>
       <c r="B9" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="C9" s="26" t="s">
+      <c r="C9" s="12" t="s">
         <v>79</v>
       </c>
-      <c r="D9" s="26" t="s">
+      <c r="D9" s="12" t="s">
         <v>46</v>
       </c>
-      <c r="E9" s="26" t="s">
+      <c r="E9" s="12" t="s">
         <v>63</v>
       </c>
-      <c r="F9" s="27" t="n">
+      <c r="F9" s="13" t="n">
         <v>1100</v>
       </c>
-      <c r="G9" s="28">
-        <v>0</v>
-      </c>
-      <c r="H9" s="29" t="n">
-        <f>IF(F9="","",IF(OR(E9="Abschreibung (AfA)",E9="Vorsteuer auf Anlagevermögen"),0,ROUND(F9*G9,2)))</f>
-        <v>0</v>
-      </c>
-      <c r="I9" s="29" t="n">
+      <c r="G9" s="21" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="H9" s="22" t="n">
+        <f aca="false">IF(F9="","",ROUND(F9*G9,2))</f>
+        <v>209</v>
+      </c>
+      <c r="I9" s="22" t="n">
         <f aca="false">IF(F9="","",F9+H9)</f>
         <v>1309</v>
       </c>
-      <c r="J9" s="26" t="inlineStr">
-        <is>
-          <t>AfA; Vorsteuer separat in Zeile 11</t>
-        </is>
+      <c r="J9" s="12" t="s">
+        <v>42</v>
       </c>
       <c r="L9" s="16" t="s">
         <v>80</v>
@@ -6039,37 +5994,37 @@
         <v>2000</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="32" hidden="false" customHeight="1" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="11" t="n">
         <v>46063</v>
       </c>
       <c r="B10" s="12" t="s">
         <v>81</v>
       </c>
-      <c r="C10" s="26" t="s">
+      <c r="C10" s="12" t="s">
         <v>82</v>
       </c>
-      <c r="D10" s="26" t="s">
+      <c r="D10" s="12" t="s">
         <v>46</v>
       </c>
-      <c r="E10" s="26" t="s">
+      <c r="E10" s="12" t="s">
         <v>83</v>
       </c>
-      <c r="F10" s="27" t="n">
+      <c r="F10" s="13" t="n">
         <v>171</v>
       </c>
-      <c r="G10" s="28" t="n">
+      <c r="G10" s="21" t="n">
         <v>0</v>
       </c>
-      <c r="H10" s="29" t="n">
-        <f>IF(F10="","",IF(OR(E10="Abschreibung (AfA)",E10="Vorsteuer auf Anlagevermögen"),0,ROUND(F10*G10,2)))</f>
+      <c r="H10" s="22" t="n">
+        <f aca="false">IF(F10="","",ROUND(F10*G10,2))</f>
         <v>0</v>
       </c>
-      <c r="I10" s="29" t="n">
+      <c r="I10" s="22" t="n">
         <f aca="false">IF(F10="","",F10+H10)</f>
         <v>171</v>
       </c>
-      <c r="J10" s="26" t="s">
+      <c r="J10" s="12" t="s">
         <v>42</v>
       </c>
       <c r="L10" s="16" t="s">
@@ -6080,49 +6035,23 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="32" hidden="false" customHeight="1" outlineLevel="0" collapsed="false">
-      <c r="A11" s="11">
-        <v>46042</v>
-      </c>
-      <c r="B11" s="12" t="inlineStr">
-        <is>
-          <t>E-001</t>
-        </is>
-      </c>
-      <c r="C11" s="26" t="inlineStr">
-        <is>
-          <t>Vorsteuer aus Laptop-Kauf</t>
-        </is>
-      </c>
-      <c r="D11" s="26" t="inlineStr">
-        <is>
-          <t>Ausgabe</t>
-        </is>
-      </c>
-      <c r="E11" s="26" t="inlineStr">
-        <is>
-          <t>Vorsteuer auf Anlagevermögen</t>
-        </is>
-      </c>
-      <c r="F11" s="27">
-        <v>209</v>
-      </c>
-      <c r="G11" s="28">
-        <v>0</v>
-      </c>
-      <c r="H11" s="29" t="n">
-        <f>IF(F11="","",IF(OR(E11="Abschreibung (AfA)",E11="Vorsteuer auf Anlagevermögen"),0,ROUND(F11*G11,2)))</f>
-        <v>0</v>
-      </c>
-      <c r="I11" s="29" t="n">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="11"/>
+      <c r="B11" s="12"/>
+      <c r="C11" s="12"/>
+      <c r="D11" s="12"/>
+      <c r="E11" s="12"/>
+      <c r="F11" s="13"/>
+      <c r="G11" s="21"/>
+      <c r="H11" s="22" t="str">
+        <f aca="false">IF(F11="","",ROUND(F11*G11,2))</f>
+        <v/>
+      </c>
+      <c r="I11" s="22" t="str">
         <f aca="false">IF(F11="","",F11+H11)</f>
-        <v>209</v>
-      </c>
-      <c r="J11" s="26" t="inlineStr">
-        <is>
-          <t>Beispiel – Eingaben löschen</t>
-        </is>
-      </c>
+        <v/>
+      </c>
+      <c r="J11" s="12"/>
       <c r="L11" s="16" t="s">
         <v>85</v>
       </c>
@@ -6140,7 +6069,7 @@
       <c r="F12" s="13"/>
       <c r="G12" s="21"/>
       <c r="H12" s="22" t="str">
-        <f>IF(F12="","",IF(OR(E12="Abschreibung (AfA)",E12="Vorsteuer auf Anlagevermögen"),0,ROUND(F12*G12,2)))</f>
+        <f aca="false">IF(F12="","",ROUND(F12*G12,2))</f>
         <v/>
       </c>
       <c r="I12" s="22" t="str">
@@ -6165,7 +6094,7 @@
       <c r="F13" s="13"/>
       <c r="G13" s="21"/>
       <c r="H13" s="22" t="str">
-        <f>IF(F13="","",IF(OR(E13="Abschreibung (AfA)",E13="Vorsteuer auf Anlagevermögen"),0,ROUND(F13*G13,2)))</f>
+        <f aca="false">IF(F13="","",ROUND(F13*G13,2))</f>
         <v/>
       </c>
       <c r="I13" s="22" t="str">
@@ -6190,7 +6119,7 @@
       <c r="F14" s="13"/>
       <c r="G14" s="21"/>
       <c r="H14" s="22" t="str">
-        <f>IF(F14="","",IF(OR(E14="Abschreibung (AfA)",E14="Vorsteuer auf Anlagevermögen"),0,ROUND(F14*G14,2)))</f>
+        <f aca="false">IF(F14="","",ROUND(F14*G14,2))</f>
         <v/>
       </c>
       <c r="I14" s="22" t="str">
@@ -6210,7 +6139,7 @@
       <c r="F15" s="13"/>
       <c r="G15" s="21"/>
       <c r="H15" s="22" t="str">
-        <f>IF(F15="","",IF(OR(E15="Abschreibung (AfA)",E15="Vorsteuer auf Anlagevermögen"),0,ROUND(F15*G15,2)))</f>
+        <f aca="false">IF(F15="","",ROUND(F15*G15,2))</f>
         <v/>
       </c>
       <c r="I15" s="22" t="str">
@@ -6232,7 +6161,7 @@
       <c r="F16" s="13"/>
       <c r="G16" s="21"/>
       <c r="H16" s="22" t="str">
-        <f>IF(F16="","",IF(OR(E16="Abschreibung (AfA)",E16="Vorsteuer auf Anlagevermögen"),0,ROUND(F16*G16,2)))</f>
+        <f aca="false">IF(F16="","",ROUND(F16*G16,2))</f>
         <v/>
       </c>
       <c r="I16" s="22" t="str">
@@ -6257,7 +6186,7 @@
       <c r="F17" s="13"/>
       <c r="G17" s="21"/>
       <c r="H17" s="22" t="str">
-        <f>IF(F17="","",IF(OR(E17="Abschreibung (AfA)",E17="Vorsteuer auf Anlagevermögen"),0,ROUND(F17*G17,2)))</f>
+        <f aca="false">IF(F17="","",ROUND(F17*G17,2))</f>
         <v/>
       </c>
       <c r="I17" s="22" t="str">
@@ -6282,7 +6211,7 @@
       <c r="F18" s="13"/>
       <c r="G18" s="21"/>
       <c r="H18" s="22" t="str">
-        <f>IF(F18="","",IF(OR(E18="Abschreibung (AfA)",E18="Vorsteuer auf Anlagevermögen"),0,ROUND(F18*G18,2)))</f>
+        <f aca="false">IF(F18="","",ROUND(F18*G18,2))</f>
         <v/>
       </c>
       <c r="I18" s="22" t="str">
@@ -6307,7 +6236,7 @@
       <c r="F19" s="13"/>
       <c r="G19" s="21"/>
       <c r="H19" s="22" t="str">
-        <f>IF(F19="","",IF(OR(E19="Abschreibung (AfA)",E19="Vorsteuer auf Anlagevermögen"),0,ROUND(F19*G19,2)))</f>
+        <f aca="false">IF(F19="","",ROUND(F19*G19,2))</f>
         <v/>
       </c>
       <c r="I19" s="22" t="str">
@@ -6332,7 +6261,7 @@
       <c r="F20" s="13"/>
       <c r="G20" s="21"/>
       <c r="H20" s="22" t="str">
-        <f>IF(F20="","",IF(OR(E20="Abschreibung (AfA)",E20="Vorsteuer auf Anlagevermögen"),0,ROUND(F20*G20,2)))</f>
+        <f aca="false">IF(F20="","",ROUND(F20*G20,2))</f>
         <v/>
       </c>
       <c r="I20" s="22" t="str">
@@ -6357,7 +6286,7 @@
       <c r="F21" s="13"/>
       <c r="G21" s="21"/>
       <c r="H21" s="22" t="str">
-        <f>IF(F21="","",IF(OR(E21="Abschreibung (AfA)",E21="Vorsteuer auf Anlagevermögen"),0,ROUND(F21*G21,2)))</f>
+        <f aca="false">IF(F21="","",ROUND(F21*G21,2))</f>
         <v/>
       </c>
       <c r="I21" s="22" t="str">
@@ -6382,7 +6311,7 @@
       <c r="F22" s="13"/>
       <c r="G22" s="21"/>
       <c r="H22" s="22" t="str">
-        <f>IF(F22="","",IF(OR(E22="Abschreibung (AfA)",E22="Vorsteuer auf Anlagevermögen"),0,ROUND(F22*G22,2)))</f>
+        <f aca="false">IF(F22="","",ROUND(F22*G22,2))</f>
         <v/>
       </c>
       <c r="I22" s="22" t="str">
@@ -6407,7 +6336,7 @@
       <c r="F23" s="13"/>
       <c r="G23" s="21"/>
       <c r="H23" s="22" t="str">
-        <f>IF(F23="","",IF(OR(E23="Abschreibung (AfA)",E23="Vorsteuer auf Anlagevermögen"),0,ROUND(F23*G23,2)))</f>
+        <f aca="false">IF(F23="","",ROUND(F23*G23,2))</f>
         <v/>
       </c>
       <c r="I23" s="22" t="str">
@@ -6432,7 +6361,7 @@
       <c r="F24" s="13"/>
       <c r="G24" s="21"/>
       <c r="H24" s="22" t="str">
-        <f>IF(F24="","",IF(OR(E24="Abschreibung (AfA)",E24="Vorsteuer auf Anlagevermögen"),0,ROUND(F24*G24,2)))</f>
+        <f aca="false">IF(F24="","",ROUND(F24*G24,2))</f>
         <v/>
       </c>
       <c r="I24" s="22" t="str">
@@ -6457,7 +6386,7 @@
       <c r="F25" s="13"/>
       <c r="G25" s="21"/>
       <c r="H25" s="22" t="str">
-        <f>IF(F25="","",IF(OR(E25="Abschreibung (AfA)",E25="Vorsteuer auf Anlagevermögen"),0,ROUND(F25*G25,2)))</f>
+        <f aca="false">IF(F25="","",ROUND(F25*G25,2))</f>
         <v/>
       </c>
       <c r="I25" s="22" t="str">
@@ -6482,7 +6411,7 @@
       <c r="F26" s="13"/>
       <c r="G26" s="21"/>
       <c r="H26" s="22" t="str">
-        <f>IF(F26="","",IF(OR(E26="Abschreibung (AfA)",E26="Vorsteuer auf Anlagevermögen"),0,ROUND(F26*G26,2)))</f>
+        <f aca="false">IF(F26="","",ROUND(F26*G26,2))</f>
         <v/>
       </c>
       <c r="I26" s="22" t="str">
@@ -6507,7 +6436,7 @@
       <c r="F27" s="13"/>
       <c r="G27" s="21"/>
       <c r="H27" s="22" t="str">
-        <f>IF(F27="","",IF(OR(E27="Abschreibung (AfA)",E27="Vorsteuer auf Anlagevermögen"),0,ROUND(F27*G27,2)))</f>
+        <f aca="false">IF(F27="","",ROUND(F27*G27,2))</f>
         <v/>
       </c>
       <c r="I27" s="22" t="str">
@@ -6532,7 +6461,7 @@
       <c r="F28" s="13"/>
       <c r="G28" s="21"/>
       <c r="H28" s="22" t="str">
-        <f>IF(F28="","",IF(OR(E28="Abschreibung (AfA)",E28="Vorsteuer auf Anlagevermögen"),0,ROUND(F28*G28,2)))</f>
+        <f aca="false">IF(F28="","",ROUND(F28*G28,2))</f>
         <v/>
       </c>
       <c r="I28" s="22" t="str">
@@ -6557,7 +6486,7 @@
       <c r="F29" s="13"/>
       <c r="G29" s="21"/>
       <c r="H29" s="22" t="str">
-        <f>IF(F29="","",IF(OR(E29="Abschreibung (AfA)",E29="Vorsteuer auf Anlagevermögen"),0,ROUND(F29*G29,2)))</f>
+        <f aca="false">IF(F29="","",ROUND(F29*G29,2))</f>
         <v/>
       </c>
       <c r="I29" s="22" t="str">
@@ -6582,7 +6511,7 @@
       <c r="F30" s="13"/>
       <c r="G30" s="21"/>
       <c r="H30" s="22" t="str">
-        <f>IF(F30="","",IF(OR(E30="Abschreibung (AfA)",E30="Vorsteuer auf Anlagevermögen"),0,ROUND(F30*G30,2)))</f>
+        <f aca="false">IF(F30="","",ROUND(F30*G30,2))</f>
         <v/>
       </c>
       <c r="I30" s="22" t="str">
@@ -6607,7 +6536,7 @@
       <c r="F31" s="13"/>
       <c r="G31" s="21"/>
       <c r="H31" s="22" t="str">
-        <f>IF(F31="","",IF(OR(E31="Abschreibung (AfA)",E31="Vorsteuer auf Anlagevermögen"),0,ROUND(F31*G31,2)))</f>
+        <f aca="false">IF(F31="","",ROUND(F31*G31,2))</f>
         <v/>
       </c>
       <c r="I31" s="22" t="str">
@@ -6619,7 +6548,7 @@
         <v>101</v>
       </c>
       <c r="M31" s="15" t="n">
-        <f>SUMIFS($H$8:$H$507,$D$8:$D$507,"Ausgabe")+SUMIFS($F$8:$F$507,$D$8:$D$507,"Ausgabe",$E$8:$E$507,"Vorsteuer auf Anlagevermögen")</f>
+        <f aca="false">SUMIFS($H$8:$H$507,$D$8:$D$507,"Ausgabe")</f>
         <v>209</v>
       </c>
     </row>
@@ -6632,7 +6561,7 @@
       <c r="F32" s="13"/>
       <c r="G32" s="21"/>
       <c r="H32" s="22" t="str">
-        <f>IF(F32="","",IF(OR(E32="Abschreibung (AfA)",E32="Vorsteuer auf Anlagevermögen"),0,ROUND(F32*G32,2)))</f>
+        <f aca="false">IF(F32="","",ROUND(F32*G32,2))</f>
         <v/>
       </c>
       <c r="I32" s="22" t="str">
@@ -6657,7 +6586,7 @@
       <c r="F33" s="13"/>
       <c r="G33" s="21"/>
       <c r="H33" s="22" t="str">
-        <f>IF(F33="","",IF(OR(E33="Abschreibung (AfA)",E33="Vorsteuer auf Anlagevermögen"),0,ROUND(F33*G33,2)))</f>
+        <f aca="false">IF(F33="","",ROUND(F33*G33,2))</f>
         <v/>
       </c>
       <c r="I33" s="22" t="str">
@@ -6682,7 +6611,7 @@
       <c r="F34" s="13"/>
       <c r="G34" s="21"/>
       <c r="H34" s="22" t="str">
-        <f>IF(F34="","",IF(OR(E34="Abschreibung (AfA)",E34="Vorsteuer auf Anlagevermögen"),0,ROUND(F34*G34,2)))</f>
+        <f aca="false">IF(F34="","",ROUND(F34*G34,2))</f>
         <v/>
       </c>
       <c r="I34" s="22" t="str">
@@ -6707,7 +6636,7 @@
       <c r="F35" s="13"/>
       <c r="G35" s="21"/>
       <c r="H35" s="22" t="str">
-        <f>IF(F35="","",IF(OR(E35="Abschreibung (AfA)",E35="Vorsteuer auf Anlagevermögen"),0,ROUND(F35*G35,2)))</f>
+        <f aca="false">IF(F35="","",ROUND(F35*G35,2))</f>
         <v/>
       </c>
       <c r="I35" s="22" t="str">
@@ -6727,7 +6656,7 @@
       <c r="F36" s="13"/>
       <c r="G36" s="21"/>
       <c r="H36" s="22" t="str">
-        <f>IF(F36="","",IF(OR(E36="Abschreibung (AfA)",E36="Vorsteuer auf Anlagevermögen"),0,ROUND(F36*G36,2)))</f>
+        <f aca="false">IF(F36="","",ROUND(F36*G36,2))</f>
         <v/>
       </c>
       <c r="I36" s="22" t="str">
@@ -6752,7 +6681,7 @@
       <c r="F37" s="13"/>
       <c r="G37" s="21"/>
       <c r="H37" s="22" t="str">
-        <f>IF(F37="","",IF(OR(E37="Abschreibung (AfA)",E37="Vorsteuer auf Anlagevermögen"),0,ROUND(F37*G37,2)))</f>
+        <f aca="false">IF(F37="","",ROUND(F37*G37,2))</f>
         <v/>
       </c>
       <c r="I37" s="22" t="str">
@@ -6772,7 +6701,7 @@
       <c r="F38" s="13"/>
       <c r="G38" s="21"/>
       <c r="H38" s="22" t="str">
-        <f>IF(F38="","",IF(OR(E38="Abschreibung (AfA)",E38="Vorsteuer auf Anlagevermögen"),0,ROUND(F38*G38,2)))</f>
+        <f aca="false">IF(F38="","",ROUND(F38*G38,2))</f>
         <v/>
       </c>
       <c r="I38" s="22" t="str">
@@ -6797,7 +6726,7 @@
       <c r="F39" s="13"/>
       <c r="G39" s="21"/>
       <c r="H39" s="22" t="str">
-        <f>IF(F39="","",IF(OR(E39="Abschreibung (AfA)",E39="Vorsteuer auf Anlagevermögen"),0,ROUND(F39*G39,2)))</f>
+        <f aca="false">IF(F39="","",ROUND(F39*G39,2))</f>
         <v/>
       </c>
       <c r="I39" s="22" t="str">
@@ -6815,7 +6744,7 @@
       <c r="F40" s="13"/>
       <c r="G40" s="21"/>
       <c r="H40" s="22" t="str">
-        <f>IF(F40="","",IF(OR(E40="Abschreibung (AfA)",E40="Vorsteuer auf Anlagevermögen"),0,ROUND(F40*G40,2)))</f>
+        <f aca="false">IF(F40="","",ROUND(F40*G40,2))</f>
         <v/>
       </c>
       <c r="I40" s="22" t="str">
@@ -6833,7 +6762,7 @@
       <c r="F41" s="13"/>
       <c r="G41" s="21"/>
       <c r="H41" s="22" t="str">
-        <f>IF(F41="","",IF(OR(E41="Abschreibung (AfA)",E41="Vorsteuer auf Anlagevermögen"),0,ROUND(F41*G41,2)))</f>
+        <f aca="false">IF(F41="","",ROUND(F41*G41,2))</f>
         <v/>
       </c>
       <c r="I41" s="22" t="str">
@@ -6851,7 +6780,7 @@
       <c r="F42" s="13"/>
       <c r="G42" s="21"/>
       <c r="H42" s="22" t="str">
-        <f>IF(F42="","",IF(OR(E42="Abschreibung (AfA)",E42="Vorsteuer auf Anlagevermögen"),0,ROUND(F42*G42,2)))</f>
+        <f aca="false">IF(F42="","",ROUND(F42*G42,2))</f>
         <v/>
       </c>
       <c r="I42" s="22" t="str">
@@ -6869,7 +6798,7 @@
       <c r="F43" s="13"/>
       <c r="G43" s="21"/>
       <c r="H43" s="22" t="str">
-        <f>IF(F43="","",IF(OR(E43="Abschreibung (AfA)",E43="Vorsteuer auf Anlagevermögen"),0,ROUND(F43*G43,2)))</f>
+        <f aca="false">IF(F43="","",ROUND(F43*G43,2))</f>
         <v/>
       </c>
       <c r="I43" s="22" t="str">
@@ -6887,7 +6816,7 @@
       <c r="F44" s="13"/>
       <c r="G44" s="21"/>
       <c r="H44" s="22" t="str">
-        <f>IF(F44="","",IF(OR(E44="Abschreibung (AfA)",E44="Vorsteuer auf Anlagevermögen"),0,ROUND(F44*G44,2)))</f>
+        <f aca="false">IF(F44="","",ROUND(F44*G44,2))</f>
         <v/>
       </c>
       <c r="I44" s="22" t="str">
@@ -6905,7 +6834,7 @@
       <c r="F45" s="13"/>
       <c r="G45" s="21"/>
       <c r="H45" s="22" t="str">
-        <f>IF(F45="","",IF(OR(E45="Abschreibung (AfA)",E45="Vorsteuer auf Anlagevermögen"),0,ROUND(F45*G45,2)))</f>
+        <f aca="false">IF(F45="","",ROUND(F45*G45,2))</f>
         <v/>
       </c>
       <c r="I45" s="22" t="str">
@@ -6923,7 +6852,7 @@
       <c r="F46" s="13"/>
       <c r="G46" s="21"/>
       <c r="H46" s="22" t="str">
-        <f>IF(F46="","",IF(OR(E46="Abschreibung (AfA)",E46="Vorsteuer auf Anlagevermögen"),0,ROUND(F46*G46,2)))</f>
+        <f aca="false">IF(F46="","",ROUND(F46*G46,2))</f>
         <v/>
       </c>
       <c r="I46" s="22" t="str">
@@ -6941,7 +6870,7 @@
       <c r="F47" s="13"/>
       <c r="G47" s="21"/>
       <c r="H47" s="22" t="str">
-        <f>IF(F47="","",IF(OR(E47="Abschreibung (AfA)",E47="Vorsteuer auf Anlagevermögen"),0,ROUND(F47*G47,2)))</f>
+        <f aca="false">IF(F47="","",ROUND(F47*G47,2))</f>
         <v/>
       </c>
       <c r="I47" s="22" t="str">
@@ -6959,7 +6888,7 @@
       <c r="F48" s="13"/>
       <c r="G48" s="21"/>
       <c r="H48" s="22" t="str">
-        <f>IF(F48="","",IF(OR(E48="Abschreibung (AfA)",E48="Vorsteuer auf Anlagevermögen"),0,ROUND(F48*G48,2)))</f>
+        <f aca="false">IF(F48="","",ROUND(F48*G48,2))</f>
         <v/>
       </c>
       <c r="I48" s="22" t="str">
@@ -6977,7 +6906,7 @@
       <c r="F49" s="13"/>
       <c r="G49" s="21"/>
       <c r="H49" s="22" t="str">
-        <f>IF(F49="","",IF(OR(E49="Abschreibung (AfA)",E49="Vorsteuer auf Anlagevermögen"),0,ROUND(F49*G49,2)))</f>
+        <f aca="false">IF(F49="","",ROUND(F49*G49,2))</f>
         <v/>
       </c>
       <c r="I49" s="22" t="str">
@@ -6995,7 +6924,7 @@
       <c r="F50" s="13"/>
       <c r="G50" s="21"/>
       <c r="H50" s="22" t="str">
-        <f>IF(F50="","",IF(OR(E50="Abschreibung (AfA)",E50="Vorsteuer auf Anlagevermögen"),0,ROUND(F50*G50,2)))</f>
+        <f aca="false">IF(F50="","",ROUND(F50*G50,2))</f>
         <v/>
       </c>
       <c r="I50" s="22" t="str">
@@ -7013,7 +6942,7 @@
       <c r="F51" s="13"/>
       <c r="G51" s="21"/>
       <c r="H51" s="22" t="str">
-        <f>IF(F51="","",IF(OR(E51="Abschreibung (AfA)",E51="Vorsteuer auf Anlagevermögen"),0,ROUND(F51*G51,2)))</f>
+        <f aca="false">IF(F51="","",ROUND(F51*G51,2))</f>
         <v/>
       </c>
       <c r="I51" s="22" t="str">
@@ -7031,7 +6960,7 @@
       <c r="F52" s="13"/>
       <c r="G52" s="21"/>
       <c r="H52" s="22" t="str">
-        <f>IF(F52="","",IF(OR(E52="Abschreibung (AfA)",E52="Vorsteuer auf Anlagevermögen"),0,ROUND(F52*G52,2)))</f>
+        <f aca="false">IF(F52="","",ROUND(F52*G52,2))</f>
         <v/>
       </c>
       <c r="I52" s="22" t="str">
@@ -7049,7 +6978,7 @@
       <c r="F53" s="13"/>
       <c r="G53" s="21"/>
       <c r="H53" s="22" t="str">
-        <f>IF(F53="","",IF(OR(E53="Abschreibung (AfA)",E53="Vorsteuer auf Anlagevermögen"),0,ROUND(F53*G53,2)))</f>
+        <f aca="false">IF(F53="","",ROUND(F53*G53,2))</f>
         <v/>
       </c>
       <c r="I53" s="22" t="str">
@@ -7067,7 +6996,7 @@
       <c r="F54" s="13"/>
       <c r="G54" s="21"/>
       <c r="H54" s="22" t="str">
-        <f>IF(F54="","",IF(OR(E54="Abschreibung (AfA)",E54="Vorsteuer auf Anlagevermögen"),0,ROUND(F54*G54,2)))</f>
+        <f aca="false">IF(F54="","",ROUND(F54*G54,2))</f>
         <v/>
       </c>
       <c r="I54" s="22" t="str">
@@ -7085,7 +7014,7 @@
       <c r="F55" s="13"/>
       <c r="G55" s="21"/>
       <c r="H55" s="22" t="str">
-        <f>IF(F55="","",IF(OR(E55="Abschreibung (AfA)",E55="Vorsteuer auf Anlagevermögen"),0,ROUND(F55*G55,2)))</f>
+        <f aca="false">IF(F55="","",ROUND(F55*G55,2))</f>
         <v/>
       </c>
       <c r="I55" s="22" t="str">
@@ -7103,7 +7032,7 @@
       <c r="F56" s="13"/>
       <c r="G56" s="21"/>
       <c r="H56" s="22" t="str">
-        <f>IF(F56="","",IF(OR(E56="Abschreibung (AfA)",E56="Vorsteuer auf Anlagevermögen"),0,ROUND(F56*G56,2)))</f>
+        <f aca="false">IF(F56="","",ROUND(F56*G56,2))</f>
         <v/>
       </c>
       <c r="I56" s="22" t="str">
@@ -7121,7 +7050,7 @@
       <c r="F57" s="13"/>
       <c r="G57" s="21"/>
       <c r="H57" s="22" t="str">
-        <f>IF(F57="","",IF(OR(E57="Abschreibung (AfA)",E57="Vorsteuer auf Anlagevermögen"),0,ROUND(F57*G57,2)))</f>
+        <f aca="false">IF(F57="","",ROUND(F57*G57,2))</f>
         <v/>
       </c>
       <c r="I57" s="22" t="str">
@@ -7139,7 +7068,7 @@
       <c r="F58" s="13"/>
       <c r="G58" s="21"/>
       <c r="H58" s="22" t="str">
-        <f>IF(F58="","",IF(OR(E58="Abschreibung (AfA)",E58="Vorsteuer auf Anlagevermögen"),0,ROUND(F58*G58,2)))</f>
+        <f aca="false">IF(F58="","",ROUND(F58*G58,2))</f>
         <v/>
       </c>
       <c r="I58" s="22" t="str">
@@ -7157,7 +7086,7 @@
       <c r="F59" s="13"/>
       <c r="G59" s="21"/>
       <c r="H59" s="22" t="str">
-        <f>IF(F59="","",IF(OR(E59="Abschreibung (AfA)",E59="Vorsteuer auf Anlagevermögen"),0,ROUND(F59*G59,2)))</f>
+        <f aca="false">IF(F59="","",ROUND(F59*G59,2))</f>
         <v/>
       </c>
       <c r="I59" s="22" t="str">
@@ -7175,7 +7104,7 @@
       <c r="F60" s="13"/>
       <c r="G60" s="21"/>
       <c r="H60" s="22" t="str">
-        <f>IF(F60="","",IF(OR(E60="Abschreibung (AfA)",E60="Vorsteuer auf Anlagevermögen"),0,ROUND(F60*G60,2)))</f>
+        <f aca="false">IF(F60="","",ROUND(F60*G60,2))</f>
         <v/>
       </c>
       <c r="I60" s="22" t="str">
@@ -7193,7 +7122,7 @@
       <c r="F61" s="13"/>
       <c r="G61" s="21"/>
       <c r="H61" s="22" t="str">
-        <f>IF(F61="","",IF(OR(E61="Abschreibung (AfA)",E61="Vorsteuer auf Anlagevermögen"),0,ROUND(F61*G61,2)))</f>
+        <f aca="false">IF(F61="","",ROUND(F61*G61,2))</f>
         <v/>
       </c>
       <c r="I61" s="22" t="str">
@@ -7211,7 +7140,7 @@
       <c r="F62" s="13"/>
       <c r="G62" s="21"/>
       <c r="H62" s="22" t="str">
-        <f>IF(F62="","",IF(OR(E62="Abschreibung (AfA)",E62="Vorsteuer auf Anlagevermögen"),0,ROUND(F62*G62,2)))</f>
+        <f aca="false">IF(F62="","",ROUND(F62*G62,2))</f>
         <v/>
       </c>
       <c r="I62" s="22" t="str">
@@ -7229,7 +7158,7 @@
       <c r="F63" s="13"/>
       <c r="G63" s="21"/>
       <c r="H63" s="22" t="str">
-        <f>IF(F63="","",IF(OR(E63="Abschreibung (AfA)",E63="Vorsteuer auf Anlagevermögen"),0,ROUND(F63*G63,2)))</f>
+        <f aca="false">IF(F63="","",ROUND(F63*G63,2))</f>
         <v/>
       </c>
       <c r="I63" s="22" t="str">
@@ -7247,7 +7176,7 @@
       <c r="F64" s="13"/>
       <c r="G64" s="21"/>
       <c r="H64" s="22" t="str">
-        <f>IF(F64="","",IF(OR(E64="Abschreibung (AfA)",E64="Vorsteuer auf Anlagevermögen"),0,ROUND(F64*G64,2)))</f>
+        <f aca="false">IF(F64="","",ROUND(F64*G64,2))</f>
         <v/>
       </c>
       <c r="I64" s="22" t="str">
@@ -7265,7 +7194,7 @@
       <c r="F65" s="13"/>
       <c r="G65" s="21"/>
       <c r="H65" s="22" t="str">
-        <f>IF(F65="","",IF(OR(E65="Abschreibung (AfA)",E65="Vorsteuer auf Anlagevermögen"),0,ROUND(F65*G65,2)))</f>
+        <f aca="false">IF(F65="","",ROUND(F65*G65,2))</f>
         <v/>
       </c>
       <c r="I65" s="22" t="str">
@@ -7283,7 +7212,7 @@
       <c r="F66" s="13"/>
       <c r="G66" s="21"/>
       <c r="H66" s="22" t="str">
-        <f>IF(F66="","",IF(OR(E66="Abschreibung (AfA)",E66="Vorsteuer auf Anlagevermögen"),0,ROUND(F66*G66,2)))</f>
+        <f aca="false">IF(F66="","",ROUND(F66*G66,2))</f>
         <v/>
       </c>
       <c r="I66" s="22" t="str">
@@ -7301,7 +7230,7 @@
       <c r="F67" s="13"/>
       <c r="G67" s="21"/>
       <c r="H67" s="22" t="str">
-        <f>IF(F67="","",IF(OR(E67="Abschreibung (AfA)",E67="Vorsteuer auf Anlagevermögen"),0,ROUND(F67*G67,2)))</f>
+        <f aca="false">IF(F67="","",ROUND(F67*G67,2))</f>
         <v/>
       </c>
       <c r="I67" s="22" t="str">
@@ -7319,7 +7248,7 @@
       <c r="F68" s="13"/>
       <c r="G68" s="21"/>
       <c r="H68" s="22" t="str">
-        <f>IF(F68="","",IF(OR(E68="Abschreibung (AfA)",E68="Vorsteuer auf Anlagevermögen"),0,ROUND(F68*G68,2)))</f>
+        <f aca="false">IF(F68="","",ROUND(F68*G68,2))</f>
         <v/>
       </c>
       <c r="I68" s="22" t="str">
@@ -7337,7 +7266,7 @@
       <c r="F69" s="13"/>
       <c r="G69" s="21"/>
       <c r="H69" s="22" t="str">
-        <f>IF(F69="","",IF(OR(E69="Abschreibung (AfA)",E69="Vorsteuer auf Anlagevermögen"),0,ROUND(F69*G69,2)))</f>
+        <f aca="false">IF(F69="","",ROUND(F69*G69,2))</f>
         <v/>
       </c>
       <c r="I69" s="22" t="str">
@@ -7355,7 +7284,7 @@
       <c r="F70" s="13"/>
       <c r="G70" s="21"/>
       <c r="H70" s="22" t="str">
-        <f>IF(F70="","",IF(OR(E70="Abschreibung (AfA)",E70="Vorsteuer auf Anlagevermögen"),0,ROUND(F70*G70,2)))</f>
+        <f aca="false">IF(F70="","",ROUND(F70*G70,2))</f>
         <v/>
       </c>
       <c r="I70" s="22" t="str">
@@ -7373,7 +7302,7 @@
       <c r="F71" s="13"/>
       <c r="G71" s="21"/>
       <c r="H71" s="22" t="str">
-        <f>IF(F71="","",IF(OR(E71="Abschreibung (AfA)",E71="Vorsteuer auf Anlagevermögen"),0,ROUND(F71*G71,2)))</f>
+        <f aca="false">IF(F71="","",ROUND(F71*G71,2))</f>
         <v/>
       </c>
       <c r="I71" s="22" t="str">
@@ -7391,7 +7320,7 @@
       <c r="F72" s="13"/>
       <c r="G72" s="21"/>
       <c r="H72" s="22" t="str">
-        <f>IF(F72="","",IF(OR(E72="Abschreibung (AfA)",E72="Vorsteuer auf Anlagevermögen"),0,ROUND(F72*G72,2)))</f>
+        <f aca="false">IF(F72="","",ROUND(F72*G72,2))</f>
         <v/>
       </c>
       <c r="I72" s="22" t="str">
@@ -7409,7 +7338,7 @@
       <c r="F73" s="13"/>
       <c r="G73" s="21"/>
       <c r="H73" s="22" t="str">
-        <f>IF(F73="","",IF(OR(E73="Abschreibung (AfA)",E73="Vorsteuer auf Anlagevermögen"),0,ROUND(F73*G73,2)))</f>
+        <f aca="false">IF(F73="","",ROUND(F73*G73,2))</f>
         <v/>
       </c>
       <c r="I73" s="22" t="str">
@@ -7427,7 +7356,7 @@
       <c r="F74" s="13"/>
       <c r="G74" s="21"/>
       <c r="H74" s="22" t="str">
-        <f>IF(F74="","",IF(OR(E74="Abschreibung (AfA)",E74="Vorsteuer auf Anlagevermögen"),0,ROUND(F74*G74,2)))</f>
+        <f aca="false">IF(F74="","",ROUND(F74*G74,2))</f>
         <v/>
       </c>
       <c r="I74" s="22" t="str">
@@ -7445,7 +7374,7 @@
       <c r="F75" s="13"/>
       <c r="G75" s="21"/>
       <c r="H75" s="22" t="str">
-        <f>IF(F75="","",IF(OR(E75="Abschreibung (AfA)",E75="Vorsteuer auf Anlagevermögen"),0,ROUND(F75*G75,2)))</f>
+        <f aca="false">IF(F75="","",ROUND(F75*G75,2))</f>
         <v/>
       </c>
       <c r="I75" s="22" t="str">
@@ -7463,7 +7392,7 @@
       <c r="F76" s="13"/>
       <c r="G76" s="21"/>
       <c r="H76" s="22" t="str">
-        <f>IF(F76="","",IF(OR(E76="Abschreibung (AfA)",E76="Vorsteuer auf Anlagevermögen"),0,ROUND(F76*G76,2)))</f>
+        <f aca="false">IF(F76="","",ROUND(F76*G76,2))</f>
         <v/>
       </c>
       <c r="I76" s="22" t="str">
@@ -7481,7 +7410,7 @@
       <c r="F77" s="13"/>
       <c r="G77" s="21"/>
       <c r="H77" s="22" t="str">
-        <f>IF(F77="","",IF(OR(E77="Abschreibung (AfA)",E77="Vorsteuer auf Anlagevermögen"),0,ROUND(F77*G77,2)))</f>
+        <f aca="false">IF(F77="","",ROUND(F77*G77,2))</f>
         <v/>
       </c>
       <c r="I77" s="22" t="str">
@@ -7499,7 +7428,7 @@
       <c r="F78" s="13"/>
       <c r="G78" s="21"/>
       <c r="H78" s="22" t="str">
-        <f>IF(F78="","",IF(OR(E78="Abschreibung (AfA)",E78="Vorsteuer auf Anlagevermögen"),0,ROUND(F78*G78,2)))</f>
+        <f aca="false">IF(F78="","",ROUND(F78*G78,2))</f>
         <v/>
       </c>
       <c r="I78" s="22" t="str">
@@ -7517,7 +7446,7 @@
       <c r="F79" s="13"/>
       <c r="G79" s="21"/>
       <c r="H79" s="22" t="str">
-        <f>IF(F79="","",IF(OR(E79="Abschreibung (AfA)",E79="Vorsteuer auf Anlagevermögen"),0,ROUND(F79*G79,2)))</f>
+        <f aca="false">IF(F79="","",ROUND(F79*G79,2))</f>
         <v/>
       </c>
       <c r="I79" s="22" t="str">
@@ -7535,7 +7464,7 @@
       <c r="F80" s="13"/>
       <c r="G80" s="21"/>
       <c r="H80" s="22" t="str">
-        <f>IF(F80="","",IF(OR(E80="Abschreibung (AfA)",E80="Vorsteuer auf Anlagevermögen"),0,ROUND(F80*G80,2)))</f>
+        <f aca="false">IF(F80="","",ROUND(F80*G80,2))</f>
         <v/>
       </c>
       <c r="I80" s="22" t="str">
@@ -7553,7 +7482,7 @@
       <c r="F81" s="13"/>
       <c r="G81" s="21"/>
       <c r="H81" s="22" t="str">
-        <f>IF(F81="","",IF(OR(E81="Abschreibung (AfA)",E81="Vorsteuer auf Anlagevermögen"),0,ROUND(F81*G81,2)))</f>
+        <f aca="false">IF(F81="","",ROUND(F81*G81,2))</f>
         <v/>
       </c>
       <c r="I81" s="22" t="str">
@@ -7571,7 +7500,7 @@
       <c r="F82" s="13"/>
       <c r="G82" s="21"/>
       <c r="H82" s="22" t="str">
-        <f>IF(F82="","",IF(OR(E82="Abschreibung (AfA)",E82="Vorsteuer auf Anlagevermögen"),0,ROUND(F82*G82,2)))</f>
+        <f aca="false">IF(F82="","",ROUND(F82*G82,2))</f>
         <v/>
       </c>
       <c r="I82" s="22" t="str">
@@ -7589,7 +7518,7 @@
       <c r="F83" s="13"/>
       <c r="G83" s="21"/>
       <c r="H83" s="22" t="str">
-        <f>IF(F83="","",IF(OR(E83="Abschreibung (AfA)",E83="Vorsteuer auf Anlagevermögen"),0,ROUND(F83*G83,2)))</f>
+        <f aca="false">IF(F83="","",ROUND(F83*G83,2))</f>
         <v/>
       </c>
       <c r="I83" s="22" t="str">
@@ -7607,7 +7536,7 @@
       <c r="F84" s="13"/>
       <c r="G84" s="21"/>
       <c r="H84" s="22" t="str">
-        <f>IF(F84="","",IF(OR(E84="Abschreibung (AfA)",E84="Vorsteuer auf Anlagevermögen"),0,ROUND(F84*G84,2)))</f>
+        <f aca="false">IF(F84="","",ROUND(F84*G84,2))</f>
         <v/>
       </c>
       <c r="I84" s="22" t="str">
@@ -7625,7 +7554,7 @@
       <c r="F85" s="13"/>
       <c r="G85" s="21"/>
       <c r="H85" s="22" t="str">
-        <f>IF(F85="","",IF(OR(E85="Abschreibung (AfA)",E85="Vorsteuer auf Anlagevermögen"),0,ROUND(F85*G85,2)))</f>
+        <f aca="false">IF(F85="","",ROUND(F85*G85,2))</f>
         <v/>
       </c>
       <c r="I85" s="22" t="str">
@@ -7643,7 +7572,7 @@
       <c r="F86" s="13"/>
       <c r="G86" s="21"/>
       <c r="H86" s="22" t="str">
-        <f>IF(F86="","",IF(OR(E86="Abschreibung (AfA)",E86="Vorsteuer auf Anlagevermögen"),0,ROUND(F86*G86,2)))</f>
+        <f aca="false">IF(F86="","",ROUND(F86*G86,2))</f>
         <v/>
       </c>
       <c r="I86" s="22" t="str">
@@ -7661,7 +7590,7 @@
       <c r="F87" s="13"/>
       <c r="G87" s="21"/>
       <c r="H87" s="22" t="str">
-        <f>IF(F87="","",IF(OR(E87="Abschreibung (AfA)",E87="Vorsteuer auf Anlagevermögen"),0,ROUND(F87*G87,2)))</f>
+        <f aca="false">IF(F87="","",ROUND(F87*G87,2))</f>
         <v/>
       </c>
       <c r="I87" s="22" t="str">
@@ -7679,7 +7608,7 @@
       <c r="F88" s="13"/>
       <c r="G88" s="21"/>
       <c r="H88" s="22" t="str">
-        <f>IF(F88="","",IF(OR(E88="Abschreibung (AfA)",E88="Vorsteuer auf Anlagevermögen"),0,ROUND(F88*G88,2)))</f>
+        <f aca="false">IF(F88="","",ROUND(F88*G88,2))</f>
         <v/>
       </c>
       <c r="I88" s="22" t="str">
@@ -7697,7 +7626,7 @@
       <c r="F89" s="13"/>
       <c r="G89" s="21"/>
       <c r="H89" s="22" t="str">
-        <f>IF(F89="","",IF(OR(E89="Abschreibung (AfA)",E89="Vorsteuer auf Anlagevermögen"),0,ROUND(F89*G89,2)))</f>
+        <f aca="false">IF(F89="","",ROUND(F89*G89,2))</f>
         <v/>
       </c>
       <c r="I89" s="22" t="str">
@@ -7715,7 +7644,7 @@
       <c r="F90" s="13"/>
       <c r="G90" s="21"/>
       <c r="H90" s="22" t="str">
-        <f>IF(F90="","",IF(OR(E90="Abschreibung (AfA)",E90="Vorsteuer auf Anlagevermögen"),0,ROUND(F90*G90,2)))</f>
+        <f aca="false">IF(F90="","",ROUND(F90*G90,2))</f>
         <v/>
       </c>
       <c r="I90" s="22" t="str">
@@ -7733,7 +7662,7 @@
       <c r="F91" s="13"/>
       <c r="G91" s="21"/>
       <c r="H91" s="22" t="str">
-        <f>IF(F91="","",IF(OR(E91="Abschreibung (AfA)",E91="Vorsteuer auf Anlagevermögen"),0,ROUND(F91*G91,2)))</f>
+        <f aca="false">IF(F91="","",ROUND(F91*G91,2))</f>
         <v/>
       </c>
       <c r="I91" s="22" t="str">
@@ -7751,7 +7680,7 @@
       <c r="F92" s="13"/>
       <c r="G92" s="21"/>
       <c r="H92" s="22" t="str">
-        <f>IF(F92="","",IF(OR(E92="Abschreibung (AfA)",E92="Vorsteuer auf Anlagevermögen"),0,ROUND(F92*G92,2)))</f>
+        <f aca="false">IF(F92="","",ROUND(F92*G92,2))</f>
         <v/>
       </c>
       <c r="I92" s="22" t="str">
@@ -7769,7 +7698,7 @@
       <c r="F93" s="13"/>
       <c r="G93" s="21"/>
       <c r="H93" s="22" t="str">
-        <f>IF(F93="","",IF(OR(E93="Abschreibung (AfA)",E93="Vorsteuer auf Anlagevermögen"),0,ROUND(F93*G93,2)))</f>
+        <f aca="false">IF(F93="","",ROUND(F93*G93,2))</f>
         <v/>
       </c>
       <c r="I93" s="22" t="str">
@@ -7787,7 +7716,7 @@
       <c r="F94" s="13"/>
       <c r="G94" s="21"/>
       <c r="H94" s="22" t="str">
-        <f>IF(F94="","",IF(OR(E94="Abschreibung (AfA)",E94="Vorsteuer auf Anlagevermögen"),0,ROUND(F94*G94,2)))</f>
+        <f aca="false">IF(F94="","",ROUND(F94*G94,2))</f>
         <v/>
       </c>
       <c r="I94" s="22" t="str">
@@ -7805,7 +7734,7 @@
       <c r="F95" s="13"/>
       <c r="G95" s="21"/>
       <c r="H95" s="22" t="str">
-        <f>IF(F95="","",IF(OR(E95="Abschreibung (AfA)",E95="Vorsteuer auf Anlagevermögen"),0,ROUND(F95*G95,2)))</f>
+        <f aca="false">IF(F95="","",ROUND(F95*G95,2))</f>
         <v/>
       </c>
       <c r="I95" s="22" t="str">
@@ -7823,7 +7752,7 @@
       <c r="F96" s="13"/>
       <c r="G96" s="21"/>
       <c r="H96" s="22" t="str">
-        <f>IF(F96="","",IF(OR(E96="Abschreibung (AfA)",E96="Vorsteuer auf Anlagevermögen"),0,ROUND(F96*G96,2)))</f>
+        <f aca="false">IF(F96="","",ROUND(F96*G96,2))</f>
         <v/>
       </c>
       <c r="I96" s="22" t="str">
@@ -7841,7 +7770,7 @@
       <c r="F97" s="13"/>
       <c r="G97" s="21"/>
       <c r="H97" s="22" t="str">
-        <f>IF(F97="","",IF(OR(E97="Abschreibung (AfA)",E97="Vorsteuer auf Anlagevermögen"),0,ROUND(F97*G97,2)))</f>
+        <f aca="false">IF(F97="","",ROUND(F97*G97,2))</f>
         <v/>
       </c>
       <c r="I97" s="22" t="str">
@@ -7859,7 +7788,7 @@
       <c r="F98" s="13"/>
       <c r="G98" s="21"/>
       <c r="H98" s="22" t="str">
-        <f>IF(F98="","",IF(OR(E98="Abschreibung (AfA)",E98="Vorsteuer auf Anlagevermögen"),0,ROUND(F98*G98,2)))</f>
+        <f aca="false">IF(F98="","",ROUND(F98*G98,2))</f>
         <v/>
       </c>
       <c r="I98" s="22" t="str">
@@ -7877,7 +7806,7 @@
       <c r="F99" s="13"/>
       <c r="G99" s="21"/>
       <c r="H99" s="22" t="str">
-        <f>IF(F99="","",IF(OR(E99="Abschreibung (AfA)",E99="Vorsteuer auf Anlagevermögen"),0,ROUND(F99*G99,2)))</f>
+        <f aca="false">IF(F99="","",ROUND(F99*G99,2))</f>
         <v/>
       </c>
       <c r="I99" s="22" t="str">
@@ -7895,7 +7824,7 @@
       <c r="F100" s="13"/>
       <c r="G100" s="21"/>
       <c r="H100" s="22" t="str">
-        <f>IF(F100="","",IF(OR(E100="Abschreibung (AfA)",E100="Vorsteuer auf Anlagevermögen"),0,ROUND(F100*G100,2)))</f>
+        <f aca="false">IF(F100="","",ROUND(F100*G100,2))</f>
         <v/>
       </c>
       <c r="I100" s="22" t="str">
@@ -7913,7 +7842,7 @@
       <c r="F101" s="13"/>
       <c r="G101" s="21"/>
       <c r="H101" s="22" t="str">
-        <f>IF(F101="","",IF(OR(E101="Abschreibung (AfA)",E101="Vorsteuer auf Anlagevermögen"),0,ROUND(F101*G101,2)))</f>
+        <f aca="false">IF(F101="","",ROUND(F101*G101,2))</f>
         <v/>
       </c>
       <c r="I101" s="22" t="str">
@@ -7931,7 +7860,7 @@
       <c r="F102" s="13"/>
       <c r="G102" s="21"/>
       <c r="H102" s="22" t="str">
-        <f>IF(F102="","",IF(OR(E102="Abschreibung (AfA)",E102="Vorsteuer auf Anlagevermögen"),0,ROUND(F102*G102,2)))</f>
+        <f aca="false">IF(F102="","",ROUND(F102*G102,2))</f>
         <v/>
       </c>
       <c r="I102" s="22" t="str">
@@ -7949,7 +7878,7 @@
       <c r="F103" s="13"/>
       <c r="G103" s="21"/>
       <c r="H103" s="22" t="str">
-        <f>IF(F103="","",IF(OR(E103="Abschreibung (AfA)",E103="Vorsteuer auf Anlagevermögen"),0,ROUND(F103*G103,2)))</f>
+        <f aca="false">IF(F103="","",ROUND(F103*G103,2))</f>
         <v/>
       </c>
       <c r="I103" s="22" t="str">
@@ -7967,7 +7896,7 @@
       <c r="F104" s="13"/>
       <c r="G104" s="21"/>
       <c r="H104" s="22" t="str">
-        <f>IF(F104="","",IF(OR(E104="Abschreibung (AfA)",E104="Vorsteuer auf Anlagevermögen"),0,ROUND(F104*G104,2)))</f>
+        <f aca="false">IF(F104="","",ROUND(F104*G104,2))</f>
         <v/>
       </c>
       <c r="I104" s="22" t="str">
@@ -7985,7 +7914,7 @@
       <c r="F105" s="13"/>
       <c r="G105" s="21"/>
       <c r="H105" s="22" t="str">
-        <f>IF(F105="","",IF(OR(E105="Abschreibung (AfA)",E105="Vorsteuer auf Anlagevermögen"),0,ROUND(F105*G105,2)))</f>
+        <f aca="false">IF(F105="","",ROUND(F105*G105,2))</f>
         <v/>
       </c>
       <c r="I105" s="22" t="str">
@@ -8003,7 +7932,7 @@
       <c r="F106" s="13"/>
       <c r="G106" s="21"/>
       <c r="H106" s="22" t="str">
-        <f>IF(F106="","",IF(OR(E106="Abschreibung (AfA)",E106="Vorsteuer auf Anlagevermögen"),0,ROUND(F106*G106,2)))</f>
+        <f aca="false">IF(F106="","",ROUND(F106*G106,2))</f>
         <v/>
       </c>
       <c r="I106" s="22" t="str">
@@ -8021,7 +7950,7 @@
       <c r="F107" s="13"/>
       <c r="G107" s="21"/>
       <c r="H107" s="22" t="str">
-        <f>IF(F107="","",IF(OR(E107="Abschreibung (AfA)",E107="Vorsteuer auf Anlagevermögen"),0,ROUND(F107*G107,2)))</f>
+        <f aca="false">IF(F107="","",ROUND(F107*G107,2))</f>
         <v/>
       </c>
       <c r="I107" s="22" t="str">
@@ -8039,7 +7968,7 @@
       <c r="F108" s="13"/>
       <c r="G108" s="21"/>
       <c r="H108" s="22" t="str">
-        <f>IF(F108="","",IF(OR(E108="Abschreibung (AfA)",E108="Vorsteuer auf Anlagevermögen"),0,ROUND(F108*G108,2)))</f>
+        <f aca="false">IF(F108="","",ROUND(F108*G108,2))</f>
         <v/>
       </c>
       <c r="I108" s="22" t="str">
@@ -8057,7 +7986,7 @@
       <c r="F109" s="13"/>
       <c r="G109" s="21"/>
       <c r="H109" s="22" t="str">
-        <f>IF(F109="","",IF(OR(E109="Abschreibung (AfA)",E109="Vorsteuer auf Anlagevermögen"),0,ROUND(F109*G109,2)))</f>
+        <f aca="false">IF(F109="","",ROUND(F109*G109,2))</f>
         <v/>
       </c>
       <c r="I109" s="22" t="str">
@@ -8075,7 +8004,7 @@
       <c r="F110" s="13"/>
       <c r="G110" s="21"/>
       <c r="H110" s="22" t="str">
-        <f>IF(F110="","",IF(OR(E110="Abschreibung (AfA)",E110="Vorsteuer auf Anlagevermögen"),0,ROUND(F110*G110,2)))</f>
+        <f aca="false">IF(F110="","",ROUND(F110*G110,2))</f>
         <v/>
       </c>
       <c r="I110" s="22" t="str">
@@ -8093,7 +8022,7 @@
       <c r="F111" s="13"/>
       <c r="G111" s="21"/>
       <c r="H111" s="22" t="str">
-        <f>IF(F111="","",IF(OR(E111="Abschreibung (AfA)",E111="Vorsteuer auf Anlagevermögen"),0,ROUND(F111*G111,2)))</f>
+        <f aca="false">IF(F111="","",ROUND(F111*G111,2))</f>
         <v/>
       </c>
       <c r="I111" s="22" t="str">
@@ -8111,7 +8040,7 @@
       <c r="F112" s="13"/>
       <c r="G112" s="21"/>
       <c r="H112" s="22" t="str">
-        <f>IF(F112="","",IF(OR(E112="Abschreibung (AfA)",E112="Vorsteuer auf Anlagevermögen"),0,ROUND(F112*G112,2)))</f>
+        <f aca="false">IF(F112="","",ROUND(F112*G112,2))</f>
         <v/>
       </c>
       <c r="I112" s="22" t="str">
@@ -8129,7 +8058,7 @@
       <c r="F113" s="13"/>
       <c r="G113" s="21"/>
       <c r="H113" s="22" t="str">
-        <f>IF(F113="","",IF(OR(E113="Abschreibung (AfA)",E113="Vorsteuer auf Anlagevermögen"),0,ROUND(F113*G113,2)))</f>
+        <f aca="false">IF(F113="","",ROUND(F113*G113,2))</f>
         <v/>
       </c>
       <c r="I113" s="22" t="str">
@@ -8147,7 +8076,7 @@
       <c r="F114" s="13"/>
       <c r="G114" s="21"/>
       <c r="H114" s="22" t="str">
-        <f>IF(F114="","",IF(OR(E114="Abschreibung (AfA)",E114="Vorsteuer auf Anlagevermögen"),0,ROUND(F114*G114,2)))</f>
+        <f aca="false">IF(F114="","",ROUND(F114*G114,2))</f>
         <v/>
       </c>
       <c r="I114" s="22" t="str">
@@ -8165,7 +8094,7 @@
       <c r="F115" s="13"/>
       <c r="G115" s="21"/>
       <c r="H115" s="22" t="str">
-        <f>IF(F115="","",IF(OR(E115="Abschreibung (AfA)",E115="Vorsteuer auf Anlagevermögen"),0,ROUND(F115*G115,2)))</f>
+        <f aca="false">IF(F115="","",ROUND(F115*G115,2))</f>
         <v/>
       </c>
       <c r="I115" s="22" t="str">
@@ -8183,7 +8112,7 @@
       <c r="F116" s="13"/>
       <c r="G116" s="21"/>
       <c r="H116" s="22" t="str">
-        <f>IF(F116="","",IF(OR(E116="Abschreibung (AfA)",E116="Vorsteuer auf Anlagevermögen"),0,ROUND(F116*G116,2)))</f>
+        <f aca="false">IF(F116="","",ROUND(F116*G116,2))</f>
         <v/>
       </c>
       <c r="I116" s="22" t="str">
@@ -8201,7 +8130,7 @@
       <c r="F117" s="13"/>
       <c r="G117" s="21"/>
       <c r="H117" s="22" t="str">
-        <f>IF(F117="","",IF(OR(E117="Abschreibung (AfA)",E117="Vorsteuer auf Anlagevermögen"),0,ROUND(F117*G117,2)))</f>
+        <f aca="false">IF(F117="","",ROUND(F117*G117,2))</f>
         <v/>
       </c>
       <c r="I117" s="22" t="str">
@@ -8219,7 +8148,7 @@
       <c r="F118" s="13"/>
       <c r="G118" s="21"/>
       <c r="H118" s="22" t="str">
-        <f>IF(F118="","",IF(OR(E118="Abschreibung (AfA)",E118="Vorsteuer auf Anlagevermögen"),0,ROUND(F118*G118,2)))</f>
+        <f aca="false">IF(F118="","",ROUND(F118*G118,2))</f>
         <v/>
       </c>
       <c r="I118" s="22" t="str">
@@ -8237,7 +8166,7 @@
       <c r="F119" s="13"/>
       <c r="G119" s="21"/>
       <c r="H119" s="22" t="str">
-        <f>IF(F119="","",IF(OR(E119="Abschreibung (AfA)",E119="Vorsteuer auf Anlagevermögen"),0,ROUND(F119*G119,2)))</f>
+        <f aca="false">IF(F119="","",ROUND(F119*G119,2))</f>
         <v/>
       </c>
       <c r="I119" s="22" t="str">
@@ -8255,7 +8184,7 @@
       <c r="F120" s="13"/>
       <c r="G120" s="21"/>
       <c r="H120" s="22" t="str">
-        <f>IF(F120="","",IF(OR(E120="Abschreibung (AfA)",E120="Vorsteuer auf Anlagevermögen"),0,ROUND(F120*G120,2)))</f>
+        <f aca="false">IF(F120="","",ROUND(F120*G120,2))</f>
         <v/>
       </c>
       <c r="I120" s="22" t="str">
@@ -8273,7 +8202,7 @@
       <c r="F121" s="13"/>
       <c r="G121" s="21"/>
       <c r="H121" s="22" t="str">
-        <f>IF(F121="","",IF(OR(E121="Abschreibung (AfA)",E121="Vorsteuer auf Anlagevermögen"),0,ROUND(F121*G121,2)))</f>
+        <f aca="false">IF(F121="","",ROUND(F121*G121,2))</f>
         <v/>
       </c>
       <c r="I121" s="22" t="str">
@@ -8291,7 +8220,7 @@
       <c r="F122" s="13"/>
       <c r="G122" s="21"/>
       <c r="H122" s="22" t="str">
-        <f>IF(F122="","",IF(OR(E122="Abschreibung (AfA)",E122="Vorsteuer auf Anlagevermögen"),0,ROUND(F122*G122,2)))</f>
+        <f aca="false">IF(F122="","",ROUND(F122*G122,2))</f>
         <v/>
       </c>
       <c r="I122" s="22" t="str">
@@ -8309,7 +8238,7 @@
       <c r="F123" s="13"/>
       <c r="G123" s="21"/>
       <c r="H123" s="22" t="str">
-        <f>IF(F123="","",IF(OR(E123="Abschreibung (AfA)",E123="Vorsteuer auf Anlagevermögen"),0,ROUND(F123*G123,2)))</f>
+        <f aca="false">IF(F123="","",ROUND(F123*G123,2))</f>
         <v/>
       </c>
       <c r="I123" s="22" t="str">
@@ -8327,7 +8256,7 @@
       <c r="F124" s="13"/>
       <c r="G124" s="21"/>
       <c r="H124" s="22" t="str">
-        <f>IF(F124="","",IF(OR(E124="Abschreibung (AfA)",E124="Vorsteuer auf Anlagevermögen"),0,ROUND(F124*G124,2)))</f>
+        <f aca="false">IF(F124="","",ROUND(F124*G124,2))</f>
         <v/>
       </c>
       <c r="I124" s="22" t="str">
@@ -8345,7 +8274,7 @@
       <c r="F125" s="13"/>
       <c r="G125" s="21"/>
       <c r="H125" s="22" t="str">
-        <f>IF(F125="","",IF(OR(E125="Abschreibung (AfA)",E125="Vorsteuer auf Anlagevermögen"),0,ROUND(F125*G125,2)))</f>
+        <f aca="false">IF(F125="","",ROUND(F125*G125,2))</f>
         <v/>
       </c>
       <c r="I125" s="22" t="str">
@@ -8363,7 +8292,7 @@
       <c r="F126" s="13"/>
       <c r="G126" s="21"/>
       <c r="H126" s="22" t="str">
-        <f>IF(F126="","",IF(OR(E126="Abschreibung (AfA)",E126="Vorsteuer auf Anlagevermögen"),0,ROUND(F126*G126,2)))</f>
+        <f aca="false">IF(F126="","",ROUND(F126*G126,2))</f>
         <v/>
       </c>
       <c r="I126" s="22" t="str">
@@ -8381,7 +8310,7 @@
       <c r="F127" s="13"/>
       <c r="G127" s="21"/>
       <c r="H127" s="22" t="str">
-        <f>IF(F127="","",IF(OR(E127="Abschreibung (AfA)",E127="Vorsteuer auf Anlagevermögen"),0,ROUND(F127*G127,2)))</f>
+        <f aca="false">IF(F127="","",ROUND(F127*G127,2))</f>
         <v/>
       </c>
       <c r="I127" s="22" t="str">
@@ -8399,7 +8328,7 @@
       <c r="F128" s="13"/>
       <c r="G128" s="21"/>
       <c r="H128" s="22" t="str">
-        <f>IF(F128="","",IF(OR(E128="Abschreibung (AfA)",E128="Vorsteuer auf Anlagevermögen"),0,ROUND(F128*G128,2)))</f>
+        <f aca="false">IF(F128="","",ROUND(F128*G128,2))</f>
         <v/>
       </c>
       <c r="I128" s="22" t="str">
@@ -8417,7 +8346,7 @@
       <c r="F129" s="13"/>
       <c r="G129" s="21"/>
       <c r="H129" s="22" t="str">
-        <f>IF(F129="","",IF(OR(E129="Abschreibung (AfA)",E129="Vorsteuer auf Anlagevermögen"),0,ROUND(F129*G129,2)))</f>
+        <f aca="false">IF(F129="","",ROUND(F129*G129,2))</f>
         <v/>
       </c>
       <c r="I129" s="22" t="str">
@@ -8435,7 +8364,7 @@
       <c r="F130" s="13"/>
       <c r="G130" s="21"/>
       <c r="H130" s="22" t="str">
-        <f>IF(F130="","",IF(OR(E130="Abschreibung (AfA)",E130="Vorsteuer auf Anlagevermögen"),0,ROUND(F130*G130,2)))</f>
+        <f aca="false">IF(F130="","",ROUND(F130*G130,2))</f>
         <v/>
       </c>
       <c r="I130" s="22" t="str">
@@ -8453,7 +8382,7 @@
       <c r="F131" s="13"/>
       <c r="G131" s="21"/>
       <c r="H131" s="22" t="str">
-        <f>IF(F131="","",IF(OR(E131="Abschreibung (AfA)",E131="Vorsteuer auf Anlagevermögen"),0,ROUND(F131*G131,2)))</f>
+        <f aca="false">IF(F131="","",ROUND(F131*G131,2))</f>
         <v/>
       </c>
       <c r="I131" s="22" t="str">
@@ -8471,7 +8400,7 @@
       <c r="F132" s="13"/>
       <c r="G132" s="21"/>
       <c r="H132" s="22" t="str">
-        <f>IF(F132="","",IF(OR(E132="Abschreibung (AfA)",E132="Vorsteuer auf Anlagevermögen"),0,ROUND(F132*G132,2)))</f>
+        <f aca="false">IF(F132="","",ROUND(F132*G132,2))</f>
         <v/>
       </c>
       <c r="I132" s="22" t="str">
@@ -8489,7 +8418,7 @@
       <c r="F133" s="13"/>
       <c r="G133" s="21"/>
       <c r="H133" s="22" t="str">
-        <f>IF(F133="","",IF(OR(E133="Abschreibung (AfA)",E133="Vorsteuer auf Anlagevermögen"),0,ROUND(F133*G133,2)))</f>
+        <f aca="false">IF(F133="","",ROUND(F133*G133,2))</f>
         <v/>
       </c>
       <c r="I133" s="22" t="str">
@@ -8507,7 +8436,7 @@
       <c r="F134" s="13"/>
       <c r="G134" s="21"/>
       <c r="H134" s="22" t="str">
-        <f>IF(F134="","",IF(OR(E134="Abschreibung (AfA)",E134="Vorsteuer auf Anlagevermögen"),0,ROUND(F134*G134,2)))</f>
+        <f aca="false">IF(F134="","",ROUND(F134*G134,2))</f>
         <v/>
       </c>
       <c r="I134" s="22" t="str">
@@ -8525,7 +8454,7 @@
       <c r="F135" s="13"/>
       <c r="G135" s="21"/>
       <c r="H135" s="22" t="str">
-        <f>IF(F135="","",IF(OR(E135="Abschreibung (AfA)",E135="Vorsteuer auf Anlagevermögen"),0,ROUND(F135*G135,2)))</f>
+        <f aca="false">IF(F135="","",ROUND(F135*G135,2))</f>
         <v/>
       </c>
       <c r="I135" s="22" t="str">
@@ -8543,7 +8472,7 @@
       <c r="F136" s="13"/>
       <c r="G136" s="21"/>
       <c r="H136" s="22" t="str">
-        <f>IF(F136="","",IF(OR(E136="Abschreibung (AfA)",E136="Vorsteuer auf Anlagevermögen"),0,ROUND(F136*G136,2)))</f>
+        <f aca="false">IF(F136="","",ROUND(F136*G136,2))</f>
         <v/>
       </c>
       <c r="I136" s="22" t="str">
@@ -8561,7 +8490,7 @@
       <c r="F137" s="13"/>
       <c r="G137" s="21"/>
       <c r="H137" s="22" t="str">
-        <f>IF(F137="","",IF(OR(E137="Abschreibung (AfA)",E137="Vorsteuer auf Anlagevermögen"),0,ROUND(F137*G137,2)))</f>
+        <f aca="false">IF(F137="","",ROUND(F137*G137,2))</f>
         <v/>
       </c>
       <c r="I137" s="22" t="str">
@@ -8579,7 +8508,7 @@
       <c r="F138" s="13"/>
       <c r="G138" s="21"/>
       <c r="H138" s="22" t="str">
-        <f>IF(F138="","",IF(OR(E138="Abschreibung (AfA)",E138="Vorsteuer auf Anlagevermögen"),0,ROUND(F138*G138,2)))</f>
+        <f aca="false">IF(F138="","",ROUND(F138*G138,2))</f>
         <v/>
       </c>
       <c r="I138" s="22" t="str">
@@ -8597,7 +8526,7 @@
       <c r="F139" s="13"/>
       <c r="G139" s="21"/>
       <c r="H139" s="22" t="str">
-        <f>IF(F139="","",IF(OR(E139="Abschreibung (AfA)",E139="Vorsteuer auf Anlagevermögen"),0,ROUND(F139*G139,2)))</f>
+        <f aca="false">IF(F139="","",ROUND(F139*G139,2))</f>
         <v/>
       </c>
       <c r="I139" s="22" t="str">
@@ -8615,7 +8544,7 @@
       <c r="F140" s="13"/>
       <c r="G140" s="21"/>
       <c r="H140" s="22" t="str">
-        <f>IF(F140="","",IF(OR(E140="Abschreibung (AfA)",E140="Vorsteuer auf Anlagevermögen"),0,ROUND(F140*G140,2)))</f>
+        <f aca="false">IF(F140="","",ROUND(F140*G140,2))</f>
         <v/>
       </c>
       <c r="I140" s="22" t="str">
@@ -8633,7 +8562,7 @@
       <c r="F141" s="13"/>
       <c r="G141" s="21"/>
       <c r="H141" s="22" t="str">
-        <f>IF(F141="","",IF(OR(E141="Abschreibung (AfA)",E141="Vorsteuer auf Anlagevermögen"),0,ROUND(F141*G141,2)))</f>
+        <f aca="false">IF(F141="","",ROUND(F141*G141,2))</f>
         <v/>
       </c>
       <c r="I141" s="22" t="str">
@@ -8651,7 +8580,7 @@
       <c r="F142" s="13"/>
       <c r="G142" s="21"/>
       <c r="H142" s="22" t="str">
-        <f>IF(F142="","",IF(OR(E142="Abschreibung (AfA)",E142="Vorsteuer auf Anlagevermögen"),0,ROUND(F142*G142,2)))</f>
+        <f aca="false">IF(F142="","",ROUND(F142*G142,2))</f>
         <v/>
       </c>
       <c r="I142" s="22" t="str">
@@ -8669,7 +8598,7 @@
       <c r="F143" s="13"/>
       <c r="G143" s="21"/>
       <c r="H143" s="22" t="str">
-        <f>IF(F143="","",IF(OR(E143="Abschreibung (AfA)",E143="Vorsteuer auf Anlagevermögen"),0,ROUND(F143*G143,2)))</f>
+        <f aca="false">IF(F143="","",ROUND(F143*G143,2))</f>
         <v/>
       </c>
       <c r="I143" s="22" t="str">
@@ -8687,7 +8616,7 @@
       <c r="F144" s="13"/>
       <c r="G144" s="21"/>
       <c r="H144" s="22" t="str">
-        <f>IF(F144="","",IF(OR(E144="Abschreibung (AfA)",E144="Vorsteuer auf Anlagevermögen"),0,ROUND(F144*G144,2)))</f>
+        <f aca="false">IF(F144="","",ROUND(F144*G144,2))</f>
         <v/>
       </c>
       <c r="I144" s="22" t="str">
@@ -8705,7 +8634,7 @@
       <c r="F145" s="13"/>
       <c r="G145" s="21"/>
       <c r="H145" s="22" t="str">
-        <f>IF(F145="","",IF(OR(E145="Abschreibung (AfA)",E145="Vorsteuer auf Anlagevermögen"),0,ROUND(F145*G145,2)))</f>
+        <f aca="false">IF(F145="","",ROUND(F145*G145,2))</f>
         <v/>
       </c>
       <c r="I145" s="22" t="str">
@@ -8723,7 +8652,7 @@
       <c r="F146" s="13"/>
       <c r="G146" s="21"/>
       <c r="H146" s="22" t="str">
-        <f>IF(F146="","",IF(OR(E146="Abschreibung (AfA)",E146="Vorsteuer auf Anlagevermögen"),0,ROUND(F146*G146,2)))</f>
+        <f aca="false">IF(F146="","",ROUND(F146*G146,2))</f>
         <v/>
       </c>
       <c r="I146" s="22" t="str">
@@ -8741,7 +8670,7 @@
       <c r="F147" s="13"/>
       <c r="G147" s="21"/>
       <c r="H147" s="22" t="str">
-        <f>IF(F147="","",IF(OR(E147="Abschreibung (AfA)",E147="Vorsteuer auf Anlagevermögen"),0,ROUND(F147*G147,2)))</f>
+        <f aca="false">IF(F147="","",ROUND(F147*G147,2))</f>
         <v/>
       </c>
       <c r="I147" s="22" t="str">
@@ -8759,7 +8688,7 @@
       <c r="F148" s="13"/>
       <c r="G148" s="21"/>
       <c r="H148" s="22" t="str">
-        <f>IF(F148="","",IF(OR(E148="Abschreibung (AfA)",E148="Vorsteuer auf Anlagevermögen"),0,ROUND(F148*G148,2)))</f>
+        <f aca="false">IF(F148="","",ROUND(F148*G148,2))</f>
         <v/>
       </c>
       <c r="I148" s="22" t="str">
@@ -8777,7 +8706,7 @@
       <c r="F149" s="13"/>
       <c r="G149" s="21"/>
       <c r="H149" s="22" t="str">
-        <f>IF(F149="","",IF(OR(E149="Abschreibung (AfA)",E149="Vorsteuer auf Anlagevermögen"),0,ROUND(F149*G149,2)))</f>
+        <f aca="false">IF(F149="","",ROUND(F149*G149,2))</f>
         <v/>
       </c>
       <c r="I149" s="22" t="str">
@@ -8795,7 +8724,7 @@
       <c r="F150" s="13"/>
       <c r="G150" s="21"/>
       <c r="H150" s="22" t="str">
-        <f>IF(F150="","",IF(OR(E150="Abschreibung (AfA)",E150="Vorsteuer auf Anlagevermögen"),0,ROUND(F150*G150,2)))</f>
+        <f aca="false">IF(F150="","",ROUND(F150*G150,2))</f>
         <v/>
       </c>
       <c r="I150" s="22" t="str">
@@ -8813,7 +8742,7 @@
       <c r="F151" s="13"/>
       <c r="G151" s="21"/>
       <c r="H151" s="22" t="str">
-        <f>IF(F151="","",IF(OR(E151="Abschreibung (AfA)",E151="Vorsteuer auf Anlagevermögen"),0,ROUND(F151*G151,2)))</f>
+        <f aca="false">IF(F151="","",ROUND(F151*G151,2))</f>
         <v/>
       </c>
       <c r="I151" s="22" t="str">
@@ -8831,7 +8760,7 @@
       <c r="F152" s="13"/>
       <c r="G152" s="21"/>
       <c r="H152" s="22" t="str">
-        <f>IF(F152="","",IF(OR(E152="Abschreibung (AfA)",E152="Vorsteuer auf Anlagevermögen"),0,ROUND(F152*G152,2)))</f>
+        <f aca="false">IF(F152="","",ROUND(F152*G152,2))</f>
         <v/>
       </c>
       <c r="I152" s="22" t="str">
@@ -8849,7 +8778,7 @@
       <c r="F153" s="13"/>
       <c r="G153" s="21"/>
       <c r="H153" s="22" t="str">
-        <f>IF(F153="","",IF(OR(E153="Abschreibung (AfA)",E153="Vorsteuer auf Anlagevermögen"),0,ROUND(F153*G153,2)))</f>
+        <f aca="false">IF(F153="","",ROUND(F153*G153,2))</f>
         <v/>
       </c>
       <c r="I153" s="22" t="str">
@@ -8867,7 +8796,7 @@
       <c r="F154" s="13"/>
       <c r="G154" s="21"/>
       <c r="H154" s="22" t="str">
-        <f>IF(F154="","",IF(OR(E154="Abschreibung (AfA)",E154="Vorsteuer auf Anlagevermögen"),0,ROUND(F154*G154,2)))</f>
+        <f aca="false">IF(F154="","",ROUND(F154*G154,2))</f>
         <v/>
       </c>
       <c r="I154" s="22" t="str">
@@ -8885,7 +8814,7 @@
       <c r="F155" s="13"/>
       <c r="G155" s="21"/>
       <c r="H155" s="22" t="str">
-        <f>IF(F155="","",IF(OR(E155="Abschreibung (AfA)",E155="Vorsteuer auf Anlagevermögen"),0,ROUND(F155*G155,2)))</f>
+        <f aca="false">IF(F155="","",ROUND(F155*G155,2))</f>
         <v/>
       </c>
       <c r="I155" s="22" t="str">
@@ -8903,7 +8832,7 @@
       <c r="F156" s="13"/>
       <c r="G156" s="21"/>
       <c r="H156" s="22" t="str">
-        <f>IF(F156="","",IF(OR(E156="Abschreibung (AfA)",E156="Vorsteuer auf Anlagevermögen"),0,ROUND(F156*G156,2)))</f>
+        <f aca="false">IF(F156="","",ROUND(F156*G156,2))</f>
         <v/>
       </c>
       <c r="I156" s="22" t="str">
@@ -8921,7 +8850,7 @@
       <c r="F157" s="13"/>
       <c r="G157" s="21"/>
       <c r="H157" s="22" t="str">
-        <f>IF(F157="","",IF(OR(E157="Abschreibung (AfA)",E157="Vorsteuer auf Anlagevermögen"),0,ROUND(F157*G157,2)))</f>
+        <f aca="false">IF(F157="","",ROUND(F157*G157,2))</f>
         <v/>
       </c>
       <c r="I157" s="22" t="str">
@@ -8939,7 +8868,7 @@
       <c r="F158" s="13"/>
       <c r="G158" s="21"/>
       <c r="H158" s="22" t="str">
-        <f>IF(F158="","",IF(OR(E158="Abschreibung (AfA)",E158="Vorsteuer auf Anlagevermögen"),0,ROUND(F158*G158,2)))</f>
+        <f aca="false">IF(F158="","",ROUND(F158*G158,2))</f>
         <v/>
       </c>
       <c r="I158" s="22" t="str">
@@ -8957,7 +8886,7 @@
       <c r="F159" s="13"/>
       <c r="G159" s="21"/>
       <c r="H159" s="22" t="str">
-        <f>IF(F159="","",IF(OR(E159="Abschreibung (AfA)",E159="Vorsteuer auf Anlagevermögen"),0,ROUND(F159*G159,2)))</f>
+        <f aca="false">IF(F159="","",ROUND(F159*G159,2))</f>
         <v/>
       </c>
       <c r="I159" s="22" t="str">
@@ -8975,7 +8904,7 @@
       <c r="F160" s="13"/>
       <c r="G160" s="21"/>
       <c r="H160" s="22" t="str">
-        <f>IF(F160="","",IF(OR(E160="Abschreibung (AfA)",E160="Vorsteuer auf Anlagevermögen"),0,ROUND(F160*G160,2)))</f>
+        <f aca="false">IF(F160="","",ROUND(F160*G160,2))</f>
         <v/>
       </c>
       <c r="I160" s="22" t="str">
@@ -8993,7 +8922,7 @@
       <c r="F161" s="13"/>
       <c r="G161" s="21"/>
       <c r="H161" s="22" t="str">
-        <f>IF(F161="","",IF(OR(E161="Abschreibung (AfA)",E161="Vorsteuer auf Anlagevermögen"),0,ROUND(F161*G161,2)))</f>
+        <f aca="false">IF(F161="","",ROUND(F161*G161,2))</f>
         <v/>
       </c>
       <c r="I161" s="22" t="str">
@@ -9011,7 +8940,7 @@
       <c r="F162" s="13"/>
       <c r="G162" s="21"/>
       <c r="H162" s="22" t="str">
-        <f>IF(F162="","",IF(OR(E162="Abschreibung (AfA)",E162="Vorsteuer auf Anlagevermögen"),0,ROUND(F162*G162,2)))</f>
+        <f aca="false">IF(F162="","",ROUND(F162*G162,2))</f>
         <v/>
       </c>
       <c r="I162" s="22" t="str">
@@ -9029,7 +8958,7 @@
       <c r="F163" s="13"/>
       <c r="G163" s="21"/>
       <c r="H163" s="22" t="str">
-        <f>IF(F163="","",IF(OR(E163="Abschreibung (AfA)",E163="Vorsteuer auf Anlagevermögen"),0,ROUND(F163*G163,2)))</f>
+        <f aca="false">IF(F163="","",ROUND(F163*G163,2))</f>
         <v/>
       </c>
       <c r="I163" s="22" t="str">
@@ -9047,7 +8976,7 @@
       <c r="F164" s="13"/>
       <c r="G164" s="21"/>
       <c r="H164" s="22" t="str">
-        <f>IF(F164="","",IF(OR(E164="Abschreibung (AfA)",E164="Vorsteuer auf Anlagevermögen"),0,ROUND(F164*G164,2)))</f>
+        <f aca="false">IF(F164="","",ROUND(F164*G164,2))</f>
         <v/>
       </c>
       <c r="I164" s="22" t="str">
@@ -9065,7 +8994,7 @@
       <c r="F165" s="13"/>
       <c r="G165" s="21"/>
       <c r="H165" s="22" t="str">
-        <f>IF(F165="","",IF(OR(E165="Abschreibung (AfA)",E165="Vorsteuer auf Anlagevermögen"),0,ROUND(F165*G165,2)))</f>
+        <f aca="false">IF(F165="","",ROUND(F165*G165,2))</f>
         <v/>
       </c>
       <c r="I165" s="22" t="str">
@@ -9083,7 +9012,7 @@
       <c r="F166" s="13"/>
       <c r="G166" s="21"/>
       <c r="H166" s="22" t="str">
-        <f>IF(F166="","",IF(OR(E166="Abschreibung (AfA)",E166="Vorsteuer auf Anlagevermögen"),0,ROUND(F166*G166,2)))</f>
+        <f aca="false">IF(F166="","",ROUND(F166*G166,2))</f>
         <v/>
       </c>
       <c r="I166" s="22" t="str">
@@ -9101,7 +9030,7 @@
       <c r="F167" s="13"/>
       <c r="G167" s="21"/>
       <c r="H167" s="22" t="str">
-        <f>IF(F167="","",IF(OR(E167="Abschreibung (AfA)",E167="Vorsteuer auf Anlagevermögen"),0,ROUND(F167*G167,2)))</f>
+        <f aca="false">IF(F167="","",ROUND(F167*G167,2))</f>
         <v/>
       </c>
       <c r="I167" s="22" t="str">
@@ -9119,7 +9048,7 @@
       <c r="F168" s="13"/>
       <c r="G168" s="21"/>
       <c r="H168" s="22" t="str">
-        <f>IF(F168="","",IF(OR(E168="Abschreibung (AfA)",E168="Vorsteuer auf Anlagevermögen"),0,ROUND(F168*G168,2)))</f>
+        <f aca="false">IF(F168="","",ROUND(F168*G168,2))</f>
         <v/>
       </c>
       <c r="I168" s="22" t="str">
@@ -9137,7 +9066,7 @@
       <c r="F169" s="13"/>
       <c r="G169" s="21"/>
       <c r="H169" s="22" t="str">
-        <f>IF(F169="","",IF(OR(E169="Abschreibung (AfA)",E169="Vorsteuer auf Anlagevermögen"),0,ROUND(F169*G169,2)))</f>
+        <f aca="false">IF(F169="","",ROUND(F169*G169,2))</f>
         <v/>
       </c>
       <c r="I169" s="22" t="str">
@@ -9155,7 +9084,7 @@
       <c r="F170" s="13"/>
       <c r="G170" s="21"/>
       <c r="H170" s="22" t="str">
-        <f>IF(F170="","",IF(OR(E170="Abschreibung (AfA)",E170="Vorsteuer auf Anlagevermögen"),0,ROUND(F170*G170,2)))</f>
+        <f aca="false">IF(F170="","",ROUND(F170*G170,2))</f>
         <v/>
       </c>
       <c r="I170" s="22" t="str">
@@ -9173,7 +9102,7 @@
       <c r="F171" s="13"/>
       <c r="G171" s="21"/>
       <c r="H171" s="22" t="str">
-        <f>IF(F171="","",IF(OR(E171="Abschreibung (AfA)",E171="Vorsteuer auf Anlagevermögen"),0,ROUND(F171*G171,2)))</f>
+        <f aca="false">IF(F171="","",ROUND(F171*G171,2))</f>
         <v/>
       </c>
       <c r="I171" s="22" t="str">
@@ -9191,7 +9120,7 @@
       <c r="F172" s="13"/>
       <c r="G172" s="21"/>
       <c r="H172" s="22" t="str">
-        <f>IF(F172="","",IF(OR(E172="Abschreibung (AfA)",E172="Vorsteuer auf Anlagevermögen"),0,ROUND(F172*G172,2)))</f>
+        <f aca="false">IF(F172="","",ROUND(F172*G172,2))</f>
         <v/>
       </c>
       <c r="I172" s="22" t="str">
@@ -9209,7 +9138,7 @@
       <c r="F173" s="13"/>
       <c r="G173" s="21"/>
       <c r="H173" s="22" t="str">
-        <f>IF(F173="","",IF(OR(E173="Abschreibung (AfA)",E173="Vorsteuer auf Anlagevermögen"),0,ROUND(F173*G173,2)))</f>
+        <f aca="false">IF(F173="","",ROUND(F173*G173,2))</f>
         <v/>
       </c>
       <c r="I173" s="22" t="str">
@@ -9227,7 +9156,7 @@
       <c r="F174" s="13"/>
       <c r="G174" s="21"/>
       <c r="H174" s="22" t="str">
-        <f>IF(F174="","",IF(OR(E174="Abschreibung (AfA)",E174="Vorsteuer auf Anlagevermögen"),0,ROUND(F174*G174,2)))</f>
+        <f aca="false">IF(F174="","",ROUND(F174*G174,2))</f>
         <v/>
       </c>
       <c r="I174" s="22" t="str">
@@ -9245,7 +9174,7 @@
       <c r="F175" s="13"/>
       <c r="G175" s="21"/>
       <c r="H175" s="22" t="str">
-        <f>IF(F175="","",IF(OR(E175="Abschreibung (AfA)",E175="Vorsteuer auf Anlagevermögen"),0,ROUND(F175*G175,2)))</f>
+        <f aca="false">IF(F175="","",ROUND(F175*G175,2))</f>
         <v/>
       </c>
       <c r="I175" s="22" t="str">
@@ -9263,7 +9192,7 @@
       <c r="F176" s="13"/>
       <c r="G176" s="21"/>
       <c r="H176" s="22" t="str">
-        <f>IF(F176="","",IF(OR(E176="Abschreibung (AfA)",E176="Vorsteuer auf Anlagevermögen"),0,ROUND(F176*G176,2)))</f>
+        <f aca="false">IF(F176="","",ROUND(F176*G176,2))</f>
         <v/>
       </c>
       <c r="I176" s="22" t="str">
@@ -9281,7 +9210,7 @@
       <c r="F177" s="13"/>
       <c r="G177" s="21"/>
       <c r="H177" s="22" t="str">
-        <f>IF(F177="","",IF(OR(E177="Abschreibung (AfA)",E177="Vorsteuer auf Anlagevermögen"),0,ROUND(F177*G177,2)))</f>
+        <f aca="false">IF(F177="","",ROUND(F177*G177,2))</f>
         <v/>
       </c>
       <c r="I177" s="22" t="str">
@@ -9299,7 +9228,7 @@
       <c r="F178" s="13"/>
       <c r="G178" s="21"/>
       <c r="H178" s="22" t="str">
-        <f>IF(F178="","",IF(OR(E178="Abschreibung (AfA)",E178="Vorsteuer auf Anlagevermögen"),0,ROUND(F178*G178,2)))</f>
+        <f aca="false">IF(F178="","",ROUND(F178*G178,2))</f>
         <v/>
       </c>
       <c r="I178" s="22" t="str">
@@ -9317,7 +9246,7 @@
       <c r="F179" s="13"/>
       <c r="G179" s="21"/>
       <c r="H179" s="22" t="str">
-        <f>IF(F179="","",IF(OR(E179="Abschreibung (AfA)",E179="Vorsteuer auf Anlagevermögen"),0,ROUND(F179*G179,2)))</f>
+        <f aca="false">IF(F179="","",ROUND(F179*G179,2))</f>
         <v/>
       </c>
       <c r="I179" s="22" t="str">
@@ -9335,7 +9264,7 @@
       <c r="F180" s="13"/>
       <c r="G180" s="21"/>
       <c r="H180" s="22" t="str">
-        <f>IF(F180="","",IF(OR(E180="Abschreibung (AfA)",E180="Vorsteuer auf Anlagevermögen"),0,ROUND(F180*G180,2)))</f>
+        <f aca="false">IF(F180="","",ROUND(F180*G180,2))</f>
         <v/>
       </c>
       <c r="I180" s="22" t="str">
@@ -9353,7 +9282,7 @@
       <c r="F181" s="13"/>
       <c r="G181" s="21"/>
       <c r="H181" s="22" t="str">
-        <f>IF(F181="","",IF(OR(E181="Abschreibung (AfA)",E181="Vorsteuer auf Anlagevermögen"),0,ROUND(F181*G181,2)))</f>
+        <f aca="false">IF(F181="","",ROUND(F181*G181,2))</f>
         <v/>
       </c>
       <c r="I181" s="22" t="str">
@@ -9371,7 +9300,7 @@
       <c r="F182" s="13"/>
       <c r="G182" s="21"/>
       <c r="H182" s="22" t="str">
-        <f>IF(F182="","",IF(OR(E182="Abschreibung (AfA)",E182="Vorsteuer auf Anlagevermögen"),0,ROUND(F182*G182,2)))</f>
+        <f aca="false">IF(F182="","",ROUND(F182*G182,2))</f>
         <v/>
       </c>
       <c r="I182" s="22" t="str">
@@ -9389,7 +9318,7 @@
       <c r="F183" s="13"/>
       <c r="G183" s="21"/>
       <c r="H183" s="22" t="str">
-        <f>IF(F183="","",IF(OR(E183="Abschreibung (AfA)",E183="Vorsteuer auf Anlagevermögen"),0,ROUND(F183*G183,2)))</f>
+        <f aca="false">IF(F183="","",ROUND(F183*G183,2))</f>
         <v/>
       </c>
       <c r="I183" s="22" t="str">
@@ -9407,7 +9336,7 @@
       <c r="F184" s="13"/>
       <c r="G184" s="21"/>
       <c r="H184" s="22" t="str">
-        <f>IF(F184="","",IF(OR(E184="Abschreibung (AfA)",E184="Vorsteuer auf Anlagevermögen"),0,ROUND(F184*G184,2)))</f>
+        <f aca="false">IF(F184="","",ROUND(F184*G184,2))</f>
         <v/>
       </c>
       <c r="I184" s="22" t="str">
@@ -9425,7 +9354,7 @@
       <c r="F185" s="13"/>
       <c r="G185" s="21"/>
       <c r="H185" s="22" t="str">
-        <f>IF(F185="","",IF(OR(E185="Abschreibung (AfA)",E185="Vorsteuer auf Anlagevermögen"),0,ROUND(F185*G185,2)))</f>
+        <f aca="false">IF(F185="","",ROUND(F185*G185,2))</f>
         <v/>
       </c>
       <c r="I185" s="22" t="str">
@@ -9443,7 +9372,7 @@
       <c r="F186" s="13"/>
       <c r="G186" s="21"/>
       <c r="H186" s="22" t="str">
-        <f>IF(F186="","",IF(OR(E186="Abschreibung (AfA)",E186="Vorsteuer auf Anlagevermögen"),0,ROUND(F186*G186,2)))</f>
+        <f aca="false">IF(F186="","",ROUND(F186*G186,2))</f>
         <v/>
       </c>
       <c r="I186" s="22" t="str">
@@ -9461,7 +9390,7 @@
       <c r="F187" s="13"/>
       <c r="G187" s="21"/>
       <c r="H187" s="22" t="str">
-        <f>IF(F187="","",IF(OR(E187="Abschreibung (AfA)",E187="Vorsteuer auf Anlagevermögen"),0,ROUND(F187*G187,2)))</f>
+        <f aca="false">IF(F187="","",ROUND(F187*G187,2))</f>
         <v/>
       </c>
       <c r="I187" s="22" t="str">
@@ -9479,7 +9408,7 @@
       <c r="F188" s="13"/>
       <c r="G188" s="21"/>
       <c r="H188" s="22" t="str">
-        <f>IF(F188="","",IF(OR(E188="Abschreibung (AfA)",E188="Vorsteuer auf Anlagevermögen"),0,ROUND(F188*G188,2)))</f>
+        <f aca="false">IF(F188="","",ROUND(F188*G188,2))</f>
         <v/>
       </c>
       <c r="I188" s="22" t="str">
@@ -9497,7 +9426,7 @@
       <c r="F189" s="13"/>
       <c r="G189" s="21"/>
       <c r="H189" s="22" t="str">
-        <f>IF(F189="","",IF(OR(E189="Abschreibung (AfA)",E189="Vorsteuer auf Anlagevermögen"),0,ROUND(F189*G189,2)))</f>
+        <f aca="false">IF(F189="","",ROUND(F189*G189,2))</f>
         <v/>
       </c>
       <c r="I189" s="22" t="str">
@@ -9515,7 +9444,7 @@
       <c r="F190" s="13"/>
       <c r="G190" s="21"/>
       <c r="H190" s="22" t="str">
-        <f>IF(F190="","",IF(OR(E190="Abschreibung (AfA)",E190="Vorsteuer auf Anlagevermögen"),0,ROUND(F190*G190,2)))</f>
+        <f aca="false">IF(F190="","",ROUND(F190*G190,2))</f>
         <v/>
       </c>
       <c r="I190" s="22" t="str">
@@ -9533,7 +9462,7 @@
       <c r="F191" s="13"/>
       <c r="G191" s="21"/>
       <c r="H191" s="22" t="str">
-        <f>IF(F191="","",IF(OR(E191="Abschreibung (AfA)",E191="Vorsteuer auf Anlagevermögen"),0,ROUND(F191*G191,2)))</f>
+        <f aca="false">IF(F191="","",ROUND(F191*G191,2))</f>
         <v/>
       </c>
       <c r="I191" s="22" t="str">
@@ -9551,7 +9480,7 @@
       <c r="F192" s="13"/>
       <c r="G192" s="21"/>
       <c r="H192" s="22" t="str">
-        <f>IF(F192="","",IF(OR(E192="Abschreibung (AfA)",E192="Vorsteuer auf Anlagevermögen"),0,ROUND(F192*G192,2)))</f>
+        <f aca="false">IF(F192="","",ROUND(F192*G192,2))</f>
         <v/>
       </c>
       <c r="I192" s="22" t="str">
@@ -9569,7 +9498,7 @@
       <c r="F193" s="13"/>
       <c r="G193" s="21"/>
       <c r="H193" s="22" t="str">
-        <f>IF(F193="","",IF(OR(E193="Abschreibung (AfA)",E193="Vorsteuer auf Anlagevermögen"),0,ROUND(F193*G193,2)))</f>
+        <f aca="false">IF(F193="","",ROUND(F193*G193,2))</f>
         <v/>
       </c>
       <c r="I193" s="22" t="str">
@@ -9587,7 +9516,7 @@
       <c r="F194" s="13"/>
       <c r="G194" s="21"/>
       <c r="H194" s="22" t="str">
-        <f>IF(F194="","",IF(OR(E194="Abschreibung (AfA)",E194="Vorsteuer auf Anlagevermögen"),0,ROUND(F194*G194,2)))</f>
+        <f aca="false">IF(F194="","",ROUND(F194*G194,2))</f>
         <v/>
       </c>
       <c r="I194" s="22" t="str">
@@ -9605,7 +9534,7 @@
       <c r="F195" s="13"/>
       <c r="G195" s="21"/>
       <c r="H195" s="22" t="str">
-        <f>IF(F195="","",IF(OR(E195="Abschreibung (AfA)",E195="Vorsteuer auf Anlagevermögen"),0,ROUND(F195*G195,2)))</f>
+        <f aca="false">IF(F195="","",ROUND(F195*G195,2))</f>
         <v/>
       </c>
       <c r="I195" s="22" t="str">
@@ -9623,7 +9552,7 @@
       <c r="F196" s="13"/>
       <c r="G196" s="21"/>
       <c r="H196" s="22" t="str">
-        <f>IF(F196="","",IF(OR(E196="Abschreibung (AfA)",E196="Vorsteuer auf Anlagevermögen"),0,ROUND(F196*G196,2)))</f>
+        <f aca="false">IF(F196="","",ROUND(F196*G196,2))</f>
         <v/>
       </c>
       <c r="I196" s="22" t="str">
@@ -9641,7 +9570,7 @@
       <c r="F197" s="13"/>
       <c r="G197" s="21"/>
       <c r="H197" s="22" t="str">
-        <f>IF(F197="","",IF(OR(E197="Abschreibung (AfA)",E197="Vorsteuer auf Anlagevermögen"),0,ROUND(F197*G197,2)))</f>
+        <f aca="false">IF(F197="","",ROUND(F197*G197,2))</f>
         <v/>
       </c>
       <c r="I197" s="22" t="str">
@@ -9659,7 +9588,7 @@
       <c r="F198" s="13"/>
       <c r="G198" s="21"/>
       <c r="H198" s="22" t="str">
-        <f>IF(F198="","",IF(OR(E198="Abschreibung (AfA)",E198="Vorsteuer auf Anlagevermögen"),0,ROUND(F198*G198,2)))</f>
+        <f aca="false">IF(F198="","",ROUND(F198*G198,2))</f>
         <v/>
       </c>
       <c r="I198" s="22" t="str">
@@ -9677,7 +9606,7 @@
       <c r="F199" s="13"/>
       <c r="G199" s="21"/>
       <c r="H199" s="22" t="str">
-        <f>IF(F199="","",IF(OR(E199="Abschreibung (AfA)",E199="Vorsteuer auf Anlagevermögen"),0,ROUND(F199*G199,2)))</f>
+        <f aca="false">IF(F199="","",ROUND(F199*G199,2))</f>
         <v/>
       </c>
       <c r="I199" s="22" t="str">
@@ -9695,7 +9624,7 @@
       <c r="F200" s="13"/>
       <c r="G200" s="21"/>
       <c r="H200" s="22" t="str">
-        <f>IF(F200="","",IF(OR(E200="Abschreibung (AfA)",E200="Vorsteuer auf Anlagevermögen"),0,ROUND(F200*G200,2)))</f>
+        <f aca="false">IF(F200="","",ROUND(F200*G200,2))</f>
         <v/>
       </c>
       <c r="I200" s="22" t="str">
@@ -9713,7 +9642,7 @@
       <c r="F201" s="13"/>
       <c r="G201" s="21"/>
       <c r="H201" s="22" t="str">
-        <f>IF(F201="","",IF(OR(E201="Abschreibung (AfA)",E201="Vorsteuer auf Anlagevermögen"),0,ROUND(F201*G201,2)))</f>
+        <f aca="false">IF(F201="","",ROUND(F201*G201,2))</f>
         <v/>
       </c>
       <c r="I201" s="22" t="str">
@@ -9731,7 +9660,7 @@
       <c r="F202" s="13"/>
       <c r="G202" s="21"/>
       <c r="H202" s="22" t="str">
-        <f>IF(F202="","",IF(OR(E202="Abschreibung (AfA)",E202="Vorsteuer auf Anlagevermögen"),0,ROUND(F202*G202,2)))</f>
+        <f aca="false">IF(F202="","",ROUND(F202*G202,2))</f>
         <v/>
       </c>
       <c r="I202" s="22" t="str">
@@ -9749,7 +9678,7 @@
       <c r="F203" s="13"/>
       <c r="G203" s="21"/>
       <c r="H203" s="22" t="str">
-        <f>IF(F203="","",IF(OR(E203="Abschreibung (AfA)",E203="Vorsteuer auf Anlagevermögen"),0,ROUND(F203*G203,2)))</f>
+        <f aca="false">IF(F203="","",ROUND(F203*G203,2))</f>
         <v/>
       </c>
       <c r="I203" s="22" t="str">
@@ -9767,7 +9696,7 @@
       <c r="F204" s="13"/>
       <c r="G204" s="21"/>
       <c r="H204" s="22" t="str">
-        <f>IF(F204="","",IF(OR(E204="Abschreibung (AfA)",E204="Vorsteuer auf Anlagevermögen"),0,ROUND(F204*G204,2)))</f>
+        <f aca="false">IF(F204="","",ROUND(F204*G204,2))</f>
         <v/>
       </c>
       <c r="I204" s="22" t="str">
@@ -9785,7 +9714,7 @@
       <c r="F205" s="13"/>
       <c r="G205" s="21"/>
       <c r="H205" s="22" t="str">
-        <f>IF(F205="","",IF(OR(E205="Abschreibung (AfA)",E205="Vorsteuer auf Anlagevermögen"),0,ROUND(F205*G205,2)))</f>
+        <f aca="false">IF(F205="","",ROUND(F205*G205,2))</f>
         <v/>
       </c>
       <c r="I205" s="22" t="str">
@@ -9803,7 +9732,7 @@
       <c r="F206" s="13"/>
       <c r="G206" s="21"/>
       <c r="H206" s="22" t="str">
-        <f>IF(F206="","",IF(OR(E206="Abschreibung (AfA)",E206="Vorsteuer auf Anlagevermögen"),0,ROUND(F206*G206,2)))</f>
+        <f aca="false">IF(F206="","",ROUND(F206*G206,2))</f>
         <v/>
       </c>
       <c r="I206" s="22" t="str">
@@ -9821,7 +9750,7 @@
       <c r="F207" s="13"/>
       <c r="G207" s="21"/>
       <c r="H207" s="22" t="str">
-        <f>IF(F207="","",IF(OR(E207="Abschreibung (AfA)",E207="Vorsteuer auf Anlagevermögen"),0,ROUND(F207*G207,2)))</f>
+        <f aca="false">IF(F207="","",ROUND(F207*G207,2))</f>
         <v/>
       </c>
       <c r="I207" s="22" t="str">
@@ -9839,7 +9768,7 @@
       <c r="F208" s="13"/>
       <c r="G208" s="21"/>
       <c r="H208" s="22" t="str">
-        <f>IF(F208="","",IF(OR(E208="Abschreibung (AfA)",E208="Vorsteuer auf Anlagevermögen"),0,ROUND(F208*G208,2)))</f>
+        <f aca="false">IF(F208="","",ROUND(F208*G208,2))</f>
         <v/>
       </c>
       <c r="I208" s="22" t="str">
@@ -9857,7 +9786,7 @@
       <c r="F209" s="13"/>
       <c r="G209" s="21"/>
       <c r="H209" s="22" t="str">
-        <f>IF(F209="","",IF(OR(E209="Abschreibung (AfA)",E209="Vorsteuer auf Anlagevermögen"),0,ROUND(F209*G209,2)))</f>
+        <f aca="false">IF(F209="","",ROUND(F209*G209,2))</f>
         <v/>
       </c>
       <c r="I209" s="22" t="str">
@@ -9875,7 +9804,7 @@
       <c r="F210" s="13"/>
       <c r="G210" s="21"/>
       <c r="H210" s="22" t="str">
-        <f>IF(F210="","",IF(OR(E210="Abschreibung (AfA)",E210="Vorsteuer auf Anlagevermögen"),0,ROUND(F210*G210,2)))</f>
+        <f aca="false">IF(F210="","",ROUND(F210*G210,2))</f>
         <v/>
       </c>
       <c r="I210" s="22" t="str">
@@ -9893,7 +9822,7 @@
       <c r="F211" s="13"/>
       <c r="G211" s="21"/>
       <c r="H211" s="22" t="str">
-        <f>IF(F211="","",IF(OR(E211="Abschreibung (AfA)",E211="Vorsteuer auf Anlagevermögen"),0,ROUND(F211*G211,2)))</f>
+        <f aca="false">IF(F211="","",ROUND(F211*G211,2))</f>
         <v/>
       </c>
       <c r="I211" s="22" t="str">
@@ -9911,7 +9840,7 @@
       <c r="F212" s="13"/>
       <c r="G212" s="21"/>
       <c r="H212" s="22" t="str">
-        <f>IF(F212="","",IF(OR(E212="Abschreibung (AfA)",E212="Vorsteuer auf Anlagevermögen"),0,ROUND(F212*G212,2)))</f>
+        <f aca="false">IF(F212="","",ROUND(F212*G212,2))</f>
         <v/>
       </c>
       <c r="I212" s="22" t="str">
@@ -9929,7 +9858,7 @@
       <c r="F213" s="13"/>
       <c r="G213" s="21"/>
       <c r="H213" s="22" t="str">
-        <f>IF(F213="","",IF(OR(E213="Abschreibung (AfA)",E213="Vorsteuer auf Anlagevermögen"),0,ROUND(F213*G213,2)))</f>
+        <f aca="false">IF(F213="","",ROUND(F213*G213,2))</f>
         <v/>
       </c>
       <c r="I213" s="22" t="str">
@@ -9947,7 +9876,7 @@
       <c r="F214" s="13"/>
       <c r="G214" s="21"/>
       <c r="H214" s="22" t="str">
-        <f>IF(F214="","",IF(OR(E214="Abschreibung (AfA)",E214="Vorsteuer auf Anlagevermögen"),0,ROUND(F214*G214,2)))</f>
+        <f aca="false">IF(F214="","",ROUND(F214*G214,2))</f>
         <v/>
       </c>
       <c r="I214" s="22" t="str">
@@ -9965,7 +9894,7 @@
       <c r="F215" s="13"/>
       <c r="G215" s="21"/>
       <c r="H215" s="22" t="str">
-        <f>IF(F215="","",IF(OR(E215="Abschreibung (AfA)",E215="Vorsteuer auf Anlagevermögen"),0,ROUND(F215*G215,2)))</f>
+        <f aca="false">IF(F215="","",ROUND(F215*G215,2))</f>
         <v/>
       </c>
       <c r="I215" s="22" t="str">
@@ -9983,7 +9912,7 @@
       <c r="F216" s="13"/>
       <c r="G216" s="21"/>
       <c r="H216" s="22" t="str">
-        <f>IF(F216="","",IF(OR(E216="Abschreibung (AfA)",E216="Vorsteuer auf Anlagevermögen"),0,ROUND(F216*G216,2)))</f>
+        <f aca="false">IF(F216="","",ROUND(F216*G216,2))</f>
         <v/>
       </c>
       <c r="I216" s="22" t="str">
@@ -10001,7 +9930,7 @@
       <c r="F217" s="13"/>
       <c r="G217" s="21"/>
       <c r="H217" s="22" t="str">
-        <f>IF(F217="","",IF(OR(E217="Abschreibung (AfA)",E217="Vorsteuer auf Anlagevermögen"),0,ROUND(F217*G217,2)))</f>
+        <f aca="false">IF(F217="","",ROUND(F217*G217,2))</f>
         <v/>
       </c>
       <c r="I217" s="22" t="str">
@@ -10019,7 +9948,7 @@
       <c r="F218" s="13"/>
       <c r="G218" s="21"/>
       <c r="H218" s="22" t="str">
-        <f>IF(F218="","",IF(OR(E218="Abschreibung (AfA)",E218="Vorsteuer auf Anlagevermögen"),0,ROUND(F218*G218,2)))</f>
+        <f aca="false">IF(F218="","",ROUND(F218*G218,2))</f>
         <v/>
       </c>
       <c r="I218" s="22" t="str">
@@ -10037,7 +9966,7 @@
       <c r="F219" s="13"/>
       <c r="G219" s="21"/>
       <c r="H219" s="22" t="str">
-        <f>IF(F219="","",IF(OR(E219="Abschreibung (AfA)",E219="Vorsteuer auf Anlagevermögen"),0,ROUND(F219*G219,2)))</f>
+        <f aca="false">IF(F219="","",ROUND(F219*G219,2))</f>
         <v/>
       </c>
       <c r="I219" s="22" t="str">
@@ -10055,7 +9984,7 @@
       <c r="F220" s="13"/>
       <c r="G220" s="21"/>
       <c r="H220" s="22" t="str">
-        <f>IF(F220="","",IF(OR(E220="Abschreibung (AfA)",E220="Vorsteuer auf Anlagevermögen"),0,ROUND(F220*G220,2)))</f>
+        <f aca="false">IF(F220="","",ROUND(F220*G220,2))</f>
         <v/>
       </c>
       <c r="I220" s="22" t="str">
@@ -10073,7 +10002,7 @@
       <c r="F221" s="13"/>
       <c r="G221" s="21"/>
       <c r="H221" s="22" t="str">
-        <f>IF(F221="","",IF(OR(E221="Abschreibung (AfA)",E221="Vorsteuer auf Anlagevermögen"),0,ROUND(F221*G221,2)))</f>
+        <f aca="false">IF(F221="","",ROUND(F221*G221,2))</f>
         <v/>
       </c>
       <c r="I221" s="22" t="str">
@@ -10091,7 +10020,7 @@
       <c r="F222" s="13"/>
       <c r="G222" s="21"/>
       <c r="H222" s="22" t="str">
-        <f>IF(F222="","",IF(OR(E222="Abschreibung (AfA)",E222="Vorsteuer auf Anlagevermögen"),0,ROUND(F222*G222,2)))</f>
+        <f aca="false">IF(F222="","",ROUND(F222*G222,2))</f>
         <v/>
       </c>
       <c r="I222" s="22" t="str">
@@ -10109,7 +10038,7 @@
       <c r="F223" s="13"/>
       <c r="G223" s="21"/>
       <c r="H223" s="22" t="str">
-        <f>IF(F223="","",IF(OR(E223="Abschreibung (AfA)",E223="Vorsteuer auf Anlagevermögen"),0,ROUND(F223*G223,2)))</f>
+        <f aca="false">IF(F223="","",ROUND(F223*G223,2))</f>
         <v/>
       </c>
       <c r="I223" s="22" t="str">
@@ -10127,7 +10056,7 @@
       <c r="F224" s="13"/>
       <c r="G224" s="21"/>
       <c r="H224" s="22" t="str">
-        <f>IF(F224="","",IF(OR(E224="Abschreibung (AfA)",E224="Vorsteuer auf Anlagevermögen"),0,ROUND(F224*G224,2)))</f>
+        <f aca="false">IF(F224="","",ROUND(F224*G224,2))</f>
         <v/>
       </c>
       <c r="I224" s="22" t="str">
@@ -10145,7 +10074,7 @@
       <c r="F225" s="13"/>
       <c r="G225" s="21"/>
       <c r="H225" s="22" t="str">
-        <f>IF(F225="","",IF(OR(E225="Abschreibung (AfA)",E225="Vorsteuer auf Anlagevermögen"),0,ROUND(F225*G225,2)))</f>
+        <f aca="false">IF(F225="","",ROUND(F225*G225,2))</f>
         <v/>
       </c>
       <c r="I225" s="22" t="str">
@@ -10163,7 +10092,7 @@
       <c r="F226" s="13"/>
       <c r="G226" s="21"/>
       <c r="H226" s="22" t="str">
-        <f>IF(F226="","",IF(OR(E226="Abschreibung (AfA)",E226="Vorsteuer auf Anlagevermögen"),0,ROUND(F226*G226,2)))</f>
+        <f aca="false">IF(F226="","",ROUND(F226*G226,2))</f>
         <v/>
       </c>
       <c r="I226" s="22" t="str">
@@ -10181,7 +10110,7 @@
       <c r="F227" s="13"/>
       <c r="G227" s="21"/>
       <c r="H227" s="22" t="str">
-        <f>IF(F227="","",IF(OR(E227="Abschreibung (AfA)",E227="Vorsteuer auf Anlagevermögen"),0,ROUND(F227*G227,2)))</f>
+        <f aca="false">IF(F227="","",ROUND(F227*G227,2))</f>
         <v/>
       </c>
       <c r="I227" s="22" t="str">
@@ -10199,7 +10128,7 @@
       <c r="F228" s="13"/>
       <c r="G228" s="21"/>
       <c r="H228" s="22" t="str">
-        <f>IF(F228="","",IF(OR(E228="Abschreibung (AfA)",E228="Vorsteuer auf Anlagevermögen"),0,ROUND(F228*G228,2)))</f>
+        <f aca="false">IF(F228="","",ROUND(F228*G228,2))</f>
         <v/>
       </c>
       <c r="I228" s="22" t="str">
@@ -10217,7 +10146,7 @@
       <c r="F229" s="13"/>
       <c r="G229" s="21"/>
       <c r="H229" s="22" t="str">
-        <f>IF(F229="","",IF(OR(E229="Abschreibung (AfA)",E229="Vorsteuer auf Anlagevermögen"),0,ROUND(F229*G229,2)))</f>
+        <f aca="false">IF(F229="","",ROUND(F229*G229,2))</f>
         <v/>
       </c>
       <c r="I229" s="22" t="str">
@@ -10235,7 +10164,7 @@
       <c r="F230" s="13"/>
       <c r="G230" s="21"/>
       <c r="H230" s="22" t="str">
-        <f>IF(F230="","",IF(OR(E230="Abschreibung (AfA)",E230="Vorsteuer auf Anlagevermögen"),0,ROUND(F230*G230,2)))</f>
+        <f aca="false">IF(F230="","",ROUND(F230*G230,2))</f>
         <v/>
       </c>
       <c r="I230" s="22" t="str">
@@ -10253,7 +10182,7 @@
       <c r="F231" s="13"/>
       <c r="G231" s="21"/>
       <c r="H231" s="22" t="str">
-        <f>IF(F231="","",IF(OR(E231="Abschreibung (AfA)",E231="Vorsteuer auf Anlagevermögen"),0,ROUND(F231*G231,2)))</f>
+        <f aca="false">IF(F231="","",ROUND(F231*G231,2))</f>
         <v/>
       </c>
       <c r="I231" s="22" t="str">
@@ -10271,7 +10200,7 @@
       <c r="F232" s="13"/>
       <c r="G232" s="21"/>
       <c r="H232" s="22" t="str">
-        <f>IF(F232="","",IF(OR(E232="Abschreibung (AfA)",E232="Vorsteuer auf Anlagevermögen"),0,ROUND(F232*G232,2)))</f>
+        <f aca="false">IF(F232="","",ROUND(F232*G232,2))</f>
         <v/>
       </c>
       <c r="I232" s="22" t="str">
@@ -10289,7 +10218,7 @@
       <c r="F233" s="13"/>
       <c r="G233" s="21"/>
       <c r="H233" s="22" t="str">
-        <f>IF(F233="","",IF(OR(E233="Abschreibung (AfA)",E233="Vorsteuer auf Anlagevermögen"),0,ROUND(F233*G233,2)))</f>
+        <f aca="false">IF(F233="","",ROUND(F233*G233,2))</f>
         <v/>
       </c>
       <c r="I233" s="22" t="str">
@@ -10307,7 +10236,7 @@
       <c r="F234" s="13"/>
       <c r="G234" s="21"/>
       <c r="H234" s="22" t="str">
-        <f>IF(F234="","",IF(OR(E234="Abschreibung (AfA)",E234="Vorsteuer auf Anlagevermögen"),0,ROUND(F234*G234,2)))</f>
+        <f aca="false">IF(F234="","",ROUND(F234*G234,2))</f>
         <v/>
       </c>
       <c r="I234" s="22" t="str">
@@ -10325,7 +10254,7 @@
       <c r="F235" s="13"/>
       <c r="G235" s="21"/>
       <c r="H235" s="22" t="str">
-        <f>IF(F235="","",IF(OR(E235="Abschreibung (AfA)",E235="Vorsteuer auf Anlagevermögen"),0,ROUND(F235*G235,2)))</f>
+        <f aca="false">IF(F235="","",ROUND(F235*G235,2))</f>
         <v/>
       </c>
       <c r="I235" s="22" t="str">
@@ -10343,7 +10272,7 @@
       <c r="F236" s="13"/>
       <c r="G236" s="21"/>
       <c r="H236" s="22" t="str">
-        <f>IF(F236="","",IF(OR(E236="Abschreibung (AfA)",E236="Vorsteuer auf Anlagevermögen"),0,ROUND(F236*G236,2)))</f>
+        <f aca="false">IF(F236="","",ROUND(F236*G236,2))</f>
         <v/>
       </c>
       <c r="I236" s="22" t="str">
@@ -10361,7 +10290,7 @@
       <c r="F237" s="13"/>
       <c r="G237" s="21"/>
       <c r="H237" s="22" t="str">
-        <f>IF(F237="","",IF(OR(E237="Abschreibung (AfA)",E237="Vorsteuer auf Anlagevermögen"),0,ROUND(F237*G237,2)))</f>
+        <f aca="false">IF(F237="","",ROUND(F237*G237,2))</f>
         <v/>
       </c>
       <c r="I237" s="22" t="str">
@@ -10379,7 +10308,7 @@
       <c r="F238" s="13"/>
       <c r="G238" s="21"/>
       <c r="H238" s="22" t="str">
-        <f>IF(F238="","",IF(OR(E238="Abschreibung (AfA)",E238="Vorsteuer auf Anlagevermögen"),0,ROUND(F238*G238,2)))</f>
+        <f aca="false">IF(F238="","",ROUND(F238*G238,2))</f>
         <v/>
       </c>
       <c r="I238" s="22" t="str">
@@ -10397,7 +10326,7 @@
       <c r="F239" s="13"/>
       <c r="G239" s="21"/>
       <c r="H239" s="22" t="str">
-        <f>IF(F239="","",IF(OR(E239="Abschreibung (AfA)",E239="Vorsteuer auf Anlagevermögen"),0,ROUND(F239*G239,2)))</f>
+        <f aca="false">IF(F239="","",ROUND(F239*G239,2))</f>
         <v/>
       </c>
       <c r="I239" s="22" t="str">
@@ -10415,7 +10344,7 @@
       <c r="F240" s="13"/>
       <c r="G240" s="21"/>
       <c r="H240" s="22" t="str">
-        <f>IF(F240="","",IF(OR(E240="Abschreibung (AfA)",E240="Vorsteuer auf Anlagevermögen"),0,ROUND(F240*G240,2)))</f>
+        <f aca="false">IF(F240="","",ROUND(F240*G240,2))</f>
         <v/>
       </c>
       <c r="I240" s="22" t="str">
@@ -10433,7 +10362,7 @@
       <c r="F241" s="13"/>
       <c r="G241" s="21"/>
       <c r="H241" s="22" t="str">
-        <f>IF(F241="","",IF(OR(E241="Abschreibung (AfA)",E241="Vorsteuer auf Anlagevermögen"),0,ROUND(F241*G241,2)))</f>
+        <f aca="false">IF(F241="","",ROUND(F241*G241,2))</f>
         <v/>
       </c>
       <c r="I241" s="22" t="str">
@@ -10451,7 +10380,7 @@
       <c r="F242" s="13"/>
       <c r="G242" s="21"/>
       <c r="H242" s="22" t="str">
-        <f>IF(F242="","",IF(OR(E242="Abschreibung (AfA)",E242="Vorsteuer auf Anlagevermögen"),0,ROUND(F242*G242,2)))</f>
+        <f aca="false">IF(F242="","",ROUND(F242*G242,2))</f>
         <v/>
       </c>
       <c r="I242" s="22" t="str">
@@ -10469,7 +10398,7 @@
       <c r="F243" s="13"/>
       <c r="G243" s="21"/>
       <c r="H243" s="22" t="str">
-        <f>IF(F243="","",IF(OR(E243="Abschreibung (AfA)",E243="Vorsteuer auf Anlagevermögen"),0,ROUND(F243*G243,2)))</f>
+        <f aca="false">IF(F243="","",ROUND(F243*G243,2))</f>
         <v/>
       </c>
       <c r="I243" s="22" t="str">
@@ -10487,7 +10416,7 @@
       <c r="F244" s="13"/>
       <c r="G244" s="21"/>
       <c r="H244" s="22" t="str">
-        <f>IF(F244="","",IF(OR(E244="Abschreibung (AfA)",E244="Vorsteuer auf Anlagevermögen"),0,ROUND(F244*G244,2)))</f>
+        <f aca="false">IF(F244="","",ROUND(F244*G244,2))</f>
         <v/>
       </c>
       <c r="I244" s="22" t="str">
@@ -10505,7 +10434,7 @@
       <c r="F245" s="13"/>
       <c r="G245" s="21"/>
       <c r="H245" s="22" t="str">
-        <f>IF(F245="","",IF(OR(E245="Abschreibung (AfA)",E245="Vorsteuer auf Anlagevermögen"),0,ROUND(F245*G245,2)))</f>
+        <f aca="false">IF(F245="","",ROUND(F245*G245,2))</f>
         <v/>
       </c>
       <c r="I245" s="22" t="str">
@@ -10523,7 +10452,7 @@
       <c r="F246" s="13"/>
       <c r="G246" s="21"/>
       <c r="H246" s="22" t="str">
-        <f>IF(F246="","",IF(OR(E246="Abschreibung (AfA)",E246="Vorsteuer auf Anlagevermögen"),0,ROUND(F246*G246,2)))</f>
+        <f aca="false">IF(F246="","",ROUND(F246*G246,2))</f>
         <v/>
       </c>
       <c r="I246" s="22" t="str">
@@ -10541,7 +10470,7 @@
       <c r="F247" s="13"/>
       <c r="G247" s="21"/>
       <c r="H247" s="22" t="str">
-        <f>IF(F247="","",IF(OR(E247="Abschreibung (AfA)",E247="Vorsteuer auf Anlagevermögen"),0,ROUND(F247*G247,2)))</f>
+        <f aca="false">IF(F247="","",ROUND(F247*G247,2))</f>
         <v/>
       </c>
       <c r="I247" s="22" t="str">
@@ -10559,7 +10488,7 @@
       <c r="F248" s="13"/>
       <c r="G248" s="21"/>
       <c r="H248" s="22" t="str">
-        <f>IF(F248="","",IF(OR(E248="Abschreibung (AfA)",E248="Vorsteuer auf Anlagevermögen"),0,ROUND(F248*G248,2)))</f>
+        <f aca="false">IF(F248="","",ROUND(F248*G248,2))</f>
         <v/>
       </c>
       <c r="I248" s="22" t="str">
@@ -10577,7 +10506,7 @@
       <c r="F249" s="13"/>
       <c r="G249" s="21"/>
       <c r="H249" s="22" t="str">
-        <f>IF(F249="","",IF(OR(E249="Abschreibung (AfA)",E249="Vorsteuer auf Anlagevermögen"),0,ROUND(F249*G249,2)))</f>
+        <f aca="false">IF(F249="","",ROUND(F249*G249,2))</f>
         <v/>
       </c>
       <c r="I249" s="22" t="str">
@@ -10595,7 +10524,7 @@
       <c r="F250" s="13"/>
       <c r="G250" s="21"/>
       <c r="H250" s="22" t="str">
-        <f>IF(F250="","",IF(OR(E250="Abschreibung (AfA)",E250="Vorsteuer auf Anlagevermögen"),0,ROUND(F250*G250,2)))</f>
+        <f aca="false">IF(F250="","",ROUND(F250*G250,2))</f>
         <v/>
       </c>
       <c r="I250" s="22" t="str">
@@ -10613,7 +10542,7 @@
       <c r="F251" s="13"/>
       <c r="G251" s="21"/>
       <c r="H251" s="22" t="str">
-        <f>IF(F251="","",IF(OR(E251="Abschreibung (AfA)",E251="Vorsteuer auf Anlagevermögen"),0,ROUND(F251*G251,2)))</f>
+        <f aca="false">IF(F251="","",ROUND(F251*G251,2))</f>
         <v/>
       </c>
       <c r="I251" s="22" t="str">
@@ -10631,7 +10560,7 @@
       <c r="F252" s="13"/>
       <c r="G252" s="21"/>
       <c r="H252" s="22" t="str">
-        <f>IF(F252="","",IF(OR(E252="Abschreibung (AfA)",E252="Vorsteuer auf Anlagevermögen"),0,ROUND(F252*G252,2)))</f>
+        <f aca="false">IF(F252="","",ROUND(F252*G252,2))</f>
         <v/>
       </c>
       <c r="I252" s="22" t="str">
@@ -10649,7 +10578,7 @@
       <c r="F253" s="13"/>
       <c r="G253" s="21"/>
       <c r="H253" s="22" t="str">
-        <f>IF(F253="","",IF(OR(E253="Abschreibung (AfA)",E253="Vorsteuer auf Anlagevermögen"),0,ROUND(F253*G253,2)))</f>
+        <f aca="false">IF(F253="","",ROUND(F253*G253,2))</f>
         <v/>
       </c>
       <c r="I253" s="22" t="str">
@@ -10667,7 +10596,7 @@
       <c r="F254" s="13"/>
       <c r="G254" s="21"/>
       <c r="H254" s="22" t="str">
-        <f>IF(F254="","",IF(OR(E254="Abschreibung (AfA)",E254="Vorsteuer auf Anlagevermögen"),0,ROUND(F254*G254,2)))</f>
+        <f aca="false">IF(F254="","",ROUND(F254*G254,2))</f>
         <v/>
       </c>
       <c r="I254" s="22" t="str">
@@ -10685,7 +10614,7 @@
       <c r="F255" s="13"/>
       <c r="G255" s="21"/>
       <c r="H255" s="22" t="str">
-        <f>IF(F255="","",IF(OR(E255="Abschreibung (AfA)",E255="Vorsteuer auf Anlagevermögen"),0,ROUND(F255*G255,2)))</f>
+        <f aca="false">IF(F255="","",ROUND(F255*G255,2))</f>
         <v/>
       </c>
       <c r="I255" s="22" t="str">
@@ -10703,7 +10632,7 @@
       <c r="F256" s="13"/>
       <c r="G256" s="21"/>
       <c r="H256" s="22" t="str">
-        <f>IF(F256="","",IF(OR(E256="Abschreibung (AfA)",E256="Vorsteuer auf Anlagevermögen"),0,ROUND(F256*G256,2)))</f>
+        <f aca="false">IF(F256="","",ROUND(F256*G256,2))</f>
         <v/>
       </c>
       <c r="I256" s="22" t="str">
@@ -10721,7 +10650,7 @@
       <c r="F257" s="13"/>
       <c r="G257" s="21"/>
       <c r="H257" s="22" t="str">
-        <f>IF(F257="","",IF(OR(E257="Abschreibung (AfA)",E257="Vorsteuer auf Anlagevermögen"),0,ROUND(F257*G257,2)))</f>
+        <f aca="false">IF(F257="","",ROUND(F257*G257,2))</f>
         <v/>
       </c>
       <c r="I257" s="22" t="str">
@@ -10739,7 +10668,7 @@
       <c r="F258" s="13"/>
       <c r="G258" s="21"/>
       <c r="H258" s="22" t="str">
-        <f>IF(F258="","",IF(OR(E258="Abschreibung (AfA)",E258="Vorsteuer auf Anlagevermögen"),0,ROUND(F258*G258,2)))</f>
+        <f aca="false">IF(F258="","",ROUND(F258*G258,2))</f>
         <v/>
       </c>
       <c r="I258" s="22" t="str">
@@ -10757,7 +10686,7 @@
       <c r="F259" s="13"/>
       <c r="G259" s="21"/>
       <c r="H259" s="22" t="str">
-        <f>IF(F259="","",IF(OR(E259="Abschreibung (AfA)",E259="Vorsteuer auf Anlagevermögen"),0,ROUND(F259*G259,2)))</f>
+        <f aca="false">IF(F259="","",ROUND(F259*G259,2))</f>
         <v/>
       </c>
       <c r="I259" s="22" t="str">
@@ -10775,7 +10704,7 @@
       <c r="F260" s="13"/>
       <c r="G260" s="21"/>
       <c r="H260" s="22" t="str">
-        <f>IF(F260="","",IF(OR(E260="Abschreibung (AfA)",E260="Vorsteuer auf Anlagevermögen"),0,ROUND(F260*G260,2)))</f>
+        <f aca="false">IF(F260="","",ROUND(F260*G260,2))</f>
         <v/>
       </c>
       <c r="I260" s="22" t="str">
@@ -10793,7 +10722,7 @@
       <c r="F261" s="13"/>
       <c r="G261" s="21"/>
       <c r="H261" s="22" t="str">
-        <f>IF(F261="","",IF(OR(E261="Abschreibung (AfA)",E261="Vorsteuer auf Anlagevermögen"),0,ROUND(F261*G261,2)))</f>
+        <f aca="false">IF(F261="","",ROUND(F261*G261,2))</f>
         <v/>
       </c>
       <c r="I261" s="22" t="str">
@@ -10811,7 +10740,7 @@
       <c r="F262" s="13"/>
       <c r="G262" s="21"/>
       <c r="H262" s="22" t="str">
-        <f>IF(F262="","",IF(OR(E262="Abschreibung (AfA)",E262="Vorsteuer auf Anlagevermögen"),0,ROUND(F262*G262,2)))</f>
+        <f aca="false">IF(F262="","",ROUND(F262*G262,2))</f>
         <v/>
       </c>
       <c r="I262" s="22" t="str">
@@ -10829,7 +10758,7 @@
       <c r="F263" s="13"/>
       <c r="G263" s="21"/>
       <c r="H263" s="22" t="str">
-        <f>IF(F263="","",IF(OR(E263="Abschreibung (AfA)",E263="Vorsteuer auf Anlagevermögen"),0,ROUND(F263*G263,2)))</f>
+        <f aca="false">IF(F263="","",ROUND(F263*G263,2))</f>
         <v/>
       </c>
       <c r="I263" s="22" t="str">
@@ -10847,7 +10776,7 @@
       <c r="F264" s="13"/>
       <c r="G264" s="21"/>
       <c r="H264" s="22" t="str">
-        <f>IF(F264="","",IF(OR(E264="Abschreibung (AfA)",E264="Vorsteuer auf Anlagevermögen"),0,ROUND(F264*G264,2)))</f>
+        <f aca="false">IF(F264="","",ROUND(F264*G264,2))</f>
         <v/>
       </c>
       <c r="I264" s="22" t="str">
@@ -10865,7 +10794,7 @@
       <c r="F265" s="13"/>
       <c r="G265" s="21"/>
       <c r="H265" s="22" t="str">
-        <f>IF(F265="","",IF(OR(E265="Abschreibung (AfA)",E265="Vorsteuer auf Anlagevermögen"),0,ROUND(F265*G265,2)))</f>
+        <f aca="false">IF(F265="","",ROUND(F265*G265,2))</f>
         <v/>
       </c>
       <c r="I265" s="22" t="str">
@@ -10883,7 +10812,7 @@
       <c r="F266" s="13"/>
       <c r="G266" s="21"/>
       <c r="H266" s="22" t="str">
-        <f>IF(F266="","",IF(OR(E266="Abschreibung (AfA)",E266="Vorsteuer auf Anlagevermögen"),0,ROUND(F266*G266,2)))</f>
+        <f aca="false">IF(F266="","",ROUND(F266*G266,2))</f>
         <v/>
       </c>
       <c r="I266" s="22" t="str">
@@ -10901,7 +10830,7 @@
       <c r="F267" s="13"/>
       <c r="G267" s="21"/>
       <c r="H267" s="22" t="str">
-        <f>IF(F267="","",IF(OR(E267="Abschreibung (AfA)",E267="Vorsteuer auf Anlagevermögen"),0,ROUND(F267*G267,2)))</f>
+        <f aca="false">IF(F267="","",ROUND(F267*G267,2))</f>
         <v/>
       </c>
       <c r="I267" s="22" t="str">
@@ -10919,7 +10848,7 @@
       <c r="F268" s="13"/>
       <c r="G268" s="21"/>
       <c r="H268" s="22" t="str">
-        <f>IF(F268="","",IF(OR(E268="Abschreibung (AfA)",E268="Vorsteuer auf Anlagevermögen"),0,ROUND(F268*G268,2)))</f>
+        <f aca="false">IF(F268="","",ROUND(F268*G268,2))</f>
         <v/>
       </c>
       <c r="I268" s="22" t="str">
@@ -10937,7 +10866,7 @@
       <c r="F269" s="13"/>
       <c r="G269" s="21"/>
       <c r="H269" s="22" t="str">
-        <f>IF(F269="","",IF(OR(E269="Abschreibung (AfA)",E269="Vorsteuer auf Anlagevermögen"),0,ROUND(F269*G269,2)))</f>
+        <f aca="false">IF(F269="","",ROUND(F269*G269,2))</f>
         <v/>
       </c>
       <c r="I269" s="22" t="str">
@@ -10955,7 +10884,7 @@
       <c r="F270" s="13"/>
       <c r="G270" s="21"/>
       <c r="H270" s="22" t="str">
-        <f>IF(F270="","",IF(OR(E270="Abschreibung (AfA)",E270="Vorsteuer auf Anlagevermögen"),0,ROUND(F270*G270,2)))</f>
+        <f aca="false">IF(F270="","",ROUND(F270*G270,2))</f>
         <v/>
       </c>
       <c r="I270" s="22" t="str">
@@ -10973,7 +10902,7 @@
       <c r="F271" s="13"/>
       <c r="G271" s="21"/>
       <c r="H271" s="22" t="str">
-        <f>IF(F271="","",IF(OR(E271="Abschreibung (AfA)",E271="Vorsteuer auf Anlagevermögen"),0,ROUND(F271*G271,2)))</f>
+        <f aca="false">IF(F271="","",ROUND(F271*G271,2))</f>
         <v/>
       </c>
       <c r="I271" s="22" t="str">
@@ -10991,7 +10920,7 @@
       <c r="F272" s="13"/>
       <c r="G272" s="21"/>
       <c r="H272" s="22" t="str">
-        <f>IF(F272="","",IF(OR(E272="Abschreibung (AfA)",E272="Vorsteuer auf Anlagevermögen"),0,ROUND(F272*G272,2)))</f>
+        <f aca="false">IF(F272="","",ROUND(F272*G272,2))</f>
         <v/>
       </c>
       <c r="I272" s="22" t="str">
@@ -11009,7 +10938,7 @@
       <c r="F273" s="13"/>
       <c r="G273" s="21"/>
       <c r="H273" s="22" t="str">
-        <f>IF(F273="","",IF(OR(E273="Abschreibung (AfA)",E273="Vorsteuer auf Anlagevermögen"),0,ROUND(F273*G273,2)))</f>
+        <f aca="false">IF(F273="","",ROUND(F273*G273,2))</f>
         <v/>
       </c>
       <c r="I273" s="22" t="str">
@@ -11027,7 +10956,7 @@
       <c r="F274" s="13"/>
       <c r="G274" s="21"/>
       <c r="H274" s="22" t="str">
-        <f>IF(F274="","",IF(OR(E274="Abschreibung (AfA)",E274="Vorsteuer auf Anlagevermögen"),0,ROUND(F274*G274,2)))</f>
+        <f aca="false">IF(F274="","",ROUND(F274*G274,2))</f>
         <v/>
       </c>
       <c r="I274" s="22" t="str">
@@ -11045,7 +10974,7 @@
       <c r="F275" s="13"/>
       <c r="G275" s="21"/>
       <c r="H275" s="22" t="str">
-        <f>IF(F275="","",IF(OR(E275="Abschreibung (AfA)",E275="Vorsteuer auf Anlagevermögen"),0,ROUND(F275*G275,2)))</f>
+        <f aca="false">IF(F275="","",ROUND(F275*G275,2))</f>
         <v/>
       </c>
       <c r="I275" s="22" t="str">
@@ -11063,7 +10992,7 @@
       <c r="F276" s="13"/>
       <c r="G276" s="21"/>
       <c r="H276" s="22" t="str">
-        <f>IF(F276="","",IF(OR(E276="Abschreibung (AfA)",E276="Vorsteuer auf Anlagevermögen"),0,ROUND(F276*G276,2)))</f>
+        <f aca="false">IF(F276="","",ROUND(F276*G276,2))</f>
         <v/>
       </c>
       <c r="I276" s="22" t="str">
@@ -11081,7 +11010,7 @@
       <c r="F277" s="13"/>
       <c r="G277" s="21"/>
       <c r="H277" s="22" t="str">
-        <f>IF(F277="","",IF(OR(E277="Abschreibung (AfA)",E277="Vorsteuer auf Anlagevermögen"),0,ROUND(F277*G277,2)))</f>
+        <f aca="false">IF(F277="","",ROUND(F277*G277,2))</f>
         <v/>
       </c>
       <c r="I277" s="22" t="str">
@@ -11099,7 +11028,7 @@
       <c r="F278" s="13"/>
       <c r="G278" s="21"/>
       <c r="H278" s="22" t="str">
-        <f>IF(F278="","",IF(OR(E278="Abschreibung (AfA)",E278="Vorsteuer auf Anlagevermögen"),0,ROUND(F278*G278,2)))</f>
+        <f aca="false">IF(F278="","",ROUND(F278*G278,2))</f>
         <v/>
       </c>
       <c r="I278" s="22" t="str">
@@ -11117,7 +11046,7 @@
       <c r="F279" s="13"/>
       <c r="G279" s="21"/>
       <c r="H279" s="22" t="str">
-        <f>IF(F279="","",IF(OR(E279="Abschreibung (AfA)",E279="Vorsteuer auf Anlagevermögen"),0,ROUND(F279*G279,2)))</f>
+        <f aca="false">IF(F279="","",ROUND(F279*G279,2))</f>
         <v/>
       </c>
       <c r="I279" s="22" t="str">
@@ -11135,7 +11064,7 @@
       <c r="F280" s="13"/>
       <c r="G280" s="21"/>
       <c r="H280" s="22" t="str">
-        <f>IF(F280="","",IF(OR(E280="Abschreibung (AfA)",E280="Vorsteuer auf Anlagevermögen"),0,ROUND(F280*G280,2)))</f>
+        <f aca="false">IF(F280="","",ROUND(F280*G280,2))</f>
         <v/>
       </c>
       <c r="I280" s="22" t="str">
@@ -11153,7 +11082,7 @@
       <c r="F281" s="13"/>
       <c r="G281" s="21"/>
       <c r="H281" s="22" t="str">
-        <f>IF(F281="","",IF(OR(E281="Abschreibung (AfA)",E281="Vorsteuer auf Anlagevermögen"),0,ROUND(F281*G281,2)))</f>
+        <f aca="false">IF(F281="","",ROUND(F281*G281,2))</f>
         <v/>
       </c>
       <c r="I281" s="22" t="str">
@@ -11171,7 +11100,7 @@
       <c r="F282" s="13"/>
       <c r="G282" s="21"/>
       <c r="H282" s="22" t="str">
-        <f>IF(F282="","",IF(OR(E282="Abschreibung (AfA)",E282="Vorsteuer auf Anlagevermögen"),0,ROUND(F282*G282,2)))</f>
+        <f aca="false">IF(F282="","",ROUND(F282*G282,2))</f>
         <v/>
       </c>
       <c r="I282" s="22" t="str">
@@ -11189,7 +11118,7 @@
       <c r="F283" s="13"/>
       <c r="G283" s="21"/>
       <c r="H283" s="22" t="str">
-        <f>IF(F283="","",IF(OR(E283="Abschreibung (AfA)",E283="Vorsteuer auf Anlagevermögen"),0,ROUND(F283*G283,2)))</f>
+        <f aca="false">IF(F283="","",ROUND(F283*G283,2))</f>
         <v/>
       </c>
       <c r="I283" s="22" t="str">
@@ -11207,7 +11136,7 @@
       <c r="F284" s="13"/>
       <c r="G284" s="21"/>
       <c r="H284" s="22" t="str">
-        <f>IF(F284="","",IF(OR(E284="Abschreibung (AfA)",E284="Vorsteuer auf Anlagevermögen"),0,ROUND(F284*G284,2)))</f>
+        <f aca="false">IF(F284="","",ROUND(F284*G284,2))</f>
         <v/>
       </c>
       <c r="I284" s="22" t="str">
@@ -11225,7 +11154,7 @@
       <c r="F285" s="13"/>
       <c r="G285" s="21"/>
       <c r="H285" s="22" t="str">
-        <f>IF(F285="","",IF(OR(E285="Abschreibung (AfA)",E285="Vorsteuer auf Anlagevermögen"),0,ROUND(F285*G285,2)))</f>
+        <f aca="false">IF(F285="","",ROUND(F285*G285,2))</f>
         <v/>
       </c>
       <c r="I285" s="22" t="str">
@@ -11243,7 +11172,7 @@
       <c r="F286" s="13"/>
       <c r="G286" s="21"/>
       <c r="H286" s="22" t="str">
-        <f>IF(F286="","",IF(OR(E286="Abschreibung (AfA)",E286="Vorsteuer auf Anlagevermögen"),0,ROUND(F286*G286,2)))</f>
+        <f aca="false">IF(F286="","",ROUND(F286*G286,2))</f>
         <v/>
       </c>
       <c r="I286" s="22" t="str">
@@ -11261,7 +11190,7 @@
       <c r="F287" s="13"/>
       <c r="G287" s="21"/>
       <c r="H287" s="22" t="str">
-        <f>IF(F287="","",IF(OR(E287="Abschreibung (AfA)",E287="Vorsteuer auf Anlagevermögen"),0,ROUND(F287*G287,2)))</f>
+        <f aca="false">IF(F287="","",ROUND(F287*G287,2))</f>
         <v/>
       </c>
       <c r="I287" s="22" t="str">
@@ -11279,7 +11208,7 @@
       <c r="F288" s="13"/>
       <c r="G288" s="21"/>
       <c r="H288" s="22" t="str">
-        <f>IF(F288="","",IF(OR(E288="Abschreibung (AfA)",E288="Vorsteuer auf Anlagevermögen"),0,ROUND(F288*G288,2)))</f>
+        <f aca="false">IF(F288="","",ROUND(F288*G288,2))</f>
         <v/>
       </c>
       <c r="I288" s="22" t="str">
@@ -11297,7 +11226,7 @@
       <c r="F289" s="13"/>
       <c r="G289" s="21"/>
       <c r="H289" s="22" t="str">
-        <f>IF(F289="","",IF(OR(E289="Abschreibung (AfA)",E289="Vorsteuer auf Anlagevermögen"),0,ROUND(F289*G289,2)))</f>
+        <f aca="false">IF(F289="","",ROUND(F289*G289,2))</f>
         <v/>
       </c>
       <c r="I289" s="22" t="str">
@@ -11315,7 +11244,7 @@
       <c r="F290" s="13"/>
       <c r="G290" s="21"/>
       <c r="H290" s="22" t="str">
-        <f>IF(F290="","",IF(OR(E290="Abschreibung (AfA)",E290="Vorsteuer auf Anlagevermögen"),0,ROUND(F290*G290,2)))</f>
+        <f aca="false">IF(F290="","",ROUND(F290*G290,2))</f>
         <v/>
       </c>
       <c r="I290" s="22" t="str">
@@ -11333,7 +11262,7 @@
       <c r="F291" s="13"/>
       <c r="G291" s="21"/>
       <c r="H291" s="22" t="str">
-        <f>IF(F291="","",IF(OR(E291="Abschreibung (AfA)",E291="Vorsteuer auf Anlagevermögen"),0,ROUND(F291*G291,2)))</f>
+        <f aca="false">IF(F291="","",ROUND(F291*G291,2))</f>
         <v/>
       </c>
       <c r="I291" s="22" t="str">
@@ -11351,7 +11280,7 @@
       <c r="F292" s="13"/>
       <c r="G292" s="21"/>
       <c r="H292" s="22" t="str">
-        <f>IF(F292="","",IF(OR(E292="Abschreibung (AfA)",E292="Vorsteuer auf Anlagevermögen"),0,ROUND(F292*G292,2)))</f>
+        <f aca="false">IF(F292="","",ROUND(F292*G292,2))</f>
         <v/>
       </c>
       <c r="I292" s="22" t="str">
@@ -11369,7 +11298,7 @@
       <c r="F293" s="13"/>
       <c r="G293" s="21"/>
       <c r="H293" s="22" t="str">
-        <f>IF(F293="","",IF(OR(E293="Abschreibung (AfA)",E293="Vorsteuer auf Anlagevermögen"),0,ROUND(F293*G293,2)))</f>
+        <f aca="false">IF(F293="","",ROUND(F293*G293,2))</f>
         <v/>
       </c>
       <c r="I293" s="22" t="str">
@@ -11387,7 +11316,7 @@
       <c r="F294" s="13"/>
       <c r="G294" s="21"/>
       <c r="H294" s="22" t="str">
-        <f>IF(F294="","",IF(OR(E294="Abschreibung (AfA)",E294="Vorsteuer auf Anlagevermögen"),0,ROUND(F294*G294,2)))</f>
+        <f aca="false">IF(F294="","",ROUND(F294*G294,2))</f>
         <v/>
       </c>
       <c r="I294" s="22" t="str">
@@ -11405,7 +11334,7 @@
       <c r="F295" s="13"/>
       <c r="G295" s="21"/>
       <c r="H295" s="22" t="str">
-        <f>IF(F295="","",IF(OR(E295="Abschreibung (AfA)",E295="Vorsteuer auf Anlagevermögen"),0,ROUND(F295*G295,2)))</f>
+        <f aca="false">IF(F295="","",ROUND(F295*G295,2))</f>
         <v/>
       </c>
       <c r="I295" s="22" t="str">
@@ -11423,7 +11352,7 @@
       <c r="F296" s="13"/>
       <c r="G296" s="21"/>
       <c r="H296" s="22" t="str">
-        <f>IF(F296="","",IF(OR(E296="Abschreibung (AfA)",E296="Vorsteuer auf Anlagevermögen"),0,ROUND(F296*G296,2)))</f>
+        <f aca="false">IF(F296="","",ROUND(F296*G296,2))</f>
         <v/>
       </c>
       <c r="I296" s="22" t="str">
@@ -11441,7 +11370,7 @@
       <c r="F297" s="13"/>
       <c r="G297" s="21"/>
       <c r="H297" s="22" t="str">
-        <f>IF(F297="","",IF(OR(E297="Abschreibung (AfA)",E297="Vorsteuer auf Anlagevermögen"),0,ROUND(F297*G297,2)))</f>
+        <f aca="false">IF(F297="","",ROUND(F297*G297,2))</f>
         <v/>
       </c>
       <c r="I297" s="22" t="str">
@@ -11459,7 +11388,7 @@
       <c r="F298" s="13"/>
       <c r="G298" s="21"/>
       <c r="H298" s="22" t="str">
-        <f>IF(F298="","",IF(OR(E298="Abschreibung (AfA)",E298="Vorsteuer auf Anlagevermögen"),0,ROUND(F298*G298,2)))</f>
+        <f aca="false">IF(F298="","",ROUND(F298*G298,2))</f>
         <v/>
       </c>
       <c r="I298" s="22" t="str">
@@ -11477,7 +11406,7 @@
       <c r="F299" s="13"/>
       <c r="G299" s="21"/>
       <c r="H299" s="22" t="str">
-        <f>IF(F299="","",IF(OR(E299="Abschreibung (AfA)",E299="Vorsteuer auf Anlagevermögen"),0,ROUND(F299*G299,2)))</f>
+        <f aca="false">IF(F299="","",ROUND(F299*G299,2))</f>
         <v/>
       </c>
       <c r="I299" s="22" t="str">
@@ -11495,7 +11424,7 @@
       <c r="F300" s="13"/>
       <c r="G300" s="21"/>
       <c r="H300" s="22" t="str">
-        <f>IF(F300="","",IF(OR(E300="Abschreibung (AfA)",E300="Vorsteuer auf Anlagevermögen"),0,ROUND(F300*G300,2)))</f>
+        <f aca="false">IF(F300="","",ROUND(F300*G300,2))</f>
         <v/>
       </c>
       <c r="I300" s="22" t="str">
@@ -11513,7 +11442,7 @@
       <c r="F301" s="13"/>
       <c r="G301" s="21"/>
       <c r="H301" s="22" t="str">
-        <f>IF(F301="","",IF(OR(E301="Abschreibung (AfA)",E301="Vorsteuer auf Anlagevermögen"),0,ROUND(F301*G301,2)))</f>
+        <f aca="false">IF(F301="","",ROUND(F301*G301,2))</f>
         <v/>
       </c>
       <c r="I301" s="22" t="str">
@@ -11531,7 +11460,7 @@
       <c r="F302" s="13"/>
       <c r="G302" s="21"/>
       <c r="H302" s="22" t="str">
-        <f>IF(F302="","",IF(OR(E302="Abschreibung (AfA)",E302="Vorsteuer auf Anlagevermögen"),0,ROUND(F302*G302,2)))</f>
+        <f aca="false">IF(F302="","",ROUND(F302*G302,2))</f>
         <v/>
       </c>
       <c r="I302" s="22" t="str">
@@ -11549,7 +11478,7 @@
       <c r="F303" s="13"/>
       <c r="G303" s="21"/>
       <c r="H303" s="22" t="str">
-        <f>IF(F303="","",IF(OR(E303="Abschreibung (AfA)",E303="Vorsteuer auf Anlagevermögen"),0,ROUND(F303*G303,2)))</f>
+        <f aca="false">IF(F303="","",ROUND(F303*G303,2))</f>
         <v/>
       </c>
       <c r="I303" s="22" t="str">
@@ -11567,7 +11496,7 @@
       <c r="F304" s="13"/>
       <c r="G304" s="21"/>
       <c r="H304" s="22" t="str">
-        <f>IF(F304="","",IF(OR(E304="Abschreibung (AfA)",E304="Vorsteuer auf Anlagevermögen"),0,ROUND(F304*G304,2)))</f>
+        <f aca="false">IF(F304="","",ROUND(F304*G304,2))</f>
         <v/>
       </c>
       <c r="I304" s="22" t="str">
@@ -11585,7 +11514,7 @@
       <c r="F305" s="13"/>
       <c r="G305" s="21"/>
       <c r="H305" s="22" t="str">
-        <f>IF(F305="","",IF(OR(E305="Abschreibung (AfA)",E305="Vorsteuer auf Anlagevermögen"),0,ROUND(F305*G305,2)))</f>
+        <f aca="false">IF(F305="","",ROUND(F305*G305,2))</f>
         <v/>
       </c>
       <c r="I305" s="22" t="str">
@@ -11603,7 +11532,7 @@
       <c r="F306" s="13"/>
       <c r="G306" s="21"/>
       <c r="H306" s="22" t="str">
-        <f>IF(F306="","",IF(OR(E306="Abschreibung (AfA)",E306="Vorsteuer auf Anlagevermögen"),0,ROUND(F306*G306,2)))</f>
+        <f aca="false">IF(F306="","",ROUND(F306*G306,2))</f>
         <v/>
       </c>
       <c r="I306" s="22" t="str">
@@ -11621,7 +11550,7 @@
       <c r="F307" s="13"/>
       <c r="G307" s="21"/>
       <c r="H307" s="22" t="str">
-        <f>IF(F307="","",IF(OR(E307="Abschreibung (AfA)",E307="Vorsteuer auf Anlagevermögen"),0,ROUND(F307*G307,2)))</f>
+        <f aca="false">IF(F307="","",ROUND(F307*G307,2))</f>
         <v/>
       </c>
       <c r="I307" s="22" t="str">
@@ -11639,7 +11568,7 @@
       <c r="F308" s="13"/>
       <c r="G308" s="21"/>
       <c r="H308" s="22" t="str">
-        <f>IF(F308="","",IF(OR(E308="Abschreibung (AfA)",E308="Vorsteuer auf Anlagevermögen"),0,ROUND(F308*G308,2)))</f>
+        <f aca="false">IF(F308="","",ROUND(F308*G308,2))</f>
         <v/>
       </c>
       <c r="I308" s="22" t="str">
@@ -11657,7 +11586,7 @@
       <c r="F309" s="13"/>
       <c r="G309" s="21"/>
       <c r="H309" s="22" t="str">
-        <f>IF(F309="","",IF(OR(E309="Abschreibung (AfA)",E309="Vorsteuer auf Anlagevermögen"),0,ROUND(F309*G309,2)))</f>
+        <f aca="false">IF(F309="","",ROUND(F309*G309,2))</f>
         <v/>
       </c>
       <c r="I309" s="22" t="str">
@@ -11675,7 +11604,7 @@
       <c r="F310" s="13"/>
       <c r="G310" s="21"/>
       <c r="H310" s="22" t="str">
-        <f>IF(F310="","",IF(OR(E310="Abschreibung (AfA)",E310="Vorsteuer auf Anlagevermögen"),0,ROUND(F310*G310,2)))</f>
+        <f aca="false">IF(F310="","",ROUND(F310*G310,2))</f>
         <v/>
       </c>
       <c r="I310" s="22" t="str">
@@ -11693,7 +11622,7 @@
       <c r="F311" s="13"/>
       <c r="G311" s="21"/>
       <c r="H311" s="22" t="str">
-        <f>IF(F311="","",IF(OR(E311="Abschreibung (AfA)",E311="Vorsteuer auf Anlagevermögen"),0,ROUND(F311*G311,2)))</f>
+        <f aca="false">IF(F311="","",ROUND(F311*G311,2))</f>
         <v/>
       </c>
       <c r="I311" s="22" t="str">
@@ -11711,7 +11640,7 @@
       <c r="F312" s="13"/>
       <c r="G312" s="21"/>
       <c r="H312" s="22" t="str">
-        <f>IF(F312="","",IF(OR(E312="Abschreibung (AfA)",E312="Vorsteuer auf Anlagevermögen"),0,ROUND(F312*G312,2)))</f>
+        <f aca="false">IF(F312="","",ROUND(F312*G312,2))</f>
         <v/>
       </c>
       <c r="I312" s="22" t="str">
@@ -11729,7 +11658,7 @@
       <c r="F313" s="13"/>
       <c r="G313" s="21"/>
       <c r="H313" s="22" t="str">
-        <f>IF(F313="","",IF(OR(E313="Abschreibung (AfA)",E313="Vorsteuer auf Anlagevermögen"),0,ROUND(F313*G313,2)))</f>
+        <f aca="false">IF(F313="","",ROUND(F313*G313,2))</f>
         <v/>
       </c>
       <c r="I313" s="22" t="str">
@@ -11747,7 +11676,7 @@
       <c r="F314" s="13"/>
       <c r="G314" s="21"/>
       <c r="H314" s="22" t="str">
-        <f>IF(F314="","",IF(OR(E314="Abschreibung (AfA)",E314="Vorsteuer auf Anlagevermögen"),0,ROUND(F314*G314,2)))</f>
+        <f aca="false">IF(F314="","",ROUND(F314*G314,2))</f>
         <v/>
       </c>
       <c r="I314" s="22" t="str">
@@ -11765,7 +11694,7 @@
       <c r="F315" s="13"/>
       <c r="G315" s="21"/>
       <c r="H315" s="22" t="str">
-        <f>IF(F315="","",IF(OR(E315="Abschreibung (AfA)",E315="Vorsteuer auf Anlagevermögen"),0,ROUND(F315*G315,2)))</f>
+        <f aca="false">IF(F315="","",ROUND(F315*G315,2))</f>
         <v/>
       </c>
       <c r="I315" s="22" t="str">
@@ -11783,7 +11712,7 @@
       <c r="F316" s="13"/>
       <c r="G316" s="21"/>
       <c r="H316" s="22" t="str">
-        <f>IF(F316="","",IF(OR(E316="Abschreibung (AfA)",E316="Vorsteuer auf Anlagevermögen"),0,ROUND(F316*G316,2)))</f>
+        <f aca="false">IF(F316="","",ROUND(F316*G316,2))</f>
         <v/>
       </c>
       <c r="I316" s="22" t="str">
@@ -11801,7 +11730,7 @@
       <c r="F317" s="13"/>
       <c r="G317" s="21"/>
       <c r="H317" s="22" t="str">
-        <f>IF(F317="","",IF(OR(E317="Abschreibung (AfA)",E317="Vorsteuer auf Anlagevermögen"),0,ROUND(F317*G317,2)))</f>
+        <f aca="false">IF(F317="","",ROUND(F317*G317,2))</f>
         <v/>
       </c>
       <c r="I317" s="22" t="str">
@@ -11819,7 +11748,7 @@
       <c r="F318" s="13"/>
       <c r="G318" s="21"/>
       <c r="H318" s="22" t="str">
-        <f>IF(F318="","",IF(OR(E318="Abschreibung (AfA)",E318="Vorsteuer auf Anlagevermögen"),0,ROUND(F318*G318,2)))</f>
+        <f aca="false">IF(F318="","",ROUND(F318*G318,2))</f>
         <v/>
       </c>
       <c r="I318" s="22" t="str">
@@ -11837,7 +11766,7 @@
       <c r="F319" s="13"/>
       <c r="G319" s="21"/>
       <c r="H319" s="22" t="str">
-        <f>IF(F319="","",IF(OR(E319="Abschreibung (AfA)",E319="Vorsteuer auf Anlagevermögen"),0,ROUND(F319*G319,2)))</f>
+        <f aca="false">IF(F319="","",ROUND(F319*G319,2))</f>
         <v/>
       </c>
       <c r="I319" s="22" t="str">
@@ -11855,7 +11784,7 @@
       <c r="F320" s="13"/>
       <c r="G320" s="21"/>
       <c r="H320" s="22" t="str">
-        <f>IF(F320="","",IF(OR(E320="Abschreibung (AfA)",E320="Vorsteuer auf Anlagevermögen"),0,ROUND(F320*G320,2)))</f>
+        <f aca="false">IF(F320="","",ROUND(F320*G320,2))</f>
         <v/>
       </c>
       <c r="I320" s="22" t="str">
@@ -11873,7 +11802,7 @@
       <c r="F321" s="13"/>
       <c r="G321" s="21"/>
       <c r="H321" s="22" t="str">
-        <f>IF(F321="","",IF(OR(E321="Abschreibung (AfA)",E321="Vorsteuer auf Anlagevermögen"),0,ROUND(F321*G321,2)))</f>
+        <f aca="false">IF(F321="","",ROUND(F321*G321,2))</f>
         <v/>
       </c>
       <c r="I321" s="22" t="str">
@@ -11891,7 +11820,7 @@
       <c r="F322" s="13"/>
       <c r="G322" s="21"/>
       <c r="H322" s="22" t="str">
-        <f>IF(F322="","",IF(OR(E322="Abschreibung (AfA)",E322="Vorsteuer auf Anlagevermögen"),0,ROUND(F322*G322,2)))</f>
+        <f aca="false">IF(F322="","",ROUND(F322*G322,2))</f>
         <v/>
       </c>
       <c r="I322" s="22" t="str">
@@ -11909,7 +11838,7 @@
       <c r="F323" s="13"/>
       <c r="G323" s="21"/>
       <c r="H323" s="22" t="str">
-        <f>IF(F323="","",IF(OR(E323="Abschreibung (AfA)",E323="Vorsteuer auf Anlagevermögen"),0,ROUND(F323*G323,2)))</f>
+        <f aca="false">IF(F323="","",ROUND(F323*G323,2))</f>
         <v/>
       </c>
       <c r="I323" s="22" t="str">
@@ -11927,7 +11856,7 @@
       <c r="F324" s="13"/>
       <c r="G324" s="21"/>
       <c r="H324" s="22" t="str">
-        <f>IF(F324="","",IF(OR(E324="Abschreibung (AfA)",E324="Vorsteuer auf Anlagevermögen"),0,ROUND(F324*G324,2)))</f>
+        <f aca="false">IF(F324="","",ROUND(F324*G324,2))</f>
         <v/>
       </c>
       <c r="I324" s="22" t="str">
@@ -11945,7 +11874,7 @@
       <c r="F325" s="13"/>
       <c r="G325" s="21"/>
       <c r="H325" s="22" t="str">
-        <f>IF(F325="","",IF(OR(E325="Abschreibung (AfA)",E325="Vorsteuer auf Anlagevermögen"),0,ROUND(F325*G325,2)))</f>
+        <f aca="false">IF(F325="","",ROUND(F325*G325,2))</f>
         <v/>
       </c>
       <c r="I325" s="22" t="str">
@@ -11963,7 +11892,7 @@
       <c r="F326" s="13"/>
       <c r="G326" s="21"/>
       <c r="H326" s="22" t="str">
-        <f>IF(F326="","",IF(OR(E326="Abschreibung (AfA)",E326="Vorsteuer auf Anlagevermögen"),0,ROUND(F326*G326,2)))</f>
+        <f aca="false">IF(F326="","",ROUND(F326*G326,2))</f>
         <v/>
       </c>
       <c r="I326" s="22" t="str">
@@ -11981,7 +11910,7 @@
       <c r="F327" s="13"/>
       <c r="G327" s="21"/>
       <c r="H327" s="22" t="str">
-        <f>IF(F327="","",IF(OR(E327="Abschreibung (AfA)",E327="Vorsteuer auf Anlagevermögen"),0,ROUND(F327*G327,2)))</f>
+        <f aca="false">IF(F327="","",ROUND(F327*G327,2))</f>
         <v/>
       </c>
       <c r="I327" s="22" t="str">
@@ -11999,7 +11928,7 @@
       <c r="F328" s="13"/>
       <c r="G328" s="21"/>
       <c r="H328" s="22" t="str">
-        <f>IF(F328="","",IF(OR(E328="Abschreibung (AfA)",E328="Vorsteuer auf Anlagevermögen"),0,ROUND(F328*G328,2)))</f>
+        <f aca="false">IF(F328="","",ROUND(F328*G328,2))</f>
         <v/>
       </c>
       <c r="I328" s="22" t="str">
@@ -12017,7 +11946,7 @@
       <c r="F329" s="13"/>
       <c r="G329" s="21"/>
       <c r="H329" s="22" t="str">
-        <f>IF(F329="","",IF(OR(E329="Abschreibung (AfA)",E329="Vorsteuer auf Anlagevermögen"),0,ROUND(F329*G329,2)))</f>
+        <f aca="false">IF(F329="","",ROUND(F329*G329,2))</f>
         <v/>
       </c>
       <c r="I329" s="22" t="str">
@@ -12035,7 +11964,7 @@
       <c r="F330" s="13"/>
       <c r="G330" s="21"/>
       <c r="H330" s="22" t="str">
-        <f>IF(F330="","",IF(OR(E330="Abschreibung (AfA)",E330="Vorsteuer auf Anlagevermögen"),0,ROUND(F330*G330,2)))</f>
+        <f aca="false">IF(F330="","",ROUND(F330*G330,2))</f>
         <v/>
       </c>
       <c r="I330" s="22" t="str">
@@ -12053,7 +11982,7 @@
       <c r="F331" s="13"/>
       <c r="G331" s="21"/>
       <c r="H331" s="22" t="str">
-        <f>IF(F331="","",IF(OR(E331="Abschreibung (AfA)",E331="Vorsteuer auf Anlagevermögen"),0,ROUND(F331*G331,2)))</f>
+        <f aca="false">IF(F331="","",ROUND(F331*G331,2))</f>
         <v/>
       </c>
       <c r="I331" s="22" t="str">
@@ -12071,7 +12000,7 @@
       <c r="F332" s="13"/>
       <c r="G332" s="21"/>
       <c r="H332" s="22" t="str">
-        <f>IF(F332="","",IF(OR(E332="Abschreibung (AfA)",E332="Vorsteuer auf Anlagevermögen"),0,ROUND(F332*G332,2)))</f>
+        <f aca="false">IF(F332="","",ROUND(F332*G332,2))</f>
         <v/>
       </c>
       <c r="I332" s="22" t="str">
@@ -12089,7 +12018,7 @@
       <c r="F333" s="13"/>
       <c r="G333" s="21"/>
       <c r="H333" s="22" t="str">
-        <f>IF(F333="","",IF(OR(E333="Abschreibung (AfA)",E333="Vorsteuer auf Anlagevermögen"),0,ROUND(F333*G333,2)))</f>
+        <f aca="false">IF(F333="","",ROUND(F333*G333,2))</f>
         <v/>
       </c>
       <c r="I333" s="22" t="str">
@@ -12107,7 +12036,7 @@
       <c r="F334" s="13"/>
       <c r="G334" s="21"/>
       <c r="H334" s="22" t="str">
-        <f>IF(F334="","",IF(OR(E334="Abschreibung (AfA)",E334="Vorsteuer auf Anlagevermögen"),0,ROUND(F334*G334,2)))</f>
+        <f aca="false">IF(F334="","",ROUND(F334*G334,2))</f>
         <v/>
       </c>
       <c r="I334" s="22" t="str">
@@ -12125,7 +12054,7 @@
       <c r="F335" s="13"/>
       <c r="G335" s="21"/>
       <c r="H335" s="22" t="str">
-        <f>IF(F335="","",IF(OR(E335="Abschreibung (AfA)",E335="Vorsteuer auf Anlagevermögen"),0,ROUND(F335*G335,2)))</f>
+        <f aca="false">IF(F335="","",ROUND(F335*G335,2))</f>
         <v/>
       </c>
       <c r="I335" s="22" t="str">
@@ -12143,7 +12072,7 @@
       <c r="F336" s="13"/>
       <c r="G336" s="21"/>
       <c r="H336" s="22" t="str">
-        <f>IF(F336="","",IF(OR(E336="Abschreibung (AfA)",E336="Vorsteuer auf Anlagevermögen"),0,ROUND(F336*G336,2)))</f>
+        <f aca="false">IF(F336="","",ROUND(F336*G336,2))</f>
         <v/>
       </c>
       <c r="I336" s="22" t="str">
@@ -12161,7 +12090,7 @@
       <c r="F337" s="13"/>
       <c r="G337" s="21"/>
       <c r="H337" s="22" t="str">
-        <f>IF(F337="","",IF(OR(E337="Abschreibung (AfA)",E337="Vorsteuer auf Anlagevermögen"),0,ROUND(F337*G337,2)))</f>
+        <f aca="false">IF(F337="","",ROUND(F337*G337,2))</f>
         <v/>
       </c>
       <c r="I337" s="22" t="str">
@@ -12179,7 +12108,7 @@
       <c r="F338" s="13"/>
       <c r="G338" s="21"/>
       <c r="H338" s="22" t="str">
-        <f>IF(F338="","",IF(OR(E338="Abschreibung (AfA)",E338="Vorsteuer auf Anlagevermögen"),0,ROUND(F338*G338,2)))</f>
+        <f aca="false">IF(F338="","",ROUND(F338*G338,2))</f>
         <v/>
       </c>
       <c r="I338" s="22" t="str">
@@ -12197,7 +12126,7 @@
       <c r="F339" s="13"/>
       <c r="G339" s="21"/>
       <c r="H339" s="22" t="str">
-        <f>IF(F339="","",IF(OR(E339="Abschreibung (AfA)",E339="Vorsteuer auf Anlagevermögen"),0,ROUND(F339*G339,2)))</f>
+        <f aca="false">IF(F339="","",ROUND(F339*G339,2))</f>
         <v/>
       </c>
       <c r="I339" s="22" t="str">
@@ -12215,7 +12144,7 @@
       <c r="F340" s="13"/>
       <c r="G340" s="21"/>
       <c r="H340" s="22" t="str">
-        <f>IF(F340="","",IF(OR(E340="Abschreibung (AfA)",E340="Vorsteuer auf Anlagevermögen"),0,ROUND(F340*G340,2)))</f>
+        <f aca="false">IF(F340="","",ROUND(F340*G340,2))</f>
         <v/>
       </c>
       <c r="I340" s="22" t="str">
@@ -12233,7 +12162,7 @@
       <c r="F341" s="13"/>
       <c r="G341" s="21"/>
       <c r="H341" s="22" t="str">
-        <f>IF(F341="","",IF(OR(E341="Abschreibung (AfA)",E341="Vorsteuer auf Anlagevermögen"),0,ROUND(F341*G341,2)))</f>
+        <f aca="false">IF(F341="","",ROUND(F341*G341,2))</f>
         <v/>
       </c>
       <c r="I341" s="22" t="str">
@@ -12251,7 +12180,7 @@
       <c r="F342" s="13"/>
       <c r="G342" s="21"/>
       <c r="H342" s="22" t="str">
-        <f>IF(F342="","",IF(OR(E342="Abschreibung (AfA)",E342="Vorsteuer auf Anlagevermögen"),0,ROUND(F342*G342,2)))</f>
+        <f aca="false">IF(F342="","",ROUND(F342*G342,2))</f>
         <v/>
       </c>
       <c r="I342" s="22" t="str">
@@ -12269,7 +12198,7 @@
       <c r="F343" s="13"/>
       <c r="G343" s="21"/>
       <c r="H343" s="22" t="str">
-        <f>IF(F343="","",IF(OR(E343="Abschreibung (AfA)",E343="Vorsteuer auf Anlagevermögen"),0,ROUND(F343*G343,2)))</f>
+        <f aca="false">IF(F343="","",ROUND(F343*G343,2))</f>
         <v/>
       </c>
       <c r="I343" s="22" t="str">
@@ -12287,7 +12216,7 @@
       <c r="F344" s="13"/>
       <c r="G344" s="21"/>
       <c r="H344" s="22" t="str">
-        <f>IF(F344="","",IF(OR(E344="Abschreibung (AfA)",E344="Vorsteuer auf Anlagevermögen"),0,ROUND(F344*G344,2)))</f>
+        <f aca="false">IF(F344="","",ROUND(F344*G344,2))</f>
         <v/>
       </c>
       <c r="I344" s="22" t="str">
@@ -12305,7 +12234,7 @@
       <c r="F345" s="13"/>
       <c r="G345" s="21"/>
       <c r="H345" s="22" t="str">
-        <f>IF(F345="","",IF(OR(E345="Abschreibung (AfA)",E345="Vorsteuer auf Anlagevermögen"),0,ROUND(F345*G345,2)))</f>
+        <f aca="false">IF(F345="","",ROUND(F345*G345,2))</f>
         <v/>
       </c>
       <c r="I345" s="22" t="str">
@@ -12323,7 +12252,7 @@
       <c r="F346" s="13"/>
       <c r="G346" s="21"/>
       <c r="H346" s="22" t="str">
-        <f>IF(F346="","",IF(OR(E346="Abschreibung (AfA)",E346="Vorsteuer auf Anlagevermögen"),0,ROUND(F346*G346,2)))</f>
+        <f aca="false">IF(F346="","",ROUND(F346*G346,2))</f>
         <v/>
       </c>
       <c r="I346" s="22" t="str">
@@ -12341,7 +12270,7 @@
       <c r="F347" s="13"/>
       <c r="G347" s="21"/>
       <c r="H347" s="22" t="str">
-        <f>IF(F347="","",IF(OR(E347="Abschreibung (AfA)",E347="Vorsteuer auf Anlagevermögen"),0,ROUND(F347*G347,2)))</f>
+        <f aca="false">IF(F347="","",ROUND(F347*G347,2))</f>
         <v/>
       </c>
       <c r="I347" s="22" t="str">
@@ -12359,7 +12288,7 @@
       <c r="F348" s="13"/>
       <c r="G348" s="21"/>
       <c r="H348" s="22" t="str">
-        <f>IF(F348="","",IF(OR(E348="Abschreibung (AfA)",E348="Vorsteuer auf Anlagevermögen"),0,ROUND(F348*G348,2)))</f>
+        <f aca="false">IF(F348="","",ROUND(F348*G348,2))</f>
         <v/>
       </c>
       <c r="I348" s="22" t="str">
@@ -12377,7 +12306,7 @@
       <c r="F349" s="13"/>
       <c r="G349" s="21"/>
       <c r="H349" s="22" t="str">
-        <f>IF(F349="","",IF(OR(E349="Abschreibung (AfA)",E349="Vorsteuer auf Anlagevermögen"),0,ROUND(F349*G349,2)))</f>
+        <f aca="false">IF(F349="","",ROUND(F349*G349,2))</f>
         <v/>
       </c>
       <c r="I349" s="22" t="str">
@@ -12395,7 +12324,7 @@
       <c r="F350" s="13"/>
       <c r="G350" s="21"/>
       <c r="H350" s="22" t="str">
-        <f>IF(F350="","",IF(OR(E350="Abschreibung (AfA)",E350="Vorsteuer auf Anlagevermögen"),0,ROUND(F350*G350,2)))</f>
+        <f aca="false">IF(F350="","",ROUND(F350*G350,2))</f>
         <v/>
       </c>
       <c r="I350" s="22" t="str">
@@ -12413,7 +12342,7 @@
       <c r="F351" s="13"/>
       <c r="G351" s="21"/>
       <c r="H351" s="22" t="str">
-        <f>IF(F351="","",IF(OR(E351="Abschreibung (AfA)",E351="Vorsteuer auf Anlagevermögen"),0,ROUND(F351*G351,2)))</f>
+        <f aca="false">IF(F351="","",ROUND(F351*G351,2))</f>
         <v/>
       </c>
       <c r="I351" s="22" t="str">
@@ -12431,7 +12360,7 @@
       <c r="F352" s="13"/>
       <c r="G352" s="21"/>
       <c r="H352" s="22" t="str">
-        <f>IF(F352="","",IF(OR(E352="Abschreibung (AfA)",E352="Vorsteuer auf Anlagevermögen"),0,ROUND(F352*G352,2)))</f>
+        <f aca="false">IF(F352="","",ROUND(F352*G352,2))</f>
         <v/>
       </c>
       <c r="I352" s="22" t="str">
@@ -12449,7 +12378,7 @@
       <c r="F353" s="13"/>
       <c r="G353" s="21"/>
       <c r="H353" s="22" t="str">
-        <f>IF(F353="","",IF(OR(E353="Abschreibung (AfA)",E353="Vorsteuer auf Anlagevermögen"),0,ROUND(F353*G353,2)))</f>
+        <f aca="false">IF(F353="","",ROUND(F353*G353,2))</f>
         <v/>
       </c>
       <c r="I353" s="22" t="str">
@@ -12467,7 +12396,7 @@
       <c r="F354" s="13"/>
       <c r="G354" s="21"/>
       <c r="H354" s="22" t="str">
-        <f>IF(F354="","",IF(OR(E354="Abschreibung (AfA)",E354="Vorsteuer auf Anlagevermögen"),0,ROUND(F354*G354,2)))</f>
+        <f aca="false">IF(F354="","",ROUND(F354*G354,2))</f>
         <v/>
       </c>
       <c r="I354" s="22" t="str">
@@ -12485,7 +12414,7 @@
       <c r="F355" s="13"/>
       <c r="G355" s="21"/>
       <c r="H355" s="22" t="str">
-        <f>IF(F355="","",IF(OR(E355="Abschreibung (AfA)",E355="Vorsteuer auf Anlagevermögen"),0,ROUND(F355*G355,2)))</f>
+        <f aca="false">IF(F355="","",ROUND(F355*G355,2))</f>
         <v/>
       </c>
       <c r="I355" s="22" t="str">
@@ -12503,7 +12432,7 @@
       <c r="F356" s="13"/>
       <c r="G356" s="21"/>
       <c r="H356" s="22" t="str">
-        <f>IF(F356="","",IF(OR(E356="Abschreibung (AfA)",E356="Vorsteuer auf Anlagevermögen"),0,ROUND(F356*G356,2)))</f>
+        <f aca="false">IF(F356="","",ROUND(F356*G356,2))</f>
         <v/>
       </c>
       <c r="I356" s="22" t="str">
@@ -12521,7 +12450,7 @@
       <c r="F357" s="13"/>
       <c r="G357" s="21"/>
       <c r="H357" s="22" t="str">
-        <f>IF(F357="","",IF(OR(E357="Abschreibung (AfA)",E357="Vorsteuer auf Anlagevermögen"),0,ROUND(F357*G357,2)))</f>
+        <f aca="false">IF(F357="","",ROUND(F357*G357,2))</f>
         <v/>
       </c>
       <c r="I357" s="22" t="str">
@@ -12539,7 +12468,7 @@
       <c r="F358" s="13"/>
       <c r="G358" s="21"/>
       <c r="H358" s="22" t="str">
-        <f>IF(F358="","",IF(OR(E358="Abschreibung (AfA)",E358="Vorsteuer auf Anlagevermögen"),0,ROUND(F358*G358,2)))</f>
+        <f aca="false">IF(F358="","",ROUND(F358*G358,2))</f>
         <v/>
       </c>
       <c r="I358" s="22" t="str">
@@ -12557,7 +12486,7 @@
       <c r="F359" s="13"/>
       <c r="G359" s="21"/>
       <c r="H359" s="22" t="str">
-        <f>IF(F359="","",IF(OR(E359="Abschreibung (AfA)",E359="Vorsteuer auf Anlagevermögen"),0,ROUND(F359*G359,2)))</f>
+        <f aca="false">IF(F359="","",ROUND(F359*G359,2))</f>
         <v/>
       </c>
       <c r="I359" s="22" t="str">
@@ -12575,7 +12504,7 @@
       <c r="F360" s="13"/>
       <c r="G360" s="21"/>
       <c r="H360" s="22" t="str">
-        <f>IF(F360="","",IF(OR(E360="Abschreibung (AfA)",E360="Vorsteuer auf Anlagevermögen"),0,ROUND(F360*G360,2)))</f>
+        <f aca="false">IF(F360="","",ROUND(F360*G360,2))</f>
         <v/>
       </c>
       <c r="I360" s="22" t="str">
@@ -12593,7 +12522,7 @@
       <c r="F361" s="13"/>
       <c r="G361" s="21"/>
       <c r="H361" s="22" t="str">
-        <f>IF(F361="","",IF(OR(E361="Abschreibung (AfA)",E361="Vorsteuer auf Anlagevermögen"),0,ROUND(F361*G361,2)))</f>
+        <f aca="false">IF(F361="","",ROUND(F361*G361,2))</f>
         <v/>
       </c>
       <c r="I361" s="22" t="str">
@@ -12611,7 +12540,7 @@
       <c r="F362" s="13"/>
       <c r="G362" s="21"/>
       <c r="H362" s="22" t="str">
-        <f>IF(F362="","",IF(OR(E362="Abschreibung (AfA)",E362="Vorsteuer auf Anlagevermögen"),0,ROUND(F362*G362,2)))</f>
+        <f aca="false">IF(F362="","",ROUND(F362*G362,2))</f>
         <v/>
       </c>
       <c r="I362" s="22" t="str">
@@ -12629,7 +12558,7 @@
       <c r="F363" s="13"/>
       <c r="G363" s="21"/>
       <c r="H363" s="22" t="str">
-        <f>IF(F363="","",IF(OR(E363="Abschreibung (AfA)",E363="Vorsteuer auf Anlagevermögen"),0,ROUND(F363*G363,2)))</f>
+        <f aca="false">IF(F363="","",ROUND(F363*G363,2))</f>
         <v/>
       </c>
       <c r="I363" s="22" t="str">
@@ -12647,7 +12576,7 @@
       <c r="F364" s="13"/>
       <c r="G364" s="21"/>
       <c r="H364" s="22" t="str">
-        <f>IF(F364="","",IF(OR(E364="Abschreibung (AfA)",E364="Vorsteuer auf Anlagevermögen"),0,ROUND(F364*G364,2)))</f>
+        <f aca="false">IF(F364="","",ROUND(F364*G364,2))</f>
         <v/>
       </c>
       <c r="I364" s="22" t="str">
@@ -12665,7 +12594,7 @@
       <c r="F365" s="13"/>
       <c r="G365" s="21"/>
       <c r="H365" s="22" t="str">
-        <f>IF(F365="","",IF(OR(E365="Abschreibung (AfA)",E365="Vorsteuer auf Anlagevermögen"),0,ROUND(F365*G365,2)))</f>
+        <f aca="false">IF(F365="","",ROUND(F365*G365,2))</f>
         <v/>
       </c>
       <c r="I365" s="22" t="str">
@@ -12683,7 +12612,7 @@
       <c r="F366" s="13"/>
       <c r="G366" s="21"/>
       <c r="H366" s="22" t="str">
-        <f>IF(F366="","",IF(OR(E366="Abschreibung (AfA)",E366="Vorsteuer auf Anlagevermögen"),0,ROUND(F366*G366,2)))</f>
+        <f aca="false">IF(F366="","",ROUND(F366*G366,2))</f>
         <v/>
       </c>
       <c r="I366" s="22" t="str">
@@ -12701,7 +12630,7 @@
       <c r="F367" s="13"/>
       <c r="G367" s="21"/>
       <c r="H367" s="22" t="str">
-        <f>IF(F367="","",IF(OR(E367="Abschreibung (AfA)",E367="Vorsteuer auf Anlagevermögen"),0,ROUND(F367*G367,2)))</f>
+        <f aca="false">IF(F367="","",ROUND(F367*G367,2))</f>
         <v/>
       </c>
       <c r="I367" s="22" t="str">
@@ -12719,7 +12648,7 @@
       <c r="F368" s="13"/>
       <c r="G368" s="21"/>
       <c r="H368" s="22" t="str">
-        <f>IF(F368="","",IF(OR(E368="Abschreibung (AfA)",E368="Vorsteuer auf Anlagevermögen"),0,ROUND(F368*G368,2)))</f>
+        <f aca="false">IF(F368="","",ROUND(F368*G368,2))</f>
         <v/>
       </c>
       <c r="I368" s="22" t="str">
@@ -12737,7 +12666,7 @@
       <c r="F369" s="13"/>
       <c r="G369" s="21"/>
       <c r="H369" s="22" t="str">
-        <f>IF(F369="","",IF(OR(E369="Abschreibung (AfA)",E369="Vorsteuer auf Anlagevermögen"),0,ROUND(F369*G369,2)))</f>
+        <f aca="false">IF(F369="","",ROUND(F369*G369,2))</f>
         <v/>
       </c>
       <c r="I369" s="22" t="str">
@@ -12755,7 +12684,7 @@
       <c r="F370" s="13"/>
       <c r="G370" s="21"/>
       <c r="H370" s="22" t="str">
-        <f>IF(F370="","",IF(OR(E370="Abschreibung (AfA)",E370="Vorsteuer auf Anlagevermögen"),0,ROUND(F370*G370,2)))</f>
+        <f aca="false">IF(F370="","",ROUND(F370*G370,2))</f>
         <v/>
       </c>
       <c r="I370" s="22" t="str">
@@ -12773,7 +12702,7 @@
       <c r="F371" s="13"/>
       <c r="G371" s="21"/>
       <c r="H371" s="22" t="str">
-        <f>IF(F371="","",IF(OR(E371="Abschreibung (AfA)",E371="Vorsteuer auf Anlagevermögen"),0,ROUND(F371*G371,2)))</f>
+        <f aca="false">IF(F371="","",ROUND(F371*G371,2))</f>
         <v/>
       </c>
       <c r="I371" s="22" t="str">
@@ -12791,7 +12720,7 @@
       <c r="F372" s="13"/>
       <c r="G372" s="21"/>
       <c r="H372" s="22" t="str">
-        <f>IF(F372="","",IF(OR(E372="Abschreibung (AfA)",E372="Vorsteuer auf Anlagevermögen"),0,ROUND(F372*G372,2)))</f>
+        <f aca="false">IF(F372="","",ROUND(F372*G372,2))</f>
         <v/>
       </c>
       <c r="I372" s="22" t="str">
@@ -12809,7 +12738,7 @@
       <c r="F373" s="13"/>
       <c r="G373" s="21"/>
       <c r="H373" s="22" t="str">
-        <f>IF(F373="","",IF(OR(E373="Abschreibung (AfA)",E373="Vorsteuer auf Anlagevermögen"),0,ROUND(F373*G373,2)))</f>
+        <f aca="false">IF(F373="","",ROUND(F373*G373,2))</f>
         <v/>
       </c>
       <c r="I373" s="22" t="str">
@@ -12827,7 +12756,7 @@
       <c r="F374" s="13"/>
       <c r="G374" s="21"/>
       <c r="H374" s="22" t="str">
-        <f>IF(F374="","",IF(OR(E374="Abschreibung (AfA)",E374="Vorsteuer auf Anlagevermögen"),0,ROUND(F374*G374,2)))</f>
+        <f aca="false">IF(F374="","",ROUND(F374*G374,2))</f>
         <v/>
       </c>
       <c r="I374" s="22" t="str">
@@ -12845,7 +12774,7 @@
       <c r="F375" s="13"/>
       <c r="G375" s="21"/>
       <c r="H375" s="22" t="str">
-        <f>IF(F375="","",IF(OR(E375="Abschreibung (AfA)",E375="Vorsteuer auf Anlagevermögen"),0,ROUND(F375*G375,2)))</f>
+        <f aca="false">IF(F375="","",ROUND(F375*G375,2))</f>
         <v/>
       </c>
       <c r="I375" s="22" t="str">
@@ -12863,7 +12792,7 @@
       <c r="F376" s="13"/>
       <c r="G376" s="21"/>
       <c r="H376" s="22" t="str">
-        <f>IF(F376="","",IF(OR(E376="Abschreibung (AfA)",E376="Vorsteuer auf Anlagevermögen"),0,ROUND(F376*G376,2)))</f>
+        <f aca="false">IF(F376="","",ROUND(F376*G376,2))</f>
         <v/>
       </c>
       <c r="I376" s="22" t="str">
@@ -12881,7 +12810,7 @@
       <c r="F377" s="13"/>
       <c r="G377" s="21"/>
       <c r="H377" s="22" t="str">
-        <f>IF(F377="","",IF(OR(E377="Abschreibung (AfA)",E377="Vorsteuer auf Anlagevermögen"),0,ROUND(F377*G377,2)))</f>
+        <f aca="false">IF(F377="","",ROUND(F377*G377,2))</f>
         <v/>
       </c>
       <c r="I377" s="22" t="str">
@@ -12899,7 +12828,7 @@
       <c r="F378" s="13"/>
       <c r="G378" s="21"/>
       <c r="H378" s="22" t="str">
-        <f>IF(F378="","",IF(OR(E378="Abschreibung (AfA)",E378="Vorsteuer auf Anlagevermögen"),0,ROUND(F378*G378,2)))</f>
+        <f aca="false">IF(F378="","",ROUND(F378*G378,2))</f>
         <v/>
       </c>
       <c r="I378" s="22" t="str">
@@ -12917,7 +12846,7 @@
       <c r="F379" s="13"/>
       <c r="G379" s="21"/>
       <c r="H379" s="22" t="str">
-        <f>IF(F379="","",IF(OR(E379="Abschreibung (AfA)",E379="Vorsteuer auf Anlagevermögen"),0,ROUND(F379*G379,2)))</f>
+        <f aca="false">IF(F379="","",ROUND(F379*G379,2))</f>
         <v/>
       </c>
       <c r="I379" s="22" t="str">
@@ -12935,7 +12864,7 @@
       <c r="F380" s="13"/>
       <c r="G380" s="21"/>
       <c r="H380" s="22" t="str">
-        <f>IF(F380="","",IF(OR(E380="Abschreibung (AfA)",E380="Vorsteuer auf Anlagevermögen"),0,ROUND(F380*G380,2)))</f>
+        <f aca="false">IF(F380="","",ROUND(F380*G380,2))</f>
         <v/>
       </c>
       <c r="I380" s="22" t="str">
@@ -12953,7 +12882,7 @@
       <c r="F381" s="13"/>
       <c r="G381" s="21"/>
       <c r="H381" s="22" t="str">
-        <f>IF(F381="","",IF(OR(E381="Abschreibung (AfA)",E381="Vorsteuer auf Anlagevermögen"),0,ROUND(F381*G381,2)))</f>
+        <f aca="false">IF(F381="","",ROUND(F381*G381,2))</f>
         <v/>
       </c>
       <c r="I381" s="22" t="str">
@@ -12971,7 +12900,7 @@
       <c r="F382" s="13"/>
       <c r="G382" s="21"/>
       <c r="H382" s="22" t="str">
-        <f>IF(F382="","",IF(OR(E382="Abschreibung (AfA)",E382="Vorsteuer auf Anlagevermögen"),0,ROUND(F382*G382,2)))</f>
+        <f aca="false">IF(F382="","",ROUND(F382*G382,2))</f>
         <v/>
       </c>
       <c r="I382" s="22" t="str">
@@ -12989,7 +12918,7 @@
       <c r="F383" s="13"/>
       <c r="G383" s="21"/>
       <c r="H383" s="22" t="str">
-        <f>IF(F383="","",IF(OR(E383="Abschreibung (AfA)",E383="Vorsteuer auf Anlagevermögen"),0,ROUND(F383*G383,2)))</f>
+        <f aca="false">IF(F383="","",ROUND(F383*G383,2))</f>
         <v/>
       </c>
       <c r="I383" s="22" t="str">
@@ -13007,7 +12936,7 @@
       <c r="F384" s="13"/>
       <c r="G384" s="21"/>
       <c r="H384" s="22" t="str">
-        <f>IF(F384="","",IF(OR(E384="Abschreibung (AfA)",E384="Vorsteuer auf Anlagevermögen"),0,ROUND(F384*G384,2)))</f>
+        <f aca="false">IF(F384="","",ROUND(F384*G384,2))</f>
         <v/>
       </c>
       <c r="I384" s="22" t="str">
@@ -13025,7 +12954,7 @@
       <c r="F385" s="13"/>
       <c r="G385" s="21"/>
       <c r="H385" s="22" t="str">
-        <f>IF(F385="","",IF(OR(E385="Abschreibung (AfA)",E385="Vorsteuer auf Anlagevermögen"),0,ROUND(F385*G385,2)))</f>
+        <f aca="false">IF(F385="","",ROUND(F385*G385,2))</f>
         <v/>
       </c>
       <c r="I385" s="22" t="str">
@@ -13043,7 +12972,7 @@
       <c r="F386" s="13"/>
       <c r="G386" s="21"/>
       <c r="H386" s="22" t="str">
-        <f>IF(F386="","",IF(OR(E386="Abschreibung (AfA)",E386="Vorsteuer auf Anlagevermögen"),0,ROUND(F386*G386,2)))</f>
+        <f aca="false">IF(F386="","",ROUND(F386*G386,2))</f>
         <v/>
       </c>
       <c r="I386" s="22" t="str">
@@ -13061,7 +12990,7 @@
       <c r="F387" s="13"/>
       <c r="G387" s="21"/>
       <c r="H387" s="22" t="str">
-        <f>IF(F387="","",IF(OR(E387="Abschreibung (AfA)",E387="Vorsteuer auf Anlagevermögen"),0,ROUND(F387*G387,2)))</f>
+        <f aca="false">IF(F387="","",ROUND(F387*G387,2))</f>
         <v/>
       </c>
       <c r="I387" s="22" t="str">
@@ -13079,7 +13008,7 @@
       <c r="F388" s="13"/>
       <c r="G388" s="21"/>
       <c r="H388" s="22" t="str">
-        <f>IF(F388="","",IF(OR(E388="Abschreibung (AfA)",E388="Vorsteuer auf Anlagevermögen"),0,ROUND(F388*G388,2)))</f>
+        <f aca="false">IF(F388="","",ROUND(F388*G388,2))</f>
         <v/>
       </c>
       <c r="I388" s="22" t="str">
@@ -13097,7 +13026,7 @@
       <c r="F389" s="13"/>
       <c r="G389" s="21"/>
       <c r="H389" s="22" t="str">
-        <f>IF(F389="","",IF(OR(E389="Abschreibung (AfA)",E389="Vorsteuer auf Anlagevermögen"),0,ROUND(F389*G389,2)))</f>
+        <f aca="false">IF(F389="","",ROUND(F389*G389,2))</f>
         <v/>
       </c>
       <c r="I389" s="22" t="str">
@@ -13115,7 +13044,7 @@
       <c r="F390" s="13"/>
       <c r="G390" s="21"/>
       <c r="H390" s="22" t="str">
-        <f>IF(F390="","",IF(OR(E390="Abschreibung (AfA)",E390="Vorsteuer auf Anlagevermögen"),0,ROUND(F390*G390,2)))</f>
+        <f aca="false">IF(F390="","",ROUND(F390*G390,2))</f>
         <v/>
       </c>
       <c r="I390" s="22" t="str">
@@ -13133,7 +13062,7 @@
       <c r="F391" s="13"/>
       <c r="G391" s="21"/>
       <c r="H391" s="22" t="str">
-        <f>IF(F391="","",IF(OR(E391="Abschreibung (AfA)",E391="Vorsteuer auf Anlagevermögen"),0,ROUND(F391*G391,2)))</f>
+        <f aca="false">IF(F391="","",ROUND(F391*G391,2))</f>
         <v/>
       </c>
       <c r="I391" s="22" t="str">
@@ -13151,7 +13080,7 @@
       <c r="F392" s="13"/>
       <c r="G392" s="21"/>
       <c r="H392" s="22" t="str">
-        <f>IF(F392="","",IF(OR(E392="Abschreibung (AfA)",E392="Vorsteuer auf Anlagevermögen"),0,ROUND(F392*G392,2)))</f>
+        <f aca="false">IF(F392="","",ROUND(F392*G392,2))</f>
         <v/>
       </c>
       <c r="I392" s="22" t="str">
@@ -13169,7 +13098,7 @@
       <c r="F393" s="13"/>
       <c r="G393" s="21"/>
       <c r="H393" s="22" t="str">
-        <f>IF(F393="","",IF(OR(E393="Abschreibung (AfA)",E393="Vorsteuer auf Anlagevermögen"),0,ROUND(F393*G393,2)))</f>
+        <f aca="false">IF(F393="","",ROUND(F393*G393,2))</f>
         <v/>
       </c>
       <c r="I393" s="22" t="str">
@@ -13187,7 +13116,7 @@
       <c r="F394" s="13"/>
       <c r="G394" s="21"/>
       <c r="H394" s="22" t="str">
-        <f>IF(F394="","",IF(OR(E394="Abschreibung (AfA)",E394="Vorsteuer auf Anlagevermögen"),0,ROUND(F394*G394,2)))</f>
+        <f aca="false">IF(F394="","",ROUND(F394*G394,2))</f>
         <v/>
       </c>
       <c r="I394" s="22" t="str">
@@ -13205,7 +13134,7 @@
       <c r="F395" s="13"/>
       <c r="G395" s="21"/>
       <c r="H395" s="22" t="str">
-        <f>IF(F395="","",IF(OR(E395="Abschreibung (AfA)",E395="Vorsteuer auf Anlagevermögen"),0,ROUND(F395*G395,2)))</f>
+        <f aca="false">IF(F395="","",ROUND(F395*G395,2))</f>
         <v/>
       </c>
       <c r="I395" s="22" t="str">
@@ -13223,7 +13152,7 @@
       <c r="F396" s="13"/>
       <c r="G396" s="21"/>
       <c r="H396" s="22" t="str">
-        <f>IF(F396="","",IF(OR(E396="Abschreibung (AfA)",E396="Vorsteuer auf Anlagevermögen"),0,ROUND(F396*G396,2)))</f>
+        <f aca="false">IF(F396="","",ROUND(F396*G396,2))</f>
         <v/>
       </c>
       <c r="I396" s="22" t="str">
@@ -13241,7 +13170,7 @@
       <c r="F397" s="13"/>
       <c r="G397" s="21"/>
       <c r="H397" s="22" t="str">
-        <f>IF(F397="","",IF(OR(E397="Abschreibung (AfA)",E397="Vorsteuer auf Anlagevermögen"),0,ROUND(F397*G397,2)))</f>
+        <f aca="false">IF(F397="","",ROUND(F397*G397,2))</f>
         <v/>
       </c>
       <c r="I397" s="22" t="str">
@@ -13259,7 +13188,7 @@
       <c r="F398" s="13"/>
       <c r="G398" s="21"/>
       <c r="H398" s="22" t="str">
-        <f>IF(F398="","",IF(OR(E398="Abschreibung (AfA)",E398="Vorsteuer auf Anlagevermögen"),0,ROUND(F398*G398,2)))</f>
+        <f aca="false">IF(F398="","",ROUND(F398*G398,2))</f>
         <v/>
       </c>
       <c r="I398" s="22" t="str">
@@ -13277,7 +13206,7 @@
       <c r="F399" s="13"/>
       <c r="G399" s="21"/>
       <c r="H399" s="22" t="str">
-        <f>IF(F399="","",IF(OR(E399="Abschreibung (AfA)",E399="Vorsteuer auf Anlagevermögen"),0,ROUND(F399*G399,2)))</f>
+        <f aca="false">IF(F399="","",ROUND(F399*G399,2))</f>
         <v/>
       </c>
       <c r="I399" s="22" t="str">
@@ -13295,7 +13224,7 @@
       <c r="F400" s="13"/>
       <c r="G400" s="21"/>
       <c r="H400" s="22" t="str">
-        <f>IF(F400="","",IF(OR(E400="Abschreibung (AfA)",E400="Vorsteuer auf Anlagevermögen"),0,ROUND(F400*G400,2)))</f>
+        <f aca="false">IF(F400="","",ROUND(F400*G400,2))</f>
         <v/>
       </c>
       <c r="I400" s="22" t="str">
@@ -13313,7 +13242,7 @@
       <c r="F401" s="13"/>
       <c r="G401" s="21"/>
       <c r="H401" s="22" t="str">
-        <f>IF(F401="","",IF(OR(E401="Abschreibung (AfA)",E401="Vorsteuer auf Anlagevermögen"),0,ROUND(F401*G401,2)))</f>
+        <f aca="false">IF(F401="","",ROUND(F401*G401,2))</f>
         <v/>
       </c>
       <c r="I401" s="22" t="str">
@@ -13331,7 +13260,7 @@
       <c r="F402" s="13"/>
       <c r="G402" s="21"/>
       <c r="H402" s="22" t="str">
-        <f>IF(F402="","",IF(OR(E402="Abschreibung (AfA)",E402="Vorsteuer auf Anlagevermögen"),0,ROUND(F402*G402,2)))</f>
+        <f aca="false">IF(F402="","",ROUND(F402*G402,2))</f>
         <v/>
       </c>
       <c r="I402" s="22" t="str">
@@ -13349,7 +13278,7 @@
       <c r="F403" s="13"/>
       <c r="G403" s="21"/>
       <c r="H403" s="22" t="str">
-        <f>IF(F403="","",IF(OR(E403="Abschreibung (AfA)",E403="Vorsteuer auf Anlagevermögen"),0,ROUND(F403*G403,2)))</f>
+        <f aca="false">IF(F403="","",ROUND(F403*G403,2))</f>
         <v/>
       </c>
       <c r="I403" s="22" t="str">
@@ -13367,7 +13296,7 @@
       <c r="F404" s="13"/>
       <c r="G404" s="21"/>
       <c r="H404" s="22" t="str">
-        <f>IF(F404="","",IF(OR(E404="Abschreibung (AfA)",E404="Vorsteuer auf Anlagevermögen"),0,ROUND(F404*G404,2)))</f>
+        <f aca="false">IF(F404="","",ROUND(F404*G404,2))</f>
         <v/>
       </c>
       <c r="I404" s="22" t="str">
@@ -13385,7 +13314,7 @@
       <c r="F405" s="13"/>
       <c r="G405" s="21"/>
       <c r="H405" s="22" t="str">
-        <f>IF(F405="","",IF(OR(E405="Abschreibung (AfA)",E405="Vorsteuer auf Anlagevermögen"),0,ROUND(F405*G405,2)))</f>
+        <f aca="false">IF(F405="","",ROUND(F405*G405,2))</f>
         <v/>
       </c>
       <c r="I405" s="22" t="str">
@@ -13403,7 +13332,7 @@
       <c r="F406" s="13"/>
       <c r="G406" s="21"/>
       <c r="H406" s="22" t="str">
-        <f>IF(F406="","",IF(OR(E406="Abschreibung (AfA)",E406="Vorsteuer auf Anlagevermögen"),0,ROUND(F406*G406,2)))</f>
+        <f aca="false">IF(F406="","",ROUND(F406*G406,2))</f>
         <v/>
       </c>
       <c r="I406" s="22" t="str">
@@ -13421,7 +13350,7 @@
       <c r="F407" s="13"/>
       <c r="G407" s="21"/>
       <c r="H407" s="22" t="str">
-        <f>IF(F407="","",IF(OR(E407="Abschreibung (AfA)",E407="Vorsteuer auf Anlagevermögen"),0,ROUND(F407*G407,2)))</f>
+        <f aca="false">IF(F407="","",ROUND(F407*G407,2))</f>
         <v/>
       </c>
       <c r="I407" s="22" t="str">
@@ -13439,7 +13368,7 @@
       <c r="F408" s="13"/>
       <c r="G408" s="21"/>
       <c r="H408" s="22" t="str">
-        <f>IF(F408="","",IF(OR(E408="Abschreibung (AfA)",E408="Vorsteuer auf Anlagevermögen"),0,ROUND(F408*G408,2)))</f>
+        <f aca="false">IF(F408="","",ROUND(F408*G408,2))</f>
         <v/>
       </c>
       <c r="I408" s="22" t="str">
@@ -13457,7 +13386,7 @@
       <c r="F409" s="13"/>
       <c r="G409" s="21"/>
       <c r="H409" s="22" t="str">
-        <f>IF(F409="","",IF(OR(E409="Abschreibung (AfA)",E409="Vorsteuer auf Anlagevermögen"),0,ROUND(F409*G409,2)))</f>
+        <f aca="false">IF(F409="","",ROUND(F409*G409,2))</f>
         <v/>
       </c>
       <c r="I409" s="22" t="str">
@@ -13475,7 +13404,7 @@
       <c r="F410" s="13"/>
       <c r="G410" s="21"/>
       <c r="H410" s="22" t="str">
-        <f>IF(F410="","",IF(OR(E410="Abschreibung (AfA)",E410="Vorsteuer auf Anlagevermögen"),0,ROUND(F410*G410,2)))</f>
+        <f aca="false">IF(F410="","",ROUND(F410*G410,2))</f>
         <v/>
       </c>
       <c r="I410" s="22" t="str">
@@ -13493,7 +13422,7 @@
       <c r="F411" s="13"/>
       <c r="G411" s="21"/>
       <c r="H411" s="22" t="str">
-        <f>IF(F411="","",IF(OR(E411="Abschreibung (AfA)",E411="Vorsteuer auf Anlagevermögen"),0,ROUND(F411*G411,2)))</f>
+        <f aca="false">IF(F411="","",ROUND(F411*G411,2))</f>
         <v/>
       </c>
       <c r="I411" s="22" t="str">
@@ -13511,7 +13440,7 @@
       <c r="F412" s="13"/>
       <c r="G412" s="21"/>
       <c r="H412" s="22" t="str">
-        <f>IF(F412="","",IF(OR(E412="Abschreibung (AfA)",E412="Vorsteuer auf Anlagevermögen"),0,ROUND(F412*G412,2)))</f>
+        <f aca="false">IF(F412="","",ROUND(F412*G412,2))</f>
         <v/>
       </c>
       <c r="I412" s="22" t="str">
@@ -13529,7 +13458,7 @@
       <c r="F413" s="13"/>
       <c r="G413" s="21"/>
       <c r="H413" s="22" t="str">
-        <f>IF(F413="","",IF(OR(E413="Abschreibung (AfA)",E413="Vorsteuer auf Anlagevermögen"),0,ROUND(F413*G413,2)))</f>
+        <f aca="false">IF(F413="","",ROUND(F413*G413,2))</f>
         <v/>
       </c>
       <c r="I413" s="22" t="str">
@@ -13547,7 +13476,7 @@
       <c r="F414" s="13"/>
       <c r="G414" s="21"/>
       <c r="H414" s="22" t="str">
-        <f>IF(F414="","",IF(OR(E414="Abschreibung (AfA)",E414="Vorsteuer auf Anlagevermögen"),0,ROUND(F414*G414,2)))</f>
+        <f aca="false">IF(F414="","",ROUND(F414*G414,2))</f>
         <v/>
       </c>
       <c r="I414" s="22" t="str">
@@ -13565,7 +13494,7 @@
       <c r="F415" s="13"/>
       <c r="G415" s="21"/>
       <c r="H415" s="22" t="str">
-        <f>IF(F415="","",IF(OR(E415="Abschreibung (AfA)",E415="Vorsteuer auf Anlagevermögen"),0,ROUND(F415*G415,2)))</f>
+        <f aca="false">IF(F415="","",ROUND(F415*G415,2))</f>
         <v/>
       </c>
       <c r="I415" s="22" t="str">
@@ -13583,7 +13512,7 @@
       <c r="F416" s="13"/>
       <c r="G416" s="21"/>
       <c r="H416" s="22" t="str">
-        <f>IF(F416="","",IF(OR(E416="Abschreibung (AfA)",E416="Vorsteuer auf Anlagevermögen"),0,ROUND(F416*G416,2)))</f>
+        <f aca="false">IF(F416="","",ROUND(F416*G416,2))</f>
         <v/>
       </c>
       <c r="I416" s="22" t="str">
@@ -13601,7 +13530,7 @@
       <c r="F417" s="13"/>
       <c r="G417" s="21"/>
       <c r="H417" s="22" t="str">
-        <f>IF(F417="","",IF(OR(E417="Abschreibung (AfA)",E417="Vorsteuer auf Anlagevermögen"),0,ROUND(F417*G417,2)))</f>
+        <f aca="false">IF(F417="","",ROUND(F417*G417,2))</f>
         <v/>
       </c>
       <c r="I417" s="22" t="str">
@@ -13619,7 +13548,7 @@
       <c r="F418" s="13"/>
       <c r="G418" s="21"/>
       <c r="H418" s="22" t="str">
-        <f>IF(F418="","",IF(OR(E418="Abschreibung (AfA)",E418="Vorsteuer auf Anlagevermögen"),0,ROUND(F418*G418,2)))</f>
+        <f aca="false">IF(F418="","",ROUND(F418*G418,2))</f>
         <v/>
       </c>
       <c r="I418" s="22" t="str">
@@ -13637,7 +13566,7 @@
       <c r="F419" s="13"/>
       <c r="G419" s="21"/>
       <c r="H419" s="22" t="str">
-        <f>IF(F419="","",IF(OR(E419="Abschreibung (AfA)",E419="Vorsteuer auf Anlagevermögen"),0,ROUND(F419*G419,2)))</f>
+        <f aca="false">IF(F419="","",ROUND(F419*G419,2))</f>
         <v/>
       </c>
       <c r="I419" s="22" t="str">
@@ -13655,7 +13584,7 @@
       <c r="F420" s="13"/>
       <c r="G420" s="21"/>
       <c r="H420" s="22" t="str">
-        <f>IF(F420="","",IF(OR(E420="Abschreibung (AfA)",E420="Vorsteuer auf Anlagevermögen"),0,ROUND(F420*G420,2)))</f>
+        <f aca="false">IF(F420="","",ROUND(F420*G420,2))</f>
         <v/>
       </c>
       <c r="I420" s="22" t="str">
@@ -13673,7 +13602,7 @@
       <c r="F421" s="13"/>
       <c r="G421" s="21"/>
       <c r="H421" s="22" t="str">
-        <f>IF(F421="","",IF(OR(E421="Abschreibung (AfA)",E421="Vorsteuer auf Anlagevermögen"),0,ROUND(F421*G421,2)))</f>
+        <f aca="false">IF(F421="","",ROUND(F421*G421,2))</f>
         <v/>
       </c>
       <c r="I421" s="22" t="str">
@@ -13691,7 +13620,7 @@
       <c r="F422" s="13"/>
       <c r="G422" s="21"/>
       <c r="H422" s="22" t="str">
-        <f>IF(F422="","",IF(OR(E422="Abschreibung (AfA)",E422="Vorsteuer auf Anlagevermögen"),0,ROUND(F422*G422,2)))</f>
+        <f aca="false">IF(F422="","",ROUND(F422*G422,2))</f>
         <v/>
       </c>
       <c r="I422" s="22" t="str">
@@ -13709,7 +13638,7 @@
       <c r="F423" s="13"/>
       <c r="G423" s="21"/>
       <c r="H423" s="22" t="str">
-        <f>IF(F423="","",IF(OR(E423="Abschreibung (AfA)",E423="Vorsteuer auf Anlagevermögen"),0,ROUND(F423*G423,2)))</f>
+        <f aca="false">IF(F423="","",ROUND(F423*G423,2))</f>
         <v/>
       </c>
       <c r="I423" s="22" t="str">
@@ -13727,7 +13656,7 @@
       <c r="F424" s="13"/>
       <c r="G424" s="21"/>
       <c r="H424" s="22" t="str">
-        <f>IF(F424="","",IF(OR(E424="Abschreibung (AfA)",E424="Vorsteuer auf Anlagevermögen"),0,ROUND(F424*G424,2)))</f>
+        <f aca="false">IF(F424="","",ROUND(F424*G424,2))</f>
         <v/>
       </c>
       <c r="I424" s="22" t="str">
@@ -13745,7 +13674,7 @@
       <c r="F425" s="13"/>
       <c r="G425" s="21"/>
       <c r="H425" s="22" t="str">
-        <f>IF(F425="","",IF(OR(E425="Abschreibung (AfA)",E425="Vorsteuer auf Anlagevermögen"),0,ROUND(F425*G425,2)))</f>
+        <f aca="false">IF(F425="","",ROUND(F425*G425,2))</f>
         <v/>
       </c>
       <c r="I425" s="22" t="str">
@@ -13763,7 +13692,7 @@
       <c r="F426" s="13"/>
       <c r="G426" s="21"/>
       <c r="H426" s="22" t="str">
-        <f>IF(F426="","",IF(OR(E426="Abschreibung (AfA)",E426="Vorsteuer auf Anlagevermögen"),0,ROUND(F426*G426,2)))</f>
+        <f aca="false">IF(F426="","",ROUND(F426*G426,2))</f>
         <v/>
       </c>
       <c r="I426" s="22" t="str">
@@ -13781,7 +13710,7 @@
       <c r="F427" s="13"/>
       <c r="G427" s="21"/>
       <c r="H427" s="22" t="str">
-        <f>IF(F427="","",IF(OR(E427="Abschreibung (AfA)",E427="Vorsteuer auf Anlagevermögen"),0,ROUND(F427*G427,2)))</f>
+        <f aca="false">IF(F427="","",ROUND(F427*G427,2))</f>
         <v/>
       </c>
       <c r="I427" s="22" t="str">
@@ -13799,7 +13728,7 @@
       <c r="F428" s="13"/>
       <c r="G428" s="21"/>
       <c r="H428" s="22" t="str">
-        <f>IF(F428="","",IF(OR(E428="Abschreibung (AfA)",E428="Vorsteuer auf Anlagevermögen"),0,ROUND(F428*G428,2)))</f>
+        <f aca="false">IF(F428="","",ROUND(F428*G428,2))</f>
         <v/>
       </c>
       <c r="I428" s="22" t="str">
@@ -13817,7 +13746,7 @@
       <c r="F429" s="13"/>
       <c r="G429" s="21"/>
       <c r="H429" s="22" t="str">
-        <f>IF(F429="","",IF(OR(E429="Abschreibung (AfA)",E429="Vorsteuer auf Anlagevermögen"),0,ROUND(F429*G429,2)))</f>
+        <f aca="false">IF(F429="","",ROUND(F429*G429,2))</f>
         <v/>
       </c>
       <c r="I429" s="22" t="str">
@@ -13835,7 +13764,7 @@
       <c r="F430" s="13"/>
       <c r="G430" s="21"/>
       <c r="H430" s="22" t="str">
-        <f>IF(F430="","",IF(OR(E430="Abschreibung (AfA)",E430="Vorsteuer auf Anlagevermögen"),0,ROUND(F430*G430,2)))</f>
+        <f aca="false">IF(F430="","",ROUND(F430*G430,2))</f>
         <v/>
       </c>
       <c r="I430" s="22" t="str">
@@ -13853,7 +13782,7 @@
       <c r="F431" s="13"/>
       <c r="G431" s="21"/>
       <c r="H431" s="22" t="str">
-        <f>IF(F431="","",IF(OR(E431="Abschreibung (AfA)",E431="Vorsteuer auf Anlagevermögen"),0,ROUND(F431*G431,2)))</f>
+        <f aca="false">IF(F431="","",ROUND(F431*G431,2))</f>
         <v/>
       </c>
       <c r="I431" s="22" t="str">
@@ -13871,7 +13800,7 @@
       <c r="F432" s="13"/>
       <c r="G432" s="21"/>
       <c r="H432" s="22" t="str">
-        <f>IF(F432="","",IF(OR(E432="Abschreibung (AfA)",E432="Vorsteuer auf Anlagevermögen"),0,ROUND(F432*G432,2)))</f>
+        <f aca="false">IF(F432="","",ROUND(F432*G432,2))</f>
         <v/>
       </c>
       <c r="I432" s="22" t="str">
@@ -13889,7 +13818,7 @@
       <c r="F433" s="13"/>
       <c r="G433" s="21"/>
       <c r="H433" s="22" t="str">
-        <f>IF(F433="","",IF(OR(E433="Abschreibung (AfA)",E433="Vorsteuer auf Anlagevermögen"),0,ROUND(F433*G433,2)))</f>
+        <f aca="false">IF(F433="","",ROUND(F433*G433,2))</f>
         <v/>
       </c>
       <c r="I433" s="22" t="str">
@@ -13907,7 +13836,7 @@
       <c r="F434" s="13"/>
       <c r="G434" s="21"/>
       <c r="H434" s="22" t="str">
-        <f>IF(F434="","",IF(OR(E434="Abschreibung (AfA)",E434="Vorsteuer auf Anlagevermögen"),0,ROUND(F434*G434,2)))</f>
+        <f aca="false">IF(F434="","",ROUND(F434*G434,2))</f>
         <v/>
       </c>
       <c r="I434" s="22" t="str">
@@ -13925,7 +13854,7 @@
       <c r="F435" s="13"/>
       <c r="G435" s="21"/>
       <c r="H435" s="22" t="str">
-        <f>IF(F435="","",IF(OR(E435="Abschreibung (AfA)",E435="Vorsteuer auf Anlagevermögen"),0,ROUND(F435*G435,2)))</f>
+        <f aca="false">IF(F435="","",ROUND(F435*G435,2))</f>
         <v/>
       </c>
       <c r="I435" s="22" t="str">
@@ -13943,7 +13872,7 @@
       <c r="F436" s="13"/>
       <c r="G436" s="21"/>
       <c r="H436" s="22" t="str">
-        <f>IF(F436="","",IF(OR(E436="Abschreibung (AfA)",E436="Vorsteuer auf Anlagevermögen"),0,ROUND(F436*G436,2)))</f>
+        <f aca="false">IF(F436="","",ROUND(F436*G436,2))</f>
         <v/>
       </c>
       <c r="I436" s="22" t="str">
@@ -13961,7 +13890,7 @@
       <c r="F437" s="13"/>
       <c r="G437" s="21"/>
       <c r="H437" s="22" t="str">
-        <f>IF(F437="","",IF(OR(E437="Abschreibung (AfA)",E437="Vorsteuer auf Anlagevermögen"),0,ROUND(F437*G437,2)))</f>
+        <f aca="false">IF(F437="","",ROUND(F437*G437,2))</f>
         <v/>
       </c>
       <c r="I437" s="22" t="str">
@@ -13979,7 +13908,7 @@
       <c r="F438" s="13"/>
       <c r="G438" s="21"/>
       <c r="H438" s="22" t="str">
-        <f>IF(F438="","",IF(OR(E438="Abschreibung (AfA)",E438="Vorsteuer auf Anlagevermögen"),0,ROUND(F438*G438,2)))</f>
+        <f aca="false">IF(F438="","",ROUND(F438*G438,2))</f>
         <v/>
       </c>
       <c r="I438" s="22" t="str">
@@ -13997,7 +13926,7 @@
       <c r="F439" s="13"/>
       <c r="G439" s="21"/>
       <c r="H439" s="22" t="str">
-        <f>IF(F439="","",IF(OR(E439="Abschreibung (AfA)",E439="Vorsteuer auf Anlagevermögen"),0,ROUND(F439*G439,2)))</f>
+        <f aca="false">IF(F439="","",ROUND(F439*G439,2))</f>
         <v/>
       </c>
       <c r="I439" s="22" t="str">
@@ -14015,7 +13944,7 @@
       <c r="F440" s="13"/>
       <c r="G440" s="21"/>
       <c r="H440" s="22" t="str">
-        <f>IF(F440="","",IF(OR(E440="Abschreibung (AfA)",E440="Vorsteuer auf Anlagevermögen"),0,ROUND(F440*G440,2)))</f>
+        <f aca="false">IF(F440="","",ROUND(F440*G440,2))</f>
         <v/>
       </c>
       <c r="I440" s="22" t="str">
@@ -14033,7 +13962,7 @@
       <c r="F441" s="13"/>
       <c r="G441" s="21"/>
       <c r="H441" s="22" t="str">
-        <f>IF(F441="","",IF(OR(E441="Abschreibung (AfA)",E441="Vorsteuer auf Anlagevermögen"),0,ROUND(F441*G441,2)))</f>
+        <f aca="false">IF(F441="","",ROUND(F441*G441,2))</f>
         <v/>
       </c>
       <c r="I441" s="22" t="str">
@@ -14051,7 +13980,7 @@
       <c r="F442" s="13"/>
       <c r="G442" s="21"/>
       <c r="H442" s="22" t="str">
-        <f>IF(F442="","",IF(OR(E442="Abschreibung (AfA)",E442="Vorsteuer auf Anlagevermögen"),0,ROUND(F442*G442,2)))</f>
+        <f aca="false">IF(F442="","",ROUND(F442*G442,2))</f>
         <v/>
       </c>
       <c r="I442" s="22" t="str">
@@ -14069,7 +13998,7 @@
       <c r="F443" s="13"/>
       <c r="G443" s="21"/>
       <c r="H443" s="22" t="str">
-        <f>IF(F443="","",IF(OR(E443="Abschreibung (AfA)",E443="Vorsteuer auf Anlagevermögen"),0,ROUND(F443*G443,2)))</f>
+        <f aca="false">IF(F443="","",ROUND(F443*G443,2))</f>
         <v/>
       </c>
       <c r="I443" s="22" t="str">
@@ -14087,7 +14016,7 @@
       <c r="F444" s="13"/>
       <c r="G444" s="21"/>
       <c r="H444" s="22" t="str">
-        <f>IF(F444="","",IF(OR(E444="Abschreibung (AfA)",E444="Vorsteuer auf Anlagevermögen"),0,ROUND(F444*G444,2)))</f>
+        <f aca="false">IF(F444="","",ROUND(F444*G444,2))</f>
         <v/>
       </c>
       <c r="I444" s="22" t="str">
@@ -14105,7 +14034,7 @@
       <c r="F445" s="13"/>
       <c r="G445" s="21"/>
       <c r="H445" s="22" t="str">
-        <f>IF(F445="","",IF(OR(E445="Abschreibung (AfA)",E445="Vorsteuer auf Anlagevermögen"),0,ROUND(F445*G445,2)))</f>
+        <f aca="false">IF(F445="","",ROUND(F445*G445,2))</f>
         <v/>
       </c>
       <c r="I445" s="22" t="str">
@@ -14123,7 +14052,7 @@
       <c r="F446" s="13"/>
       <c r="G446" s="21"/>
       <c r="H446" s="22" t="str">
-        <f>IF(F446="","",IF(OR(E446="Abschreibung (AfA)",E446="Vorsteuer auf Anlagevermögen"),0,ROUND(F446*G446,2)))</f>
+        <f aca="false">IF(F446="","",ROUND(F446*G446,2))</f>
         <v/>
       </c>
       <c r="I446" s="22" t="str">
@@ -14141,7 +14070,7 @@
       <c r="F447" s="13"/>
       <c r="G447" s="21"/>
       <c r="H447" s="22" t="str">
-        <f>IF(F447="","",IF(OR(E447="Abschreibung (AfA)",E447="Vorsteuer auf Anlagevermögen"),0,ROUND(F447*G447,2)))</f>
+        <f aca="false">IF(F447="","",ROUND(F447*G447,2))</f>
         <v/>
       </c>
       <c r="I447" s="22" t="str">
@@ -14159,7 +14088,7 @@
       <c r="F448" s="13"/>
       <c r="G448" s="21"/>
       <c r="H448" s="22" t="str">
-        <f>IF(F448="","",IF(OR(E448="Abschreibung (AfA)",E448="Vorsteuer auf Anlagevermögen"),0,ROUND(F448*G448,2)))</f>
+        <f aca="false">IF(F448="","",ROUND(F448*G448,2))</f>
         <v/>
       </c>
       <c r="I448" s="22" t="str">
@@ -14177,7 +14106,7 @@
       <c r="F449" s="13"/>
       <c r="G449" s="21"/>
       <c r="H449" s="22" t="str">
-        <f>IF(F449="","",IF(OR(E449="Abschreibung (AfA)",E449="Vorsteuer auf Anlagevermögen"),0,ROUND(F449*G449,2)))</f>
+        <f aca="false">IF(F449="","",ROUND(F449*G449,2))</f>
         <v/>
       </c>
       <c r="I449" s="22" t="str">
@@ -14195,7 +14124,7 @@
       <c r="F450" s="13"/>
       <c r="G450" s="21"/>
       <c r="H450" s="22" t="str">
-        <f>IF(F450="","",IF(OR(E450="Abschreibung (AfA)",E450="Vorsteuer auf Anlagevermögen"),0,ROUND(F450*G450,2)))</f>
+        <f aca="false">IF(F450="","",ROUND(F450*G450,2))</f>
         <v/>
       </c>
       <c r="I450" s="22" t="str">
@@ -14213,7 +14142,7 @@
       <c r="F451" s="13"/>
       <c r="G451" s="21"/>
       <c r="H451" s="22" t="str">
-        <f>IF(F451="","",IF(OR(E451="Abschreibung (AfA)",E451="Vorsteuer auf Anlagevermögen"),0,ROUND(F451*G451,2)))</f>
+        <f aca="false">IF(F451="","",ROUND(F451*G451,2))</f>
         <v/>
       </c>
       <c r="I451" s="22" t="str">
@@ -14231,7 +14160,7 @@
       <c r="F452" s="13"/>
       <c r="G452" s="21"/>
       <c r="H452" s="22" t="str">
-        <f>IF(F452="","",IF(OR(E452="Abschreibung (AfA)",E452="Vorsteuer auf Anlagevermögen"),0,ROUND(F452*G452,2)))</f>
+        <f aca="false">IF(F452="","",ROUND(F452*G452,2))</f>
         <v/>
       </c>
       <c r="I452" s="22" t="str">
@@ -14249,7 +14178,7 @@
       <c r="F453" s="13"/>
       <c r="G453" s="21"/>
       <c r="H453" s="22" t="str">
-        <f>IF(F453="","",IF(OR(E453="Abschreibung (AfA)",E453="Vorsteuer auf Anlagevermögen"),0,ROUND(F453*G453,2)))</f>
+        <f aca="false">IF(F453="","",ROUND(F453*G453,2))</f>
         <v/>
       </c>
       <c r="I453" s="22" t="str">
@@ -14267,7 +14196,7 @@
       <c r="F454" s="13"/>
       <c r="G454" s="21"/>
       <c r="H454" s="22" t="str">
-        <f>IF(F454="","",IF(OR(E454="Abschreibung (AfA)",E454="Vorsteuer auf Anlagevermögen"),0,ROUND(F454*G454,2)))</f>
+        <f aca="false">IF(F454="","",ROUND(F454*G454,2))</f>
         <v/>
       </c>
       <c r="I454" s="22" t="str">
@@ -14285,7 +14214,7 @@
       <c r="F455" s="13"/>
       <c r="G455" s="21"/>
       <c r="H455" s="22" t="str">
-        <f>IF(F455="","",IF(OR(E455="Abschreibung (AfA)",E455="Vorsteuer auf Anlagevermögen"),0,ROUND(F455*G455,2)))</f>
+        <f aca="false">IF(F455="","",ROUND(F455*G455,2))</f>
         <v/>
       </c>
       <c r="I455" s="22" t="str">
@@ -14303,7 +14232,7 @@
       <c r="F456" s="13"/>
       <c r="G456" s="21"/>
       <c r="H456" s="22" t="str">
-        <f>IF(F456="","",IF(OR(E456="Abschreibung (AfA)",E456="Vorsteuer auf Anlagevermögen"),0,ROUND(F456*G456,2)))</f>
+        <f aca="false">IF(F456="","",ROUND(F456*G456,2))</f>
         <v/>
       </c>
       <c r="I456" s="22" t="str">
@@ -14321,7 +14250,7 @@
       <c r="F457" s="13"/>
       <c r="G457" s="21"/>
       <c r="H457" s="22" t="str">
-        <f>IF(F457="","",IF(OR(E457="Abschreibung (AfA)",E457="Vorsteuer auf Anlagevermögen"),0,ROUND(F457*G457,2)))</f>
+        <f aca="false">IF(F457="","",ROUND(F457*G457,2))</f>
         <v/>
       </c>
       <c r="I457" s="22" t="str">
@@ -14339,7 +14268,7 @@
       <c r="F458" s="13"/>
       <c r="G458" s="21"/>
       <c r="H458" s="22" t="str">
-        <f>IF(F458="","",IF(OR(E458="Abschreibung (AfA)",E458="Vorsteuer auf Anlagevermögen"),0,ROUND(F458*G458,2)))</f>
+        <f aca="false">IF(F458="","",ROUND(F458*G458,2))</f>
         <v/>
       </c>
       <c r="I458" s="22" t="str">
@@ -14357,7 +14286,7 @@
       <c r="F459" s="13"/>
       <c r="G459" s="21"/>
       <c r="H459" s="22" t="str">
-        <f>IF(F459="","",IF(OR(E459="Abschreibung (AfA)",E459="Vorsteuer auf Anlagevermögen"),0,ROUND(F459*G459,2)))</f>
+        <f aca="false">IF(F459="","",ROUND(F459*G459,2))</f>
         <v/>
       </c>
       <c r="I459" s="22" t="str">
@@ -14375,7 +14304,7 @@
       <c r="F460" s="13"/>
       <c r="G460" s="21"/>
       <c r="H460" s="22" t="str">
-        <f>IF(F460="","",IF(OR(E460="Abschreibung (AfA)",E460="Vorsteuer auf Anlagevermögen"),0,ROUND(F460*G460,2)))</f>
+        <f aca="false">IF(F460="","",ROUND(F460*G460,2))</f>
         <v/>
       </c>
       <c r="I460" s="22" t="str">
@@ -14393,7 +14322,7 @@
       <c r="F461" s="13"/>
       <c r="G461" s="21"/>
       <c r="H461" s="22" t="str">
-        <f>IF(F461="","",IF(OR(E461="Abschreibung (AfA)",E461="Vorsteuer auf Anlagevermögen"),0,ROUND(F461*G461,2)))</f>
+        <f aca="false">IF(F461="","",ROUND(F461*G461,2))</f>
         <v/>
       </c>
       <c r="I461" s="22" t="str">
@@ -14411,7 +14340,7 @@
       <c r="F462" s="13"/>
       <c r="G462" s="21"/>
       <c r="H462" s="22" t="str">
-        <f>IF(F462="","",IF(OR(E462="Abschreibung (AfA)",E462="Vorsteuer auf Anlagevermögen"),0,ROUND(F462*G462,2)))</f>
+        <f aca="false">IF(F462="","",ROUND(F462*G462,2))</f>
         <v/>
       </c>
       <c r="I462" s="22" t="str">
@@ -14429,7 +14358,7 @@
       <c r="F463" s="13"/>
       <c r="G463" s="21"/>
       <c r="H463" s="22" t="str">
-        <f>IF(F463="","",IF(OR(E463="Abschreibung (AfA)",E463="Vorsteuer auf Anlagevermögen"),0,ROUND(F463*G463,2)))</f>
+        <f aca="false">IF(F463="","",ROUND(F463*G463,2))</f>
         <v/>
       </c>
       <c r="I463" s="22" t="str">
@@ -14447,7 +14376,7 @@
       <c r="F464" s="13"/>
       <c r="G464" s="21"/>
       <c r="H464" s="22" t="str">
-        <f>IF(F464="","",IF(OR(E464="Abschreibung (AfA)",E464="Vorsteuer auf Anlagevermögen"),0,ROUND(F464*G464,2)))</f>
+        <f aca="false">IF(F464="","",ROUND(F464*G464,2))</f>
         <v/>
       </c>
       <c r="I464" s="22" t="str">
@@ -14465,7 +14394,7 @@
       <c r="F465" s="13"/>
       <c r="G465" s="21"/>
       <c r="H465" s="22" t="str">
-        <f>IF(F465="","",IF(OR(E465="Abschreibung (AfA)",E465="Vorsteuer auf Anlagevermögen"),0,ROUND(F465*G465,2)))</f>
+        <f aca="false">IF(F465="","",ROUND(F465*G465,2))</f>
         <v/>
       </c>
       <c r="I465" s="22" t="str">
@@ -14483,7 +14412,7 @@
       <c r="F466" s="13"/>
       <c r="G466" s="21"/>
       <c r="H466" s="22" t="str">
-        <f>IF(F466="","",IF(OR(E466="Abschreibung (AfA)",E466="Vorsteuer auf Anlagevermögen"),0,ROUND(F466*G466,2)))</f>
+        <f aca="false">IF(F466="","",ROUND(F466*G466,2))</f>
         <v/>
       </c>
       <c r="I466" s="22" t="str">
@@ -14501,7 +14430,7 @@
       <c r="F467" s="13"/>
       <c r="G467" s="21"/>
       <c r="H467" s="22" t="str">
-        <f>IF(F467="","",IF(OR(E467="Abschreibung (AfA)",E467="Vorsteuer auf Anlagevermögen"),0,ROUND(F467*G467,2)))</f>
+        <f aca="false">IF(F467="","",ROUND(F467*G467,2))</f>
         <v/>
       </c>
       <c r="I467" s="22" t="str">
@@ -14519,7 +14448,7 @@
       <c r="F468" s="13"/>
       <c r="G468" s="21"/>
       <c r="H468" s="22" t="str">
-        <f>IF(F468="","",IF(OR(E468="Abschreibung (AfA)",E468="Vorsteuer auf Anlagevermögen"),0,ROUND(F468*G468,2)))</f>
+        <f aca="false">IF(F468="","",ROUND(F468*G468,2))</f>
         <v/>
       </c>
       <c r="I468" s="22" t="str">
@@ -14537,7 +14466,7 @@
       <c r="F469" s="13"/>
       <c r="G469" s="21"/>
       <c r="H469" s="22" t="str">
-        <f>IF(F469="","",IF(OR(E469="Abschreibung (AfA)",E469="Vorsteuer auf Anlagevermögen"),0,ROUND(F469*G469,2)))</f>
+        <f aca="false">IF(F469="","",ROUND(F469*G469,2))</f>
         <v/>
       </c>
       <c r="I469" s="22" t="str">
@@ -14555,7 +14484,7 @@
       <c r="F470" s="13"/>
       <c r="G470" s="21"/>
       <c r="H470" s="22" t="str">
-        <f>IF(F470="","",IF(OR(E470="Abschreibung (AfA)",E470="Vorsteuer auf Anlagevermögen"),0,ROUND(F470*G470,2)))</f>
+        <f aca="false">IF(F470="","",ROUND(F470*G470,2))</f>
         <v/>
       </c>
       <c r="I470" s="22" t="str">
@@ -14573,7 +14502,7 @@
       <c r="F471" s="13"/>
       <c r="G471" s="21"/>
       <c r="H471" s="22" t="str">
-        <f>IF(F471="","",IF(OR(E471="Abschreibung (AfA)",E471="Vorsteuer auf Anlagevermögen"),0,ROUND(F471*G471,2)))</f>
+        <f aca="false">IF(F471="","",ROUND(F471*G471,2))</f>
         <v/>
       </c>
       <c r="I471" s="22" t="str">
@@ -14591,7 +14520,7 @@
       <c r="F472" s="13"/>
       <c r="G472" s="21"/>
       <c r="H472" s="22" t="str">
-        <f>IF(F472="","",IF(OR(E472="Abschreibung (AfA)",E472="Vorsteuer auf Anlagevermögen"),0,ROUND(F472*G472,2)))</f>
+        <f aca="false">IF(F472="","",ROUND(F472*G472,2))</f>
         <v/>
       </c>
       <c r="I472" s="22" t="str">
@@ -14609,7 +14538,7 @@
       <c r="F473" s="13"/>
       <c r="G473" s="21"/>
       <c r="H473" s="22" t="str">
-        <f>IF(F473="","",IF(OR(E473="Abschreibung (AfA)",E473="Vorsteuer auf Anlagevermögen"),0,ROUND(F473*G473,2)))</f>
+        <f aca="false">IF(F473="","",ROUND(F473*G473,2))</f>
         <v/>
       </c>
       <c r="I473" s="22" t="str">
@@ -14627,7 +14556,7 @@
       <c r="F474" s="13"/>
       <c r="G474" s="21"/>
       <c r="H474" s="22" t="str">
-        <f>IF(F474="","",IF(OR(E474="Abschreibung (AfA)",E474="Vorsteuer auf Anlagevermögen"),0,ROUND(F474*G474,2)))</f>
+        <f aca="false">IF(F474="","",ROUND(F474*G474,2))</f>
         <v/>
       </c>
       <c r="I474" s="22" t="str">
@@ -14645,7 +14574,7 @@
       <c r="F475" s="13"/>
       <c r="G475" s="21"/>
       <c r="H475" s="22" t="str">
-        <f>IF(F475="","",IF(OR(E475="Abschreibung (AfA)",E475="Vorsteuer auf Anlagevermögen"),0,ROUND(F475*G475,2)))</f>
+        <f aca="false">IF(F475="","",ROUND(F475*G475,2))</f>
         <v/>
       </c>
       <c r="I475" s="22" t="str">
@@ -14663,7 +14592,7 @@
       <c r="F476" s="13"/>
       <c r="G476" s="21"/>
       <c r="H476" s="22" t="str">
-        <f>IF(F476="","",IF(OR(E476="Abschreibung (AfA)",E476="Vorsteuer auf Anlagevermögen"),0,ROUND(F476*G476,2)))</f>
+        <f aca="false">IF(F476="","",ROUND(F476*G476,2))</f>
         <v/>
       </c>
       <c r="I476" s="22" t="str">
@@ -14681,7 +14610,7 @@
       <c r="F477" s="13"/>
       <c r="G477" s="21"/>
       <c r="H477" s="22" t="str">
-        <f>IF(F477="","",IF(OR(E477="Abschreibung (AfA)",E477="Vorsteuer auf Anlagevermögen"),0,ROUND(F477*G477,2)))</f>
+        <f aca="false">IF(F477="","",ROUND(F477*G477,2))</f>
         <v/>
       </c>
       <c r="I477" s="22" t="str">
@@ -14699,7 +14628,7 @@
       <c r="F478" s="13"/>
       <c r="G478" s="21"/>
       <c r="H478" s="22" t="str">
-        <f>IF(F478="","",IF(OR(E478="Abschreibung (AfA)",E478="Vorsteuer auf Anlagevermögen"),0,ROUND(F478*G478,2)))</f>
+        <f aca="false">IF(F478="","",ROUND(F478*G478,2))</f>
         <v/>
       </c>
       <c r="I478" s="22" t="str">
@@ -14717,7 +14646,7 @@
       <c r="F479" s="13"/>
       <c r="G479" s="21"/>
       <c r="H479" s="22" t="str">
-        <f>IF(F479="","",IF(OR(E479="Abschreibung (AfA)",E479="Vorsteuer auf Anlagevermögen"),0,ROUND(F479*G479,2)))</f>
+        <f aca="false">IF(F479="","",ROUND(F479*G479,2))</f>
         <v/>
       </c>
       <c r="I479" s="22" t="str">
@@ -14735,7 +14664,7 @@
       <c r="F480" s="13"/>
       <c r="G480" s="21"/>
       <c r="H480" s="22" t="str">
-        <f>IF(F480="","",IF(OR(E480="Abschreibung (AfA)",E480="Vorsteuer auf Anlagevermögen"),0,ROUND(F480*G480,2)))</f>
+        <f aca="false">IF(F480="","",ROUND(F480*G480,2))</f>
         <v/>
       </c>
       <c r="I480" s="22" t="str">
@@ -14753,7 +14682,7 @@
       <c r="F481" s="13"/>
       <c r="G481" s="21"/>
       <c r="H481" s="22" t="str">
-        <f>IF(F481="","",IF(OR(E481="Abschreibung (AfA)",E481="Vorsteuer auf Anlagevermögen"),0,ROUND(F481*G481,2)))</f>
+        <f aca="false">IF(F481="","",ROUND(F481*G481,2))</f>
         <v/>
       </c>
       <c r="I481" s="22" t="str">
@@ -14771,7 +14700,7 @@
       <c r="F482" s="13"/>
       <c r="G482" s="21"/>
       <c r="H482" s="22" t="str">
-        <f>IF(F482="","",IF(OR(E482="Abschreibung (AfA)",E482="Vorsteuer auf Anlagevermögen"),0,ROUND(F482*G482,2)))</f>
+        <f aca="false">IF(F482="","",ROUND(F482*G482,2))</f>
         <v/>
       </c>
       <c r="I482" s="22" t="str">
@@ -14789,7 +14718,7 @@
       <c r="F483" s="13"/>
       <c r="G483" s="21"/>
       <c r="H483" s="22" t="str">
-        <f>IF(F483="","",IF(OR(E483="Abschreibung (AfA)",E483="Vorsteuer auf Anlagevermögen"),0,ROUND(F483*G483,2)))</f>
+        <f aca="false">IF(F483="","",ROUND(F483*G483,2))</f>
         <v/>
       </c>
       <c r="I483" s="22" t="str">
@@ -14807,7 +14736,7 @@
       <c r="F484" s="13"/>
       <c r="G484" s="21"/>
       <c r="H484" s="22" t="str">
-        <f>IF(F484="","",IF(OR(E484="Abschreibung (AfA)",E484="Vorsteuer auf Anlagevermögen"),0,ROUND(F484*G484,2)))</f>
+        <f aca="false">IF(F484="","",ROUND(F484*G484,2))</f>
         <v/>
       </c>
       <c r="I484" s="22" t="str">
@@ -14825,7 +14754,7 @@
       <c r="F485" s="13"/>
       <c r="G485" s="21"/>
       <c r="H485" s="22" t="str">
-        <f>IF(F485="","",IF(OR(E485="Abschreibung (AfA)",E485="Vorsteuer auf Anlagevermögen"),0,ROUND(F485*G485,2)))</f>
+        <f aca="false">IF(F485="","",ROUND(F485*G485,2))</f>
         <v/>
       </c>
       <c r="I485" s="22" t="str">
@@ -14843,7 +14772,7 @@
       <c r="F486" s="13"/>
       <c r="G486" s="21"/>
       <c r="H486" s="22" t="str">
-        <f>IF(F486="","",IF(OR(E486="Abschreibung (AfA)",E486="Vorsteuer auf Anlagevermögen"),0,ROUND(F486*G486,2)))</f>
+        <f aca="false">IF(F486="","",ROUND(F486*G486,2))</f>
         <v/>
       </c>
       <c r="I486" s="22" t="str">
@@ -14861,7 +14790,7 @@
       <c r="F487" s="13"/>
       <c r="G487" s="21"/>
       <c r="H487" s="22" t="str">
-        <f>IF(F487="","",IF(OR(E487="Abschreibung (AfA)",E487="Vorsteuer auf Anlagevermögen"),0,ROUND(F487*G487,2)))</f>
+        <f aca="false">IF(F487="","",ROUND(F487*G487,2))</f>
         <v/>
       </c>
       <c r="I487" s="22" t="str">
@@ -14879,7 +14808,7 @@
       <c r="F488" s="13"/>
       <c r="G488" s="21"/>
       <c r="H488" s="22" t="str">
-        <f>IF(F488="","",IF(OR(E488="Abschreibung (AfA)",E488="Vorsteuer auf Anlagevermögen"),0,ROUND(F488*G488,2)))</f>
+        <f aca="false">IF(F488="","",ROUND(F488*G488,2))</f>
         <v/>
       </c>
       <c r="I488" s="22" t="str">
@@ -14897,7 +14826,7 @@
       <c r="F489" s="13"/>
       <c r="G489" s="21"/>
       <c r="H489" s="22" t="str">
-        <f>IF(F489="","",IF(OR(E489="Abschreibung (AfA)",E489="Vorsteuer auf Anlagevermögen"),0,ROUND(F489*G489,2)))</f>
+        <f aca="false">IF(F489="","",ROUND(F489*G489,2))</f>
         <v/>
       </c>
       <c r="I489" s="22" t="str">
@@ -14915,7 +14844,7 @@
       <c r="F490" s="13"/>
       <c r="G490" s="21"/>
       <c r="H490" s="22" t="str">
-        <f>IF(F490="","",IF(OR(E490="Abschreibung (AfA)",E490="Vorsteuer auf Anlagevermögen"),0,ROUND(F490*G490,2)))</f>
+        <f aca="false">IF(F490="","",ROUND(F490*G490,2))</f>
         <v/>
       </c>
       <c r="I490" s="22" t="str">
@@ -14933,7 +14862,7 @@
       <c r="F491" s="13"/>
       <c r="G491" s="21"/>
       <c r="H491" s="22" t="str">
-        <f>IF(F491="","",IF(OR(E491="Abschreibung (AfA)",E491="Vorsteuer auf Anlagevermögen"),0,ROUND(F491*G491,2)))</f>
+        <f aca="false">IF(F491="","",ROUND(F491*G491,2))</f>
         <v/>
       </c>
       <c r="I491" s="22" t="str">
@@ -14951,7 +14880,7 @@
       <c r="F492" s="13"/>
       <c r="G492" s="21"/>
       <c r="H492" s="22" t="str">
-        <f>IF(F492="","",IF(OR(E492="Abschreibung (AfA)",E492="Vorsteuer auf Anlagevermögen"),0,ROUND(F492*G492,2)))</f>
+        <f aca="false">IF(F492="","",ROUND(F492*G492,2))</f>
         <v/>
       </c>
       <c r="I492" s="22" t="str">
@@ -14969,7 +14898,7 @@
       <c r="F493" s="13"/>
       <c r="G493" s="21"/>
       <c r="H493" s="22" t="str">
-        <f>IF(F493="","",IF(OR(E493="Abschreibung (AfA)",E493="Vorsteuer auf Anlagevermögen"),0,ROUND(F493*G493,2)))</f>
+        <f aca="false">IF(F493="","",ROUND(F493*G493,2))</f>
         <v/>
       </c>
       <c r="I493" s="22" t="str">
@@ -14987,7 +14916,7 @@
       <c r="F494" s="13"/>
       <c r="G494" s="21"/>
       <c r="H494" s="22" t="str">
-        <f>IF(F494="","",IF(OR(E494="Abschreibung (AfA)",E494="Vorsteuer auf Anlagevermögen"),0,ROUND(F494*G494,2)))</f>
+        <f aca="false">IF(F494="","",ROUND(F494*G494,2))</f>
         <v/>
       </c>
       <c r="I494" s="22" t="str">
@@ -15005,7 +14934,7 @@
       <c r="F495" s="13"/>
       <c r="G495" s="21"/>
       <c r="H495" s="22" t="str">
-        <f>IF(F495="","",IF(OR(E495="Abschreibung (AfA)",E495="Vorsteuer auf Anlagevermögen"),0,ROUND(F495*G495,2)))</f>
+        <f aca="false">IF(F495="","",ROUND(F495*G495,2))</f>
         <v/>
       </c>
       <c r="I495" s="22" t="str">
@@ -15023,7 +14952,7 @@
       <c r="F496" s="13"/>
       <c r="G496" s="21"/>
       <c r="H496" s="22" t="str">
-        <f>IF(F496="","",IF(OR(E496="Abschreibung (AfA)",E496="Vorsteuer auf Anlagevermögen"),0,ROUND(F496*G496,2)))</f>
+        <f aca="false">IF(F496="","",ROUND(F496*G496,2))</f>
         <v/>
       </c>
       <c r="I496" s="22" t="str">
@@ -15041,7 +14970,7 @@
       <c r="F497" s="13"/>
       <c r="G497" s="21"/>
       <c r="H497" s="22" t="str">
-        <f>IF(F497="","",IF(OR(E497="Abschreibung (AfA)",E497="Vorsteuer auf Anlagevermögen"),0,ROUND(F497*G497,2)))</f>
+        <f aca="false">IF(F497="","",ROUND(F497*G497,2))</f>
         <v/>
       </c>
       <c r="I497" s="22" t="str">
@@ -15059,7 +14988,7 @@
       <c r="F498" s="13"/>
       <c r="G498" s="21"/>
       <c r="H498" s="22" t="str">
-        <f>IF(F498="","",IF(OR(E498="Abschreibung (AfA)",E498="Vorsteuer auf Anlagevermögen"),0,ROUND(F498*G498,2)))</f>
+        <f aca="false">IF(F498="","",ROUND(F498*G498,2))</f>
         <v/>
       </c>
       <c r="I498" s="22" t="str">
@@ -15077,7 +15006,7 @@
       <c r="F499" s="13"/>
       <c r="G499" s="21"/>
       <c r="H499" s="22" t="str">
-        <f>IF(F499="","",IF(OR(E499="Abschreibung (AfA)",E499="Vorsteuer auf Anlagevermögen"),0,ROUND(F499*G499,2)))</f>
+        <f aca="false">IF(F499="","",ROUND(F499*G499,2))</f>
         <v/>
       </c>
       <c r="I499" s="22" t="str">
@@ -15095,7 +15024,7 @@
       <c r="F500" s="13"/>
       <c r="G500" s="21"/>
       <c r="H500" s="22" t="str">
-        <f>IF(F500="","",IF(OR(E500="Abschreibung (AfA)",E500="Vorsteuer auf Anlagevermögen"),0,ROUND(F500*G500,2)))</f>
+        <f aca="false">IF(F500="","",ROUND(F500*G500,2))</f>
         <v/>
       </c>
       <c r="I500" s="22" t="str">
@@ -15113,7 +15042,7 @@
       <c r="F501" s="13"/>
       <c r="G501" s="21"/>
       <c r="H501" s="22" t="str">
-        <f>IF(F501="","",IF(OR(E501="Abschreibung (AfA)",E501="Vorsteuer auf Anlagevermögen"),0,ROUND(F501*G501,2)))</f>
+        <f aca="false">IF(F501="","",ROUND(F501*G501,2))</f>
         <v/>
       </c>
       <c r="I501" s="22" t="str">
@@ -15131,7 +15060,7 @@
       <c r="F502" s="13"/>
       <c r="G502" s="21"/>
       <c r="H502" s="22" t="str">
-        <f>IF(F502="","",IF(OR(E502="Abschreibung (AfA)",E502="Vorsteuer auf Anlagevermögen"),0,ROUND(F502*G502,2)))</f>
+        <f aca="false">IF(F502="","",ROUND(F502*G502,2))</f>
         <v/>
       </c>
       <c r="I502" s="22" t="str">
@@ -15149,7 +15078,7 @@
       <c r="F503" s="13"/>
       <c r="G503" s="21"/>
       <c r="H503" s="22" t="str">
-        <f>IF(F503="","",IF(OR(E503="Abschreibung (AfA)",E503="Vorsteuer auf Anlagevermögen"),0,ROUND(F503*G503,2)))</f>
+        <f aca="false">IF(F503="","",ROUND(F503*G503,2))</f>
         <v/>
       </c>
       <c r="I503" s="22" t="str">
@@ -15167,7 +15096,7 @@
       <c r="F504" s="13"/>
       <c r="G504" s="21"/>
       <c r="H504" s="22" t="str">
-        <f>IF(F504="","",IF(OR(E504="Abschreibung (AfA)",E504="Vorsteuer auf Anlagevermögen"),0,ROUND(F504*G504,2)))</f>
+        <f aca="false">IF(F504="","",ROUND(F504*G504,2))</f>
         <v/>
       </c>
       <c r="I504" s="22" t="str">
@@ -15185,7 +15114,7 @@
       <c r="F505" s="13"/>
       <c r="G505" s="21"/>
       <c r="H505" s="22" t="str">
-        <f>IF(F505="","",IF(OR(E505="Abschreibung (AfA)",E505="Vorsteuer auf Anlagevermögen"),0,ROUND(F505*G505,2)))</f>
+        <f aca="false">IF(F505="","",ROUND(F505*G505,2))</f>
         <v/>
       </c>
       <c r="I505" s="22" t="str">
@@ -15203,7 +15132,7 @@
       <c r="F506" s="13"/>
       <c r="G506" s="21"/>
       <c r="H506" s="22" t="str">
-        <f>IF(F506="","",IF(OR(E506="Abschreibung (AfA)",E506="Vorsteuer auf Anlagevermögen"),0,ROUND(F506*G506,2)))</f>
+        <f aca="false">IF(F506="","",ROUND(F506*G506,2))</f>
         <v/>
       </c>
       <c r="I506" s="22" t="str">
@@ -15221,7 +15150,7 @@
       <c r="F507" s="13"/>
       <c r="G507" s="21"/>
       <c r="H507" s="22" t="str">
-        <f>IF(F507="","",IF(OR(E507="Abschreibung (AfA)",E507="Vorsteuer auf Anlagevermögen"),0,ROUND(F507*G507,2)))</f>
+        <f aca="false">IF(F507="","",ROUND(F507*G507,2))</f>
         <v/>
       </c>
       <c r="I507" s="22" t="str">
@@ -15237,7 +15166,7 @@
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" error="Bitte einen Wert aus der Liste wählen." errorStyle="stop" errorTitle="Ungültiger Eintrag" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E8:E507" type="list">
-      <formula1>'Listen'!$C$2:$C$21</formula1>
+      <formula1>Listen!$C$2:$C$20</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" error="Bitte einen Wert aus der Liste wählen." errorStyle="stop" errorTitle="Ungültiger Eintrag" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="G8:G507" type="list">
@@ -15260,7 +15189,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:D20"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15472,13 +15401,6 @@
         <v>83</v>
       </c>
       <c r="D20" s="23"/>
-    </row>
-    <row r="21">
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>Vorsteuer auf Anlagevermögen</t>
-        </is>
-      </c>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>